<commit_message>
Até 4 etiquetas por bloco e painéis do totem com cor e etiqueta próprias
- Pirâmide e mesas mostram até 4 etiquetas; a linha de cada bloco da gôndola e
  de cada frente das mesas também (ETIQUETAS_POR_BLOCO). Blocos vizinhos só se
  juntam quando todas as etiquetas são iguais.
- Totem: espaços PAINEL-1 a 3 (o 1 é o de cima), cada um com cor e Etiqueta 1;
  a etiqueta fica ao lado do totem, com linha-guia até o painel.
- Planilha base e instruções atualizadas; ciclo de exemplo mostra o totem com
  3 cores e um bloco de gôndola com 2 etiquetas (VERSAO_EXEMPLO 5).
- Versão de visualização e index.html gerados de novo.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019BmnBNRucVHCBVjZaoSiJv
</commit_message>
<xml_diff>
--- a/visualizador/Planilha base - Visualizador.xlsx
+++ b/visualizador/Planilha base - Visualizador.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="777" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="802" uniqueCount="297">
   <si>
     <t>Ciclo</t>
   </si>
@@ -120,6 +120,9 @@
     <t>LIQUIDA QDB</t>
   </si>
   <si>
+    <t>JUICY MOOD</t>
+  </si>
+  <si>
     <t>GONDOLA 1/MEIO-A</t>
   </si>
   <si>
@@ -213,9 +216,6 @@
     <t>BOT+QDB</t>
   </si>
   <si>
-    <t>JUICY MOOD</t>
-  </si>
-  <si>
     <t>MOVEL DE FILA 2</t>
   </si>
   <si>
@@ -240,7 +240,25 @@
     <t>Totem 1 · vale para ER P, ER M, ER G, ER GG</t>
   </si>
   <si>
+    <t>TOTEM 1/PAINEL-1</t>
+  </si>
+  <si>
+    <t>Totem 1 – Painel 1</t>
+  </si>
+  <si>
     <t>LÇTO UOMINI</t>
+  </si>
+  <si>
+    <t>TOTEM 1/PAINEL-2</t>
+  </si>
+  <si>
+    <t>Totem 1 – Painel 2</t>
+  </si>
+  <si>
+    <t>TOTEM 1/PAINEL-3</t>
+  </si>
+  <si>
+    <t>Totem 1 – Painel 3</t>
   </si>
   <si>
     <t>EXTRA-CESTINHAS</t>
@@ -765,7 +783,7 @@
     <t>Planilha base — Plano de Varejo</t>
   </si>
   <si>
-    <t>Gerada em 06/10/2026, 08:23:36 a partir do ciclo "Ciclo exemplo".</t>
+    <t>Gerada em 06/10/2026, 09:17:13 a partir do ciclo "Ciclo exemplo".</t>
   </si>
   <si>
     <t>Como preencher</t>
@@ -780,7 +798,7 @@
     <t>3. "Marca do Móvel" define a cor do móvel na planta. Deixe vazio (ou NEUTRO) para o móvel aparecer branco.</t>
   </si>
   <si>
-    <t>4. "Etiqueta 1…4" são as caixas de texto do móvel; "Marca Etiqueta N" define a cor de cada uma (vazio = cor do móvel). Pirâmide e mesa destaque mostram só 1 etiqueta (as colunas que não aparecem na planta ficam cinza).</t>
+    <t>4. "Etiqueta 1…4" são as caixas de texto do móvel; "Marca Etiqueta N" define a cor de cada uma (vazio = cor do móvel). Pirâmide e mesa destaque mostram até 4 etiquetas, empilhadas (as colunas que não aparecem na planta ficam cinza).</t>
   </si>
   <si>
     <t>5. "Símbolo" é opcional e aparece ao lado da primeira etiqueta (tabela abaixo).</t>
@@ -792,10 +810,10 @@
     <t>6.1 Gôndolas têm uma linha para a gôndola inteira e uma por espaço (ex.: GONDOLA 1/LADO-A, GONDOLA 1/MEIO-A). Espaço preenchido tem prioridade; espaço vazio usa a linha da gôndola inteira (para deixar um espaço branco, use NEUTRO). Para dividir um meio em dois movimentos, preencha também a linha da metade 2 (ex.: GONDOLA 1/MEIO-A-2): a linha do meio passa a valer para a metade 1 e a planta mostra o meio dividido.</t>
   </si>
   <si>
-    <t>6.2 A gôndola mostra uma etiqueta por bloco. Na linha da gôndola inteira: Etiqueta 1 = Lado A, Etiqueta 2 = Meio A, Etiqueta 3 = Meio B, Etiqueta 4 = Lado B ("A" é sempre o lado virado para quem olha a planta). A Etiqueta 1 da linha de um espaço substitui a etiqueta daquele bloco.</t>
-  </si>
-  <si>
-    <t>6.3 Mesa destaque (FRENTE-1 e 2), mesa 3 frentes (FRENTE-1 a 3) e móvel make (TESTEIRA-1 a 4) têm uma linha por bloco, com cor e etiqueta próprias. Blocos vizinhos com o mesmo texto e cor ficam com uma etiqueta só, no centro. O balcão recepção tem uma cor só; Etiqueta 1, 2 e 3 vão para o bloco 1, o canto e o bloco 3.</t>
+    <t>6.2 Etiquetas da gôndola. Na linha da gôndola inteira: Etiqueta 1 = Lado A, Etiqueta 2 = Meio A, Etiqueta 3 = Meio B, Etiqueta 4 = Lado B ("A" é sempre o lado virado para quem olha a planta). A linha de um espaço mostra até 4 etiquetas empilhadas em cima daquele bloco (Etiqueta 1 a 4) e substitui a etiqueta que viria da gôndola inteira.</t>
+  </si>
+  <si>
+    <t>6.3 Mesa destaque (FRENTE-1 e 2), mesa 3 frentes (FRENTE-1 a 3), totem (PAINEL-1 a 3, o 1 é o painel de cima) e móvel make (TESTEIRA-1 a 4) têm uma linha por bloco, com cor e etiqueta próprias. Cada frente das mesas mostra até 4 etiquetas; cada painel do totem e cada testeira, 1. Bloco sem linha própria usa a cor do móvel inteiro. Blocos vizinhos com as mesmas etiquetas e cor ficam com uma pilha só, no centro. O balcão recepção tem uma cor só; Etiqueta 1, 2 e 3 vão para o bloco 1, o canto e o bloco 3.</t>
   </si>
   <si>
     <t>7. Na coluna "Planta" vale o nome (ex.: ER P) ou o número (01). Cascata: o que é definido numa planta vale também para as seguintes (ER P → ER M → ER G → ER GG), por isso cada móvel aparece uma vez só, na primeira planta que o tem ("vale para…" na coluna Móvel). Para mudar um móvel só a partir de uma planta, acrescente uma linha com o mesmo ID Móvel e essa planta. Planta = TODAS vale para todas.</t>
@@ -1762,7 +1780,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O382"/>
+  <dimension ref="A1:O385"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="13" style="1" customWidth="1"/>
@@ -1928,12 +1946,14 @@
       <c r="G4" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="H4" s="5"/>
-      <c r="I4" s="5"/>
-      <c r="J4" s="5"/>
-      <c r="K4" s="5"/>
-      <c r="L4" s="5"/>
-      <c r="M4" s="5"/>
+      <c r="H4" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="K4" s="1"/>
+      <c r="M4" s="1"/>
       <c r="N4" s="1" t="s">
         <v>24</v>
       </c>
@@ -1949,19 +1969,16 @@
         <v>16</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E5" s="1"/>
       <c r="G5" s="1"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
-      <c r="J5" s="5"/>
-      <c r="K5" s="5"/>
-      <c r="L5" s="5"/>
-      <c r="M5" s="5"/>
+      <c r="I5" s="1"/>
+      <c r="K5" s="1"/>
+      <c r="M5" s="1"/>
       <c r="N5" s="1"/>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
@@ -1972,19 +1989,16 @@
         <v>16</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E6" s="1"/>
       <c r="G6" s="1"/>
-      <c r="H6" s="5"/>
-      <c r="I6" s="5"/>
-      <c r="J6" s="5"/>
-      <c r="K6" s="5"/>
-      <c r="L6" s="5"/>
-      <c r="M6" s="5"/>
+      <c r="I6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="M6" s="1"/>
       <c r="N6" s="1"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
@@ -1995,19 +2009,16 @@
         <v>16</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E7" s="1"/>
       <c r="G7" s="1"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="5"/>
-      <c r="J7" s="5"/>
-      <c r="K7" s="5"/>
-      <c r="L7" s="5"/>
-      <c r="M7" s="5"/>
+      <c r="I7" s="1"/>
+      <c r="K7" s="1"/>
+      <c r="M7" s="1"/>
       <c r="N7" s="1"/>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
@@ -2018,19 +2029,16 @@
         <v>16</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E8" s="1"/>
       <c r="G8" s="1"/>
-      <c r="H8" s="5"/>
-      <c r="I8" s="5"/>
-      <c r="J8" s="5"/>
-      <c r="K8" s="5"/>
-      <c r="L8" s="5"/>
-      <c r="M8" s="5"/>
+      <c r="I8" s="1"/>
+      <c r="K8" s="1"/>
+      <c r="M8" s="1"/>
       <c r="N8" s="1"/>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
@@ -2041,19 +2049,16 @@
         <v>16</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E9" s="1"/>
       <c r="G9" s="1"/>
-      <c r="H9" s="5"/>
-      <c r="I9" s="5"/>
-      <c r="J9" s="5"/>
-      <c r="K9" s="5"/>
-      <c r="L9" s="5"/>
-      <c r="M9" s="5"/>
+      <c r="I9" s="1"/>
+      <c r="K9" s="1"/>
+      <c r="M9" s="1"/>
       <c r="N9" s="1"/>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
@@ -2064,13 +2069,13 @@
         <v>16</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>22</v>
@@ -2078,12 +2083,9 @@
       <c r="G10" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="H10" s="5"/>
-      <c r="I10" s="5"/>
-      <c r="J10" s="5"/>
-      <c r="K10" s="5"/>
-      <c r="L10" s="5"/>
-      <c r="M10" s="5"/>
+      <c r="I10" s="1"/>
+      <c r="K10" s="1"/>
+      <c r="M10" s="1"/>
       <c r="N10" s="1" t="s">
         <v>24</v>
       </c>
@@ -2099,26 +2101,23 @@
         <v>16</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>21</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G11" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5"/>
-      <c r="J11" s="5"/>
-      <c r="K11" s="5"/>
-      <c r="L11" s="5"/>
-      <c r="M11" s="5"/>
+      <c r="I11" s="1"/>
+      <c r="K11" s="1"/>
+      <c r="M11" s="1"/>
       <c r="N11" s="1" t="s">
         <v>24</v>
       </c>
@@ -2134,21 +2133,18 @@
         <v>16</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>23</v>
       </c>
       <c r="G12" s="1"/>
-      <c r="H12" s="5"/>
-      <c r="I12" s="5"/>
-      <c r="J12" s="5"/>
-      <c r="K12" s="5"/>
-      <c r="L12" s="5"/>
-      <c r="M12" s="5"/>
+      <c r="I12" s="1"/>
+      <c r="K12" s="1"/>
+      <c r="M12" s="1"/>
       <c r="N12" s="1" t="s">
         <v>24</v>
       </c>
@@ -2164,26 +2160,23 @@
         <v>16</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>21</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G13" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H13" s="5"/>
-      <c r="I13" s="5"/>
-      <c r="J13" s="5"/>
-      <c r="K13" s="5"/>
-      <c r="L13" s="5"/>
-      <c r="M13" s="5"/>
+      <c r="I13" s="1"/>
+      <c r="K13" s="1"/>
+      <c r="M13" s="1"/>
       <c r="N13" s="1" t="s">
         <v>24</v>
       </c>
@@ -2199,26 +2192,23 @@
         <v>16</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="H14" s="5"/>
-      <c r="I14" s="5"/>
-      <c r="J14" s="5"/>
-      <c r="K14" s="5"/>
-      <c r="L14" s="5"/>
-      <c r="M14" s="5"/>
+        <v>48</v>
+      </c>
+      <c r="I14" s="1"/>
+      <c r="K14" s="1"/>
+      <c r="M14" s="1"/>
       <c r="N14" s="1" t="s">
         <v>24</v>
       </c>
@@ -2234,19 +2224,19 @@
         <v>16</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I15" s="1"/>
       <c r="K15" s="1"/>
@@ -2266,31 +2256,31 @@
         <v>16</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>21</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>66</v>
+        <v>35</v>
       </c>
       <c r="I16" s="1" t="s">
         <v>33</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="L16" s="5"/>
       <c r="M16" s="5"/>
@@ -2347,13 +2337,13 @@
         <v>71</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>72</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I18" s="1"/>
       <c r="K18" s="1"/>
@@ -2381,18 +2371,8 @@
       <c r="E19" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="F19" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="G19" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="H19" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="I19" s="1" t="s">
-        <v>21</v>
-      </c>
+      <c r="G19" s="1"/>
+      <c r="I19" s="1"/>
       <c r="K19" s="1"/>
       <c r="M19" s="1"/>
       <c r="N19" s="1" t="s">
@@ -2410,23 +2390,26 @@
         <v>16</v>
       </c>
       <c r="C20" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="D20" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="E20" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F20" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="E20" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>64</v>
-      </c>
       <c r="G20" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="I20" s="1"/>
-      <c r="K20" s="1"/>
-      <c r="M20" s="1"/>
+        <v>21</v>
+      </c>
+      <c r="H20" s="5"/>
+      <c r="I20" s="5"/>
+      <c r="J20" s="5"/>
+      <c r="K20" s="5"/>
+      <c r="L20" s="5"/>
+      <c r="M20" s="5"/>
       <c r="N20" s="1" t="s">
         <v>24</v>
       </c>
@@ -2448,22 +2431,20 @@
         <v>79</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="G21" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H21" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="I21" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="K21" s="1"/>
-      <c r="M21" s="1"/>
+      <c r="H21" s="5"/>
+      <c r="I21" s="5"/>
+      <c r="J21" s="5"/>
+      <c r="K21" s="5"/>
+      <c r="L21" s="5"/>
+      <c r="M21" s="5"/>
       <c r="N21" s="1" t="s">
         <v>24</v>
       </c>
@@ -2479,23 +2460,26 @@
         <v>16</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>61</v>
+        <v>34</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="I22" s="1"/>
-      <c r="K22" s="1"/>
-      <c r="M22" s="1"/>
+        <v>33</v>
+      </c>
+      <c r="H22" s="5"/>
+      <c r="I22" s="5"/>
+      <c r="J22" s="5"/>
+      <c r="K22" s="5"/>
+      <c r="L22" s="5"/>
+      <c r="M22" s="5"/>
       <c r="N22" s="1" t="s">
         <v>24</v>
       </c>
@@ -2511,19 +2495,19 @@
         <v>16</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>19</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>86</v>
+        <v>65</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>23</v>
+        <v>66</v>
       </c>
       <c r="I23" s="1"/>
       <c r="K23" s="1"/>
@@ -2543,21 +2527,28 @@
         <v>16</v>
       </c>
       <c r="C24" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H24" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="D24" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="G24" s="1"/>
-      <c r="H24" s="5"/>
-      <c r="I24" s="5"/>
-      <c r="J24" s="5"/>
-      <c r="K24" s="5"/>
-      <c r="L24" s="5"/>
-      <c r="M24" s="5"/>
+      <c r="I24" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="K24" s="1"/>
+      <c r="M24" s="1"/>
       <c r="N24" s="1" t="s">
         <v>24</v>
       </c>
@@ -2573,26 +2564,23 @@
         <v>16</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>80</v>
+        <v>62</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="H25" s="5"/>
-      <c r="I25" s="5"/>
-      <c r="J25" s="5"/>
-      <c r="K25" s="5"/>
-      <c r="L25" s="5"/>
-      <c r="M25" s="5"/>
+        <v>48</v>
+      </c>
+      <c r="I25" s="1"/>
+      <c r="K25" s="1"/>
+      <c r="M25" s="1"/>
       <c r="N25" s="1" t="s">
         <v>24</v>
       </c>
@@ -2608,26 +2596,23 @@
         <v>16</v>
       </c>
       <c r="C26" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F26" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D26" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>80</v>
-      </c>
       <c r="G26" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="H26" s="5"/>
-      <c r="I26" s="5"/>
-      <c r="J26" s="5"/>
-      <c r="K26" s="5"/>
-      <c r="L26" s="5"/>
-      <c r="M26" s="5"/>
+        <v>23</v>
+      </c>
+      <c r="I26" s="1"/>
+      <c r="K26" s="1"/>
+      <c r="M26" s="1"/>
       <c r="N26" s="1" t="s">
         <v>24</v>
       </c>
@@ -2643,13 +2628,13 @@
         <v>16</v>
       </c>
       <c r="C27" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="D27" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="D27" s="4" t="s">
+      <c r="E27" s="1" t="s">
         <v>95</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>47</v>
       </c>
       <c r="G27" s="1"/>
       <c r="H27" s="5"/>
@@ -2679,22 +2664,20 @@
         <v>97</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="G28" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H28" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="I28" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="K28" s="1"/>
-      <c r="M28" s="1"/>
+      <c r="H28" s="5"/>
+      <c r="I28" s="5"/>
+      <c r="J28" s="5"/>
+      <c r="K28" s="5"/>
+      <c r="L28" s="5"/>
+      <c r="M28" s="5"/>
       <c r="N28" s="1" t="s">
         <v>24</v>
       </c>
@@ -2710,28 +2693,26 @@
         <v>16</v>
       </c>
       <c r="C29" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="D29" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="D29" s="4" t="s">
-        <v>100</v>
-      </c>
       <c r="E29" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>101</v>
+        <v>86</v>
       </c>
       <c r="G29" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H29" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="I29" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="K29" s="1"/>
-      <c r="M29" s="1"/>
+      <c r="H29" s="5"/>
+      <c r="I29" s="5"/>
+      <c r="J29" s="5"/>
+      <c r="K29" s="5"/>
+      <c r="L29" s="5"/>
+      <c r="M29" s="5"/>
       <c r="N29" s="1" t="s">
         <v>24</v>
       </c>
@@ -2747,176 +2728,187 @@
         <v>16</v>
       </c>
       <c r="C30" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G30" s="1"/>
+      <c r="H30" s="5"/>
+      <c r="I30" s="5"/>
+      <c r="J30" s="5"/>
+      <c r="K30" s="5"/>
+      <c r="L30" s="5"/>
+      <c r="M30" s="5"/>
+      <c r="N30" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O30" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C31" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="D30" s="4" t="s">
+      <c r="D31" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="E30" s="1" t="s">
+      <c r="E31" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="F30" s="1" t="s">
+      <c r="F31" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="G30" s="1" t="s">
+      <c r="G31" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H30" s="1" t="s">
+      <c r="H31" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="I30" s="1" t="s">
+      <c r="I31" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="K30" s="1"/>
-      <c r="M30" s="1"/>
-      <c r="N30" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="O30" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A31" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B31" s="6" t="s">
+      <c r="K31" s="1"/>
+      <c r="M31" s="1"/>
+      <c r="N31" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O31" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A32" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C32" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="C31" s="6" t="s">
+      <c r="D32" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="D31" s="7" t="s">
+      <c r="E32" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F32" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="E31" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="G31" s="1"/>
-      <c r="H31" s="1" t="s">
+      <c r="G32" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I32" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="K32" s="1"/>
+      <c r="M32" s="1"/>
+      <c r="N32" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O32" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A33" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C33" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="I31" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="J31" s="1" t="s">
+      <c r="D33" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="K31" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="L31" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="M31" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="N31" s="1" t="s">
+      <c r="E33" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F33" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="O31" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A32" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B32" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="C32" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="D32" s="7" t="s">
-        <v>112</v>
-      </c>
-      <c r="E32" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="F32" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="G32" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="H32" s="5"/>
-      <c r="I32" s="5"/>
-      <c r="J32" s="5"/>
-      <c r="K32" s="5"/>
-      <c r="L32" s="5"/>
-      <c r="M32" s="5"/>
-      <c r="N32" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="O32" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A33" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B33" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="C33" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="D33" s="7" t="s">
-        <v>114</v>
-      </c>
-      <c r="E33" s="1"/>
-      <c r="G33" s="1"/>
-      <c r="H33" s="5"/>
-      <c r="I33" s="5"/>
-      <c r="J33" s="5"/>
-      <c r="K33" s="5"/>
-      <c r="L33" s="5"/>
-      <c r="M33" s="5"/>
-      <c r="N33" s="1"/>
+      <c r="G33" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H33" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I33" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="K33" s="1"/>
+      <c r="M33" s="1"/>
+      <c r="N33" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O33" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="C34" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="D34" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G34" s="1"/>
+      <c r="H34" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="I34" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="J34" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="D34" s="7" t="s">
+      <c r="K34" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="L34" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="M34" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="N34" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="E34" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F34" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="G34" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="H34" s="5"/>
-      <c r="I34" s="5"/>
-      <c r="J34" s="5"/>
-      <c r="K34" s="5"/>
-      <c r="L34" s="5"/>
-      <c r="M34" s="5"/>
-      <c r="N34" s="1" t="s">
-        <v>110</v>
-      </c>
       <c r="O34" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="C35" s="6" t="s">
         <v>117</v>
@@ -2924,22 +2916,31 @@
       <c r="D35" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="E35" s="1"/>
-      <c r="G35" s="1"/>
-      <c r="H35" s="5"/>
-      <c r="I35" s="5"/>
-      <c r="J35" s="5"/>
-      <c r="K35" s="5"/>
-      <c r="L35" s="5"/>
-      <c r="M35" s="5"/>
-      <c r="N35" s="1"/>
+      <c r="E35" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I35" s="1"/>
+      <c r="K35" s="1"/>
+      <c r="M35" s="1"/>
+      <c r="N35" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O35" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="C36" s="6" t="s">
         <v>119</v>
@@ -2949,20 +2950,17 @@
       </c>
       <c r="E36" s="1"/>
       <c r="G36" s="1"/>
-      <c r="H36" s="5"/>
-      <c r="I36" s="5"/>
-      <c r="J36" s="5"/>
-      <c r="K36" s="5"/>
-      <c r="L36" s="5"/>
-      <c r="M36" s="5"/>
+      <c r="I36" s="1"/>
+      <c r="K36" s="1"/>
+      <c r="M36" s="1"/>
       <c r="N36" s="1"/>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="C37" s="6" t="s">
         <v>121</v>
@@ -2970,22 +2968,31 @@
       <c r="D37" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="E37" s="1"/>
-      <c r="G37" s="1"/>
-      <c r="H37" s="5"/>
-      <c r="I37" s="5"/>
-      <c r="J37" s="5"/>
-      <c r="K37" s="5"/>
-      <c r="L37" s="5"/>
-      <c r="M37" s="5"/>
-      <c r="N37" s="1"/>
-    </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="E37" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="I37" s="1"/>
+      <c r="K37" s="1"/>
+      <c r="M37" s="1"/>
+      <c r="N37" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="O37" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A38" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="C38" s="6" t="s">
         <v>123</v>
@@ -2993,31 +3000,19 @@
       <c r="D38" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="E38" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F38" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="G38" s="1" t="s">
-        <v>21</v>
-      </c>
+      <c r="E38" s="1"/>
+      <c r="G38" s="1"/>
       <c r="I38" s="1"/>
       <c r="K38" s="1"/>
       <c r="M38" s="1"/>
-      <c r="N38" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="O38" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N38" s="1"/>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A39" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="C39" s="6" t="s">
         <v>125</v>
@@ -3025,31 +3020,19 @@
       <c r="D39" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="E39" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="F39" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="G39" s="1" t="s">
-        <v>33</v>
-      </c>
+      <c r="E39" s="1"/>
+      <c r="G39" s="1"/>
       <c r="I39" s="1"/>
       <c r="K39" s="1"/>
       <c r="M39" s="1"/>
-      <c r="N39" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="O39" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N39" s="1"/>
+    </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A40" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="C40" s="6" t="s">
         <v>127</v>
@@ -3057,52 +3040,40 @@
       <c r="D40" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="E40" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="F40" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="G40" s="1" t="s">
-        <v>129</v>
-      </c>
+      <c r="E40" s="1"/>
+      <c r="G40" s="1"/>
       <c r="I40" s="1"/>
       <c r="K40" s="1"/>
       <c r="M40" s="1"/>
-      <c r="N40" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="O40" s="1" t="s">
-        <v>24</v>
-      </c>
+      <c r="N40" s="1"/>
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="D41" s="7" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>129</v>
+        <v>21</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>134</v>
+        <v>69</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>129</v>
+        <v>21</v>
       </c>
       <c r="I41" s="1"/>
       <c r="K41" s="1"/>
       <c r="M41" s="1"/>
       <c r="N41" s="1" t="s">
-        <v>131</v>
+        <v>24</v>
       </c>
       <c r="O41" s="1" t="s">
         <v>24</v>
@@ -3113,185 +3084,209 @@
         <v>15</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="C42" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="D42" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G42" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I42" s="1"/>
+      <c r="K42" s="1"/>
+      <c r="M42" s="1"/>
+      <c r="N42" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O42" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A43" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B43" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="C43" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="D43" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="E43" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="D42" s="7" t="s">
+      <c r="F43" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="E42" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="F42" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="G42" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="H42" s="5"/>
-      <c r="I42" s="5"/>
-      <c r="J42" s="5"/>
-      <c r="K42" s="5"/>
-      <c r="L42" s="5"/>
-      <c r="M42" s="5"/>
-      <c r="N42" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="O42" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A43" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B43" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="C43" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="D43" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="E43" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F43" s="1" t="s">
-        <v>69</v>
-      </c>
       <c r="G43" s="1" t="s">
-        <v>21</v>
+        <v>135</v>
       </c>
       <c r="I43" s="1"/>
       <c r="K43" s="1"/>
       <c r="M43" s="1"/>
       <c r="N43" s="1" t="s">
-        <v>24</v>
+        <v>137</v>
       </c>
       <c r="O43" s="1" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="44" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A44" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B44" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="C44" s="3" t="s">
+      <c r="A44" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B44" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="C44" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="D44" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="F44" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="D44" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="E44" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F44" s="1" t="s">
-        <v>22</v>
-      </c>
       <c r="G44" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="H44" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="I44" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="J44" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="K44" s="1" t="s">
-        <v>23</v>
-      </c>
+        <v>135</v>
+      </c>
+      <c r="I44" s="1"/>
+      <c r="K44" s="1"/>
       <c r="M44" s="1"/>
       <c r="N44" s="1" t="s">
-        <v>110</v>
+        <v>137</v>
       </c>
       <c r="O44" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A45" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B45" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="C45" s="3" t="s">
+    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A45" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B45" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="C45" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="D45" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G45" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I45" s="1"/>
+      <c r="K45" s="1"/>
+      <c r="M45" s="1"/>
+      <c r="N45" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O45" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A46" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="C46" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="D45" s="4" t="s">
+      <c r="D46" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="E45" s="1"/>
-      <c r="G45" s="1"/>
-      <c r="H45" s="5"/>
-      <c r="I45" s="5"/>
-      <c r="J45" s="5"/>
-      <c r="K45" s="5"/>
-      <c r="L45" s="5"/>
-      <c r="M45" s="5"/>
-      <c r="N45" s="1"/>
-    </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A46" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B46" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="C46" s="3" t="s">
+      <c r="E46" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="G46" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="I46" s="1"/>
+      <c r="K46" s="1"/>
+      <c r="M46" s="1"/>
+      <c r="N46" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O46" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="47" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A47" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="C47" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="D46" s="4" t="s">
+      <c r="D47" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="E46" s="1"/>
-      <c r="G46" s="1"/>
-      <c r="H46" s="5"/>
-      <c r="I46" s="5"/>
-      <c r="J46" s="5"/>
-      <c r="K46" s="5"/>
-      <c r="L46" s="5"/>
-      <c r="M46" s="5"/>
-      <c r="N46" s="1"/>
-    </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A47" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B47" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="C47" s="3" t="s">
+      <c r="E47" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F47" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G47" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H47" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="D47" s="4" t="s">
+      <c r="I47" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="J47" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="E47" s="1"/>
-      <c r="G47" s="1"/>
-      <c r="H47" s="5"/>
-      <c r="I47" s="5"/>
-      <c r="J47" s="5"/>
-      <c r="K47" s="5"/>
-      <c r="L47" s="5"/>
-      <c r="M47" s="5"/>
-      <c r="N47" s="1"/>
+      <c r="K47" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="M47" s="1"/>
+      <c r="N47" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="O47" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="C48" s="3" t="s">
         <v>150</v>
@@ -3301,12 +3296,9 @@
       </c>
       <c r="E48" s="1"/>
       <c r="G48" s="1"/>
-      <c r="H48" s="5"/>
-      <c r="I48" s="5"/>
-      <c r="J48" s="5"/>
-      <c r="K48" s="5"/>
-      <c r="L48" s="5"/>
-      <c r="M48" s="5"/>
+      <c r="I48" s="1"/>
+      <c r="K48" s="1"/>
+      <c r="M48" s="1"/>
       <c r="N48" s="1"/>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.25">
@@ -3314,7 +3306,7 @@
         <v>15</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="C49" s="3" t="s">
         <v>152</v>
@@ -3324,12 +3316,9 @@
       </c>
       <c r="E49" s="1"/>
       <c r="G49" s="1"/>
-      <c r="H49" s="5"/>
-      <c r="I49" s="5"/>
-      <c r="J49" s="5"/>
-      <c r="K49" s="5"/>
-      <c r="L49" s="5"/>
-      <c r="M49" s="5"/>
+      <c r="I49" s="1"/>
+      <c r="K49" s="1"/>
+      <c r="M49" s="1"/>
       <c r="N49" s="1"/>
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.25">
@@ -3337,7 +3326,7 @@
         <v>15</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="C50" s="3" t="s">
         <v>154</v>
@@ -3347,12 +3336,9 @@
       </c>
       <c r="E50" s="1"/>
       <c r="G50" s="1"/>
-      <c r="H50" s="5"/>
-      <c r="I50" s="5"/>
-      <c r="J50" s="5"/>
-      <c r="K50" s="5"/>
-      <c r="L50" s="5"/>
-      <c r="M50" s="5"/>
+      <c r="I50" s="1"/>
+      <c r="K50" s="1"/>
+      <c r="M50" s="1"/>
       <c r="N50" s="1"/>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.25">
@@ -3360,7 +3346,7 @@
         <v>15</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="C51" s="3" t="s">
         <v>156</v>
@@ -3380,7 +3366,7 @@
         <v>15</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="C52" s="3" t="s">
         <v>158</v>
@@ -3395,12 +3381,12 @@
       <c r="M52" s="1"/>
       <c r="N52" s="1"/>
     </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="C53" s="3" t="s">
         <v>160</v>
@@ -3408,31 +3394,19 @@
       <c r="D53" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="E53" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="F53" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="G53" s="1" t="s">
-        <v>33</v>
-      </c>
+      <c r="E53" s="1"/>
+      <c r="G53" s="1"/>
       <c r="I53" s="1"/>
       <c r="K53" s="1"/>
       <c r="M53" s="1"/>
-      <c r="N53" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="O53" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N53" s="1"/>
+    </row>
+    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="C54" s="3" t="s">
         <v>162</v>
@@ -3440,26 +3414,19 @@
       <c r="D54" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="E54" s="1" t="s">
-        <v>23</v>
-      </c>
+      <c r="E54" s="1"/>
       <c r="G54" s="1"/>
       <c r="I54" s="1"/>
       <c r="K54" s="1"/>
       <c r="M54" s="1"/>
-      <c r="N54" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="O54" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N54" s="1"/>
+    </row>
+    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="C55" s="3" t="s">
         <v>164</v>
@@ -3467,34 +3434,19 @@
       <c r="D55" s="4" t="s">
         <v>165</v>
       </c>
-      <c r="E55" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F55" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="G55" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="H55" s="5"/>
-      <c r="I55" s="5"/>
-      <c r="J55" s="5"/>
-      <c r="K55" s="5"/>
-      <c r="L55" s="5"/>
-      <c r="M55" s="5"/>
-      <c r="N55" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="O55" s="1" t="s">
-        <v>24</v>
-      </c>
+      <c r="E55" s="1"/>
+      <c r="G55" s="1"/>
+      <c r="I55" s="1"/>
+      <c r="K55" s="1"/>
+      <c r="M55" s="1"/>
+      <c r="N55" s="1"/>
     </row>
     <row r="56" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="C56" s="3" t="s">
         <v>166</v>
@@ -3503,20 +3455,17 @@
         <v>167</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>168</v>
+        <v>34</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="H56" s="5"/>
-      <c r="I56" s="5"/>
-      <c r="J56" s="5"/>
-      <c r="K56" s="5"/>
-      <c r="L56" s="5"/>
-      <c r="M56" s="5"/>
+        <v>33</v>
+      </c>
+      <c r="I56" s="1"/>
+      <c r="K56" s="1"/>
+      <c r="M56" s="1"/>
       <c r="N56" s="1" t="s">
         <v>24</v>
       </c>
@@ -3529,143 +3478,162 @@
         <v>15</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="C57" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="D57" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="D57" s="4" t="s">
+      <c r="E57" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G57" s="1"/>
+      <c r="I57" s="1"/>
+      <c r="K57" s="1"/>
+      <c r="M57" s="1"/>
+      <c r="N57" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O57" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="58" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A58" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B58" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="C58" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="E57" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="F57" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="G57" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="H57" s="5"/>
-      <c r="I57" s="5"/>
-      <c r="J57" s="5"/>
-      <c r="K57" s="5"/>
-      <c r="L57" s="5"/>
-      <c r="M57" s="5"/>
-      <c r="N57" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="O57" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A58" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B58" s="6" t="s">
+      <c r="D58" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="C58" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="D58" s="7" t="s">
-        <v>173</v>
-      </c>
       <c r="E58" s="1" t="s">
-        <v>129</v>
+        <v>21</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>174</v>
+        <v>56</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>129</v>
+        <v>21</v>
       </c>
       <c r="I58" s="1"/>
       <c r="K58" s="1"/>
       <c r="M58" s="1"/>
       <c r="N58" s="1" t="s">
-        <v>110</v>
+        <v>24</v>
       </c>
       <c r="O58" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A59" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B59" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="C59" s="6" t="s">
+    <row r="59" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A59" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="C59" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="D59" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="E59" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F59" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="G59" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I59" s="1"/>
+      <c r="K59" s="1"/>
+      <c r="M59" s="1"/>
+      <c r="N59" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O59" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="60" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A60" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="C60" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="D59" s="7" t="s">
+      <c r="D60" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="E59" s="1"/>
-      <c r="G59" s="1"/>
-      <c r="H59" s="5"/>
-      <c r="I59" s="5"/>
-      <c r="J59" s="5"/>
-      <c r="K59" s="5"/>
-      <c r="L59" s="5"/>
-      <c r="M59" s="5"/>
-      <c r="N59" s="1"/>
-    </row>
-    <row r="60" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A60" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B60" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="C60" s="6" t="s">
+      <c r="E60" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F60" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="G60" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="I60" s="1"/>
+      <c r="K60" s="1"/>
+      <c r="M60" s="1"/>
+      <c r="N60" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O60" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="61" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A61" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B61" s="6" t="s">
         <v>177</v>
       </c>
-      <c r="D60" s="7" t="s">
+      <c r="C61" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="E60" s="1"/>
-      <c r="G60" s="1"/>
-      <c r="H60" s="5"/>
-      <c r="I60" s="5"/>
-      <c r="J60" s="5"/>
-      <c r="K60" s="5"/>
-      <c r="L60" s="5"/>
-      <c r="M60" s="5"/>
-      <c r="N60" s="1"/>
-    </row>
-    <row r="61" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A61" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B61" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="C61" s="6" t="s">
+      <c r="D61" s="7" t="s">
         <v>179</v>
       </c>
-      <c r="D61" s="7" t="s">
+      <c r="E61" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="F61" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="E61" s="1"/>
-      <c r="G61" s="1"/>
-      <c r="H61" s="5"/>
-      <c r="I61" s="5"/>
-      <c r="J61" s="5"/>
-      <c r="K61" s="5"/>
-      <c r="L61" s="5"/>
-      <c r="M61" s="5"/>
-      <c r="N61" s="1"/>
+      <c r="G61" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="I61" s="1"/>
+      <c r="K61" s="1"/>
+      <c r="M61" s="1"/>
+      <c r="N61" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="O61" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A62" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B62" s="6" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="C62" s="6" t="s">
         <v>181</v>
@@ -3675,12 +3643,9 @@
       </c>
       <c r="E62" s="1"/>
       <c r="G62" s="1"/>
-      <c r="H62" s="5"/>
-      <c r="I62" s="5"/>
-      <c r="J62" s="5"/>
-      <c r="K62" s="5"/>
-      <c r="L62" s="5"/>
-      <c r="M62" s="5"/>
+      <c r="I62" s="1"/>
+      <c r="K62" s="1"/>
+      <c r="M62" s="1"/>
       <c r="N62" s="1"/>
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.25">
@@ -3688,7 +3653,7 @@
         <v>15</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="C63" s="6" t="s">
         <v>183</v>
@@ -3698,12 +3663,9 @@
       </c>
       <c r="E63" s="1"/>
       <c r="G63" s="1"/>
-      <c r="H63" s="5"/>
-      <c r="I63" s="5"/>
-      <c r="J63" s="5"/>
-      <c r="K63" s="5"/>
-      <c r="L63" s="5"/>
-      <c r="M63" s="5"/>
+      <c r="I63" s="1"/>
+      <c r="K63" s="1"/>
+      <c r="M63" s="1"/>
       <c r="N63" s="1"/>
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.25">
@@ -3711,7 +3673,7 @@
         <v>15</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="C64" s="6" t="s">
         <v>185</v>
@@ -3721,20 +3683,17 @@
       </c>
       <c r="E64" s="1"/>
       <c r="G64" s="1"/>
-      <c r="H64" s="5"/>
-      <c r="I64" s="5"/>
-      <c r="J64" s="5"/>
-      <c r="K64" s="5"/>
-      <c r="L64" s="5"/>
-      <c r="M64" s="5"/>
+      <c r="I64" s="1"/>
+      <c r="K64" s="1"/>
+      <c r="M64" s="1"/>
       <c r="N64" s="1"/>
     </row>
-    <row r="65" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A65" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="C65" s="6" t="s">
         <v>187</v>
@@ -3742,31 +3701,19 @@
       <c r="D65" s="7" t="s">
         <v>188</v>
       </c>
-      <c r="E65" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="F65" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="G65" s="1" t="s">
-        <v>33</v>
-      </c>
+      <c r="E65" s="1"/>
+      <c r="G65" s="1"/>
       <c r="I65" s="1"/>
       <c r="K65" s="1"/>
       <c r="M65" s="1"/>
-      <c r="N65" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="O65" s="1" t="s">
-        <v>24</v>
-      </c>
+      <c r="N65" s="1"/>
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A66" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="C66" s="6" t="s">
         <v>189</v>
@@ -3776,12 +3723,9 @@
       </c>
       <c r="E66" s="1"/>
       <c r="G66" s="1"/>
-      <c r="H66" s="5"/>
-      <c r="I66" s="5"/>
-      <c r="J66" s="5"/>
-      <c r="K66" s="5"/>
-      <c r="L66" s="5"/>
-      <c r="M66" s="5"/>
+      <c r="I66" s="1"/>
+      <c r="K66" s="1"/>
+      <c r="M66" s="1"/>
       <c r="N66" s="1"/>
     </row>
     <row r="67" spans="1:14" x14ac:dyDescent="0.25">
@@ -3789,7 +3733,7 @@
         <v>15</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="C67" s="6" t="s">
         <v>191</v>
@@ -3799,20 +3743,17 @@
       </c>
       <c r="E67" s="1"/>
       <c r="G67" s="1"/>
-      <c r="H67" s="5"/>
-      <c r="I67" s="5"/>
-      <c r="J67" s="5"/>
-      <c r="K67" s="5"/>
-      <c r="L67" s="5"/>
-      <c r="M67" s="5"/>
+      <c r="I67" s="1"/>
+      <c r="K67" s="1"/>
+      <c r="M67" s="1"/>
       <c r="N67" s="1"/>
     </row>
-    <row r="68" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A68" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="C68" s="6" t="s">
         <v>193</v>
@@ -3820,22 +3761,31 @@
       <c r="D68" s="7" t="s">
         <v>194</v>
       </c>
-      <c r="E68" s="1"/>
-      <c r="G68" s="1"/>
-      <c r="H68" s="5"/>
-      <c r="I68" s="5"/>
-      <c r="J68" s="5"/>
-      <c r="K68" s="5"/>
-      <c r="L68" s="5"/>
-      <c r="M68" s="5"/>
-      <c r="N68" s="1"/>
+      <c r="E68" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F68" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G68" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I68" s="1"/>
+      <c r="K68" s="1"/>
+      <c r="M68" s="1"/>
+      <c r="N68" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O68" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="69" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A69" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="C69" s="6" t="s">
         <v>195</v>
@@ -3845,12 +3795,9 @@
       </c>
       <c r="E69" s="1"/>
       <c r="G69" s="1"/>
-      <c r="H69" s="5"/>
-      <c r="I69" s="5"/>
-      <c r="J69" s="5"/>
-      <c r="K69" s="5"/>
-      <c r="L69" s="5"/>
-      <c r="M69" s="5"/>
+      <c r="I69" s="1"/>
+      <c r="K69" s="1"/>
+      <c r="M69" s="1"/>
       <c r="N69" s="1"/>
     </row>
     <row r="70" spans="1:14" x14ac:dyDescent="0.25">
@@ -3858,7 +3805,7 @@
         <v>15</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="C70" s="6" t="s">
         <v>197</v>
@@ -3868,12 +3815,9 @@
       </c>
       <c r="E70" s="1"/>
       <c r="G70" s="1"/>
-      <c r="H70" s="5"/>
-      <c r="I70" s="5"/>
-      <c r="J70" s="5"/>
-      <c r="K70" s="5"/>
-      <c r="L70" s="5"/>
-      <c r="M70" s="5"/>
+      <c r="I70" s="1"/>
+      <c r="K70" s="1"/>
+      <c r="M70" s="1"/>
       <c r="N70" s="1"/>
     </row>
     <row r="71" spans="1:14" x14ac:dyDescent="0.25">
@@ -3881,7 +3825,7 @@
         <v>15</v>
       </c>
       <c r="B71" s="6" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="C71" s="6" t="s">
         <v>199</v>
@@ -3891,20 +3835,17 @@
       </c>
       <c r="E71" s="1"/>
       <c r="G71" s="1"/>
-      <c r="H71" s="5"/>
-      <c r="I71" s="5"/>
-      <c r="J71" s="5"/>
-      <c r="K71" s="5"/>
-      <c r="L71" s="5"/>
-      <c r="M71" s="5"/>
+      <c r="I71" s="1"/>
+      <c r="K71" s="1"/>
+      <c r="M71" s="1"/>
       <c r="N71" s="1"/>
     </row>
-    <row r="72" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A72" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="C72" s="6" t="s">
         <v>201</v>
@@ -3912,46 +3853,31 @@
       <c r="D72" s="7" t="s">
         <v>202</v>
       </c>
-      <c r="E72" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="F72" s="1" t="s">
-        <v>203</v>
-      </c>
-      <c r="G72" s="1" t="s">
-        <v>47</v>
-      </c>
+      <c r="E72" s="1"/>
+      <c r="G72" s="1"/>
       <c r="I72" s="1"/>
       <c r="K72" s="1"/>
       <c r="M72" s="1"/>
-      <c r="N72" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="O72" s="1" t="s">
-        <v>24</v>
-      </c>
+      <c r="N72" s="1"/>
     </row>
     <row r="73" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A73" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B73" s="6" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="C73" s="6" t="s">
+        <v>203</v>
+      </c>
+      <c r="D73" s="7" t="s">
         <v>204</v>
-      </c>
-      <c r="D73" s="7" t="s">
-        <v>205</v>
       </c>
       <c r="E73" s="1"/>
       <c r="G73" s="1"/>
-      <c r="H73" s="5"/>
-      <c r="I73" s="5"/>
-      <c r="J73" s="5"/>
-      <c r="K73" s="5"/>
-      <c r="L73" s="5"/>
-      <c r="M73" s="5"/>
+      <c r="I73" s="1"/>
+      <c r="K73" s="1"/>
+      <c r="M73" s="1"/>
       <c r="N73" s="1"/>
     </row>
     <row r="74" spans="1:14" x14ac:dyDescent="0.25">
@@ -3959,53 +3885,59 @@
         <v>15</v>
       </c>
       <c r="B74" s="6" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="C74" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="D74" s="7" t="s">
         <v>206</v>
-      </c>
-      <c r="D74" s="7" t="s">
-        <v>207</v>
       </c>
       <c r="E74" s="1"/>
       <c r="G74" s="1"/>
-      <c r="H74" s="5"/>
-      <c r="I74" s="5"/>
-      <c r="J74" s="5"/>
-      <c r="K74" s="5"/>
-      <c r="L74" s="5"/>
-      <c r="M74" s="5"/>
+      <c r="I74" s="1"/>
+      <c r="K74" s="1"/>
+      <c r="M74" s="1"/>
       <c r="N74" s="1"/>
     </row>
-    <row r="75" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A75" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B75" s="6" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="C75" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="D75" s="7" t="s">
         <v>208</v>
       </c>
-      <c r="D75" s="7" t="s">
+      <c r="E75" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F75" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="E75" s="1"/>
-      <c r="G75" s="1"/>
-      <c r="H75" s="5"/>
-      <c r="I75" s="5"/>
-      <c r="J75" s="5"/>
-      <c r="K75" s="5"/>
-      <c r="L75" s="5"/>
-      <c r="M75" s="5"/>
-      <c r="N75" s="1"/>
+      <c r="G75" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="I75" s="1"/>
+      <c r="K75" s="1"/>
+      <c r="M75" s="1"/>
+      <c r="N75" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="O75" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="76" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A76" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B76" s="6" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="C76" s="6" t="s">
         <v>210</v>
@@ -4015,12 +3947,9 @@
       </c>
       <c r="E76" s="1"/>
       <c r="G76" s="1"/>
-      <c r="H76" s="5"/>
-      <c r="I76" s="5"/>
-      <c r="J76" s="5"/>
-      <c r="K76" s="5"/>
-      <c r="L76" s="5"/>
-      <c r="M76" s="5"/>
+      <c r="I76" s="1"/>
+      <c r="K76" s="1"/>
+      <c r="M76" s="1"/>
       <c r="N76" s="1"/>
     </row>
     <row r="77" spans="1:14" x14ac:dyDescent="0.25">
@@ -4028,7 +3957,7 @@
         <v>15</v>
       </c>
       <c r="B77" s="6" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="C77" s="6" t="s">
         <v>212</v>
@@ -4038,12 +3967,9 @@
       </c>
       <c r="E77" s="1"/>
       <c r="G77" s="1"/>
-      <c r="H77" s="5"/>
-      <c r="I77" s="5"/>
-      <c r="J77" s="5"/>
-      <c r="K77" s="5"/>
-      <c r="L77" s="5"/>
-      <c r="M77" s="5"/>
+      <c r="I77" s="1"/>
+      <c r="K77" s="1"/>
+      <c r="M77" s="1"/>
       <c r="N77" s="1"/>
     </row>
     <row r="78" spans="1:14" x14ac:dyDescent="0.25">
@@ -4051,7 +3977,7 @@
         <v>15</v>
       </c>
       <c r="B78" s="6" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="C78" s="6" t="s">
         <v>214</v>
@@ -4061,20 +3987,17 @@
       </c>
       <c r="E78" s="1"/>
       <c r="G78" s="1"/>
-      <c r="H78" s="5"/>
-      <c r="I78" s="5"/>
-      <c r="J78" s="5"/>
-      <c r="K78" s="5"/>
-      <c r="L78" s="5"/>
-      <c r="M78" s="5"/>
+      <c r="I78" s="1"/>
+      <c r="K78" s="1"/>
+      <c r="M78" s="1"/>
       <c r="N78" s="1"/>
     </row>
-    <row r="79" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A79" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B79" s="6" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="C79" s="6" t="s">
         <v>216</v>
@@ -4082,106 +4005,59 @@
       <c r="D79" s="7" t="s">
         <v>217</v>
       </c>
-      <c r="E79" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F79" s="1" t="s">
+      <c r="E79" s="1"/>
+      <c r="G79" s="1"/>
+      <c r="I79" s="1"/>
+      <c r="K79" s="1"/>
+      <c r="M79" s="1"/>
+      <c r="N79" s="1"/>
+    </row>
+    <row r="80" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A80" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B80" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="C80" s="6" t="s">
         <v>218</v>
       </c>
-      <c r="G79" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="H79" s="5"/>
-      <c r="I79" s="5"/>
-      <c r="J79" s="5"/>
-      <c r="K79" s="5"/>
-      <c r="L79" s="5"/>
-      <c r="M79" s="5"/>
-      <c r="N79" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="O79" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="80" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A80" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B80" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="C80" s="6" t="s">
+      <c r="D80" s="7" t="s">
         <v>219</v>
       </c>
-      <c r="D80" s="7" t="s">
+      <c r="E80" s="1"/>
+      <c r="G80" s="1"/>
+      <c r="I80" s="1"/>
+      <c r="K80" s="1"/>
+      <c r="M80" s="1"/>
+      <c r="N80" s="1"/>
+    </row>
+    <row r="81" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A81" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B81" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="C81" s="6" t="s">
         <v>220</v>
-      </c>
-      <c r="E80" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F80" s="1" t="s">
-        <v>218</v>
-      </c>
-      <c r="G80" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="H80" s="5"/>
-      <c r="I80" s="5"/>
-      <c r="J80" s="5"/>
-      <c r="K80" s="5"/>
-      <c r="L80" s="5"/>
-      <c r="M80" s="5"/>
-      <c r="N80" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="O80" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="81" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A81" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B81" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="C81" s="6" t="s">
-        <v>102</v>
       </c>
       <c r="D81" s="7" t="s">
         <v>221</v>
       </c>
-      <c r="E81" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F81" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="G81" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="H81" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="I81" s="1" t="s">
-        <v>23</v>
-      </c>
+      <c r="E81" s="1"/>
+      <c r="G81" s="1"/>
+      <c r="I81" s="1"/>
       <c r="K81" s="1"/>
       <c r="M81" s="1"/>
-      <c r="N81" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="O81" s="1" t="s">
-        <v>24</v>
-      </c>
+      <c r="N81" s="1"/>
     </row>
     <row r="82" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A82" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B82" s="6" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="C82" s="6" t="s">
         <v>222</v>
@@ -4190,52 +4066,129 @@
         <v>223</v>
       </c>
       <c r="E82" s="1" t="s">
-        <v>129</v>
+        <v>23</v>
       </c>
       <c r="F82" s="1" t="s">
-        <v>130</v>
+        <v>224</v>
       </c>
       <c r="G82" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="H82" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="I82" s="1" t="s">
-        <v>129</v>
-      </c>
+        <v>48</v>
+      </c>
+      <c r="I82" s="1"/>
       <c r="K82" s="1"/>
       <c r="M82" s="1"/>
       <c r="N82" s="1" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="O82" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="83" spans="5:14" x14ac:dyDescent="0.25">
-      <c r="E83" s="1"/>
-      <c r="G83" s="1"/>
+    <row r="83" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A83" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B83" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="C83" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="D83" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="E83" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F83" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="G83" s="1" t="s">
+        <v>21</v>
+      </c>
       <c r="I83" s="1"/>
       <c r="K83" s="1"/>
       <c r="M83" s="1"/>
-      <c r="N83" s="1"/>
-    </row>
-    <row r="84" spans="5:14" x14ac:dyDescent="0.25">
-      <c r="E84" s="1"/>
-      <c r="G84" s="1"/>
-      <c r="I84" s="1"/>
+      <c r="N83" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="O83" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="84" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A84" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B84" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="C84" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="D84" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="E84" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F84" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G84" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H84" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I84" s="1" t="s">
+        <v>23</v>
+      </c>
       <c r="K84" s="1"/>
       <c r="M84" s="1"/>
-      <c r="N84" s="1"/>
-    </row>
-    <row r="85" spans="5:14" x14ac:dyDescent="0.25">
-      <c r="E85" s="1"/>
-      <c r="G85" s="1"/>
-      <c r="I85" s="1"/>
+      <c r="N84" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O84" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="85" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A85" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B85" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="C85" s="6" t="s">
+        <v>228</v>
+      </c>
+      <c r="D85" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="E85" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="F85" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="G85" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="H85" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="I85" s="1" t="s">
+        <v>135</v>
+      </c>
       <c r="K85" s="1"/>
       <c r="M85" s="1"/>
-      <c r="N85" s="1"/>
+      <c r="N85" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="O85" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="86" spans="5:14" x14ac:dyDescent="0.25">
       <c r="E86" s="1"/>
@@ -6613,9 +6566,33 @@
       <c r="M382" s="1"/>
       <c r="N382" s="1"/>
     </row>
+    <row r="383" spans="5:14" x14ac:dyDescent="0.25">
+      <c r="E383" s="1"/>
+      <c r="G383" s="1"/>
+      <c r="I383" s="1"/>
+      <c r="K383" s="1"/>
+      <c r="M383" s="1"/>
+      <c r="N383" s="1"/>
+    </row>
+    <row r="384" spans="5:14" x14ac:dyDescent="0.25">
+      <c r="E384" s="1"/>
+      <c r="G384" s="1"/>
+      <c r="I384" s="1"/>
+      <c r="K384" s="1"/>
+      <c r="M384" s="1"/>
+      <c r="N384" s="1"/>
+    </row>
+    <row r="385" spans="5:14" x14ac:dyDescent="0.25">
+      <c r="E385" s="1"/>
+      <c r="G385" s="1"/>
+      <c r="I385" s="1"/>
+      <c r="K385" s="1"/>
+      <c r="M385" s="1"/>
+      <c r="N385" s="1"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O1"/>
-  <conditionalFormatting sqref="E2:E382">
+  <conditionalFormatting sqref="E2:E385">
     <cfRule type="containsText" dxfId="0" priority="1">
       <formula>NOT(ISERROR(SEARCH("BOT",E2)))</formula>
     </cfRule>
@@ -6635,7 +6612,7 @@
       <formula>NOT(ISERROR(SEARCH("NEUTRO",E2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G382">
+  <conditionalFormatting sqref="G2:G385">
     <cfRule type="containsText" dxfId="6" priority="1">
       <formula>NOT(ISERROR(SEARCH("BOT",G2)))</formula>
     </cfRule>
@@ -6655,7 +6632,7 @@
       <formula>NOT(ISERROR(SEARCH("NEUTRO",G2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I382">
+  <conditionalFormatting sqref="I2:I385">
     <cfRule type="containsText" dxfId="12" priority="1">
       <formula>NOT(ISERROR(SEARCH("BOT",I2)))</formula>
     </cfRule>
@@ -6675,7 +6652,7 @@
       <formula>NOT(ISERROR(SEARCH("NEUTRO",I2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K2:K382">
+  <conditionalFormatting sqref="K2:K385">
     <cfRule type="containsText" dxfId="18" priority="1">
       <formula>NOT(ISERROR(SEARCH("BOT",K2)))</formula>
     </cfRule>
@@ -6695,7 +6672,7 @@
       <formula>NOT(ISERROR(SEARCH("NEUTRO",K2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M2:M382">
+  <conditionalFormatting sqref="M2:M385">
     <cfRule type="containsText" dxfId="24" priority="1">
       <formula>NOT(ISERROR(SEARCH("BOT",M2)))</formula>
     </cfRule>
@@ -6716,40 +6693,40 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="12">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca do Móvel" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca do Móvel" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="E10:E382">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca do Móvel" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca do Móvel" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="E10:E385">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca do Móvel" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca do Móvel" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="E2:E382">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca do Móvel" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca do Móvel" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="E2:E385">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 1" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 1" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="G10:G382">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 1" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 1" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="G10:G385">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 1" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 1" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="G2:G382">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 1" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 1" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="G2:G385">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 2" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 2" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="I10:I382">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 2" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 2" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="I10:I385">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 2" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 2" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="I2:I382">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 2" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 2" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="I2:I385">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 3" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 3" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="K10:K382">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 3" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 3" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="K10:K385">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 3" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 3" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="K2:K382">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 3" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 3" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="K2:K385">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 4" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 4" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="M10:M382">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 4" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 4" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="M10:M385">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 4" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 4" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="M2:M382">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 4" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 4" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="M2:M385">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo" prompt="MOVIMENTO = Movimento definido nesta planta; FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo" error="MOVIMENTO = Movimento definido nesta planta; FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" sqref="N10:N382">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo" prompt="MOVIMENTO = Movimento definido nesta planta; FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo" error="MOVIMENTO = Movimento definido nesta planta; FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" sqref="N10:N385">
       <formula1>"MOVIMENTO,FIXO,EXPOSICAO,NOVO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo" prompt="MOVIMENTO = Movimento definido nesta planta; FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo" error="MOVIMENTO = Movimento definido nesta planta; FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" sqref="N2:N382">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo" prompt="MOVIMENTO = Movimento definido nesta planta; FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo" error="MOVIMENTO = Movimento definido nesta planta; FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" sqref="N2:N385">
       <formula1>"MOVIMENTO,FIXO,EXPOSICAO,NOVO"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6777,16 +6754,16 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>224</v>
+        <v>230</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>226</v>
+        <v>232</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>227</v>
+        <v>233</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -6794,13 +6771,13 @@
         <v>15</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>228</v>
+        <v>234</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>23</v>
@@ -6814,10 +6791,10 @@
         <v>15</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>228</v>
+        <v>234</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
       <c r="D3" s="8" t="s">
         <v>69</v>
@@ -6834,16 +6811,16 @@
         <v>15</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>228</v>
+        <v>234</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>24</v>
@@ -6854,13 +6831,13 @@
         <v>15</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>228</v>
+        <v>234</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>21</v>
@@ -6874,13 +6851,13 @@
         <v>15</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>228</v>
+        <v>234</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>21</v>
@@ -6894,16 +6871,16 @@
         <v>15</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>228</v>
+        <v>234</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>234</v>
+        <v>240</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>24</v>
@@ -6914,16 +6891,16 @@
         <v>15</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>228</v>
+        <v>234</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>24</v>
@@ -6934,13 +6911,13 @@
         <v>15</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>228</v>
+        <v>234</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>23</v>
@@ -6954,19 +6931,19 @@
         <v>15</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>228</v>
+        <v>234</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>237</v>
+        <v>243</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>23</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -6974,19 +6951,19 @@
         <v>15</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>228</v>
+        <v>234</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>237</v>
+        <v>243</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>239</v>
+        <v>245</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>21</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -6994,19 +6971,19 @@
         <v>15</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>228</v>
+        <v>234</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>237</v>
+        <v>243</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -7017,10 +6994,10 @@
         <v>16</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>24</v>
@@ -7037,10 +7014,10 @@
         <v>16</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>243</v>
+        <v>249</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>24</v>
@@ -7054,13 +7031,13 @@
         <v>15</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>24</v>
@@ -7074,13 +7051,13 @@
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>24</v>
@@ -7094,13 +7071,13 @@
         <v>15</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>24</v>
@@ -7114,13 +7091,13 @@
         <v>15</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>24</v>
@@ -7134,13 +7111,13 @@
         <v>15</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>24</v>
@@ -7154,13 +7131,13 @@
         <v>15</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>24</v>
@@ -7174,13 +7151,13 @@
         <v>15</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>24</v>
@@ -8443,108 +8420,108 @@
   <sheetData>
     <row r="1" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B1" s="9" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B2" s="10" t="s">
-        <v>248</v>
+        <v>254</v>
       </c>
       <c r="C2" s="10"/>
       <c r="D2" s="10"/>
     </row>
     <row r="4" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B4" s="11" t="s">
-        <v>249</v>
+        <v>255</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B5" s="10" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="C5" s="10"/>
       <c r="D5" s="10"/>
     </row>
     <row r="6" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B6" s="10" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="C6" s="10"/>
       <c r="D6" s="10"/>
     </row>
     <row r="7" ht="16" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B7" s="10" t="s">
-        <v>252</v>
+        <v>258</v>
       </c>
       <c r="C7" s="10"/>
       <c r="D7" s="10"/>
     </row>
-    <row r="8" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="8" ht="45" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B8" s="10" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="C8" s="10"/>
       <c r="D8" s="10"/>
     </row>
     <row r="9" ht="16" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B9" s="10" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="C9" s="10"/>
       <c r="D9" s="10"/>
     </row>
     <row r="10" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B10" s="10" t="s">
-        <v>255</v>
+        <v>261</v>
       </c>
       <c r="C10" s="10"/>
       <c r="D10" s="10"/>
     </row>
     <row r="11" ht="60" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B11" s="10" t="s">
-        <v>256</v>
+        <v>262</v>
       </c>
       <c r="C11" s="10"/>
       <c r="D11" s="10"/>
     </row>
-    <row r="12" ht="45" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="12" ht="60" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B12" s="10" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="C12" s="10"/>
       <c r="D12" s="10"/>
     </row>
-    <row r="13" ht="45" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="13" ht="75" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B13" s="10" t="s">
-        <v>258</v>
+        <v>264</v>
       </c>
       <c r="C13" s="10"/>
       <c r="D13" s="10"/>
     </row>
     <row r="14" ht="60" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B14" s="10" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
       <c r="C14" s="10"/>
       <c r="D14" s="10"/>
     </row>
     <row r="15" ht="45" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B15" s="10" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="C15" s="10"/>
       <c r="D15" s="10"/>
     </row>
     <row r="16" ht="45" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B16" s="10" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="C16" s="10"/>
       <c r="D16" s="10"/>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B18" s="11" t="s">
-        <v>262</v>
+        <v>268</v>
       </c>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.25">
@@ -8552,10 +8529,10 @@
         <v>21</v>
       </c>
       <c r="C19" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.25">
@@ -8563,32 +8540,32 @@
         <v>33</v>
       </c>
       <c r="C20" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B21" s="12" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C21" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="D21" s="15" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="22" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B22" s="12" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="C22" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>270</v>
+        <v>276</v>
       </c>
     </row>
     <row r="23" spans="2:4" x14ac:dyDescent="0.25">
@@ -8596,10 +8573,10 @@
         <v>23</v>
       </c>
       <c r="C23" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="D23" s="17" t="s">
-        <v>272</v>
+        <v>278</v>
       </c>
     </row>
     <row r="24" spans="2:4" x14ac:dyDescent="0.25">
@@ -8607,26 +8584,26 @@
         <v>19</v>
       </c>
       <c r="C24" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
       <c r="D24" s="18" t="s">
-        <v>274</v>
+        <v>280</v>
       </c>
     </row>
     <row r="26" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B26" s="11" t="s">
-        <v>275</v>
+        <v>281</v>
       </c>
     </row>
     <row r="27" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B27" s="12" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="C27" t="s">
-        <v>276</v>
+        <v>282</v>
       </c>
       <c r="D27" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
     </row>
     <row r="28" spans="2:4" x14ac:dyDescent="0.25">
@@ -8634,81 +8611,81 @@
         <v>30</v>
       </c>
       <c r="C28" t="s">
-        <v>278</v>
+        <v>284</v>
       </c>
       <c r="D28" t="s">
-        <v>279</v>
+        <v>285</v>
       </c>
     </row>
     <row r="29" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B29" s="12" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="C29" t="s">
-        <v>280</v>
+        <v>286</v>
       </c>
       <c r="D29" t="s">
-        <v>281</v>
+        <v>287</v>
       </c>
     </row>
     <row r="30" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B30" s="12" t="s">
-        <v>282</v>
+        <v>288</v>
       </c>
       <c r="C30" t="s">
-        <v>283</v>
+        <v>289</v>
       </c>
       <c r="D30" t="s">
-        <v>284</v>
+        <v>290</v>
       </c>
     </row>
     <row r="32" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B32" s="11" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
     </row>
     <row r="33" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B33" s="12" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
       <c r="C33" t="s">
-        <v>286</v>
+        <v>292</v>
       </c>
       <c r="D33"/>
     </row>
     <row r="34" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B34" s="12" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
       <c r="C34" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="D34"/>
     </row>
     <row r="35" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B35" s="12" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="C35" t="s">
-        <v>288</v>
+        <v>294</v>
       </c>
       <c r="D35"/>
     </row>
     <row r="36" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B36" s="12" t="s">
-        <v>237</v>
+        <v>243</v>
       </c>
       <c r="C36" t="s">
-        <v>289</v>
+        <v>295</v>
       </c>
       <c r="D36"/>
     </row>
     <row r="37" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B37" s="12" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="C37" t="s">
-        <v>290</v>
+        <v>296</v>
       </c>
       <c r="D37"/>
     </row>

</xml_diff>

<commit_message>
Totem: etiquetas e cores dos painéis pela linha do próprio totem
- Na linha TOTEM 1, Etiqueta 1–3 vão para o painel de cima, do meio e de baixo
  (ao lado do totem, com linha-guia) e a Marca Etiqueta N pinta o painel N.
  Funciona em planilhas que não têm as linhas TOTEM 1/PAINEL-N, que continuam
  aceitas e têm prioridade.
- IDs de espaço aceitam variações de digitação ("Totem 1 / painel 1",
  "PAINEL1", "LADO A", "MEIO_A_2").
- Planilha base sem as linhas de painel; ciclo de exemplo com o totem em uma
  linha (VERSAO_EXEMPLO 6).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019BmnBNRucVHCBVjZaoSiJv
</commit_message>
<xml_diff>
--- a/visualizador/Planilha base - Visualizador.xlsx
+++ b/visualizador/Planilha base - Visualizador.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="802" uniqueCount="297">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="782" uniqueCount="292">
   <si>
     <t>Ciclo</t>
   </si>
@@ -237,28 +237,10 @@
     <t>TOTEM 1</t>
   </si>
   <si>
-    <t>Totem 1 · vale para ER P, ER M, ER G, ER GG</t>
-  </si>
-  <si>
-    <t>TOTEM 1/PAINEL-1</t>
-  </si>
-  <si>
-    <t>Totem 1 – Painel 1</t>
+    <t>Totem 1 (Etiqueta 1–3 = painel de cima, do meio e de baixo; Marca Etiqueta N = cor do painel N) · vale para ER P, ER M, ER G, ER GG</t>
   </si>
   <si>
     <t>LÇTO UOMINI</t>
-  </si>
-  <si>
-    <t>TOTEM 1/PAINEL-2</t>
-  </si>
-  <si>
-    <t>Totem 1 – Painel 2</t>
-  </si>
-  <si>
-    <t>TOTEM 1/PAINEL-3</t>
-  </si>
-  <si>
-    <t>Totem 1 – Painel 3</t>
   </si>
   <si>
     <t>EXTRA-CESTINHAS</t>
@@ -783,7 +765,7 @@
     <t>Planilha base — Plano de Varejo</t>
   </si>
   <si>
-    <t>Gerada em 06/10/2026, 09:17:13 a partir do ciclo "Ciclo exemplo".</t>
+    <t>Gerada em 06/10/2026, 09:43:08 a partir do ciclo "Ciclo exemplo".</t>
   </si>
   <si>
     <t>Como preencher</t>
@@ -813,7 +795,10 @@
     <t>6.2 Etiquetas da gôndola. Na linha da gôndola inteira: Etiqueta 1 = Lado A, Etiqueta 2 = Meio A, Etiqueta 3 = Meio B, Etiqueta 4 = Lado B ("A" é sempre o lado virado para quem olha a planta). A linha de um espaço mostra até 4 etiquetas empilhadas em cima daquele bloco (Etiqueta 1 a 4) e substitui a etiqueta que viria da gôndola inteira.</t>
   </si>
   <si>
-    <t>6.3 Mesa destaque (FRENTE-1 e 2), mesa 3 frentes (FRENTE-1 a 3), totem (PAINEL-1 a 3, o 1 é o painel de cima) e móvel make (TESTEIRA-1 a 4) têm uma linha por bloco, com cor e etiqueta próprias. Cada frente das mesas mostra até 4 etiquetas; cada painel do totem e cada testeira, 1. Bloco sem linha própria usa a cor do móvel inteiro. Blocos vizinhos com as mesmas etiquetas e cor ficam com uma pilha só, no centro. O balcão recepção tem uma cor só; Etiqueta 1, 2 e 3 vão para o bloco 1, o canto e o bloco 3.</t>
+    <t>6.3 Mesa destaque (FRENTE-1 e 2), mesa 3 frentes (FRENTE-1 a 3) e móvel make (TESTEIRA-1 a 4) têm uma linha por bloco, com cor e etiqueta próprias. Cada frente das mesas mostra até 4 etiquetas; cada testeira, 1. Bloco sem linha própria usa a cor do móvel inteiro. Blocos vizinhos com as mesmas etiquetas e cor ficam com uma pilha só, no centro. O balcão recepção tem uma cor só; Etiqueta 1, 2 e 3 vão para o bloco 1, o canto e o bloco 3.</t>
+  </si>
+  <si>
+    <t>6.4 Totem: na linha do totem, Etiqueta 1, 2 e 3 vão para o painel de cima, o do meio e o de baixo (cada uma ao lado do seu painel), e a "Marca Etiqueta N" pinta o painel N. Painel sem etiqueta usa a "Marca do Móvel". Se preferir, uma linha TOTEM 1/PAINEL-1 (a 3) define cor e etiqueta de um painel e tem prioridade.</t>
   </si>
   <si>
     <t>7. Na coluna "Planta" vale o nome (ex.: ER P) ou o número (01). Cascata: o que é definido numa planta vale também para as seguintes (ER P → ER M → ER G → ER GG), por isso cada móvel aparece uma vez só, na primeira planta que o tem ("vale para…" na coluna Móvel). Para mudar um móvel só a partir de uma planta, acrescente uma linha com o mesmo ID Móvel e essa planta. Planta = TODAS vale para todas.</t>
@@ -1780,7 +1765,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O385"/>
+  <dimension ref="A1:O382"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="13" style="1" customWidth="1"/>
@@ -2371,10 +2356,26 @@
       <c r="E19" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G19" s="1"/>
-      <c r="I19" s="1"/>
-      <c r="K19" s="1"/>
-      <c r="M19" s="1"/>
+      <c r="F19" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="I19" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="J19" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="K19" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="L19" s="5"/>
+      <c r="M19" s="5"/>
       <c r="N19" s="1" t="s">
         <v>24</v>
       </c>
@@ -2390,26 +2391,23 @@
         <v>16</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="H20" s="5"/>
-      <c r="I20" s="5"/>
-      <c r="J20" s="5"/>
-      <c r="K20" s="5"/>
-      <c r="L20" s="5"/>
-      <c r="M20" s="5"/>
+        <v>66</v>
+      </c>
+      <c r="I20" s="1"/>
+      <c r="K20" s="1"/>
+      <c r="M20" s="1"/>
       <c r="N20" s="1" t="s">
         <v>24</v>
       </c>
@@ -2431,20 +2429,22 @@
         <v>79</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="G21" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H21" s="5"/>
-      <c r="I21" s="5"/>
-      <c r="J21" s="5"/>
-      <c r="K21" s="5"/>
-      <c r="L21" s="5"/>
-      <c r="M21" s="5"/>
+      <c r="H21" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="K21" s="1"/>
+      <c r="M21" s="1"/>
       <c r="N21" s="1" t="s">
         <v>24</v>
       </c>
@@ -2460,26 +2460,23 @@
         <v>16</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>34</v>
+        <v>62</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="H22" s="5"/>
-      <c r="I22" s="5"/>
-      <c r="J22" s="5"/>
-      <c r="K22" s="5"/>
-      <c r="L22" s="5"/>
-      <c r="M22" s="5"/>
+        <v>48</v>
+      </c>
+      <c r="I22" s="1"/>
+      <c r="K22" s="1"/>
+      <c r="M22" s="1"/>
       <c r="N22" s="1" t="s">
         <v>24</v>
       </c>
@@ -2495,19 +2492,19 @@
         <v>16</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>19</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>65</v>
+        <v>86</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>66</v>
+        <v>23</v>
       </c>
       <c r="I23" s="1"/>
       <c r="K23" s="1"/>
@@ -2527,28 +2524,21 @@
         <v>16</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F24" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="G24" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="H24" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="I24" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="K24" s="1"/>
-      <c r="M24" s="1"/>
+        <v>89</v>
+      </c>
+      <c r="G24" s="1"/>
+      <c r="H24" s="5"/>
+      <c r="I24" s="5"/>
+      <c r="J24" s="5"/>
+      <c r="K24" s="5"/>
+      <c r="L24" s="5"/>
+      <c r="M24" s="5"/>
       <c r="N24" s="1" t="s">
         <v>24</v>
       </c>
@@ -2564,23 +2554,26 @@
         <v>16</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>62</v>
+        <v>80</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="I25" s="1"/>
-      <c r="K25" s="1"/>
-      <c r="M25" s="1"/>
+        <v>21</v>
+      </c>
+      <c r="H25" s="5"/>
+      <c r="I25" s="5"/>
+      <c r="J25" s="5"/>
+      <c r="K25" s="5"/>
+      <c r="L25" s="5"/>
+      <c r="M25" s="5"/>
       <c r="N25" s="1" t="s">
         <v>24</v>
       </c>
@@ -2596,23 +2589,26 @@
         <v>16</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I26" s="1"/>
-      <c r="K26" s="1"/>
-      <c r="M26" s="1"/>
+        <v>21</v>
+      </c>
+      <c r="H26" s="5"/>
+      <c r="I26" s="5"/>
+      <c r="J26" s="5"/>
+      <c r="K26" s="5"/>
+      <c r="L26" s="5"/>
+      <c r="M26" s="5"/>
       <c r="N26" s="1" t="s">
         <v>24</v>
       </c>
@@ -2628,13 +2624,13 @@
         <v>16</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>95</v>
+        <v>48</v>
       </c>
       <c r="G27" s="1"/>
       <c r="H27" s="5"/>
@@ -2664,20 +2660,22 @@
         <v>97</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="G28" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H28" s="5"/>
-      <c r="I28" s="5"/>
-      <c r="J28" s="5"/>
-      <c r="K28" s="5"/>
-      <c r="L28" s="5"/>
-      <c r="M28" s="5"/>
+      <c r="H28" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I28" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="K28" s="1"/>
+      <c r="M28" s="1"/>
       <c r="N28" s="1" t="s">
         <v>24</v>
       </c>
@@ -2693,26 +2691,28 @@
         <v>16</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>86</v>
+        <v>101</v>
       </c>
       <c r="G29" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H29" s="5"/>
-      <c r="I29" s="5"/>
-      <c r="J29" s="5"/>
-      <c r="K29" s="5"/>
-      <c r="L29" s="5"/>
-      <c r="M29" s="5"/>
+      <c r="H29" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I29" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="K29" s="1"/>
+      <c r="M29" s="1"/>
       <c r="N29" s="1" t="s">
         <v>24</v>
       </c>
@@ -2728,93 +2728,100 @@
         <v>16</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E30" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H30" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I30" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="K30" s="1"/>
+      <c r="M30" s="1"/>
+      <c r="N30" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O30" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A31" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="D31" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="E31" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="G30" s="1"/>
-      <c r="H30" s="5"/>
-      <c r="I30" s="5"/>
-      <c r="J30" s="5"/>
-      <c r="K30" s="5"/>
-      <c r="L30" s="5"/>
-      <c r="M30" s="5"/>
-      <c r="N30" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="O30" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A31" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C31" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="D31" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="E31" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F31" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="G31" s="1" t="s">
-        <v>21</v>
-      </c>
+      <c r="G31" s="1"/>
       <c r="H31" s="1" t="s">
-        <v>22</v>
+        <v>108</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="K31" s="1"/>
-      <c r="M31" s="1"/>
+        <v>48</v>
+      </c>
+      <c r="J31" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="K31" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="L31" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="M31" s="1" t="s">
+        <v>48</v>
+      </c>
       <c r="N31" s="1" t="s">
-        <v>24</v>
+        <v>110</v>
       </c>
       <c r="O31" s="1" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A32" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B32" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C32" s="3" t="s">
+      <c r="A32" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B32" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="D32" s="4" t="s">
-        <v>106</v>
+      <c r="C32" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="D32" s="7" t="s">
+        <v>112</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>107</v>
+        <v>34</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="H32" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="I32" s="1" t="s">
-        <v>23</v>
-      </c>
+        <v>33</v>
+      </c>
+      <c r="I32" s="1"/>
       <c r="K32" s="1"/>
       <c r="M32" s="1"/>
       <c r="N32" s="1" t="s">
@@ -2824,91 +2831,64 @@
         <v>24</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A33" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B33" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C33" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="D33" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="E33" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F33" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="G33" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="H33" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="I33" s="1" t="s">
-        <v>23</v>
-      </c>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A33" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="D33" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="E33" s="1"/>
+      <c r="G33" s="1"/>
+      <c r="I33" s="1"/>
       <c r="K33" s="1"/>
       <c r="M33" s="1"/>
-      <c r="N33" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="O33" s="1" t="s">
-        <v>24</v>
-      </c>
+      <c r="N33" s="1"/>
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="G34" s="1"/>
-      <c r="H34" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="I34" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="J34" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="K34" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="L34" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="M34" s="1" t="s">
-        <v>48</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="G34" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="I34" s="1"/>
+      <c r="K34" s="1"/>
+      <c r="M34" s="1"/>
       <c r="N34" s="1" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="O34" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="C35" s="6" t="s">
         <v>117</v>
@@ -2916,31 +2896,19 @@
       <c r="D35" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="E35" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="F35" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="G35" s="1" t="s">
-        <v>33</v>
-      </c>
+      <c r="E35" s="1"/>
+      <c r="G35" s="1"/>
       <c r="I35" s="1"/>
       <c r="K35" s="1"/>
       <c r="M35" s="1"/>
-      <c r="N35" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="O35" s="1" t="s">
-        <v>24</v>
-      </c>
+      <c r="N35" s="1"/>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="C36" s="6" t="s">
         <v>119</v>
@@ -2955,12 +2923,12 @@
       <c r="M36" s="1"/>
       <c r="N36" s="1"/>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="C37" s="6" t="s">
         <v>121</v>
@@ -2968,31 +2936,19 @@
       <c r="D37" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="E37" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F37" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="G37" s="1" t="s">
-        <v>21</v>
-      </c>
+      <c r="E37" s="1"/>
+      <c r="G37" s="1"/>
       <c r="I37" s="1"/>
       <c r="K37" s="1"/>
       <c r="M37" s="1"/>
-      <c r="N37" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="O37" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N37" s="1"/>
+    </row>
+    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="C38" s="6" t="s">
         <v>123</v>
@@ -3000,19 +2956,31 @@
       <c r="D38" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="E38" s="1"/>
-      <c r="G38" s="1"/>
+      <c r="E38" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>21</v>
+      </c>
       <c r="I38" s="1"/>
       <c r="K38" s="1"/>
       <c r="M38" s="1"/>
-      <c r="N38" s="1"/>
-    </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N38" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O38" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="C39" s="6" t="s">
         <v>125</v>
@@ -3020,19 +2988,31 @@
       <c r="D39" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="E39" s="1"/>
-      <c r="G39" s="1"/>
+      <c r="E39" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F39" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G39" s="1" t="s">
+        <v>33</v>
+      </c>
       <c r="I39" s="1"/>
       <c r="K39" s="1"/>
       <c r="M39" s="1"/>
-      <c r="N39" s="1"/>
-    </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N39" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O39" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="C40" s="6" t="s">
         <v>127</v>
@@ -3040,40 +3020,52 @@
       <c r="D40" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="E40" s="1"/>
-      <c r="G40" s="1"/>
+      <c r="E40" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="G40" s="1" t="s">
+        <v>129</v>
+      </c>
       <c r="I40" s="1"/>
       <c r="K40" s="1"/>
       <c r="M40" s="1"/>
-      <c r="N40" s="1"/>
+      <c r="N40" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="O40" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="C41" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="D41" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="E41" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="D41" s="7" t="s">
-        <v>130</v>
-      </c>
-      <c r="E41" s="1" t="s">
-        <v>21</v>
-      </c>
       <c r="F41" s="1" t="s">
-        <v>69</v>
+        <v>134</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>21</v>
+        <v>129</v>
       </c>
       <c r="I41" s="1"/>
       <c r="K41" s="1"/>
       <c r="M41" s="1"/>
       <c r="N41" s="1" t="s">
-        <v>24</v>
+        <v>131</v>
       </c>
       <c r="O41" s="1" t="s">
         <v>24</v>
@@ -3084,22 +3076,22 @@
         <v>15</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="D42" s="7" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>33</v>
+        <v>48</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="I42" s="1"/>
       <c r="K42" s="1"/>
@@ -3112,181 +3104,145 @@
       </c>
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A43" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B43" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="C43" s="6" t="s">
-        <v>133</v>
-      </c>
-      <c r="D43" s="7" t="s">
-        <v>134</v>
+      <c r="A43" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="C43" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="D43" s="4" t="s">
+        <v>139</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>135</v>
+        <v>21</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>136</v>
+        <v>69</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>135</v>
+        <v>21</v>
       </c>
       <c r="I43" s="1"/>
       <c r="K43" s="1"/>
       <c r="M43" s="1"/>
       <c r="N43" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O43" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A44" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B44" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="O43" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A44" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B44" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="C44" s="6" t="s">
-        <v>138</v>
-      </c>
-      <c r="D44" s="7" t="s">
-        <v>139</v>
+      <c r="C44" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="D44" s="4" t="s">
+        <v>141</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>135</v>
+        <v>23</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>140</v>
+        <v>22</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="I44" s="1"/>
-      <c r="K44" s="1"/>
+        <v>23</v>
+      </c>
+      <c r="H44" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="I44" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="J44" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="K44" s="1" t="s">
+        <v>23</v>
+      </c>
       <c r="M44" s="1"/>
       <c r="N44" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="O44" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A45" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B45" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="O44" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A45" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B45" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="C45" s="6" t="s">
-        <v>141</v>
-      </c>
-      <c r="D45" s="7" t="s">
-        <v>142</v>
-      </c>
-      <c r="E45" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F45" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="G45" s="1" t="s">
-        <v>23</v>
-      </c>
+      <c r="C45" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="E45" s="1"/>
+      <c r="G45" s="1"/>
       <c r="I45" s="1"/>
       <c r="K45" s="1"/>
       <c r="M45" s="1"/>
-      <c r="N45" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="O45" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N45" s="1"/>
+    </row>
+    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="E46" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F46" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="G46" s="1" t="s">
-        <v>21</v>
-      </c>
+        <v>147</v>
+      </c>
+      <c r="E46" s="1"/>
+      <c r="G46" s="1"/>
       <c r="I46" s="1"/>
       <c r="K46" s="1"/>
       <c r="M46" s="1"/>
-      <c r="N46" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="O46" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N46" s="1"/>
+    </row>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="E47" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F47" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="G47" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="H47" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="I47" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="J47" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="K47" s="1" t="s">
-        <v>23</v>
-      </c>
+      <c r="E47" s="1"/>
+      <c r="G47" s="1"/>
+      <c r="I47" s="1"/>
+      <c r="K47" s="1"/>
       <c r="M47" s="1"/>
-      <c r="N47" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="O47" s="1" t="s">
-        <v>24</v>
-      </c>
+      <c r="N47" s="1"/>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="C48" s="3" t="s">
         <v>150</v>
@@ -3306,7 +3262,7 @@
         <v>15</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="C49" s="3" t="s">
         <v>152</v>
@@ -3326,7 +3282,7 @@
         <v>15</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="C50" s="3" t="s">
         <v>154</v>
@@ -3346,7 +3302,7 @@
         <v>15</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="C51" s="3" t="s">
         <v>156</v>
@@ -3366,7 +3322,7 @@
         <v>15</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="C52" s="3" t="s">
         <v>158</v>
@@ -3381,12 +3337,12 @@
       <c r="M52" s="1"/>
       <c r="N52" s="1"/>
     </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="C53" s="3" t="s">
         <v>160</v>
@@ -3394,19 +3350,31 @@
       <c r="D53" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="E53" s="1"/>
-      <c r="G53" s="1"/>
+      <c r="E53" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F53" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G53" s="1" t="s">
+        <v>33</v>
+      </c>
       <c r="I53" s="1"/>
       <c r="K53" s="1"/>
       <c r="M53" s="1"/>
-      <c r="N53" s="1"/>
-    </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N53" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O53" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="54" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="C54" s="3" t="s">
         <v>162</v>
@@ -3414,19 +3382,26 @@
       <c r="D54" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="E54" s="1"/>
+      <c r="E54" s="1" t="s">
+        <v>23</v>
+      </c>
       <c r="G54" s="1"/>
       <c r="I54" s="1"/>
       <c r="K54" s="1"/>
       <c r="M54" s="1"/>
-      <c r="N54" s="1"/>
-    </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N54" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O54" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="55" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="C55" s="3" t="s">
         <v>164</v>
@@ -3434,19 +3409,31 @@
       <c r="D55" s="4" t="s">
         <v>165</v>
       </c>
-      <c r="E55" s="1"/>
-      <c r="G55" s="1"/>
+      <c r="E55" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F55" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="G55" s="1" t="s">
+        <v>21</v>
+      </c>
       <c r="I55" s="1"/>
       <c r="K55" s="1"/>
       <c r="M55" s="1"/>
-      <c r="N55" s="1"/>
+      <c r="N55" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O55" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="56" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="C56" s="3" t="s">
         <v>166</v>
@@ -3455,13 +3442,13 @@
         <v>167</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>34</v>
+        <v>168</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="I56" s="1"/>
       <c r="K56" s="1"/>
@@ -3478,18 +3465,23 @@
         <v>15</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D57" s="4" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="G57" s="1"/>
+        <v>48</v>
+      </c>
+      <c r="F57" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="G57" s="1" t="s">
+        <v>48</v>
+      </c>
       <c r="I57" s="1"/>
       <c r="K57" s="1"/>
       <c r="M57" s="1"/>
@@ -3501,139 +3493,103 @@
       </c>
     </row>
     <row r="58" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A58" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B58" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="C58" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="D58" s="4" t="s">
+      <c r="A58" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B58" s="6" t="s">
         <v>171</v>
       </c>
+      <c r="C58" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="D58" s="7" t="s">
+        <v>173</v>
+      </c>
       <c r="E58" s="1" t="s">
-        <v>21</v>
+        <v>129</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>56</v>
+        <v>174</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>21</v>
+        <v>129</v>
       </c>
       <c r="I58" s="1"/>
       <c r="K58" s="1"/>
       <c r="M58" s="1"/>
       <c r="N58" s="1" t="s">
-        <v>24</v>
+        <v>110</v>
       </c>
       <c r="O58" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="59" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A59" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B59" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="C59" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="D59" s="4" t="s">
-        <v>173</v>
-      </c>
-      <c r="E59" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F59" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="G59" s="1" t="s">
-        <v>23</v>
-      </c>
+    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A59" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B59" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="C59" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="D59" s="7" t="s">
+        <v>176</v>
+      </c>
+      <c r="E59" s="1"/>
+      <c r="G59" s="1"/>
       <c r="I59" s="1"/>
       <c r="K59" s="1"/>
       <c r="M59" s="1"/>
-      <c r="N59" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="O59" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="60" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A60" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B60" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="C60" s="3" t="s">
-        <v>175</v>
-      </c>
-      <c r="D60" s="4" t="s">
-        <v>176</v>
-      </c>
-      <c r="E60" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F60" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="G60" s="1" t="s">
-        <v>48</v>
-      </c>
+      <c r="N59" s="1"/>
+    </row>
+    <row r="60" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A60" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B60" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="C60" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="D60" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="E60" s="1"/>
+      <c r="G60" s="1"/>
       <c r="I60" s="1"/>
       <c r="K60" s="1"/>
       <c r="M60" s="1"/>
-      <c r="N60" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="O60" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="61" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N60" s="1"/>
+    </row>
+    <row r="61" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A61" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B61" s="6" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D61" s="7" t="s">
-        <v>179</v>
-      </c>
-      <c r="E61" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="F61" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="G61" s="1" t="s">
-        <v>135</v>
-      </c>
+      <c r="E61" s="1"/>
+      <c r="G61" s="1"/>
       <c r="I61" s="1"/>
       <c r="K61" s="1"/>
       <c r="M61" s="1"/>
-      <c r="N61" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="O61" s="1" t="s">
-        <v>24</v>
-      </c>
+      <c r="N61" s="1"/>
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A62" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B62" s="6" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="C62" s="6" t="s">
         <v>181</v>
@@ -3653,7 +3609,7 @@
         <v>15</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="C63" s="6" t="s">
         <v>183</v>
@@ -3673,7 +3629,7 @@
         <v>15</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="C64" s="6" t="s">
         <v>185</v>
@@ -3688,12 +3644,12 @@
       <c r="M64" s="1"/>
       <c r="N64" s="1"/>
     </row>
-    <row r="65" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A65" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="C65" s="6" t="s">
         <v>187</v>
@@ -3701,19 +3657,31 @@
       <c r="D65" s="7" t="s">
         <v>188</v>
       </c>
-      <c r="E65" s="1"/>
-      <c r="G65" s="1"/>
+      <c r="E65" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F65" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G65" s="1" t="s">
+        <v>33</v>
+      </c>
       <c r="I65" s="1"/>
       <c r="K65" s="1"/>
       <c r="M65" s="1"/>
-      <c r="N65" s="1"/>
+      <c r="N65" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O65" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A66" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="C66" s="6" t="s">
         <v>189</v>
@@ -3733,7 +3701,7 @@
         <v>15</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="C67" s="6" t="s">
         <v>191</v>
@@ -3748,12 +3716,12 @@
       <c r="M67" s="1"/>
       <c r="N67" s="1"/>
     </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A68" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="C68" s="6" t="s">
         <v>193</v>
@@ -3761,31 +3729,19 @@
       <c r="D68" s="7" t="s">
         <v>194</v>
       </c>
-      <c r="E68" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="F68" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="G68" s="1" t="s">
-        <v>33</v>
-      </c>
+      <c r="E68" s="1"/>
+      <c r="G68" s="1"/>
       <c r="I68" s="1"/>
       <c r="K68" s="1"/>
       <c r="M68" s="1"/>
-      <c r="N68" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="O68" s="1" t="s">
-        <v>24</v>
-      </c>
+      <c r="N68" s="1"/>
     </row>
     <row r="69" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A69" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="C69" s="6" t="s">
         <v>195</v>
@@ -3805,7 +3761,7 @@
         <v>15</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="C70" s="6" t="s">
         <v>197</v>
@@ -3825,7 +3781,7 @@
         <v>15</v>
       </c>
       <c r="B71" s="6" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="C71" s="6" t="s">
         <v>199</v>
@@ -3840,12 +3796,12 @@
       <c r="M71" s="1"/>
       <c r="N71" s="1"/>
     </row>
-    <row r="72" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A72" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="C72" s="6" t="s">
         <v>201</v>
@@ -3853,25 +3809,37 @@
       <c r="D72" s="7" t="s">
         <v>202</v>
       </c>
-      <c r="E72" s="1"/>
-      <c r="G72" s="1"/>
+      <c r="E72" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F72" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="G72" s="1" t="s">
+        <v>48</v>
+      </c>
       <c r="I72" s="1"/>
       <c r="K72" s="1"/>
       <c r="M72" s="1"/>
-      <c r="N72" s="1"/>
+      <c r="N72" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="O72" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="73" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A73" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B73" s="6" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="C73" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D73" s="7" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="E73" s="1"/>
       <c r="G73" s="1"/>
@@ -3885,13 +3853,13 @@
         <v>15</v>
       </c>
       <c r="B74" s="6" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="C74" s="6" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D74" s="7" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E74" s="1"/>
       <c r="G74" s="1"/>
@@ -3900,44 +3868,32 @@
       <c r="M74" s="1"/>
       <c r="N74" s="1"/>
     </row>
-    <row r="75" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A75" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B75" s="6" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="C75" s="6" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="D75" s="7" t="s">
-        <v>208</v>
-      </c>
-      <c r="E75" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F75" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="G75" s="1" t="s">
-        <v>48</v>
-      </c>
+      <c r="E75" s="1"/>
+      <c r="G75" s="1"/>
       <c r="I75" s="1"/>
       <c r="K75" s="1"/>
       <c r="M75" s="1"/>
-      <c r="N75" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="O75" s="1" t="s">
-        <v>24</v>
-      </c>
+      <c r="N75" s="1"/>
     </row>
     <row r="76" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A76" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B76" s="6" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="C76" s="6" t="s">
         <v>210</v>
@@ -3957,7 +3913,7 @@
         <v>15</v>
       </c>
       <c r="B77" s="6" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="C77" s="6" t="s">
         <v>212</v>
@@ -3977,7 +3933,7 @@
         <v>15</v>
       </c>
       <c r="B78" s="6" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="C78" s="6" t="s">
         <v>214</v>
@@ -3992,12 +3948,12 @@
       <c r="M78" s="1"/>
       <c r="N78" s="1"/>
     </row>
-    <row r="79" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A79" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B79" s="6" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="C79" s="6" t="s">
         <v>216</v>
@@ -4005,59 +3961,100 @@
       <c r="D79" s="7" t="s">
         <v>217</v>
       </c>
-      <c r="E79" s="1"/>
-      <c r="G79" s="1"/>
+      <c r="E79" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F79" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="G79" s="1" t="s">
+        <v>48</v>
+      </c>
       <c r="I79" s="1"/>
       <c r="K79" s="1"/>
       <c r="M79" s="1"/>
-      <c r="N79" s="1"/>
-    </row>
-    <row r="80" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N79" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="O79" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="80" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A80" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B80" s="6" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="C80" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="D80" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="E80" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F80" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="D80" s="7" t="s">
-        <v>219</v>
-      </c>
-      <c r="E80" s="1"/>
-      <c r="G80" s="1"/>
+      <c r="G80" s="1" t="s">
+        <v>21</v>
+      </c>
       <c r="I80" s="1"/>
       <c r="K80" s="1"/>
       <c r="M80" s="1"/>
-      <c r="N80" s="1"/>
-    </row>
-    <row r="81" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N80" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="O80" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="81" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A81" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B81" s="6" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="C81" s="6" t="s">
-        <v>220</v>
+        <v>102</v>
       </c>
       <c r="D81" s="7" t="s">
         <v>221</v>
       </c>
-      <c r="E81" s="1"/>
-      <c r="G81" s="1"/>
-      <c r="I81" s="1"/>
+      <c r="E81" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F81" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G81" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H81" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I81" s="1" t="s">
+        <v>23</v>
+      </c>
       <c r="K81" s="1"/>
       <c r="M81" s="1"/>
-      <c r="N81" s="1"/>
+      <c r="N81" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O81" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="82" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A82" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B82" s="6" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="C82" s="6" t="s">
         <v>222</v>
@@ -4066,129 +4063,52 @@
         <v>223</v>
       </c>
       <c r="E82" s="1" t="s">
-        <v>23</v>
+        <v>129</v>
       </c>
       <c r="F82" s="1" t="s">
-        <v>224</v>
+        <v>130</v>
       </c>
       <c r="G82" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="I82" s="1"/>
+        <v>129</v>
+      </c>
+      <c r="H82" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="I82" s="1" t="s">
+        <v>129</v>
+      </c>
       <c r="K82" s="1"/>
       <c r="M82" s="1"/>
       <c r="N82" s="1" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="O82" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="83" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A83" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B83" s="6" t="s">
-        <v>177</v>
-      </c>
-      <c r="C83" s="6" t="s">
-        <v>225</v>
-      </c>
-      <c r="D83" s="7" t="s">
-        <v>226</v>
-      </c>
-      <c r="E83" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F83" s="1" t="s">
-        <v>224</v>
-      </c>
-      <c r="G83" s="1" t="s">
-        <v>21</v>
-      </c>
+    <row r="83" spans="5:14" x14ac:dyDescent="0.25">
+      <c r="E83" s="1"/>
+      <c r="G83" s="1"/>
       <c r="I83" s="1"/>
       <c r="K83" s="1"/>
       <c r="M83" s="1"/>
-      <c r="N83" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="O83" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="84" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A84" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B84" s="6" t="s">
-        <v>177</v>
-      </c>
-      <c r="C84" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="D84" s="7" t="s">
-        <v>227</v>
-      </c>
-      <c r="E84" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F84" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="G84" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="H84" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="I84" s="1" t="s">
-        <v>23</v>
-      </c>
+      <c r="N83" s="1"/>
+    </row>
+    <row r="84" spans="5:14" x14ac:dyDescent="0.25">
+      <c r="E84" s="1"/>
+      <c r="G84" s="1"/>
+      <c r="I84" s="1"/>
       <c r="K84" s="1"/>
       <c r="M84" s="1"/>
-      <c r="N84" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="O84" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="85" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A85" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B85" s="6" t="s">
-        <v>177</v>
-      </c>
-      <c r="C85" s="6" t="s">
-        <v>228</v>
-      </c>
-      <c r="D85" s="7" t="s">
-        <v>229</v>
-      </c>
-      <c r="E85" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="F85" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="G85" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="H85" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="I85" s="1" t="s">
-        <v>135</v>
-      </c>
+      <c r="N84" s="1"/>
+    </row>
+    <row r="85" spans="5:14" x14ac:dyDescent="0.25">
+      <c r="E85" s="1"/>
+      <c r="G85" s="1"/>
+      <c r="I85" s="1"/>
       <c r="K85" s="1"/>
       <c r="M85" s="1"/>
-      <c r="N85" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="O85" s="1" t="s">
-        <v>24</v>
-      </c>
+      <c r="N85" s="1"/>
     </row>
     <row r="86" spans="5:14" x14ac:dyDescent="0.25">
       <c r="E86" s="1"/>
@@ -6566,33 +6486,9 @@
       <c r="M382" s="1"/>
       <c r="N382" s="1"/>
     </row>
-    <row r="383" spans="5:14" x14ac:dyDescent="0.25">
-      <c r="E383" s="1"/>
-      <c r="G383" s="1"/>
-      <c r="I383" s="1"/>
-      <c r="K383" s="1"/>
-      <c r="M383" s="1"/>
-      <c r="N383" s="1"/>
-    </row>
-    <row r="384" spans="5:14" x14ac:dyDescent="0.25">
-      <c r="E384" s="1"/>
-      <c r="G384" s="1"/>
-      <c r="I384" s="1"/>
-      <c r="K384" s="1"/>
-      <c r="M384" s="1"/>
-      <c r="N384" s="1"/>
-    </row>
-    <row r="385" spans="5:14" x14ac:dyDescent="0.25">
-      <c r="E385" s="1"/>
-      <c r="G385" s="1"/>
-      <c r="I385" s="1"/>
-      <c r="K385" s="1"/>
-      <c r="M385" s="1"/>
-      <c r="N385" s="1"/>
-    </row>
   </sheetData>
   <autoFilter ref="A1:O1"/>
-  <conditionalFormatting sqref="E2:E385">
+  <conditionalFormatting sqref="E2:E382">
     <cfRule type="containsText" dxfId="0" priority="1">
       <formula>NOT(ISERROR(SEARCH("BOT",E2)))</formula>
     </cfRule>
@@ -6612,7 +6508,7 @@
       <formula>NOT(ISERROR(SEARCH("NEUTRO",E2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G385">
+  <conditionalFormatting sqref="G2:G382">
     <cfRule type="containsText" dxfId="6" priority="1">
       <formula>NOT(ISERROR(SEARCH("BOT",G2)))</formula>
     </cfRule>
@@ -6632,7 +6528,7 @@
       <formula>NOT(ISERROR(SEARCH("NEUTRO",G2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I385">
+  <conditionalFormatting sqref="I2:I382">
     <cfRule type="containsText" dxfId="12" priority="1">
       <formula>NOT(ISERROR(SEARCH("BOT",I2)))</formula>
     </cfRule>
@@ -6652,7 +6548,7 @@
       <formula>NOT(ISERROR(SEARCH("NEUTRO",I2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K2:K385">
+  <conditionalFormatting sqref="K2:K382">
     <cfRule type="containsText" dxfId="18" priority="1">
       <formula>NOT(ISERROR(SEARCH("BOT",K2)))</formula>
     </cfRule>
@@ -6672,7 +6568,7 @@
       <formula>NOT(ISERROR(SEARCH("NEUTRO",K2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M2:M385">
+  <conditionalFormatting sqref="M2:M382">
     <cfRule type="containsText" dxfId="24" priority="1">
       <formula>NOT(ISERROR(SEARCH("BOT",M2)))</formula>
     </cfRule>
@@ -6693,40 +6589,40 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="12">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca do Móvel" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca do Móvel" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="E10:E385">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca do Móvel" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca do Móvel" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="E10:E382">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca do Móvel" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca do Móvel" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="E2:E385">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca do Móvel" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca do Móvel" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="E2:E382">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 1" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 1" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="G10:G385">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 1" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 1" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="G10:G382">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 1" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 1" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="G2:G385">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 1" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 1" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="G2:G382">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 2" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 2" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="I10:I385">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 2" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 2" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="I10:I382">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 2" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 2" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="I2:I385">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 2" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 2" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="I2:I382">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 3" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 3" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="K10:K385">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 3" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 3" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="K10:K382">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 3" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 3" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="K2:K385">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 3" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 3" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="K2:K382">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 4" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 4" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="M10:M385">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 4" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 4" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="M10:M382">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 4" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 4" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="M2:M385">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 4" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 4" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="M2:M382">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo" prompt="MOVIMENTO = Movimento definido nesta planta; FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo" error="MOVIMENTO = Movimento definido nesta planta; FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" sqref="N10:N385">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo" prompt="MOVIMENTO = Movimento definido nesta planta; FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo" error="MOVIMENTO = Movimento definido nesta planta; FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" sqref="N10:N382">
       <formula1>"MOVIMENTO,FIXO,EXPOSICAO,NOVO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo" prompt="MOVIMENTO = Movimento definido nesta planta; FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo" error="MOVIMENTO = Movimento definido nesta planta; FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" sqref="N2:N385">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo" prompt="MOVIMENTO = Movimento definido nesta planta; FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo" error="MOVIMENTO = Movimento definido nesta planta; FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" sqref="N2:N382">
       <formula1>"MOVIMENTO,FIXO,EXPOSICAO,NOVO"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6754,16 +6650,16 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -6771,13 +6667,13 @@
         <v>15</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>23</v>
@@ -6791,10 +6687,10 @@
         <v>15</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="D3" s="8" t="s">
         <v>69</v>
@@ -6811,13 +6707,13 @@
         <v>15</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>48</v>
@@ -6831,13 +6727,13 @@
         <v>15</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>21</v>
@@ -6851,10 +6747,10 @@
         <v>15</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
       <c r="D6" s="8" t="s">
         <v>65</v>
@@ -6871,13 +6767,13 @@
         <v>15</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="D7" s="8" t="s">
         <v>234</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>239</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>240</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>48</v>
@@ -6891,16 +6787,16 @@
         <v>15</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>24</v>
@@ -6911,13 +6807,13 @@
         <v>15</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>23</v>
@@ -6931,19 +6827,19 @@
         <v>15</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>23</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -6951,19 +6847,19 @@
         <v>15</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>21</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -6971,19 +6867,19 @@
         <v>15</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>48</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -6994,10 +6890,10 @@
         <v>16</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>24</v>
@@ -7014,10 +6910,10 @@
         <v>16</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>24</v>
@@ -7031,13 +6927,13 @@
         <v>15</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>24</v>
@@ -7051,13 +6947,13 @@
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>24</v>
@@ -7071,13 +6967,13 @@
         <v>15</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>24</v>
@@ -7091,13 +6987,13 @@
         <v>15</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>24</v>
@@ -7111,13 +7007,13 @@
         <v>15</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>24</v>
@@ -7131,13 +7027,13 @@
         <v>15</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>252</v>
+        <v>246</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>24</v>
@@ -7151,13 +7047,13 @@
         <v>15</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>24</v>
@@ -8409,7 +8305,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:D37"/>
+  <dimension ref="B1:D38"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -8420,277 +8316,284 @@
   <sheetData>
     <row r="1" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B1" s="9" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B2" s="10" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="C2" s="10"/>
       <c r="D2" s="10"/>
     </row>
     <row r="4" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B4" s="11" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B5" s="10" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="C5" s="10"/>
       <c r="D5" s="10"/>
     </row>
     <row r="6" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B6" s="10" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="C6" s="10"/>
       <c r="D6" s="10"/>
     </row>
     <row r="7" ht="16" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B7" s="10" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="C7" s="10"/>
       <c r="D7" s="10"/>
     </row>
     <row r="8" ht="45" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B8" s="10" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="C8" s="10"/>
       <c r="D8" s="10"/>
     </row>
     <row r="9" ht="16" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B9" s="10" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="C9" s="10"/>
       <c r="D9" s="10"/>
     </row>
     <row r="10" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B10" s="10" t="s">
-        <v>261</v>
+        <v>255</v>
       </c>
       <c r="C10" s="10"/>
       <c r="D10" s="10"/>
     </row>
     <row r="11" ht="60" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B11" s="10" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
       <c r="C11" s="10"/>
       <c r="D11" s="10"/>
     </row>
     <row r="12" ht="60" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B12" s="10" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="C12" s="10"/>
       <c r="D12" s="10"/>
     </row>
-    <row r="13" ht="75" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="13" ht="60" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B13" s="10" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="C13" s="10"/>
       <c r="D13" s="10"/>
     </row>
-    <row r="14" ht="60" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="14" ht="45" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B14" s="10" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
       <c r="C14" s="10"/>
       <c r="D14" s="10"/>
     </row>
-    <row r="15" ht="45" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="15" ht="60" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B15" s="10" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="C15" s="10"/>
       <c r="D15" s="10"/>
     </row>
     <row r="16" ht="45" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B16" s="10" t="s">
-        <v>267</v>
+        <v>261</v>
       </c>
       <c r="C16" s="10"/>
       <c r="D16" s="10"/>
     </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B18" s="11" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B19" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="C19" t="s">
-        <v>269</v>
-      </c>
-      <c r="D19" s="13" t="s">
-        <v>270</v>
+    <row r="17" ht="45" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B17" s="10" t="s">
+        <v>262</v>
+      </c>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+    </row>
+    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B19" s="11" t="s">
+        <v>263</v>
       </c>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B20" s="12" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="C20" t="s">
-        <v>271</v>
-      </c>
-      <c r="D20" s="14" t="s">
-        <v>272</v>
+        <v>264</v>
+      </c>
+      <c r="D20" s="13" t="s">
+        <v>265</v>
       </c>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B21" s="12" t="s">
-        <v>48</v>
+        <v>33</v>
       </c>
       <c r="C21" t="s">
-        <v>273</v>
-      </c>
-      <c r="D21" s="15" t="s">
-        <v>274</v>
+        <v>266</v>
+      </c>
+      <c r="D21" s="14" t="s">
+        <v>267</v>
       </c>
     </row>
     <row r="22" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B22" s="12" t="s">
-        <v>135</v>
+        <v>48</v>
       </c>
       <c r="C22" t="s">
-        <v>275</v>
-      </c>
-      <c r="D22" s="16" t="s">
-        <v>276</v>
+        <v>268</v>
+      </c>
+      <c r="D22" s="15" t="s">
+        <v>269</v>
       </c>
     </row>
     <row r="23" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B23" s="12" t="s">
-        <v>23</v>
+        <v>129</v>
       </c>
       <c r="C23" t="s">
-        <v>277</v>
-      </c>
-      <c r="D23" s="17" t="s">
-        <v>278</v>
+        <v>270</v>
+      </c>
+      <c r="D23" s="16" t="s">
+        <v>271</v>
       </c>
     </row>
     <row r="24" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B24" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C24" t="s">
+        <v>272</v>
+      </c>
+      <c r="D24" s="17" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="25" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B25" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="C24" t="s">
-        <v>279</v>
-      </c>
-      <c r="D24" s="18" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="26" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B26" s="11" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="27" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B27" s="12" t="s">
-        <v>116</v>
-      </c>
-      <c r="C27" t="s">
-        <v>282</v>
-      </c>
-      <c r="D27" t="s">
-        <v>283</v>
+      <c r="C25" t="s">
+        <v>274</v>
+      </c>
+      <c r="D25" s="18" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="27" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B27" s="11" t="s">
+        <v>276</v>
       </c>
     </row>
     <row r="28" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B28" s="12" t="s">
-        <v>30</v>
+        <v>110</v>
       </c>
       <c r="C28" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
       <c r="D28" t="s">
-        <v>285</v>
+        <v>278</v>
       </c>
     </row>
     <row r="29" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B29" s="12" t="s">
-        <v>137</v>
+        <v>30</v>
       </c>
       <c r="C29" t="s">
-        <v>286</v>
+        <v>279</v>
       </c>
       <c r="D29" t="s">
-        <v>287</v>
+        <v>280</v>
       </c>
     </row>
     <row r="30" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B30" s="12" t="s">
-        <v>288</v>
+        <v>131</v>
       </c>
       <c r="C30" t="s">
-        <v>289</v>
+        <v>281</v>
       </c>
       <c r="D30" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="32" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B32" s="11" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="33" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B33" s="12" t="s">
-        <v>235</v>
-      </c>
-      <c r="C33" t="s">
-        <v>292</v>
-      </c>
-      <c r="D33"/>
+        <v>282</v>
+      </c>
+    </row>
+    <row r="31" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B31" s="12" t="s">
+        <v>283</v>
+      </c>
+      <c r="C31" t="s">
+        <v>284</v>
+      </c>
+      <c r="D31" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="33" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B33" s="11" t="s">
+        <v>286</v>
+      </c>
     </row>
     <row r="34" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B34" s="12" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="C34" t="s">
-        <v>293</v>
+        <v>287</v>
       </c>
       <c r="D34"/>
     </row>
     <row r="35" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B35" s="12" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="C35" t="s">
-        <v>294</v>
+        <v>288</v>
       </c>
       <c r="D35"/>
     </row>
     <row r="36" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B36" s="12" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="C36" t="s">
-        <v>295</v>
+        <v>289</v>
       </c>
       <c r="D36"/>
     </row>
     <row r="37" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B37" s="12" t="s">
-        <v>247</v>
+        <v>237</v>
       </c>
       <c r="C37" t="s">
-        <v>296</v>
+        <v>290</v>
       </c>
       <c r="D37"/>
     </row>
+    <row r="38" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B38" s="12" t="s">
+        <v>241</v>
+      </c>
+      <c r="C38" t="s">
+        <v>291</v>
+      </c>
+      <c r="D38"/>
+    </row>
   </sheetData>
-  <mergeCells count="18">
+  <mergeCells count="19">
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="B6:D6"/>
@@ -8704,11 +8607,12 @@
     <mergeCell ref="B14:D14"/>
     <mergeCell ref="B15:D15"/>
     <mergeCell ref="B16:D16"/>
-    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="B17:D17"/>
     <mergeCell ref="C34:D34"/>
     <mergeCell ref="C35:D35"/>
     <mergeCell ref="C36:D36"/>
     <mergeCell ref="C37:D37"/>
+    <mergeCell ref="C38:D38"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Transferência de espaços entre plantas: Gôndola 2 (ER M) → Gôndola 3 (ER G/GG)
A partir da ER G, o lado B e o meio B da Gôndola 2 da ER M passam a ser o
lado A e o meio A da Gôndola 3; esses espaços da Gôndola 2 ficam livres
(brancos) para outros movimentos. Regra configurável em TRANSFERENCIAS
(Config.gs). Planilha base indica a origem e os espaços livres.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NsHPzcvz8rbUjBrgUMFTLU
</commit_message>
<xml_diff>
--- a/visualizador/Planilha base - Visualizador.xlsx
+++ b/visualizador/Planilha base - Visualizador.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="782" uniqueCount="292">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="787" uniqueCount="294">
   <si>
     <t>Ciclo</t>
   </si>
@@ -435,28 +435,31 @@
     <t>Móvel de fila 6 · vale para ER G, ER GG</t>
   </si>
   <si>
+    <t>Gôndola 2 – Meio B (inteiro, ou metade 1 se a metade 2 for preenchida) · ESPAÇO LIVRE: o que estava aqui na ER M foi para GONDOLA 3/MEIO-A; preencha com o novo movimento</t>
+  </si>
+  <si>
+    <t>Gôndola 2 – Lado B · ESPAÇO LIVRE: o que estava aqui na ER M foi para GONDOLA 3/LADO-A; preencha com o novo movimento</t>
+  </si>
+  <si>
     <t>GONDOLA 3</t>
   </si>
   <si>
     <t>Gôndola 3 (gôndola inteira; Etiqueta 1–4 = Lado A, Meio A, Meio B, Lado B) · vale para ER G, ER GG</t>
   </si>
   <si>
-    <t>CURTO PRAZO</t>
-  </si>
-  <si>
     <t>+PEC REGIONAL</t>
   </si>
   <si>
     <t>GONDOLA 3/LADO-A</t>
   </si>
   <si>
-    <t>Gôndola 3 – Lado A</t>
+    <t>Gôndola 3 – Lado A · VEM DE GONDOLA 2/LADO-B da ER M (preencha só para trocar)</t>
   </si>
   <si>
     <t>GONDOLA 3/MEIO-A</t>
   </si>
   <si>
-    <t>Gôndola 3 – Meio A (inteiro, ou metade 1 se a metade 2 for preenchida)</t>
+    <t>Gôndola 3 – Meio A (inteiro, ou metade 1 se a metade 2 for preenchida) · VEM DE GONDOLA 2/MEIO-B da ER M (preencha só para trocar)</t>
   </si>
   <si>
     <t>GONDOLA 3/MEIO-A-2</t>
@@ -765,7 +768,7 @@
     <t>Planilha base — Plano de Varejo</t>
   </si>
   <si>
-    <t>Gerada em 06/10/2026, 09:43:08 a partir do ciclo "Ciclo exemplo".</t>
+    <t>Gerada em 06/10/2026, 12:39:19 a partir do ciclo "Ciclo exemplo".</t>
   </si>
   <si>
     <t>Como preencher</t>
@@ -802,6 +805,9 @@
   </si>
   <si>
     <t>7. Na coluna "Planta" vale o nome (ex.: ER P) ou o número (01). Cascata: o que é definido numa planta vale também para as seguintes (ER P → ER M → ER G → ER GG), por isso cada móvel aparece uma vez só, na primeira planta que o tem ("vale para…" na coluna Móvel). Para mudar um móvel só a partir de uma planta, acrescente uma linha com o mesmo ID Móvel e essa planta. Planta = TODAS vale para todas.</t>
+  </si>
+  <si>
+    <t>7.1 Espaços que mudam de móvel na cascata: a partir da ER G, GONDOLA 3/LADO-A mostra o que GONDOLA 2/LADO-B tinha na ER M; a partir da ER G, GONDOLA 3/MEIO-A mostra o que GONDOLA 2/MEIO-B tinha na ER M. Nessas plantas o espaço de origem fica livre (branco): preencha a linha dele com o novo movimento. Uma linha própria do espaço de destino tem prioridade sobre a transferência.</t>
   </si>
   <si>
     <t>8. Todos os ciclos ficam nesta mesma planilha. Para criar um ciclo novo, copie as linhas de um ciclo existente (nas abas "Movimentos" e "Painéis"), cole no fim e troque o "Ciclo". Cada nome diferente de ciclo aparece no seletor do visualizador.</t>
@@ -1765,7 +1771,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O382"/>
+  <dimension ref="A1:O384"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="13" style="1" customWidth="1"/>
@@ -3135,7 +3141,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
         <v>15</v>
       </c>
@@ -3143,39 +3149,17 @@
         <v>137</v>
       </c>
       <c r="C44" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="D44" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="D44" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="E44" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F44" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="G44" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="H44" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="I44" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="J44" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="K44" s="1" t="s">
-        <v>23</v>
-      </c>
+      <c r="E44" s="1"/>
+      <c r="G44" s="1"/>
+      <c r="I44" s="1"/>
+      <c r="K44" s="1"/>
       <c r="M44" s="1"/>
-      <c r="N44" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="O44" s="1" t="s">
-        <v>24</v>
-      </c>
+      <c r="N44" s="1"/>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
@@ -3185,10 +3169,10 @@
         <v>137</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>144</v>
+        <v>121</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="E45" s="1"/>
       <c r="G45" s="1"/>
@@ -3197,7 +3181,7 @@
       <c r="M45" s="1"/>
       <c r="N45" s="1"/>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
         <v>15</v>
       </c>
@@ -3205,17 +3189,29 @@
         <v>137</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="E46" s="1"/>
+        <v>143</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>23</v>
+      </c>
       <c r="G46" s="1"/>
       <c r="I46" s="1"/>
-      <c r="K46" s="1"/>
+      <c r="J46" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="K46" s="1" t="s">
+        <v>23</v>
+      </c>
       <c r="M46" s="1"/>
-      <c r="N46" s="1"/>
+      <c r="N46" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="O46" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
@@ -3225,10 +3221,10 @@
         <v>137</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="E47" s="1"/>
       <c r="G47" s="1"/>
@@ -3245,10 +3241,10 @@
         <v>137</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="E48" s="1"/>
       <c r="G48" s="1"/>
@@ -3265,10 +3261,10 @@
         <v>137</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="D49" s="4" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="E49" s="1"/>
       <c r="G49" s="1"/>
@@ -3285,10 +3281,10 @@
         <v>137</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="E50" s="1"/>
       <c r="G50" s="1"/>
@@ -3305,10 +3301,10 @@
         <v>137</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="E51" s="1"/>
       <c r="G51" s="1"/>
@@ -3325,10 +3321,10 @@
         <v>137</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="E52" s="1"/>
       <c r="G52" s="1"/>
@@ -3337,7 +3333,7 @@
       <c r="M52" s="1"/>
       <c r="N52" s="1"/>
     </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
         <v>15</v>
       </c>
@@ -3345,31 +3341,19 @@
         <v>137</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="E53" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="F53" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="G53" s="1" t="s">
-        <v>33</v>
-      </c>
+        <v>158</v>
+      </c>
+      <c r="E53" s="1"/>
+      <c r="G53" s="1"/>
       <c r="I53" s="1"/>
       <c r="K53" s="1"/>
       <c r="M53" s="1"/>
-      <c r="N53" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="O53" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N53" s="1"/>
+    </row>
+    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
         <v>15</v>
       </c>
@@ -3377,24 +3361,17 @@
         <v>137</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="D54" s="4" t="s">
-        <v>163</v>
-      </c>
-      <c r="E54" s="1" t="s">
-        <v>23</v>
-      </c>
+        <v>160</v>
+      </c>
+      <c r="E54" s="1"/>
       <c r="G54" s="1"/>
       <c r="I54" s="1"/>
       <c r="K54" s="1"/>
       <c r="M54" s="1"/>
-      <c r="N54" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="O54" s="1" t="s">
-        <v>24</v>
-      </c>
+      <c r="N54" s="1"/>
     </row>
     <row r="55" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
@@ -3404,19 +3381,19 @@
         <v>137</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="D55" s="4" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="I55" s="1"/>
       <c r="K55" s="1"/>
@@ -3436,20 +3413,15 @@
         <v>137</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="D56" s="4" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="E56" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F56" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="G56" s="1" t="s">
-        <v>23</v>
-      </c>
+      <c r="G56" s="1"/>
       <c r="I56" s="1"/>
       <c r="K56" s="1"/>
       <c r="M56" s="1"/>
@@ -3468,19 +3440,19 @@
         <v>137</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="D57" s="4" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>48</v>
+        <v>21</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>48</v>
+        <v>21</v>
       </c>
       <c r="I57" s="1"/>
       <c r="K57" s="1"/>
@@ -3493,89 +3465,113 @@
       </c>
     </row>
     <row r="58" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A58" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B58" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="C58" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="D58" s="7" t="s">
-        <v>173</v>
+      <c r="A58" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B58" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="C58" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="D58" s="4" t="s">
+        <v>168</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>129</v>
+        <v>23</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>129</v>
+        <v>23</v>
       </c>
       <c r="I58" s="1"/>
       <c r="K58" s="1"/>
       <c r="M58" s="1"/>
       <c r="N58" s="1" t="s">
-        <v>110</v>
+        <v>24</v>
       </c>
       <c r="O58" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A59" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B59" s="6" t="s">
+    <row r="59" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A59" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="C59" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="D59" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="C59" s="6" t="s">
-        <v>175</v>
-      </c>
-      <c r="D59" s="7" t="s">
-        <v>176</v>
-      </c>
-      <c r="E59" s="1"/>
-      <c r="G59" s="1"/>
+      <c r="E59" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F59" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="G59" s="1" t="s">
+        <v>48</v>
+      </c>
       <c r="I59" s="1"/>
       <c r="K59" s="1"/>
       <c r="M59" s="1"/>
-      <c r="N59" s="1"/>
-    </row>
-    <row r="60" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N59" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O59" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="60" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A60" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B60" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D60" s="7" t="s">
-        <v>178</v>
-      </c>
-      <c r="E60" s="1"/>
-      <c r="G60" s="1"/>
+        <v>174</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="F60" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="G60" s="1" t="s">
+        <v>129</v>
+      </c>
       <c r="I60" s="1"/>
       <c r="K60" s="1"/>
       <c r="M60" s="1"/>
-      <c r="N60" s="1"/>
+      <c r="N60" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="O60" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A61" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B61" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="D61" s="7" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="E61" s="1"/>
       <c r="G61" s="1"/>
@@ -3589,13 +3585,13 @@
         <v>15</v>
       </c>
       <c r="B62" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="D62" s="7" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="E62" s="1"/>
       <c r="G62" s="1"/>
@@ -3609,13 +3605,13 @@
         <v>15</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="D63" s="7" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="E63" s="1"/>
       <c r="G63" s="1"/>
@@ -3629,13 +3625,13 @@
         <v>15</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="D64" s="7" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="E64" s="1"/>
       <c r="G64" s="1"/>
@@ -3644,50 +3640,38 @@
       <c r="M64" s="1"/>
       <c r="N64" s="1"/>
     </row>
-    <row r="65" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A65" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="D65" s="7" t="s">
-        <v>188</v>
-      </c>
-      <c r="E65" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="F65" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="G65" s="1" t="s">
-        <v>33</v>
-      </c>
+        <v>185</v>
+      </c>
+      <c r="E65" s="1"/>
+      <c r="G65" s="1"/>
       <c r="I65" s="1"/>
       <c r="K65" s="1"/>
       <c r="M65" s="1"/>
-      <c r="N65" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="O65" s="1" t="s">
-        <v>24</v>
-      </c>
+      <c r="N65" s="1"/>
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A66" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="D66" s="7" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="E66" s="1"/>
       <c r="G66" s="1"/>
@@ -3696,38 +3680,50 @@
       <c r="M66" s="1"/>
       <c r="N66" s="1"/>
     </row>
-    <row r="67" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A67" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="D67" s="7" t="s">
-        <v>192</v>
-      </c>
-      <c r="E67" s="1"/>
-      <c r="G67" s="1"/>
+        <v>189</v>
+      </c>
+      <c r="E67" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F67" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G67" s="1" t="s">
+        <v>33</v>
+      </c>
       <c r="I67" s="1"/>
       <c r="K67" s="1"/>
       <c r="M67" s="1"/>
-      <c r="N67" s="1"/>
+      <c r="N67" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O67" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="68" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A68" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="D68" s="7" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="E68" s="1"/>
       <c r="G68" s="1"/>
@@ -3741,13 +3737,13 @@
         <v>15</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="D69" s="7" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="E69" s="1"/>
       <c r="G69" s="1"/>
@@ -3761,13 +3757,13 @@
         <v>15</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C70" s="6" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D70" s="7" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="E70" s="1"/>
       <c r="G70" s="1"/>
@@ -3781,13 +3777,13 @@
         <v>15</v>
       </c>
       <c r="B71" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C71" s="6" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="D71" s="7" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="E71" s="1"/>
       <c r="G71" s="1"/>
@@ -3796,50 +3792,38 @@
       <c r="M71" s="1"/>
       <c r="N71" s="1"/>
     </row>
-    <row r="72" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A72" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C72" s="6" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="D72" s="7" t="s">
-        <v>202</v>
-      </c>
-      <c r="E72" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F72" s="1" t="s">
-        <v>203</v>
-      </c>
-      <c r="G72" s="1" t="s">
-        <v>48</v>
-      </c>
+        <v>199</v>
+      </c>
+      <c r="E72" s="1"/>
+      <c r="G72" s="1"/>
       <c r="I72" s="1"/>
       <c r="K72" s="1"/>
       <c r="M72" s="1"/>
-      <c r="N72" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="O72" s="1" t="s">
-        <v>24</v>
-      </c>
+      <c r="N72" s="1"/>
     </row>
     <row r="73" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A73" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B73" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C73" s="6" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="D73" s="7" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="E73" s="1"/>
       <c r="G73" s="1"/>
@@ -3848,38 +3832,50 @@
       <c r="M73" s="1"/>
       <c r="N73" s="1"/>
     </row>
-    <row r="74" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A74" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B74" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C74" s="6" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="D74" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="E74" s="1"/>
-      <c r="G74" s="1"/>
+        <v>203</v>
+      </c>
+      <c r="E74" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F74" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="G74" s="1" t="s">
+        <v>48</v>
+      </c>
       <c r="I74" s="1"/>
       <c r="K74" s="1"/>
       <c r="M74" s="1"/>
-      <c r="N74" s="1"/>
+      <c r="N74" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="O74" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="75" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A75" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B75" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C75" s="6" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="D75" s="7" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="E75" s="1"/>
       <c r="G75" s="1"/>
@@ -3893,13 +3889,13 @@
         <v>15</v>
       </c>
       <c r="B76" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C76" s="6" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="D76" s="7" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="E76" s="1"/>
       <c r="G76" s="1"/>
@@ -3913,13 +3909,13 @@
         <v>15</v>
       </c>
       <c r="B77" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C77" s="6" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="D77" s="7" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="E77" s="1"/>
       <c r="G77" s="1"/>
@@ -3933,13 +3929,13 @@
         <v>15</v>
       </c>
       <c r="B78" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C78" s="6" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="D78" s="7" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="E78" s="1"/>
       <c r="G78" s="1"/>
@@ -3948,102 +3944,73 @@
       <c r="M78" s="1"/>
       <c r="N78" s="1"/>
     </row>
-    <row r="79" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A79" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B79" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C79" s="6" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="D79" s="7" t="s">
-        <v>217</v>
-      </c>
-      <c r="E79" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F79" s="1" t="s">
-        <v>218</v>
-      </c>
-      <c r="G79" s="1" t="s">
-        <v>48</v>
-      </c>
+        <v>214</v>
+      </c>
+      <c r="E79" s="1"/>
+      <c r="G79" s="1"/>
       <c r="I79" s="1"/>
       <c r="K79" s="1"/>
       <c r="M79" s="1"/>
-      <c r="N79" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="O79" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="80" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N79" s="1"/>
+    </row>
+    <row r="80" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A80" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B80" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C80" s="6" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="D80" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="E80" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F80" s="1" t="s">
-        <v>218</v>
-      </c>
-      <c r="G80" s="1" t="s">
-        <v>21</v>
-      </c>
+        <v>216</v>
+      </c>
+      <c r="E80" s="1"/>
+      <c r="G80" s="1"/>
       <c r="I80" s="1"/>
       <c r="K80" s="1"/>
       <c r="M80" s="1"/>
-      <c r="N80" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="O80" s="1" t="s">
-        <v>24</v>
-      </c>
+      <c r="N80" s="1"/>
     </row>
     <row r="81" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A81" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B81" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C81" s="6" t="s">
-        <v>102</v>
+        <v>217</v>
       </c>
       <c r="D81" s="7" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="F81" s="1" t="s">
-        <v>20</v>
+        <v>219</v>
       </c>
       <c r="G81" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="H81" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="I81" s="1" t="s">
-        <v>23</v>
-      </c>
+        <v>48</v>
+      </c>
+      <c r="I81" s="1"/>
       <c r="K81" s="1"/>
       <c r="M81" s="1"/>
       <c r="N81" s="1" t="s">
-        <v>24</v>
+        <v>110</v>
       </c>
       <c r="O81" s="1" t="s">
         <v>24</v>
@@ -4054,53 +4021,106 @@
         <v>15</v>
       </c>
       <c r="B82" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C82" s="6" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="D82" s="7" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="E82" s="1" t="s">
-        <v>129</v>
+        <v>21</v>
       </c>
       <c r="F82" s="1" t="s">
-        <v>130</v>
+        <v>219</v>
       </c>
       <c r="G82" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="H82" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="I82" s="1" t="s">
-        <v>129</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="I82" s="1"/>
       <c r="K82" s="1"/>
       <c r="M82" s="1"/>
       <c r="N82" s="1" t="s">
-        <v>131</v>
+        <v>110</v>
       </c>
       <c r="O82" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="83" spans="5:14" x14ac:dyDescent="0.25">
-      <c r="E83" s="1"/>
-      <c r="G83" s="1"/>
-      <c r="I83" s="1"/>
+    <row r="83" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A83" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B83" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="C83" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="D83" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="E83" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F83" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G83" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H83" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I83" s="1" t="s">
+        <v>23</v>
+      </c>
       <c r="K83" s="1"/>
       <c r="M83" s="1"/>
-      <c r="N83" s="1"/>
-    </row>
-    <row r="84" spans="5:14" x14ac:dyDescent="0.25">
-      <c r="E84" s="1"/>
-      <c r="G84" s="1"/>
-      <c r="I84" s="1"/>
+      <c r="N83" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O83" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="84" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A84" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B84" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="C84" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="D84" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="E84" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="F84" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="G84" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="H84" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="I84" s="1" t="s">
+        <v>129</v>
+      </c>
       <c r="K84" s="1"/>
       <c r="M84" s="1"/>
-      <c r="N84" s="1"/>
+      <c r="N84" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="O84" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="85" spans="5:14" x14ac:dyDescent="0.25">
       <c r="E85" s="1"/>
@@ -6486,9 +6506,25 @@
       <c r="M382" s="1"/>
       <c r="N382" s="1"/>
     </row>
+    <row r="383" spans="5:14" x14ac:dyDescent="0.25">
+      <c r="E383" s="1"/>
+      <c r="G383" s="1"/>
+      <c r="I383" s="1"/>
+      <c r="K383" s="1"/>
+      <c r="M383" s="1"/>
+      <c r="N383" s="1"/>
+    </row>
+    <row r="384" spans="5:14" x14ac:dyDescent="0.25">
+      <c r="E384" s="1"/>
+      <c r="G384" s="1"/>
+      <c r="I384" s="1"/>
+      <c r="K384" s="1"/>
+      <c r="M384" s="1"/>
+      <c r="N384" s="1"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O1"/>
-  <conditionalFormatting sqref="E2:E382">
+  <conditionalFormatting sqref="E2:E384">
     <cfRule type="containsText" dxfId="0" priority="1">
       <formula>NOT(ISERROR(SEARCH("BOT",E2)))</formula>
     </cfRule>
@@ -6508,7 +6544,7 @@
       <formula>NOT(ISERROR(SEARCH("NEUTRO",E2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G382">
+  <conditionalFormatting sqref="G2:G384">
     <cfRule type="containsText" dxfId="6" priority="1">
       <formula>NOT(ISERROR(SEARCH("BOT",G2)))</formula>
     </cfRule>
@@ -6528,7 +6564,7 @@
       <formula>NOT(ISERROR(SEARCH("NEUTRO",G2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I382">
+  <conditionalFormatting sqref="I2:I384">
     <cfRule type="containsText" dxfId="12" priority="1">
       <formula>NOT(ISERROR(SEARCH("BOT",I2)))</formula>
     </cfRule>
@@ -6548,7 +6584,7 @@
       <formula>NOT(ISERROR(SEARCH("NEUTRO",I2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K2:K382">
+  <conditionalFormatting sqref="K2:K384">
     <cfRule type="containsText" dxfId="18" priority="1">
       <formula>NOT(ISERROR(SEARCH("BOT",K2)))</formula>
     </cfRule>
@@ -6568,7 +6604,7 @@
       <formula>NOT(ISERROR(SEARCH("NEUTRO",K2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M2:M382">
+  <conditionalFormatting sqref="M2:M384">
     <cfRule type="containsText" dxfId="24" priority="1">
       <formula>NOT(ISERROR(SEARCH("BOT",M2)))</formula>
     </cfRule>
@@ -6589,40 +6625,40 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="12">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca do Móvel" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca do Móvel" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="E10:E382">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca do Móvel" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca do Móvel" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="E10:E384">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca do Móvel" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca do Móvel" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="E2:E382">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca do Móvel" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca do Móvel" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="E2:E384">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 1" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 1" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="G10:G382">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 1" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 1" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="G10:G384">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 1" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 1" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="G2:G382">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 1" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 1" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="G2:G384">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 2" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 2" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="I10:I382">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 2" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 2" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="I10:I384">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 2" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 2" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="I2:I382">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 2" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 2" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="I2:I384">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 3" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 3" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="K10:K382">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 3" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 3" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="K10:K384">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 3" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 3" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="K2:K382">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 3" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 3" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="K2:K384">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 4" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 4" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="M10:M382">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 4" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 4" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="M10:M384">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 4" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 4" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="M2:M382">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 4" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 4" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="M2:M384">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo" prompt="MOVIMENTO = Movimento definido nesta planta; FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo" error="MOVIMENTO = Movimento definido nesta planta; FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" sqref="N10:N382">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo" prompt="MOVIMENTO = Movimento definido nesta planta; FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo" error="MOVIMENTO = Movimento definido nesta planta; FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" sqref="N10:N384">
       <formula1>"MOVIMENTO,FIXO,EXPOSICAO,NOVO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo" prompt="MOVIMENTO = Movimento definido nesta planta; FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo" error="MOVIMENTO = Movimento definido nesta planta; FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" sqref="N2:N382">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo" prompt="MOVIMENTO = Movimento definido nesta planta; FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo" error="MOVIMENTO = Movimento definido nesta planta; FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" sqref="N2:N384">
       <formula1>"MOVIMENTO,FIXO,EXPOSICAO,NOVO"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6650,16 +6686,16 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -6667,13 +6703,13 @@
         <v>15</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>23</v>
@@ -6687,10 +6723,10 @@
         <v>15</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D3" s="8" t="s">
         <v>69</v>
@@ -6707,13 +6743,13 @@
         <v>15</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>48</v>
@@ -6727,10 +6763,10 @@
         <v>15</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D5" s="8" t="s">
         <v>75</v>
@@ -6747,10 +6783,10 @@
         <v>15</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D6" s="8" t="s">
         <v>65</v>
@@ -6767,13 +6803,13 @@
         <v>15</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>48</v>
@@ -6787,13 +6823,13 @@
         <v>15</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>129</v>
@@ -6807,13 +6843,13 @@
         <v>15</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>23</v>
@@ -6827,13 +6863,13 @@
         <v>15</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>23</v>
@@ -6847,13 +6883,13 @@
         <v>15</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>21</v>
@@ -6867,13 +6903,13 @@
         <v>15</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>48</v>
@@ -6890,10 +6926,10 @@
         <v>16</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>24</v>
@@ -6910,10 +6946,10 @@
         <v>16</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>24</v>
@@ -6930,10 +6966,10 @@
         <v>105</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>24</v>
@@ -6950,10 +6986,10 @@
         <v>105</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>24</v>
@@ -6970,10 +7006,10 @@
         <v>137</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>24</v>
@@ -6990,10 +7026,10 @@
         <v>137</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>24</v>
@@ -7007,13 +7043,13 @@
         <v>15</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>24</v>
@@ -7027,13 +7063,13 @@
         <v>15</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>24</v>
@@ -7047,13 +7083,13 @@
         <v>15</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>24</v>
@@ -8305,7 +8341,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:D38"/>
+  <dimension ref="B1:D39"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -8316,202 +8352,198 @@
   <sheetData>
     <row r="1" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B1" s="9" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B2" s="10" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C2" s="10"/>
       <c r="D2" s="10"/>
     </row>
     <row r="4" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B4" s="11" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B5" s="10" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C5" s="10"/>
       <c r="D5" s="10"/>
     </row>
     <row r="6" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B6" s="10" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C6" s="10"/>
       <c r="D6" s="10"/>
     </row>
     <row r="7" ht="16" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B7" s="10" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C7" s="10"/>
       <c r="D7" s="10"/>
     </row>
     <row r="8" ht="45" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B8" s="10" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C8" s="10"/>
       <c r="D8" s="10"/>
     </row>
     <row r="9" ht="16" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B9" s="10" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C9" s="10"/>
       <c r="D9" s="10"/>
     </row>
     <row r="10" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B10" s="10" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C10" s="10"/>
       <c r="D10" s="10"/>
     </row>
     <row r="11" ht="60" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B11" s="10" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C11" s="10"/>
       <c r="D11" s="10"/>
     </row>
     <row r="12" ht="60" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B12" s="10" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C12" s="10"/>
       <c r="D12" s="10"/>
     </row>
     <row r="13" ht="60" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B13" s="10" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C13" s="10"/>
       <c r="D13" s="10"/>
     </row>
     <row r="14" ht="45" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B14" s="10" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C14" s="10"/>
       <c r="D14" s="10"/>
     </row>
     <row r="15" ht="60" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B15" s="10" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C15" s="10"/>
       <c r="D15" s="10"/>
     </row>
-    <row r="16" ht="45" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="16" ht="60" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B16" s="10" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C16" s="10"/>
       <c r="D16" s="10"/>
     </row>
     <row r="17" ht="45" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B17" s="10" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C17" s="10"/>
       <c r="D17" s="10"/>
     </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B19" s="11" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B20" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="C20" t="s">
+    <row r="18" ht="45" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B18" s="10" t="s">
         <v>264</v>
       </c>
-      <c r="D20" s="13" t="s">
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+    </row>
+    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B20" s="11" t="s">
         <v>265</v>
       </c>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B21" s="12" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="C21" t="s">
         <v>266</v>
       </c>
-      <c r="D21" s="14" t="s">
+      <c r="D21" s="13" t="s">
         <v>267</v>
       </c>
     </row>
     <row r="22" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B22" s="12" t="s">
-        <v>48</v>
+        <v>33</v>
       </c>
       <c r="C22" t="s">
         <v>268</v>
       </c>
-      <c r="D22" s="15" t="s">
+      <c r="D22" s="14" t="s">
         <v>269</v>
       </c>
     </row>
     <row r="23" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B23" s="12" t="s">
-        <v>129</v>
+        <v>48</v>
       </c>
       <c r="C23" t="s">
         <v>270</v>
       </c>
-      <c r="D23" s="16" t="s">
+      <c r="D23" s="15" t="s">
         <v>271</v>
       </c>
     </row>
     <row r="24" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B24" s="12" t="s">
-        <v>23</v>
+        <v>129</v>
       </c>
       <c r="C24" t="s">
         <v>272</v>
       </c>
-      <c r="D24" s="17" t="s">
+      <c r="D24" s="16" t="s">
         <v>273</v>
       </c>
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B25" s="12" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C25" t="s">
         <v>274</v>
       </c>
-      <c r="D25" s="18" t="s">
+      <c r="D25" s="17" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="27" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B27" s="11" t="s">
+    <row r="26" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B26" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C26" t="s">
         <v>276</v>
       </c>
-    </row>
-    <row r="28" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B28" s="12" t="s">
-        <v>110</v>
-      </c>
-      <c r="C28" t="s">
+      <c r="D26" s="18" t="s">
         <v>277</v>
       </c>
-      <c r="D28" t="s">
+    </row>
+    <row r="28" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B28" s="11" t="s">
         <v>278</v>
       </c>
     </row>
     <row r="29" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B29" s="12" t="s">
-        <v>30</v>
+        <v>110</v>
       </c>
       <c r="C29" t="s">
         <v>279</v>
@@ -8522,7 +8554,7 @@
     </row>
     <row r="30" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B30" s="12" t="s">
-        <v>131</v>
+        <v>30</v>
       </c>
       <c r="C30" t="s">
         <v>281</v>
@@ -8533,67 +8565,78 @@
     </row>
     <row r="31" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B31" s="12" t="s">
+        <v>131</v>
+      </c>
+      <c r="C31" t="s">
         <v>283</v>
       </c>
-      <c r="C31" t="s">
+      <c r="D31" t="s">
         <v>284</v>
       </c>
-      <c r="D31" t="s">
+    </row>
+    <row r="32" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B32" s="12" t="s">
         <v>285</v>
       </c>
-    </row>
-    <row r="33" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B33" s="11" t="s">
+      <c r="C32" t="s">
         <v>286</v>
       </c>
-    </row>
-    <row r="34" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B34" s="12" t="s">
-        <v>229</v>
-      </c>
-      <c r="C34" t="s">
+      <c r="D32" t="s">
         <v>287</v>
       </c>
-      <c r="D34"/>
+    </row>
+    <row r="34" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B34" s="11" t="s">
+        <v>288</v>
+      </c>
     </row>
     <row r="35" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B35" s="12" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C35" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D35"/>
     </row>
     <row r="36" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B36" s="12" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C36" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D36"/>
     </row>
     <row r="37" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B37" s="12" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="C37" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D37"/>
     </row>
     <row r="38" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B38" s="12" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="C38" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="D38"/>
     </row>
+    <row r="39" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B39" s="12" t="s">
+        <v>242</v>
+      </c>
+      <c r="C39" t="s">
+        <v>293</v>
+      </c>
+      <c r="D39"/>
+    </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="20">
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="B6:D6"/>
@@ -8608,11 +8651,12 @@
     <mergeCell ref="B15:D15"/>
     <mergeCell ref="B16:D16"/>
     <mergeCell ref="B17:D17"/>
-    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="B18:D18"/>
     <mergeCell ref="C35:D35"/>
     <mergeCell ref="C36:D36"/>
     <mergeCell ref="C37:D37"/>
     <mergeCell ref="C38:D38"/>
+    <mergeCell ref="C39:D39"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Transferência Gôndola 2 → Gôndola 3 também com linhas próprias nas plantas maiores
O destino (Gôndola 3 lado A / meio A na ER G e ER GG) recebe sempre o conteúdo
da origem na ER M, mesmo com linha própria; e a origem descarta o que repete o
movimento transferido, para ele não aparecer nos dois móveis. Versão 2026.10.06-4.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NsHPzcvz8rbUjBrgUMFTLU
</commit_message>
<xml_diff>
--- a/visualizador/Planilha base - Visualizador.xlsx
+++ b/visualizador/Planilha base - Visualizador.xlsx
@@ -339,13 +339,13 @@
     <t>GONDOLA 3/LADO-A</t>
   </si>
   <si>
-    <t>Gôndola 3 – Lado A · VEM DE GONDOLA 2/LADO-B da ER M (preencha só para trocar)</t>
+    <t>Gôndola 3 – Lado A · VEM DE GONDOLA 2/LADO-B da ER M (automático: para mudar, mude a GONDOLA 2/LADO-B na ER M)</t>
   </si>
   <si>
     <t>GONDOLA 3/MEIO-A</t>
   </si>
   <si>
-    <t>Gôndola 3 – Meio A (inteiro, ou metade 1 se a metade 2 for preenchida) · VEM DE GONDOLA 2/MEIO-B da ER M (preencha só para trocar)</t>
+    <t>Gôndola 3 – Meio A (inteiro, ou metade 1 se a metade 2 for preenchida) · VEM DE GONDOLA 2/MEIO-B da ER M (automático: para mudar, mude a GONDOLA 2/MEIO-B na ER M)</t>
   </si>
   <si>
     <t>GONDOLA 3/MEIO-A-2</t>
@@ -576,7 +576,7 @@
     <t>Planilha base — Plano de Varejo</t>
   </si>
   <si>
-    <t>Gerada em 06/10/2026, 12:51:21 (em branco).</t>
+    <t>Gerada em 06/10/2026, 13:05:45 (em branco).</t>
   </si>
   <si>
     <t>Como preencher</t>
@@ -615,7 +615,7 @@
     <t>7. Na coluna "Planta" vale o nome (ex.: ER P) ou o número (01). Cascata: o que é definido numa planta vale também para as seguintes (ER P → ER M → ER G → ER GG), por isso cada móvel aparece uma vez só, na primeira planta que o tem ("vale para…" na coluna Móvel). Para mudar um móvel só a partir de uma planta, acrescente uma linha com o mesmo ID Móvel e essa planta. Planta = TODAS vale para todas.</t>
   </si>
   <si>
-    <t>7.1 Espaços que mudam de móvel na cascata: a partir da ER G, GONDOLA 3/LADO-A mostra o que GONDOLA 2/LADO-B tinha na ER M; a partir da ER G, GONDOLA 3/MEIO-A mostra o que GONDOLA 2/MEIO-B tinha na ER M. Nessas plantas o espaço de origem fica livre (branco): preencha a linha dele com o novo movimento. Uma linha própria do espaço de destino tem prioridade sobre a transferência.</t>
+    <t>7.1 Espaços que mudam de móvel na cascata: a partir da ER G, GONDOLA 3/LADO-A mostra o que GONDOLA 2/LADO-B tinha na ER M; a partir da ER G, GONDOLA 3/MEIO-A mostra o que GONDOLA 2/MEIO-B tinha na ER M. Nessas plantas o espaço de destino recebe sempre o conteúdo da planta anterior (a linha própria dele só vale se a origem estiver vazia) e o espaço de origem fica livre (branco): preencha a linha dele com o novo movimento. Se a linha da planta maior repetir o movimento que foi transferido, ele é ignorado ali, para não aparecer nos dois móveis.</t>
   </si>
   <si>
     <t>8. Todos os ciclos ficam nesta mesma planilha. No primeiro ciclo, preencha o "Ciclo" nas linhas já prontas (linhas sem ciclo e sem conteúdo são ignoradas). Para criar um ciclo novo, copie as linhas de um ciclo existente (nas abas "Movimentos" e "Painéis"), cole no fim e troque o "Ciclo". Cada nome diferente de ciclo aparece no seletor do visualizador.</t>
@@ -7247,7 +7247,7 @@
       <c r="C15" s="9"/>
       <c r="D15" s="9"/>
     </row>
-    <row r="16" ht="60" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="16" ht="75" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B16" s="9" t="s">
         <v>200</v>
       </c>

</xml_diff>

<commit_message>
Móveis com espaços preenchidos só por espaço (sem linha do móvel inteiro)
- Gôndola, mesas destaque, totem e móvel make: só valem as linhas dos espaços
  (lados/meios, frentes, painéis, testeiras); espaço sem linha fica branco. A linha
  do móvel inteiro é ignorada na leitura, com aviso. Móveis de um espaço só e o
  balcão continuam com uma linha.
- Planta, dica, espaço por marca, tela do móvel e planograma sem a herança do
  móvel inteiro; corpo do móvel make fica sem marca.
- Planilha base: uma linha por espaço (o totem passa a ter PAINEL-1 a 3) e
  instruções atualizadas; ciclo de exemplo convertido (VERSAO_EXEMPLO 7).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QG98EBYtnpUCaCwXswk4sP
</commit_message>
<xml_diff>
--- a/visualizador/Planilha base - Visualizador.xlsx
+++ b/visualizador/Planilha base - Visualizador.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="782" uniqueCount="292">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="797" uniqueCount="278">
   <si>
     <t>Ciclo</t>
   </si>
@@ -90,69 +90,63 @@
     <t/>
   </si>
   <si>
-    <t>GONDOLA 1</t>
-  </si>
-  <si>
-    <t>Gôndola 1 (gôndola inteira; Etiqueta 1–4 = Lado A, Meio A, Meio B, Lado B) · vale para ER P, ER M, ER G, ER GG</t>
+    <t>GONDOLA 1/LADO-A</t>
+  </si>
+  <si>
+    <t>Gôndola 1 – Lado A · vale para ER P, ER M, ER G, ER GG</t>
+  </si>
+  <si>
+    <t>QDB</t>
+  </si>
+  <si>
+    <t>LIQUIDA QDB</t>
+  </si>
+  <si>
+    <t>JUICY MOOD</t>
+  </si>
+  <si>
+    <t>GONDOLA 1/MEIO-A</t>
+  </si>
+  <si>
+    <t>Gôndola 1 – Meio A (ou metade 1, se a metade 2 for preenchida)</t>
   </si>
   <si>
     <t>BOTIK</t>
   </si>
   <si>
+    <t>FIXO</t>
+  </si>
+  <si>
+    <t>GONDOLA 1/MEIO-A-2</t>
+  </si>
+  <si>
+    <t>Gôndola 1 – Meio A – metade 2 (preencha só para dividir o meio em dois)</t>
+  </si>
+  <si>
+    <t>GONDOLA 1/MEIO-B</t>
+  </si>
+  <si>
+    <t>Gôndola 1 – Meio B (ou metade 1, se a metade 2 for preenchida)</t>
+  </si>
+  <si>
     <t>UOMINI HERO</t>
   </si>
   <si>
+    <t>GONDOLA 1/MEIO-B-2</t>
+  </si>
+  <si>
+    <t>Gôndola 1 – Meio B – metade 2 (preencha só para dividir o meio em dois)</t>
+  </si>
+  <si>
+    <t>GONDOLA 1/LADO-B</t>
+  </si>
+  <si>
+    <t>Gôndola 1 – Lado B</t>
+  </si>
+  <si>
     <t>BOTI PROMO</t>
   </si>
   <si>
-    <t>FIXO</t>
-  </si>
-  <si>
-    <t>GONDOLA 1/LADO-A</t>
-  </si>
-  <si>
-    <t>Gôndola 1 – Lado A</t>
-  </si>
-  <si>
-    <t>QDB</t>
-  </si>
-  <si>
-    <t>LIQUIDA QDB</t>
-  </si>
-  <si>
-    <t>JUICY MOOD</t>
-  </si>
-  <si>
-    <t>GONDOLA 1/MEIO-A</t>
-  </si>
-  <si>
-    <t>Gôndola 1 – Meio A (inteiro, ou metade 1 se a metade 2 for preenchida)</t>
-  </si>
-  <si>
-    <t>GONDOLA 1/MEIO-A-2</t>
-  </si>
-  <si>
-    <t>Gôndola 1 – Meio A – metade 2 (preencha só para dividir o meio em dois)</t>
-  </si>
-  <si>
-    <t>GONDOLA 1/MEIO-B</t>
-  </si>
-  <si>
-    <t>Gôndola 1 – Meio B (inteiro, ou metade 1 se a metade 2 for preenchida)</t>
-  </si>
-  <si>
-    <t>GONDOLA 1/MEIO-B-2</t>
-  </si>
-  <si>
-    <t>Gôndola 1 – Meio B – metade 2 (preencha só para dividir o meio em dois)</t>
-  </si>
-  <si>
-    <t>GONDOLA 1/LADO-B</t>
-  </si>
-  <si>
-    <t>Gôndola 1 – Lado B</t>
-  </si>
-  <si>
     <t>PIRAMIDE 1</t>
   </si>
   <si>
@@ -171,16 +165,10 @@
     <t>PRINCIPAIS OPORTUNIDADES</t>
   </si>
   <si>
-    <t>MESA DESTAQUE 1</t>
-  </si>
-  <si>
-    <t>Mesa destaque 1 · vale para ER P, ER M</t>
-  </si>
-  <si>
     <t>MESA DESTAQUE 1/FRENTE-1</t>
   </si>
   <si>
-    <t>Mesa destaque 1 – Frente 1</t>
+    <t>Mesa destaque 1 – Frente 1 · vale para ER P, ER M</t>
   </si>
   <si>
     <t>UOMINI GLORIFICADO</t>
@@ -234,15 +222,27 @@
     <t>OUTLET EUD</t>
   </si>
   <si>
-    <t>TOTEM 1</t>
-  </si>
-  <si>
-    <t>Totem 1 (Etiqueta 1–3 = painel de cima, do meio e de baixo; Marca Etiqueta N = cor do painel N) · vale para ER P, ER M, ER G, ER GG</t>
+    <t>TOTEM 1/PAINEL-1</t>
+  </si>
+  <si>
+    <t>Totem 1 – Painel 1 · vale para ER P, ER M, ER G, ER GG</t>
   </si>
   <si>
     <t>LÇTO UOMINI</t>
   </si>
   <si>
+    <t>TOTEM 1/PAINEL-2</t>
+  </si>
+  <si>
+    <t>Totem 1 – Painel 2</t>
+  </si>
+  <si>
+    <t>TOTEM 1/PAINEL-3</t>
+  </si>
+  <si>
+    <t>Totem 1 – Painel 3</t>
+  </si>
+  <si>
     <t>EXTRA-CESTINHAS</t>
   </si>
   <si>
@@ -267,469 +267,427 @@
     <t>Cavalete · vale para ER P, ER M, ER G, ER GG</t>
   </si>
   <si>
+    <t>MOVEL MAKE 1/TESTEIRA-1</t>
+  </si>
+  <si>
+    <t>Móvel make 1 – Testeira 1 · vale para ER P, ER M, ER G, ER GG</t>
+  </si>
+  <si>
+    <t>#1F1F1F</t>
+  </si>
+  <si>
+    <t>MOVEL MAKE 1/TESTEIRA-2</t>
+  </si>
+  <si>
+    <t>Móvel make 1 – Testeira 2</t>
+  </si>
+  <si>
+    <t>MOVEL MAKE 1/TESTEIRA-3</t>
+  </si>
+  <si>
+    <t>Móvel make 1 – Testeira 3</t>
+  </si>
+  <si>
+    <t>MOVEL MAKE 1/TESTEIRA-4</t>
+  </si>
+  <si>
+    <t>Móvel make 1 – Testeira 4</t>
+  </si>
+  <si>
+    <t>MOVEL DE PAREDE 2</t>
+  </si>
+  <si>
+    <t>Móvel de parede 2 · vale para ER P, ER M, ER G, ER GG</t>
+  </si>
+  <si>
+    <t>PERF MASC</t>
+  </si>
+  <si>
+    <t>MOVEL DE PAREDE 3</t>
+  </si>
+  <si>
+    <t>Móvel de parede 3 · vale para ER P, ER M, ER G, ER GG</t>
+  </si>
+  <si>
+    <t>CUIDADOS (CBEM)</t>
+  </si>
+  <si>
+    <t>MOVEL DE PAREDE 4</t>
+  </si>
+  <si>
+    <t>Móvel de parede 4 · vale para ER P, ER M, ER G, ER GG</t>
+  </si>
+  <si>
+    <t>PERF FEM</t>
+  </si>
+  <si>
+    <t>ER M</t>
+  </si>
+  <si>
+    <t>GONDOLA 2/LADO-A</t>
+  </si>
+  <si>
+    <t>Gôndola 2 – Lado A · vale para ER M, ER G, ER GG</t>
+  </si>
+  <si>
+    <t>GONDOLA 2/MEIO-A</t>
+  </si>
+  <si>
+    <t>Gôndola 2 – Meio A (ou metade 1, se a metade 2 for preenchida)</t>
+  </si>
+  <si>
+    <t>PERFUMARIA</t>
+  </si>
+  <si>
+    <t>MOVIMENTO</t>
+  </si>
+  <si>
+    <t>GONDOLA 2/MEIO-A-2</t>
+  </si>
+  <si>
+    <t>Gôndola 2 – Meio A – metade 2 (preencha só para dividir o meio em dois)</t>
+  </si>
+  <si>
+    <t>GONDOLA 2/MEIO-B</t>
+  </si>
+  <si>
+    <t>Gôndola 2 – Meio B (ou metade 1, se a metade 2 for preenchida)</t>
+  </si>
+  <si>
+    <t>CUIDADOS</t>
+  </si>
+  <si>
+    <t>GONDOLA 2/MEIO-B-2</t>
+  </si>
+  <si>
+    <t>Gôndola 2 – Meio B – metade 2 (preencha só para dividir o meio em dois)</t>
+  </si>
+  <si>
+    <t>GONDOLA 2/LADO-B</t>
+  </si>
+  <si>
+    <t>Gôndola 2 – Lado B</t>
+  </si>
+  <si>
+    <t>MOVEL DE FILA 3</t>
+  </si>
+  <si>
+    <t>Móvel de fila 3 · vale para ER M, ER G, ER GG</t>
+  </si>
+  <si>
+    <t>MOVEL DE FILA 4</t>
+  </si>
+  <si>
+    <t>Móvel de fila 4 · vale para ER M, ER G, ER GG</t>
+  </si>
+  <si>
+    <t>PAREDE OUI 1</t>
+  </si>
+  <si>
+    <t>Parede O.U.i 1 · vale para ER M, ER G</t>
+  </si>
+  <si>
+    <t>OUI</t>
+  </si>
+  <si>
+    <t>MON AMIE + LOÇÃO</t>
+  </si>
+  <si>
+    <t>EXPOSICAO</t>
+  </si>
+  <si>
+    <t>TOTEM OUI 1</t>
+  </si>
+  <si>
+    <t>Totem O.U.i 1 · vale para ER M, ER G, ER GG</t>
+  </si>
+  <si>
+    <t>Hôtel de Ville 193</t>
+  </si>
+  <si>
+    <t>PIRAMIDE 3</t>
+  </si>
+  <si>
+    <t>Pirâmide 3 · vale para ER M, ER G, ER GG</t>
+  </si>
+  <si>
+    <t>ER G</t>
+  </si>
+  <si>
+    <t>MOVEL DE FILA 6</t>
+  </si>
+  <si>
+    <t>Móvel de fila 6 · vale para ER G, ER GG</t>
+  </si>
+  <si>
+    <t>GONDOLA 3/LADO-A</t>
+  </si>
+  <si>
+    <t>Gôndola 3 – Lado A · vale para ER G, ER GG</t>
+  </si>
+  <si>
+    <t>GONDOLA 3/MEIO-A</t>
+  </si>
+  <si>
+    <t>Gôndola 3 – Meio A (ou metade 1, se a metade 2 for preenchida)</t>
+  </si>
+  <si>
+    <t>CURTO PRAZO</t>
+  </si>
+  <si>
+    <t>GONDOLA 3/MEIO-A-2</t>
+  </si>
+  <si>
+    <t>Gôndola 3 – Meio A – metade 2 (preencha só para dividir o meio em dois)</t>
+  </si>
+  <si>
+    <t>GONDOLA 3/MEIO-B</t>
+  </si>
+  <si>
+    <t>Gôndola 3 – Meio B (ou metade 1, se a metade 2 for preenchida)</t>
+  </si>
+  <si>
+    <t>+PEC REGIONAL</t>
+  </si>
+  <si>
+    <t>GONDOLA 3/MEIO-B-2</t>
+  </si>
+  <si>
+    <t>Gôndola 3 – Meio B – metade 2 (preencha só para dividir o meio em dois)</t>
+  </si>
+  <si>
+    <t>GONDOLA 3/LADO-B</t>
+  </si>
+  <si>
+    <t>Gôndola 3 – Lado B</t>
+  </si>
+  <si>
+    <t>MOVEL DE FILA 7</t>
+  </si>
+  <si>
+    <t>Móvel de fila 7 · vale para ER G, ER GG</t>
+  </si>
+  <si>
+    <t>MOVEL DE FILA 5</t>
+  </si>
+  <si>
+    <t>Móvel de fila 5 · vale para ER G, ER GG</t>
+  </si>
+  <si>
+    <t>MOVEL DE FILA 8</t>
+  </si>
+  <si>
+    <t>Móvel de fila 8 · vale para ER G, ER GG</t>
+  </si>
+  <si>
+    <t>MESA DESTAQUE 3 FRENTES 1/FRENTE-1</t>
+  </si>
+  <si>
+    <t>Mesa destaque 3 frentes 1 – Frente 1 · vale para ER G, ER GG</t>
+  </si>
+  <si>
+    <t>MESA DESTAQUE 3 FRENTES 1/FRENTE-2</t>
+  </si>
+  <si>
+    <t>Mesa destaque 3 frentes 1 – Frente 2</t>
+  </si>
+  <si>
+    <t>VM PERMANENTE MULTI PROMO</t>
+  </si>
+  <si>
+    <t>MESA DESTAQUE 3 FRENTES 1/FRENTE-3</t>
+  </si>
+  <si>
+    <t>Mesa destaque 3 frentes 1 – Frente 3</t>
+  </si>
+  <si>
+    <t>ER GG</t>
+  </si>
+  <si>
+    <t>GONDOLA 4/LADO-A</t>
+  </si>
+  <si>
+    <t>Gôndola 4 – Lado A</t>
+  </si>
+  <si>
+    <t>EXAUSTÃO OUI</t>
+  </si>
+  <si>
+    <t>GONDOLA 4/MEIO-A</t>
+  </si>
+  <si>
+    <t>Gôndola 4 – Meio A (ou metade 1, se a metade 2 for preenchida)</t>
+  </si>
+  <si>
+    <t>GONDOLA 4/MEIO-A-2</t>
+  </si>
+  <si>
+    <t>Gôndola 4 – Meio A – metade 2 (preencha só para dividir o meio em dois)</t>
+  </si>
+  <si>
+    <t>GONDOLA 4/MEIO-B</t>
+  </si>
+  <si>
+    <t>Gôndola 4 – Meio B (ou metade 1, se a metade 2 for preenchida)</t>
+  </si>
+  <si>
+    <t>GONDOLA 4/MEIO-B-2</t>
+  </si>
+  <si>
+    <t>Gôndola 4 – Meio B – metade 2 (preencha só para dividir o meio em dois)</t>
+  </si>
+  <si>
+    <t>GONDOLA 4/LADO-B</t>
+  </si>
+  <si>
+    <t>Gôndola 4 – Lado B</t>
+  </si>
+  <si>
+    <t>GONDOLA 5/LADO-A</t>
+  </si>
+  <si>
+    <t>Gôndola 5 – Lado A</t>
+  </si>
+  <si>
+    <t>GONDOLA 5/MEIO-A</t>
+  </si>
+  <si>
+    <t>Gôndola 5 – Meio A (ou metade 1, se a metade 2 for preenchida)</t>
+  </si>
+  <si>
+    <t>GONDOLA 5/MEIO-A-2</t>
+  </si>
+  <si>
+    <t>Gôndola 5 – Meio A – metade 2 (preencha só para dividir o meio em dois)</t>
+  </si>
+  <si>
+    <t>GONDOLA 5/MEIO-B</t>
+  </si>
+  <si>
+    <t>Gôndola 5 – Meio B (ou metade 1, se a metade 2 for preenchida)</t>
+  </si>
+  <si>
+    <t>GONDOLA 5/MEIO-B-2</t>
+  </si>
+  <si>
+    <t>Gôndola 5 – Meio B – metade 2 (preencha só para dividir o meio em dois)</t>
+  </si>
+  <si>
+    <t>GONDOLA 5/LADO-B</t>
+  </si>
+  <si>
+    <t>Gôndola 5 – Lado B</t>
+  </si>
+  <si>
+    <t>GONDOLA 6/LADO-A</t>
+  </si>
+  <si>
+    <t>Gôndola 6 – Lado A</t>
+  </si>
+  <si>
+    <t>EXAUSTÃO EUD</t>
+  </si>
+  <si>
+    <t>GONDOLA 6/MEIO-A</t>
+  </si>
+  <si>
+    <t>Gôndola 6 – Meio A (ou metade 1, se a metade 2 for preenchida)</t>
+  </si>
+  <si>
+    <t>GONDOLA 6/MEIO-A-2</t>
+  </si>
+  <si>
+    <t>Gôndola 6 – Meio A – metade 2 (preencha só para dividir o meio em dois)</t>
+  </si>
+  <si>
+    <t>GONDOLA 6/MEIO-B</t>
+  </si>
+  <si>
+    <t>Gôndola 6 – Meio B (ou metade 1, se a metade 2 for preenchida)</t>
+  </si>
+  <si>
+    <t>GONDOLA 6/MEIO-B-2</t>
+  </si>
+  <si>
+    <t>Gôndola 6 – Meio B – metade 2 (preencha só para dividir o meio em dois)</t>
+  </si>
+  <si>
+    <t>GONDOLA 6/LADO-B</t>
+  </si>
+  <si>
+    <t>Gôndola 6 – Lado B</t>
+  </si>
+  <si>
+    <t>PIRAMIDE 4</t>
+  </si>
+  <si>
+    <t>Pirâmide 4</t>
+  </si>
+  <si>
+    <t>ISCAS EXAUSTÃO</t>
+  </si>
+  <si>
+    <t>PIRAMIDE 5</t>
+  </si>
+  <si>
+    <t>Pirâmide 5</t>
+  </si>
+  <si>
+    <t>Móvel de parede 4</t>
+  </si>
+  <si>
+    <t>ILHA PREMIUM OUI 1</t>
+  </si>
+  <si>
+    <t>Ilha premium O.U.i 1</t>
+  </si>
+  <si>
+    <t>Seção</t>
+  </si>
+  <si>
+    <t>Texto</t>
+  </si>
+  <si>
+    <t>Marca</t>
+  </si>
+  <si>
+    <t>Aponta para (ID Móvel)</t>
+  </si>
+  <si>
+    <t>TODAS</t>
+  </si>
+  <si>
+    <t>TV</t>
+  </si>
+  <si>
+    <t>GRADE CURTO PRAZO</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>OUTLET EUDORA</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>LÇTO SIÀGE</t>
+  </si>
+  <si>
+    <t>LÇTO MON AMIE</t>
+  </si>
+  <si>
+    <t>COMUNICAÇÃO INSTITUCIONAL PERMANENTE (3)</t>
+  </si>
+  <si>
+    <t>CALLOUT</t>
+  </si>
+  <si>
+    <t>TESTEIRA MAKE MULTIPROMO - BOTI COM BOTIPROMO MAKE.B EUDORA COM OUTLET E QDB COM LIQUIDA</t>
+  </si>
+  <si>
     <t>MOVEL MAKE 1</t>
-  </si>
-  <si>
-    <t>Móvel make 1 · vale para ER P, ER M, ER G, ER GG</t>
-  </si>
-  <si>
-    <t>TESTEIRA MAKE MULTIPROMO</t>
-  </si>
-  <si>
-    <t>MOVEL MAKE 1/TESTEIRA-1</t>
-  </si>
-  <si>
-    <t>Móvel make 1 – Testeira 1</t>
-  </si>
-  <si>
-    <t>#1F1F1F</t>
-  </si>
-  <si>
-    <t>MOVEL MAKE 1/TESTEIRA-2</t>
-  </si>
-  <si>
-    <t>Móvel make 1 – Testeira 2</t>
-  </si>
-  <si>
-    <t>MOVEL MAKE 1/TESTEIRA-3</t>
-  </si>
-  <si>
-    <t>Móvel make 1 – Testeira 3</t>
-  </si>
-  <si>
-    <t>MOVEL MAKE 1/TESTEIRA-4</t>
-  </si>
-  <si>
-    <t>Móvel make 1 – Testeira 4</t>
-  </si>
-  <si>
-    <t>MOVEL DE PAREDE 2</t>
-  </si>
-  <si>
-    <t>Móvel de parede 2 · vale para ER P, ER M, ER G, ER GG</t>
-  </si>
-  <si>
-    <t>PERF MASC</t>
-  </si>
-  <si>
-    <t>MOVEL DE PAREDE 3</t>
-  </si>
-  <si>
-    <t>Móvel de parede 3 · vale para ER P, ER M, ER G, ER GG</t>
-  </si>
-  <si>
-    <t>CUIDADOS (CBEM)</t>
-  </si>
-  <si>
-    <t>MOVEL DE PAREDE 4</t>
-  </si>
-  <si>
-    <t>Móvel de parede 4 · vale para ER P, ER M, ER G, ER GG</t>
-  </si>
-  <si>
-    <t>PERF FEM</t>
-  </si>
-  <si>
-    <t>ER M</t>
-  </si>
-  <si>
-    <t>GONDOLA 2</t>
-  </si>
-  <si>
-    <t>Gôndola 2 (gôndola inteira; Etiqueta 1–4 = Lado A, Meio A, Meio B, Lado B) · vale para ER M, ER G, ER GG</t>
-  </si>
-  <si>
-    <t>PERFUMARIA</t>
-  </si>
-  <si>
-    <t>CUIDADOS</t>
-  </si>
-  <si>
-    <t>MOVIMENTO</t>
-  </si>
-  <si>
-    <t>GONDOLA 2/LADO-A</t>
-  </si>
-  <si>
-    <t>Gôndola 2 – Lado A</t>
-  </si>
-  <si>
-    <t>GONDOLA 2/MEIO-A</t>
-  </si>
-  <si>
-    <t>Gôndola 2 – Meio A (inteiro, ou metade 1 se a metade 2 for preenchida)</t>
-  </si>
-  <si>
-    <t>GONDOLA 2/MEIO-A-2</t>
-  </si>
-  <si>
-    <t>Gôndola 2 – Meio A – metade 2 (preencha só para dividir o meio em dois)</t>
-  </si>
-  <si>
-    <t>GONDOLA 2/MEIO-B</t>
-  </si>
-  <si>
-    <t>Gôndola 2 – Meio B (inteiro, ou metade 1 se a metade 2 for preenchida)</t>
-  </si>
-  <si>
-    <t>GONDOLA 2/MEIO-B-2</t>
-  </si>
-  <si>
-    <t>Gôndola 2 – Meio B – metade 2 (preencha só para dividir o meio em dois)</t>
-  </si>
-  <si>
-    <t>GONDOLA 2/LADO-B</t>
-  </si>
-  <si>
-    <t>Gôndola 2 – Lado B</t>
-  </si>
-  <si>
-    <t>MOVEL DE FILA 3</t>
-  </si>
-  <si>
-    <t>Móvel de fila 3 · vale para ER M, ER G, ER GG</t>
-  </si>
-  <si>
-    <t>MOVEL DE FILA 4</t>
-  </si>
-  <si>
-    <t>Móvel de fila 4 · vale para ER M, ER G, ER GG</t>
-  </si>
-  <si>
-    <t>PAREDE OUI 1</t>
-  </si>
-  <si>
-    <t>Parede O.U.i 1 · vale para ER M, ER G</t>
-  </si>
-  <si>
-    <t>OUI</t>
-  </si>
-  <si>
-    <t>MON AMIE + LOÇÃO</t>
-  </si>
-  <si>
-    <t>EXPOSICAO</t>
-  </si>
-  <si>
-    <t>TOTEM OUI 1</t>
-  </si>
-  <si>
-    <t>Totem O.U.i 1 · vale para ER M, ER G, ER GG</t>
-  </si>
-  <si>
-    <t>Hôtel de Ville 193</t>
-  </si>
-  <si>
-    <t>PIRAMIDE 3</t>
-  </si>
-  <si>
-    <t>Pirâmide 3 · vale para ER M, ER G, ER GG</t>
-  </si>
-  <si>
-    <t>ER G</t>
-  </si>
-  <si>
-    <t>MOVEL DE FILA 6</t>
-  </si>
-  <si>
-    <t>Móvel de fila 6 · vale para ER G, ER GG</t>
-  </si>
-  <si>
-    <t>GONDOLA 3</t>
-  </si>
-  <si>
-    <t>Gôndola 3 (gôndola inteira; Etiqueta 1–4 = Lado A, Meio A, Meio B, Lado B) · vale para ER G, ER GG</t>
-  </si>
-  <si>
-    <t>CURTO PRAZO</t>
-  </si>
-  <si>
-    <t>+PEC REGIONAL</t>
-  </si>
-  <si>
-    <t>GONDOLA 3/LADO-A</t>
-  </si>
-  <si>
-    <t>Gôndola 3 – Lado A</t>
-  </si>
-  <si>
-    <t>GONDOLA 3/MEIO-A</t>
-  </si>
-  <si>
-    <t>Gôndola 3 – Meio A (inteiro, ou metade 1 se a metade 2 for preenchida)</t>
-  </si>
-  <si>
-    <t>GONDOLA 3/MEIO-A-2</t>
-  </si>
-  <si>
-    <t>Gôndola 3 – Meio A – metade 2 (preencha só para dividir o meio em dois)</t>
-  </si>
-  <si>
-    <t>GONDOLA 3/MEIO-B</t>
-  </si>
-  <si>
-    <t>Gôndola 3 – Meio B (inteiro, ou metade 1 se a metade 2 for preenchida)</t>
-  </si>
-  <si>
-    <t>GONDOLA 3/MEIO-B-2</t>
-  </si>
-  <si>
-    <t>Gôndola 3 – Meio B – metade 2 (preencha só para dividir o meio em dois)</t>
-  </si>
-  <si>
-    <t>GONDOLA 3/LADO-B</t>
-  </si>
-  <si>
-    <t>Gôndola 3 – Lado B</t>
-  </si>
-  <si>
-    <t>MOVEL DE FILA 7</t>
-  </si>
-  <si>
-    <t>Móvel de fila 7 · vale para ER G, ER GG</t>
-  </si>
-  <si>
-    <t>MOVEL DE FILA 5</t>
-  </si>
-  <si>
-    <t>Móvel de fila 5 · vale para ER G, ER GG</t>
-  </si>
-  <si>
-    <t>MOVEL DE FILA 8</t>
-  </si>
-  <si>
-    <t>Móvel de fila 8 · vale para ER G, ER GG</t>
-  </si>
-  <si>
-    <t>MESA DESTAQUE 3 FRENTES 1</t>
-  </si>
-  <si>
-    <t>Mesa destaque 3 frentes 1 · vale para ER G, ER GG</t>
-  </si>
-  <si>
-    <t>MESA DESTAQUE 3 FRENTES 1/FRENTE-1</t>
-  </si>
-  <si>
-    <t>Mesa destaque 3 frentes 1 – Frente 1</t>
-  </si>
-  <si>
-    <t>MESA DESTAQUE 3 FRENTES 1/FRENTE-2</t>
-  </si>
-  <si>
-    <t>Mesa destaque 3 frentes 1 – Frente 2</t>
-  </si>
-  <si>
-    <t>VM PERMANENTE MULTI PROMO</t>
-  </si>
-  <si>
-    <t>MESA DESTAQUE 3 FRENTES 1/FRENTE-3</t>
-  </si>
-  <si>
-    <t>Mesa destaque 3 frentes 1 – Frente 3</t>
-  </si>
-  <si>
-    <t>ER GG</t>
-  </si>
-  <si>
-    <t>GONDOLA 4</t>
-  </si>
-  <si>
-    <t>Gôndola 4 (gôndola inteira; Etiqueta 1–4 = Lado A, Meio A, Meio B, Lado B)</t>
-  </si>
-  <si>
-    <t>EXAUSTÃO OUI</t>
-  </si>
-  <si>
-    <t>GONDOLA 4/LADO-A</t>
-  </si>
-  <si>
-    <t>Gôndola 4 – Lado A</t>
-  </si>
-  <si>
-    <t>GONDOLA 4/MEIO-A</t>
-  </si>
-  <si>
-    <t>Gôndola 4 – Meio A (inteiro, ou metade 1 se a metade 2 for preenchida)</t>
-  </si>
-  <si>
-    <t>GONDOLA 4/MEIO-A-2</t>
-  </si>
-  <si>
-    <t>Gôndola 4 – Meio A – metade 2 (preencha só para dividir o meio em dois)</t>
-  </si>
-  <si>
-    <t>GONDOLA 4/MEIO-B</t>
-  </si>
-  <si>
-    <t>Gôndola 4 – Meio B (inteiro, ou metade 1 se a metade 2 for preenchida)</t>
-  </si>
-  <si>
-    <t>GONDOLA 4/MEIO-B-2</t>
-  </si>
-  <si>
-    <t>Gôndola 4 – Meio B – metade 2 (preencha só para dividir o meio em dois)</t>
-  </si>
-  <si>
-    <t>GONDOLA 4/LADO-B</t>
-  </si>
-  <si>
-    <t>Gôndola 4 – Lado B</t>
-  </si>
-  <si>
-    <t>GONDOLA 5</t>
-  </si>
-  <si>
-    <t>Gôndola 5 (gôndola inteira; Etiqueta 1–4 = Lado A, Meio A, Meio B, Lado B)</t>
-  </si>
-  <si>
-    <t>GONDOLA 5/LADO-A</t>
-  </si>
-  <si>
-    <t>Gôndola 5 – Lado A</t>
-  </si>
-  <si>
-    <t>GONDOLA 5/MEIO-A</t>
-  </si>
-  <si>
-    <t>Gôndola 5 – Meio A (inteiro, ou metade 1 se a metade 2 for preenchida)</t>
-  </si>
-  <si>
-    <t>GONDOLA 5/MEIO-A-2</t>
-  </si>
-  <si>
-    <t>Gôndola 5 – Meio A – metade 2 (preencha só para dividir o meio em dois)</t>
-  </si>
-  <si>
-    <t>GONDOLA 5/MEIO-B</t>
-  </si>
-  <si>
-    <t>Gôndola 5 – Meio B (inteiro, ou metade 1 se a metade 2 for preenchida)</t>
-  </si>
-  <si>
-    <t>GONDOLA 5/MEIO-B-2</t>
-  </si>
-  <si>
-    <t>Gôndola 5 – Meio B – metade 2 (preencha só para dividir o meio em dois)</t>
-  </si>
-  <si>
-    <t>GONDOLA 5/LADO-B</t>
-  </si>
-  <si>
-    <t>Gôndola 5 – Lado B</t>
-  </si>
-  <si>
-    <t>GONDOLA 6</t>
-  </si>
-  <si>
-    <t>Gôndola 6 (gôndola inteira; Etiqueta 1–4 = Lado A, Meio A, Meio B, Lado B)</t>
-  </si>
-  <si>
-    <t>EXAUSTÃO EUD</t>
-  </si>
-  <si>
-    <t>GONDOLA 6/LADO-A</t>
-  </si>
-  <si>
-    <t>Gôndola 6 – Lado A</t>
-  </si>
-  <si>
-    <t>GONDOLA 6/MEIO-A</t>
-  </si>
-  <si>
-    <t>Gôndola 6 – Meio A (inteiro, ou metade 1 se a metade 2 for preenchida)</t>
-  </si>
-  <si>
-    <t>GONDOLA 6/MEIO-A-2</t>
-  </si>
-  <si>
-    <t>Gôndola 6 – Meio A – metade 2 (preencha só para dividir o meio em dois)</t>
-  </si>
-  <si>
-    <t>GONDOLA 6/MEIO-B</t>
-  </si>
-  <si>
-    <t>Gôndola 6 – Meio B (inteiro, ou metade 1 se a metade 2 for preenchida)</t>
-  </si>
-  <si>
-    <t>GONDOLA 6/MEIO-B-2</t>
-  </si>
-  <si>
-    <t>Gôndola 6 – Meio B – metade 2 (preencha só para dividir o meio em dois)</t>
-  </si>
-  <si>
-    <t>GONDOLA 6/LADO-B</t>
-  </si>
-  <si>
-    <t>Gôndola 6 – Lado B</t>
-  </si>
-  <si>
-    <t>PIRAMIDE 4</t>
-  </si>
-  <si>
-    <t>Pirâmide 4</t>
-  </si>
-  <si>
-    <t>ISCAS EXAUSTÃO</t>
-  </si>
-  <si>
-    <t>PIRAMIDE 5</t>
-  </si>
-  <si>
-    <t>Pirâmide 5</t>
-  </si>
-  <si>
-    <t>Móvel de parede 4</t>
-  </si>
-  <si>
-    <t>ILHA PREMIUM OUI 1</t>
-  </si>
-  <si>
-    <t>Ilha premium O.U.i 1</t>
-  </si>
-  <si>
-    <t>Seção</t>
-  </si>
-  <si>
-    <t>Texto</t>
-  </si>
-  <si>
-    <t>Marca</t>
-  </si>
-  <si>
-    <t>Aponta para (ID Móvel)</t>
-  </si>
-  <si>
-    <t>TODAS</t>
-  </si>
-  <si>
-    <t>TV</t>
-  </si>
-  <si>
-    <t>GRADE CURTO PRAZO</t>
-  </si>
-  <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>OUTLET EUDORA</t>
-  </si>
-  <si>
-    <t>C</t>
-  </si>
-  <si>
-    <t>LÇTO SIÀGE</t>
-  </si>
-  <si>
-    <t>LÇTO MON AMIE</t>
-  </si>
-  <si>
-    <t>COMUNICAÇÃO INSTITUCIONAL PERMANENTE (3)</t>
-  </si>
-  <si>
-    <t>CALLOUT</t>
-  </si>
-  <si>
-    <t>TESTEIRA MAKE MULTIPROMO - BOTI COM BOTIPROMO MAKE.B EUDORA COM OUTLET E QDB COM LIQUIDA</t>
   </si>
   <si>
     <t xml:space="preserve">- MATERIAIS COMPLEMENTARES PARA BOTIPROMO DESTACANDO AS ISCAS COMERCIAIS: “ATÉ 52% DE DD” / “ITENS A PARTIR DE”.
@@ -765,7 +723,7 @@
     <t>Planilha base — Plano de Varejo</t>
   </si>
   <si>
-    <t>Gerada em 06/10/2026, 09:43:08 a partir do ciclo "Ciclo exemplo".</t>
+    <t>Gerada em 08/10/2026, 22:39:28 a partir do ciclo "Ciclo exemplo".</t>
   </si>
   <si>
     <t>Como preencher</t>
@@ -777,10 +735,10 @@
     <t>2. Preencha "Ciclo" em todas as linhas com o nome do ciclo (ex.: C15/2026). É esse nome que aparece no seletor de ciclos.</t>
   </si>
   <si>
-    <t>3. "Marca do Móvel" define a cor do móvel na planta. Deixe vazio (ou NEUTRO) para o móvel aparecer branco.</t>
-  </si>
-  <si>
-    <t>4. "Etiqueta 1…4" são as caixas de texto do móvel; "Marca Etiqueta N" define a cor de cada uma (vazio = cor do móvel). Pirâmide e mesa destaque mostram até 4 etiquetas, empilhadas (as colunas que não aparecem na planta ficam cinza).</t>
+    <t>3. "Marca do Móvel" define a cor do móvel (ou do espaço) na planta. Deixe vazio (ou NEUTRO) para ele aparecer branco.</t>
+  </si>
+  <si>
+    <t>4. "Etiqueta 1…4" são as caixas de texto; "Marca Etiqueta N" define a cor de cada uma (vazio = cor da linha). Pirâmide e cada espaço da gôndola e das mesas mostram até 4 etiquetas, empilhadas (as colunas que não aparecem na planta ficam cinza).</t>
   </si>
   <si>
     <t>5. "Símbolo" é opcional e aparece ao lado da primeira etiqueta (tabela abaixo).</t>
@@ -789,16 +747,16 @@
     <t>6. Na aba "Painéis" ficam os textos fora dos móveis: listas TV / A / C, caixas de destaque (CALLOUT, que podem apontar para um ID Móvel) e notas (NOTA).</t>
   </si>
   <si>
-    <t>6.1 Gôndolas têm uma linha para a gôndola inteira e uma por espaço (ex.: GONDOLA 1/LADO-A, GONDOLA 1/MEIO-A). Espaço preenchido tem prioridade; espaço vazio usa a linha da gôndola inteira (para deixar um espaço branco, use NEUTRO). Para dividir um meio em dois movimentos, preencha também a linha da metade 2 (ex.: GONDOLA 1/MEIO-A-2): a linha do meio passa a valer para a metade 1 e a planta mostra o meio dividido.</t>
-  </si>
-  <si>
-    <t>6.2 Etiquetas da gôndola. Na linha da gôndola inteira: Etiqueta 1 = Lado A, Etiqueta 2 = Meio A, Etiqueta 3 = Meio B, Etiqueta 4 = Lado B ("A" é sempre o lado virado para quem olha a planta). A linha de um espaço mostra até 4 etiquetas empilhadas em cima daquele bloco (Etiqueta 1 a 4) e substitui a etiqueta que viria da gôndola inteira.</t>
-  </si>
-  <si>
-    <t>6.3 Mesa destaque (FRENTE-1 e 2), mesa 3 frentes (FRENTE-1 a 3) e móvel make (TESTEIRA-1 a 4) têm uma linha por bloco, com cor e etiqueta próprias. Cada frente das mesas mostra até 4 etiquetas; cada testeira, 1. Bloco sem linha própria usa a cor do móvel inteiro. Blocos vizinhos com as mesmas etiquetas e cor ficam com uma pilha só, no centro. O balcão recepção tem uma cor só; Etiqueta 1, 2 e 3 vão para o bloco 1, o canto e o bloco 3.</t>
-  </si>
-  <si>
-    <t>6.4 Totem: na linha do totem, Etiqueta 1, 2 e 3 vão para o painel de cima, o do meio e o de baixo (cada uma ao lado do seu painel), e a "Marca Etiqueta N" pinta o painel N. Painel sem etiqueta usa a "Marca do Móvel". Se preferir, uma linha TOTEM 1/PAINEL-1 (a 3) define cor e etiqueta de um painel e tem prioridade.</t>
+    <t>6.1 Gôndola, mesas, totem e móvel make são preenchidos espaço por espaço: não há linha do móvel inteiro (se houver, ela é ignorada). Espaço sem linha fica branco.</t>
+  </si>
+  <si>
+    <t>6.2 Gôndola: uma linha por espaço — GONDOLA 1/LADO-A, MEIO-A, MEIO-B e LADO-B ("A" é sempre o lado virado para quem olha a planta). Cada espaço mostra até 4 etiquetas empilhadas em cima dele. Para dividir um meio em dois movimentos, preencha também a linha da metade 2 (ex.: GONDOLA 1/MEIO-A-2): a linha do meio passa a valer para a metade 1 e a planta mostra o meio dividido.</t>
+  </si>
+  <si>
+    <t>6.3 Mesa destaque (FRENTE-1 e 2), mesa 3 frentes (FRENTE-1 a 3), totem (PAINEL-1 a 3; o 1 é o de cima) e móvel make (TESTEIRA-1 a 4): uma linha por bloco, com cor e etiqueta próprias. Cada frente das mesas mostra até 4 etiquetas; cada painel e cada testeira, 1. Blocos vizinhos com as mesmas etiquetas e cor ficam com uma pilha só, no centro. As etiquetas do totem ficam ao lado do painel, com linha-guia.</t>
+  </si>
+  <si>
+    <t>6.4 Móveis de um espaço só (pirâmide, móvel de fila, móvel de parede, PDV, O.U.i…) têm uma linha. O balcão recepção tem uma cor só; Etiqueta 1, 2 e 3 vão para o bloco 1, o canto e o bloco 3.</t>
   </si>
   <si>
     <t>7. Na coluna "Planta" vale o nome (ex.: ER P) ou o número (01). Cascata: o que é definido numa planta vale também para as seguintes (ER P → ER M → ER G → ER GG), por isso cada móvel aparece uma vez só, na primeira planta que o tem ("vale para…" na coluna Móvel). Para mudar um móvel só a partir de uma planta, acrescente uma linha com o mesmo ID Móvel e essa planta. Planta = TODAS vale para todas.</t>
@@ -1765,7 +1723,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O382"/>
+  <dimension ref="A1:O375"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="13" style="1" customWidth="1"/>
@@ -1881,29 +1839,24 @@
         <v>26</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="G3" s="1"/>
+        <v>27</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>27</v>
+      </c>
       <c r="H3" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="I3" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="I3" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="M3" s="1" t="s">
-        <v>21</v>
-      </c>
+      <c r="K3" s="1"/>
+      <c r="M3" s="1"/>
       <c r="N3" s="1" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="O3" s="1" t="s">
         <v>24</v>
@@ -1917,30 +1870,25 @@
         <v>16</v>
       </c>
       <c r="C4" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="E4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E4" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>34</v>
-      </c>
       <c r="G4" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>33</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="I4" s="1"/>
       <c r="K4" s="1"/>
       <c r="M4" s="1"/>
       <c r="N4" s="1" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="O4" s="1" t="s">
         <v>24</v>
@@ -1954,10 +1902,10 @@
         <v>16</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E5" s="1"/>
       <c r="G5" s="1"/>
@@ -1966,7 +1914,7 @@
       <c r="M5" s="1"/>
       <c r="N5" s="1"/>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>15</v>
       </c>
@@ -1974,17 +1922,29 @@
         <v>16</v>
       </c>
       <c r="C6" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F6" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D6" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="E6" s="1"/>
-      <c r="G6" s="1"/>
+      <c r="G6" s="1" t="s">
+        <v>21</v>
+      </c>
       <c r="I6" s="1"/>
       <c r="K6" s="1"/>
       <c r="M6" s="1"/>
-      <c r="N6" s="1"/>
+      <c r="N6" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="O6" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
@@ -1994,10 +1954,10 @@
         <v>16</v>
       </c>
       <c r="C7" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>40</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>41</v>
       </c>
       <c r="E7" s="1"/>
       <c r="G7" s="1"/>
@@ -2006,7 +1966,7 @@
       <c r="M7" s="1"/>
       <c r="N7" s="1"/>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>15</v>
       </c>
@@ -2014,19 +1974,31 @@
         <v>16</v>
       </c>
       <c r="C8" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D8" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="E8" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E8" s="1"/>
-      <c r="G8" s="1"/>
+      <c r="G8" s="1" t="s">
+        <v>21</v>
+      </c>
       <c r="I8" s="1"/>
       <c r="K8" s="1"/>
       <c r="M8" s="1"/>
-      <c r="N8" s="1"/>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N8" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="O8" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>15</v>
       </c>
@@ -2039,12 +2011,24 @@
       <c r="D9" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="E9" s="1"/>
-      <c r="G9" s="1"/>
+      <c r="E9" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>23</v>
+      </c>
       <c r="I9" s="1"/>
       <c r="K9" s="1"/>
       <c r="M9" s="1"/>
-      <c r="N9" s="1"/>
+      <c r="N9" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O9" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
@@ -2054,19 +2038,19 @@
         <v>16</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>48</v>
+        <v>21</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>22</v>
+        <v>49</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I10" s="1"/>
       <c r="K10" s="1"/>
@@ -2086,16 +2070,16 @@
         <v>16</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>21</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G11" s="1" t="s">
         <v>21</v>
@@ -2118,15 +2102,20 @@
         <v>16</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="G12" s="1"/>
+        <v>46</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>46</v>
+      </c>
       <c r="I12" s="1"/>
       <c r="K12" s="1"/>
       <c r="M12" s="1"/>
@@ -2145,19 +2134,19 @@
         <v>16</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="I13" s="1"/>
       <c r="K13" s="1"/>
@@ -2177,23 +2166,34 @@
         <v>16</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D14" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J14" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="E14" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="I14" s="1"/>
-      <c r="K14" s="1"/>
-      <c r="M14" s="1"/>
+      <c r="K14" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="L14" s="5"/>
+      <c r="M14" s="5"/>
       <c r="N14" s="1" t="s">
         <v>24</v>
       </c>
@@ -2209,19 +2209,19 @@
         <v>16</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>48</v>
+        <v>21</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>48</v>
+        <v>21</v>
       </c>
       <c r="I15" s="1"/>
       <c r="K15" s="1"/>
@@ -2241,34 +2241,23 @@
         <v>16</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="H16" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="I16" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="J16" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="K16" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="L16" s="5"/>
-      <c r="M16" s="5"/>
+        <v>46</v>
+      </c>
+      <c r="I16" s="1"/>
+      <c r="K16" s="1"/>
+      <c r="M16" s="1"/>
       <c r="N16" s="1" t="s">
         <v>24</v>
       </c>
@@ -2284,23 +2273,26 @@
         <v>16</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>21</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="G17" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="I17" s="1"/>
-      <c r="K17" s="1"/>
-      <c r="M17" s="1"/>
+      <c r="H17" s="5"/>
+      <c r="I17" s="5"/>
+      <c r="J17" s="5"/>
+      <c r="K17" s="5"/>
+      <c r="L17" s="5"/>
+      <c r="M17" s="5"/>
       <c r="N17" s="1" t="s">
         <v>24</v>
       </c>
@@ -2316,23 +2308,26 @@
         <v>16</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>48</v>
+        <v>21</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="I18" s="1"/>
-      <c r="K18" s="1"/>
-      <c r="M18" s="1"/>
+        <v>21</v>
+      </c>
+      <c r="H18" s="5"/>
+      <c r="I18" s="5"/>
+      <c r="J18" s="5"/>
+      <c r="K18" s="5"/>
+      <c r="L18" s="5"/>
+      <c r="M18" s="5"/>
       <c r="N18" s="1" t="s">
         <v>24</v>
       </c>
@@ -2348,32 +2343,24 @@
         <v>16</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>75</v>
+        <v>28</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="H19" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="I19" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="J19" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="K19" s="1" t="s">
-        <v>33</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="H19" s="5"/>
+      <c r="I19" s="5"/>
+      <c r="J19" s="5"/>
+      <c r="K19" s="5"/>
       <c r="L19" s="5"/>
       <c r="M19" s="5"/>
       <c r="N19" s="1" t="s">
@@ -2400,10 +2387,10 @@
         <v>19</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="I20" s="1"/>
       <c r="K20" s="1"/>
@@ -2441,7 +2428,7 @@
         <v>81</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="K21" s="1"/>
       <c r="M21" s="1"/>
@@ -2469,10 +2456,10 @@
         <v>19</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="I22" s="1"/>
       <c r="K22" s="1"/>
@@ -2498,17 +2485,15 @@
         <v>85</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F23" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="G23" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I23" s="1"/>
-      <c r="K23" s="1"/>
-      <c r="M23" s="1"/>
+      <c r="G23" s="1"/>
+      <c r="H23" s="5"/>
+      <c r="I23" s="5"/>
+      <c r="J23" s="5"/>
+      <c r="K23" s="5"/>
+      <c r="L23" s="5"/>
+      <c r="M23" s="5"/>
       <c r="N23" s="1" t="s">
         <v>24</v>
       </c>
@@ -2530,9 +2515,14 @@
         <v>88</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="G24" s="1"/>
+        <v>21</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>21</v>
+      </c>
       <c r="H24" s="5"/>
       <c r="I24" s="5"/>
       <c r="J24" s="5"/>
@@ -2554,10 +2544,10 @@
         <v>16</v>
       </c>
       <c r="C25" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="D25" s="4" t="s">
         <v>90</v>
-      </c>
-      <c r="D25" s="4" t="s">
-        <v>91</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>21</v>
@@ -2589,20 +2579,15 @@
         <v>16</v>
       </c>
       <c r="C26" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="D26" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="D26" s="4" t="s">
-        <v>93</v>
-      </c>
       <c r="E26" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="G26" s="1" t="s">
-        <v>21</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="G26" s="1"/>
       <c r="H26" s="5"/>
       <c r="I26" s="5"/>
       <c r="J26" s="5"/>
@@ -2624,21 +2609,28 @@
         <v>16</v>
       </c>
       <c r="C27" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="D27" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="D27" s="4" t="s">
+      <c r="E27" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F27" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="E27" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="G27" s="1"/>
-      <c r="H27" s="5"/>
-      <c r="I27" s="5"/>
-      <c r="J27" s="5"/>
-      <c r="K27" s="5"/>
-      <c r="L27" s="5"/>
-      <c r="M27" s="5"/>
+      <c r="G27" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I27" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="K27" s="1"/>
+      <c r="M27" s="1"/>
       <c r="N27" s="1" t="s">
         <v>24</v>
       </c>
@@ -2721,33 +2713,28 @@
       </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A30" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C30" s="3" t="s">
+      <c r="A30" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B30" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="D30" s="4" t="s">
+      <c r="C30" s="6" t="s">
         <v>103</v>
       </c>
+      <c r="D30" s="7" t="s">
+        <v>104</v>
+      </c>
       <c r="E30" s="1" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>104</v>
+        <v>28</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="H30" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="I30" s="1" t="s">
-        <v>23</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="I30" s="1"/>
       <c r="K30" s="1"/>
       <c r="M30" s="1"/>
       <c r="N30" s="1" t="s">
@@ -2762,38 +2749,28 @@
         <v>15</v>
       </c>
       <c r="B31" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C31" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="C31" s="6" t="s">
+      <c r="D31" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="D31" s="7" t="s">
+      <c r="E31" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F31" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="E31" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="G31" s="1"/>
-      <c r="H31" s="1" t="s">
+      <c r="G31" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="I31" s="1"/>
+      <c r="K31" s="1"/>
+      <c r="M31" s="1"/>
+      <c r="N31" s="1" t="s">
         <v>108</v>
-      </c>
-      <c r="I31" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="J31" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="K31" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="L31" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="M31" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="N31" s="1" t="s">
-        <v>110</v>
       </c>
       <c r="O31" s="1" t="s">
         <v>24</v>
@@ -2804,172 +2781,208 @@
         <v>15</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D32" s="7" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="I32" s="1"/>
       <c r="K32" s="1"/>
       <c r="M32" s="1"/>
       <c r="N32" s="1" t="s">
-        <v>24</v>
+        <v>108</v>
       </c>
       <c r="O32" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C33" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="D33" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F33" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="D33" s="7" t="s">
-        <v>114</v>
-      </c>
-      <c r="E33" s="1"/>
-      <c r="G33" s="1"/>
+      <c r="G33" s="1" t="s">
+        <v>46</v>
+      </c>
       <c r="I33" s="1"/>
       <c r="K33" s="1"/>
       <c r="M33" s="1"/>
-      <c r="N33" s="1"/>
-    </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N33" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="O33" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C34" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="D34" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="D34" s="7" t="s">
-        <v>116</v>
-      </c>
-      <c r="E34" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F34" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="G34" s="1" t="s">
-        <v>21</v>
-      </c>
+      <c r="E34" s="1"/>
+      <c r="G34" s="1"/>
       <c r="I34" s="1"/>
       <c r="K34" s="1"/>
       <c r="M34" s="1"/>
-      <c r="N34" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="O34" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N34" s="1"/>
+    </row>
+    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C35" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="D35" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="D35" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="E35" s="1"/>
-      <c r="G35" s="1"/>
+      <c r="E35" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>46</v>
+      </c>
       <c r="I35" s="1"/>
       <c r="K35" s="1"/>
       <c r="M35" s="1"/>
-      <c r="N35" s="1"/>
-    </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N35" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="O35" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C36" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="D36" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="D36" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="E36" s="1"/>
-      <c r="G36" s="1"/>
+      <c r="E36" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>21</v>
+      </c>
       <c r="I36" s="1"/>
       <c r="K36" s="1"/>
       <c r="M36" s="1"/>
-      <c r="N36" s="1"/>
-    </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N36" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O36" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C37" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="D37" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="D37" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="E37" s="1"/>
-      <c r="G37" s="1"/>
+      <c r="E37" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>27</v>
+      </c>
       <c r="I37" s="1"/>
       <c r="K37" s="1"/>
       <c r="M37" s="1"/>
-      <c r="N37" s="1"/>
+      <c r="N37" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O37" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C38" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="D38" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="D38" s="7" t="s">
+      <c r="E38" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="E38" s="1" t="s">
-        <v>21</v>
-      </c>
       <c r="F38" s="1" t="s">
-        <v>69</v>
+        <v>125</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>21</v>
+        <v>124</v>
       </c>
       <c r="I38" s="1"/>
       <c r="K38" s="1"/>
       <c r="M38" s="1"/>
       <c r="N38" s="1" t="s">
-        <v>24</v>
+        <v>126</v>
       </c>
       <c r="O38" s="1" t="s">
         <v>24</v>
@@ -2980,28 +2993,28 @@
         <v>15</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>33</v>
+        <v>124</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>34</v>
+        <v>129</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>33</v>
+        <v>124</v>
       </c>
       <c r="I39" s="1"/>
       <c r="K39" s="1"/>
       <c r="M39" s="1"/>
       <c r="N39" s="1" t="s">
-        <v>24</v>
+        <v>126</v>
       </c>
       <c r="O39" s="1" t="s">
         <v>24</v>
@@ -3012,80 +3025,80 @@
         <v>15</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="D40" s="7" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>129</v>
+        <v>46</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>130</v>
+        <v>22</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>129</v>
+        <v>23</v>
       </c>
       <c r="I40" s="1"/>
       <c r="K40" s="1"/>
       <c r="M40" s="1"/>
       <c r="N40" s="1" t="s">
-        <v>131</v>
+        <v>24</v>
       </c>
       <c r="O40" s="1" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A41" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B41" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="C41" s="6" t="s">
+      <c r="A41" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B41" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="D41" s="7" t="s">
+      <c r="C41" s="3" t="s">
         <v>133</v>
       </c>
+      <c r="D41" s="4" t="s">
+        <v>134</v>
+      </c>
       <c r="E41" s="1" t="s">
-        <v>129</v>
+        <v>21</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>134</v>
+        <v>65</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>129</v>
+        <v>21</v>
       </c>
       <c r="I41" s="1"/>
       <c r="K41" s="1"/>
       <c r="M41" s="1"/>
       <c r="N41" s="1" t="s">
-        <v>131</v>
+        <v>24</v>
       </c>
       <c r="O41" s="1" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A42" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B42" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="C42" s="6" t="s">
+      <c r="A42" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="C42" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="D42" s="7" t="s">
+      <c r="D42" s="4" t="s">
         <v>136</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>48</v>
+        <v>23</v>
       </c>
       <c r="F42" s="1" t="s">
         <v>22</v>
@@ -3097,7 +3110,7 @@
       <c r="K42" s="1"/>
       <c r="M42" s="1"/>
       <c r="N42" s="1" t="s">
-        <v>24</v>
+        <v>108</v>
       </c>
       <c r="O42" s="1" t="s">
         <v>24</v>
@@ -3108,39 +3121,39 @@
         <v>15</v>
       </c>
       <c r="B43" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="C43" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="C43" s="3" t="s">
+      <c r="D43" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="D43" s="4" t="s">
+      <c r="E43" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F43" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="E43" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F43" s="1" t="s">
-        <v>69</v>
-      </c>
       <c r="G43" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I43" s="1"/>
       <c r="K43" s="1"/>
       <c r="M43" s="1"/>
       <c r="N43" s="1" t="s">
-        <v>24</v>
+        <v>108</v>
       </c>
       <c r="O43" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="C44" s="3" t="s">
         <v>140</v>
@@ -3148,67 +3161,57 @@
       <c r="D44" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="E44" s="1" t="s">
+      <c r="E44" s="1"/>
+      <c r="G44" s="1"/>
+      <c r="I44" s="1"/>
+      <c r="K44" s="1"/>
+      <c r="M44" s="1"/>
+      <c r="N44" s="1"/>
+    </row>
+    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A45" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="C45" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="E45" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F44" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="G44" s="1" t="s">
+      <c r="F45" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="G45" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="H44" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="I44" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="J44" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="K44" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="M44" s="1"/>
-      <c r="N44" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="O44" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A45" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B45" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="C45" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="D45" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="E45" s="1"/>
-      <c r="G45" s="1"/>
       <c r="I45" s="1"/>
       <c r="K45" s="1"/>
       <c r="M45" s="1"/>
-      <c r="N45" s="1"/>
+      <c r="N45" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="O45" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="C46" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="D46" s="4" t="s">
         <v>146</v>
-      </c>
-      <c r="D46" s="4" t="s">
-        <v>147</v>
       </c>
       <c r="E46" s="1"/>
       <c r="G46" s="1"/>
@@ -3217,38 +3220,45 @@
       <c r="M46" s="1"/>
       <c r="N46" s="1"/>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="C47" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="D47" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="D47" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="E47" s="1"/>
+      <c r="E47" s="1" t="s">
+        <v>23</v>
+      </c>
       <c r="G47" s="1"/>
       <c r="I47" s="1"/>
       <c r="K47" s="1"/>
       <c r="M47" s="1"/>
-      <c r="N47" s="1"/>
+      <c r="N47" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="O47" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="C48" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="D48" s="4" t="s">
         <v>150</v>
-      </c>
-      <c r="D48" s="4" t="s">
-        <v>151</v>
       </c>
       <c r="E48" s="1"/>
       <c r="G48" s="1"/>
@@ -3262,13 +3272,13 @@
         <v>15</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="C49" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="D49" s="4" t="s">
         <v>152</v>
-      </c>
-      <c r="D49" s="4" t="s">
-        <v>153</v>
       </c>
       <c r="E49" s="1"/>
       <c r="G49" s="1"/>
@@ -3277,72 +3287,108 @@
       <c r="M49" s="1"/>
       <c r="N49" s="1"/>
     </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="C50" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D50" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="D50" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="E50" s="1"/>
-      <c r="G50" s="1"/>
+      <c r="E50" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F50" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G50" s="1" t="s">
+        <v>27</v>
+      </c>
       <c r="I50" s="1"/>
       <c r="K50" s="1"/>
       <c r="M50" s="1"/>
-      <c r="N50" s="1"/>
-    </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N50" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O50" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="51" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="C51" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="D51" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="D51" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="E51" s="1"/>
-      <c r="G51" s="1"/>
+      <c r="E51" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F51" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="G51" s="1" t="s">
+        <v>21</v>
+      </c>
       <c r="I51" s="1"/>
       <c r="K51" s="1"/>
       <c r="M51" s="1"/>
-      <c r="N51" s="1"/>
-    </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N51" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O51" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="52" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="C52" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="D52" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="D52" s="4" t="s">
+      <c r="E52" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F52" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="E52" s="1"/>
-      <c r="G52" s="1"/>
+      <c r="G52" s="1" t="s">
+        <v>23</v>
+      </c>
       <c r="I52" s="1"/>
       <c r="K52" s="1"/>
       <c r="M52" s="1"/>
-      <c r="N52" s="1"/>
+      <c r="N52" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O52" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="53" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="C53" s="3" t="s">
         <v>160</v>
@@ -3351,13 +3397,13 @@
         <v>161</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>34</v>
+        <v>55</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="I53" s="1"/>
       <c r="K53" s="1"/>
@@ -3370,134 +3416,117 @@
       </c>
     </row>
     <row r="54" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A54" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B54" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="C54" s="3" t="s">
+      <c r="A54" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B54" s="6" t="s">
         <v>162</v>
       </c>
-      <c r="D54" s="4" t="s">
+      <c r="C54" s="6" t="s">
         <v>163</v>
       </c>
+      <c r="D54" s="7" t="s">
+        <v>164</v>
+      </c>
       <c r="E54" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="G54" s="1"/>
+        <v>124</v>
+      </c>
+      <c r="F54" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="G54" s="1" t="s">
+        <v>124</v>
+      </c>
       <c r="I54" s="1"/>
       <c r="K54" s="1"/>
       <c r="M54" s="1"/>
       <c r="N54" s="1" t="s">
-        <v>24</v>
+        <v>108</v>
       </c>
       <c r="O54" s="1" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="55" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A55" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B55" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="C55" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="D55" s="4" t="s">
-        <v>165</v>
+      <c r="A55" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B55" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="C55" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="D55" s="7" t="s">
+        <v>167</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F55" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="G55" s="1" t="s">
-        <v>21</v>
-      </c>
+        <v>124</v>
+      </c>
+      <c r="G55" s="1"/>
       <c r="I55" s="1"/>
       <c r="K55" s="1"/>
       <c r="M55" s="1"/>
       <c r="N55" s="1" t="s">
-        <v>24</v>
+        <v>108</v>
       </c>
       <c r="O55" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A56" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B56" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="C56" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="D56" s="4" t="s">
-        <v>167</v>
-      </c>
-      <c r="E56" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F56" s="1" t="s">
+    <row r="56" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A56" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B56" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="C56" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="G56" s="1" t="s">
-        <v>23</v>
-      </c>
+      <c r="D56" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="E56" s="1"/>
+      <c r="G56" s="1"/>
       <c r="I56" s="1"/>
       <c r="K56" s="1"/>
       <c r="M56" s="1"/>
-      <c r="N56" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="O56" s="1" t="s">
-        <v>24</v>
-      </c>
+      <c r="N56" s="1"/>
     </row>
     <row r="57" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A57" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B57" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="C57" s="3" t="s">
-        <v>169</v>
-      </c>
-      <c r="D57" s="4" t="s">
+      <c r="A57" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B57" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="C57" s="6" t="s">
         <v>170</v>
       </c>
+      <c r="D57" s="7" t="s">
+        <v>171</v>
+      </c>
       <c r="E57" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F57" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="G57" s="1" t="s">
-        <v>48</v>
-      </c>
+        <v>124</v>
+      </c>
+      <c r="G57" s="1"/>
       <c r="I57" s="1"/>
       <c r="K57" s="1"/>
       <c r="M57" s="1"/>
       <c r="N57" s="1" t="s">
-        <v>24</v>
+        <v>108</v>
       </c>
       <c r="O57" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A58" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="C58" s="6" t="s">
         <v>172</v>
@@ -3505,97 +3534,111 @@
       <c r="D58" s="7" t="s">
         <v>173</v>
       </c>
-      <c r="E58" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="F58" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="G58" s="1" t="s">
-        <v>129</v>
-      </c>
+      <c r="E58" s="1"/>
+      <c r="G58" s="1"/>
       <c r="I58" s="1"/>
       <c r="K58" s="1"/>
       <c r="M58" s="1"/>
-      <c r="N58" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="O58" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N58" s="1"/>
+    </row>
+    <row r="59" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A59" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="C59" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="D59" s="7" t="s">
         <v>175</v>
       </c>
-      <c r="D59" s="7" t="s">
-        <v>176</v>
-      </c>
-      <c r="E59" s="1"/>
+      <c r="E59" s="1" t="s">
+        <v>124</v>
+      </c>
       <c r="G59" s="1"/>
       <c r="I59" s="1"/>
       <c r="K59" s="1"/>
       <c r="M59" s="1"/>
-      <c r="N59" s="1"/>
-    </row>
-    <row r="60" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N59" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="O59" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="60" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A60" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B60" s="6" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="C60" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="D60" s="7" t="s">
         <v>177</v>
       </c>
-      <c r="D60" s="7" t="s">
-        <v>178</v>
-      </c>
-      <c r="E60" s="1"/>
-      <c r="G60" s="1"/>
+      <c r="E60" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F60" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G60" s="1" t="s">
+        <v>27</v>
+      </c>
       <c r="I60" s="1"/>
       <c r="K60" s="1"/>
       <c r="M60" s="1"/>
-      <c r="N60" s="1"/>
-    </row>
-    <row r="61" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N60" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O60" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="61" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A61" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B61" s="6" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="C61" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="D61" s="7" t="s">
         <v>179</v>
       </c>
-      <c r="D61" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="E61" s="1"/>
+      <c r="E61" s="1" t="s">
+        <v>27</v>
+      </c>
       <c r="G61" s="1"/>
       <c r="I61" s="1"/>
       <c r="K61" s="1"/>
       <c r="M61" s="1"/>
-      <c r="N61" s="1"/>
+      <c r="N61" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O61" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A62" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B62" s="6" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="C62" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="D62" s="7" t="s">
         <v>181</v>
-      </c>
-      <c r="D62" s="7" t="s">
-        <v>182</v>
       </c>
       <c r="E62" s="1"/>
       <c r="G62" s="1"/>
@@ -3604,38 +3647,45 @@
       <c r="M62" s="1"/>
       <c r="N62" s="1"/>
     </row>
-    <row r="63" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A63" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="C63" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="D63" s="7" t="s">
         <v>183</v>
       </c>
-      <c r="D63" s="7" t="s">
-        <v>184</v>
-      </c>
-      <c r="E63" s="1"/>
+      <c r="E63" s="1" t="s">
+        <v>27</v>
+      </c>
       <c r="G63" s="1"/>
       <c r="I63" s="1"/>
       <c r="K63" s="1"/>
       <c r="M63" s="1"/>
-      <c r="N63" s="1"/>
+      <c r="N63" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O63" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A64" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="C64" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="D64" s="7" t="s">
         <v>185</v>
-      </c>
-      <c r="D64" s="7" t="s">
-        <v>186</v>
       </c>
       <c r="E64" s="1"/>
       <c r="G64" s="1"/>
@@ -3649,23 +3699,18 @@
         <v>15</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="C65" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="D65" s="7" t="s">
         <v>187</v>
       </c>
-      <c r="D65" s="7" t="s">
-        <v>188</v>
-      </c>
       <c r="E65" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="F65" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="G65" s="1" t="s">
-        <v>33</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="G65" s="1"/>
       <c r="I65" s="1"/>
       <c r="K65" s="1"/>
       <c r="M65" s="1"/>
@@ -3676,32 +3721,44 @@
         <v>24</v>
       </c>
     </row>
-    <row r="66" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A66" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="C66" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="D66" s="7" t="s">
         <v>189</v>
       </c>
-      <c r="D66" s="7" t="s">
+      <c r="E66" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F66" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="E66" s="1"/>
-      <c r="G66" s="1"/>
+      <c r="G66" s="1" t="s">
+        <v>46</v>
+      </c>
       <c r="I66" s="1"/>
       <c r="K66" s="1"/>
       <c r="M66" s="1"/>
-      <c r="N66" s="1"/>
-    </row>
-    <row r="67" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N66" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="O66" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="67" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A67" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="C67" s="6" t="s">
         <v>191</v>
@@ -3709,19 +3766,26 @@
       <c r="D67" s="7" t="s">
         <v>192</v>
       </c>
-      <c r="E67" s="1"/>
+      <c r="E67" s="1" t="s">
+        <v>46</v>
+      </c>
       <c r="G67" s="1"/>
       <c r="I67" s="1"/>
       <c r="K67" s="1"/>
       <c r="M67" s="1"/>
-      <c r="N67" s="1"/>
+      <c r="N67" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="O67" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="68" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A68" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="C68" s="6" t="s">
         <v>193</v>
@@ -3736,12 +3800,12 @@
       <c r="M68" s="1"/>
       <c r="N68" s="1"/>
     </row>
-    <row r="69" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A69" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="C69" s="6" t="s">
         <v>195</v>
@@ -3749,19 +3813,26 @@
       <c r="D69" s="7" t="s">
         <v>196</v>
       </c>
-      <c r="E69" s="1"/>
+      <c r="E69" s="1" t="s">
+        <v>46</v>
+      </c>
       <c r="G69" s="1"/>
       <c r="I69" s="1"/>
       <c r="K69" s="1"/>
       <c r="M69" s="1"/>
-      <c r="N69" s="1"/>
+      <c r="N69" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="O69" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="70" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A70" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="C70" s="6" t="s">
         <v>197</v>
@@ -3776,12 +3847,12 @@
       <c r="M70" s="1"/>
       <c r="N70" s="1"/>
     </row>
-    <row r="71" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A71" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B71" s="6" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="C71" s="6" t="s">
         <v>199</v>
@@ -3789,19 +3860,26 @@
       <c r="D71" s="7" t="s">
         <v>200</v>
       </c>
-      <c r="E71" s="1"/>
+      <c r="E71" s="1" t="s">
+        <v>46</v>
+      </c>
       <c r="G71" s="1"/>
       <c r="I71" s="1"/>
       <c r="K71" s="1"/>
       <c r="M71" s="1"/>
-      <c r="N71" s="1"/>
+      <c r="N71" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="O71" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="72" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A72" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="C72" s="6" t="s">
         <v>201</v>
@@ -3810,30 +3888,30 @@
         <v>202</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>48</v>
+        <v>23</v>
       </c>
       <c r="F72" s="1" t="s">
         <v>203</v>
       </c>
       <c r="G72" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="I72" s="1"/>
       <c r="K72" s="1"/>
       <c r="M72" s="1"/>
       <c r="N72" s="1" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="O72" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="73" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A73" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B73" s="6" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="C73" s="6" t="s">
         <v>204</v>
@@ -3841,66 +3919,100 @@
       <c r="D73" s="7" t="s">
         <v>205</v>
       </c>
-      <c r="E73" s="1"/>
-      <c r="G73" s="1"/>
+      <c r="E73" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F73" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="G73" s="1" t="s">
+        <v>21</v>
+      </c>
       <c r="I73" s="1"/>
       <c r="K73" s="1"/>
       <c r="M73" s="1"/>
-      <c r="N73" s="1"/>
-    </row>
-    <row r="74" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N73" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="O73" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="74" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A74" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B74" s="6" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="C74" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="D74" s="7" t="s">
         <v>206</v>
       </c>
-      <c r="D74" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="E74" s="1"/>
-      <c r="G74" s="1"/>
-      <c r="I74" s="1"/>
+      <c r="E74" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F74" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G74" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H74" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I74" s="1" t="s">
+        <v>23</v>
+      </c>
       <c r="K74" s="1"/>
       <c r="M74" s="1"/>
-      <c r="N74" s="1"/>
-    </row>
-    <row r="75" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N74" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O74" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="75" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A75" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B75" s="6" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="C75" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="D75" s="7" t="s">
         <v>208</v>
       </c>
-      <c r="D75" s="7" t="s">
-        <v>209</v>
-      </c>
-      <c r="E75" s="1"/>
-      <c r="G75" s="1"/>
-      <c r="I75" s="1"/>
+      <c r="E75" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="F75" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="G75" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="H75" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="I75" s="1" t="s">
+        <v>124</v>
+      </c>
       <c r="K75" s="1"/>
       <c r="M75" s="1"/>
-      <c r="N75" s="1"/>
-    </row>
-    <row r="76" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A76" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B76" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="C76" s="6" t="s">
-        <v>210</v>
-      </c>
-      <c r="D76" s="7" t="s">
-        <v>211</v>
-      </c>
+      <c r="N75" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="O75" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="76" spans="5:14" x14ac:dyDescent="0.25">
       <c r="E76" s="1"/>
       <c r="G76" s="1"/>
       <c r="I76" s="1"/>
@@ -3908,19 +4020,7 @@
       <c r="M76" s="1"/>
       <c r="N76" s="1"/>
     </row>
-    <row r="77" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A77" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B77" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="C77" s="6" t="s">
-        <v>212</v>
-      </c>
-      <c r="D77" s="7" t="s">
-        <v>213</v>
-      </c>
+    <row r="77" spans="5:14" x14ac:dyDescent="0.25">
       <c r="E77" s="1"/>
       <c r="G77" s="1"/>
       <c r="I77" s="1"/>
@@ -3928,19 +4028,7 @@
       <c r="M77" s="1"/>
       <c r="N77" s="1"/>
     </row>
-    <row r="78" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A78" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B78" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="C78" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="D78" s="7" t="s">
-        <v>215</v>
-      </c>
+    <row r="78" spans="5:14" x14ac:dyDescent="0.25">
       <c r="E78" s="1"/>
       <c r="G78" s="1"/>
       <c r="I78" s="1"/>
@@ -3948,143 +4036,37 @@
       <c r="M78" s="1"/>
       <c r="N78" s="1"/>
     </row>
-    <row r="79" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A79" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B79" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="C79" s="6" t="s">
-        <v>216</v>
-      </c>
-      <c r="D79" s="7" t="s">
-        <v>217</v>
-      </c>
-      <c r="E79" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F79" s="1" t="s">
-        <v>218</v>
-      </c>
-      <c r="G79" s="1" t="s">
-        <v>48</v>
-      </c>
+    <row r="79" spans="5:14" x14ac:dyDescent="0.25">
+      <c r="E79" s="1"/>
+      <c r="G79" s="1"/>
       <c r="I79" s="1"/>
       <c r="K79" s="1"/>
       <c r="M79" s="1"/>
-      <c r="N79" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="O79" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="80" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A80" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B80" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="C80" s="6" t="s">
-        <v>219</v>
-      </c>
-      <c r="D80" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="E80" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F80" s="1" t="s">
-        <v>218</v>
-      </c>
-      <c r="G80" s="1" t="s">
-        <v>21</v>
-      </c>
+      <c r="N79" s="1"/>
+    </row>
+    <row r="80" spans="5:14" x14ac:dyDescent="0.25">
+      <c r="E80" s="1"/>
+      <c r="G80" s="1"/>
       <c r="I80" s="1"/>
       <c r="K80" s="1"/>
       <c r="M80" s="1"/>
-      <c r="N80" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="O80" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="81" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A81" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B81" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="C81" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="D81" s="7" t="s">
-        <v>221</v>
-      </c>
-      <c r="E81" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F81" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="G81" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="H81" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="I81" s="1" t="s">
-        <v>23</v>
-      </c>
+      <c r="N80" s="1"/>
+    </row>
+    <row r="81" spans="5:14" x14ac:dyDescent="0.25">
+      <c r="E81" s="1"/>
+      <c r="G81" s="1"/>
+      <c r="I81" s="1"/>
       <c r="K81" s="1"/>
       <c r="M81" s="1"/>
-      <c r="N81" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="O81" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="82" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A82" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B82" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="C82" s="6" t="s">
-        <v>222</v>
-      </c>
-      <c r="D82" s="7" t="s">
-        <v>223</v>
-      </c>
-      <c r="E82" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="F82" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="G82" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="H82" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="I82" s="1" t="s">
-        <v>129</v>
-      </c>
+      <c r="N81" s="1"/>
+    </row>
+    <row r="82" spans="5:14" x14ac:dyDescent="0.25">
+      <c r="E82" s="1"/>
+      <c r="G82" s="1"/>
+      <c r="I82" s="1"/>
       <c r="K82" s="1"/>
       <c r="M82" s="1"/>
-      <c r="N82" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="O82" s="1" t="s">
-        <v>24</v>
-      </c>
+      <c r="N82" s="1"/>
     </row>
     <row r="83" spans="5:14" x14ac:dyDescent="0.25">
       <c r="E83" s="1"/>
@@ -6430,65 +6412,9 @@
       <c r="M375" s="1"/>
       <c r="N375" s="1"/>
     </row>
-    <row r="376" spans="5:14" x14ac:dyDescent="0.25">
-      <c r="E376" s="1"/>
-      <c r="G376" s="1"/>
-      <c r="I376" s="1"/>
-      <c r="K376" s="1"/>
-      <c r="M376" s="1"/>
-      <c r="N376" s="1"/>
-    </row>
-    <row r="377" spans="5:14" x14ac:dyDescent="0.25">
-      <c r="E377" s="1"/>
-      <c r="G377" s="1"/>
-      <c r="I377" s="1"/>
-      <c r="K377" s="1"/>
-      <c r="M377" s="1"/>
-      <c r="N377" s="1"/>
-    </row>
-    <row r="378" spans="5:14" x14ac:dyDescent="0.25">
-      <c r="E378" s="1"/>
-      <c r="G378" s="1"/>
-      <c r="I378" s="1"/>
-      <c r="K378" s="1"/>
-      <c r="M378" s="1"/>
-      <c r="N378" s="1"/>
-    </row>
-    <row r="379" spans="5:14" x14ac:dyDescent="0.25">
-      <c r="E379" s="1"/>
-      <c r="G379" s="1"/>
-      <c r="I379" s="1"/>
-      <c r="K379" s="1"/>
-      <c r="M379" s="1"/>
-      <c r="N379" s="1"/>
-    </row>
-    <row r="380" spans="5:14" x14ac:dyDescent="0.25">
-      <c r="E380" s="1"/>
-      <c r="G380" s="1"/>
-      <c r="I380" s="1"/>
-      <c r="K380" s="1"/>
-      <c r="M380" s="1"/>
-      <c r="N380" s="1"/>
-    </row>
-    <row r="381" spans="5:14" x14ac:dyDescent="0.25">
-      <c r="E381" s="1"/>
-      <c r="G381" s="1"/>
-      <c r="I381" s="1"/>
-      <c r="K381" s="1"/>
-      <c r="M381" s="1"/>
-      <c r="N381" s="1"/>
-    </row>
-    <row r="382" spans="5:14" x14ac:dyDescent="0.25">
-      <c r="E382" s="1"/>
-      <c r="G382" s="1"/>
-      <c r="I382" s="1"/>
-      <c r="K382" s="1"/>
-      <c r="M382" s="1"/>
-      <c r="N382" s="1"/>
-    </row>
   </sheetData>
   <autoFilter ref="A1:O1"/>
-  <conditionalFormatting sqref="E2:E382">
+  <conditionalFormatting sqref="E2:E375">
     <cfRule type="containsText" dxfId="0" priority="1">
       <formula>NOT(ISERROR(SEARCH("BOT",E2)))</formula>
     </cfRule>
@@ -6508,7 +6434,7 @@
       <formula>NOT(ISERROR(SEARCH("NEUTRO",E2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G382">
+  <conditionalFormatting sqref="G2:G375">
     <cfRule type="containsText" dxfId="6" priority="1">
       <formula>NOT(ISERROR(SEARCH("BOT",G2)))</formula>
     </cfRule>
@@ -6528,7 +6454,7 @@
       <formula>NOT(ISERROR(SEARCH("NEUTRO",G2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I382">
+  <conditionalFormatting sqref="I2:I375">
     <cfRule type="containsText" dxfId="12" priority="1">
       <formula>NOT(ISERROR(SEARCH("BOT",I2)))</formula>
     </cfRule>
@@ -6548,7 +6474,7 @@
       <formula>NOT(ISERROR(SEARCH("NEUTRO",I2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K2:K382">
+  <conditionalFormatting sqref="K2:K375">
     <cfRule type="containsText" dxfId="18" priority="1">
       <formula>NOT(ISERROR(SEARCH("BOT",K2)))</formula>
     </cfRule>
@@ -6568,7 +6494,7 @@
       <formula>NOT(ISERROR(SEARCH("NEUTRO",K2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M2:M382">
+  <conditionalFormatting sqref="M2:M375">
     <cfRule type="containsText" dxfId="24" priority="1">
       <formula>NOT(ISERROR(SEARCH("BOT",M2)))</formula>
     </cfRule>
@@ -6589,40 +6515,40 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="12">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca do Móvel" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca do Móvel" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="E10:E382">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca do Móvel" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca do Móvel" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="E10:E375">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca do Móvel" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca do Móvel" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="E2:E382">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca do Móvel" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca do Móvel" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="E2:E375">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 1" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 1" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="G10:G382">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 1" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 1" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="G10:G375">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 1" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 1" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="G2:G382">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 1" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 1" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="G2:G375">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 2" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 2" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="I10:I382">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 2" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 2" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="I10:I375">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 2" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 2" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="I2:I382">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 2" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 2" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="I2:I375">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 3" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 3" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="K10:K382">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 3" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 3" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="K10:K375">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 3" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 3" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="K2:K382">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 3" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 3" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="K2:K375">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 4" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 4" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="M10:M382">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 4" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 4" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="M10:M375">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 4" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 4" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="M2:M382">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 4" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 4" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="M2:M375">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo" prompt="MOVIMENTO = Movimento definido nesta planta; FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo" error="MOVIMENTO = Movimento definido nesta planta; FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" sqref="N10:N382">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo" prompt="MOVIMENTO = Movimento definido nesta planta; FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo" error="MOVIMENTO = Movimento definido nesta planta; FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" sqref="N10:N375">
       <formula1>"MOVIMENTO,FIXO,EXPOSICAO,NOVO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo" prompt="MOVIMENTO = Movimento definido nesta planta; FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo" error="MOVIMENTO = Movimento definido nesta planta; FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" sqref="N2:N382">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo" prompt="MOVIMENTO = Movimento definido nesta planta; FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo" error="MOVIMENTO = Movimento definido nesta planta; FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" sqref="N2:N375">
       <formula1>"MOVIMENTO,FIXO,EXPOSICAO,NOVO"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6650,16 +6576,16 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>224</v>
+        <v>209</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>225</v>
+        <v>210</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>226</v>
+        <v>211</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>227</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -6667,13 +6593,13 @@
         <v>15</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>228</v>
+        <v>213</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>229</v>
+        <v>214</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>230</v>
+        <v>215</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>23</v>
@@ -6687,13 +6613,13 @@
         <v>15</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>228</v>
+        <v>213</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>231</v>
+        <v>216</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>21</v>
@@ -6707,16 +6633,16 @@
         <v>15</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>228</v>
+        <v>213</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>231</v>
+        <v>216</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>232</v>
+        <v>217</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>24</v>
@@ -6727,13 +6653,13 @@
         <v>15</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>228</v>
+        <v>213</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>233</v>
+        <v>218</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>21</v>
@@ -6747,13 +6673,13 @@
         <v>15</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>228</v>
+        <v>213</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>233</v>
+        <v>218</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>21</v>
@@ -6767,16 +6693,16 @@
         <v>15</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>228</v>
+        <v>213</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>233</v>
+        <v>218</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>234</v>
+        <v>219</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>24</v>
@@ -6787,16 +6713,16 @@
         <v>15</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>228</v>
+        <v>213</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>233</v>
+        <v>218</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>235</v>
+        <v>220</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>24</v>
@@ -6807,13 +6733,13 @@
         <v>15</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>228</v>
+        <v>213</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>233</v>
+        <v>218</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>236</v>
+        <v>221</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>23</v>
@@ -6827,19 +6753,19 @@
         <v>15</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>228</v>
+        <v>213</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>237</v>
+        <v>222</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>238</v>
+        <v>223</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>23</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>84</v>
+        <v>224</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -6847,19 +6773,19 @@
         <v>15</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>228</v>
+        <v>213</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>237</v>
+        <v>222</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>239</v>
+        <v>225</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>21</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -6867,19 +6793,19 @@
         <v>15</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>228</v>
+        <v>213</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>237</v>
+        <v>222</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>240</v>
+        <v>226</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -6890,10 +6816,10 @@
         <v>16</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>241</v>
+        <v>227</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>242</v>
+        <v>228</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>24</v>
@@ -6910,10 +6836,10 @@
         <v>16</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>241</v>
+        <v>227</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>243</v>
+        <v>229</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>24</v>
@@ -6927,13 +6853,13 @@
         <v>15</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>241</v>
+        <v>227</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>244</v>
+        <v>230</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>24</v>
@@ -6947,13 +6873,13 @@
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>241</v>
+        <v>227</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>245</v>
+        <v>231</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>24</v>
@@ -6967,13 +6893,13 @@
         <v>15</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>241</v>
+        <v>227</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>244</v>
+        <v>230</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>24</v>
@@ -6987,13 +6913,13 @@
         <v>15</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>241</v>
+        <v>227</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>245</v>
+        <v>231</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>24</v>
@@ -7007,13 +6933,13 @@
         <v>15</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>241</v>
+        <v>227</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>244</v>
+        <v>230</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>24</v>
@@ -7027,13 +6953,13 @@
         <v>15</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>241</v>
+        <v>227</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>246</v>
+        <v>232</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>24</v>
@@ -7047,13 +6973,13 @@
         <v>15</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>241</v>
+        <v>227</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>245</v>
+        <v>231</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>24</v>
@@ -8316,115 +8242,115 @@
   <sheetData>
     <row r="1" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B1" s="9" t="s">
-        <v>247</v>
+        <v>233</v>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B2" s="10" t="s">
-        <v>248</v>
+        <v>234</v>
       </c>
       <c r="C2" s="10"/>
       <c r="D2" s="10"/>
     </row>
     <row r="4" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B4" s="11" t="s">
-        <v>249</v>
+        <v>235</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B5" s="10" t="s">
-        <v>250</v>
+        <v>236</v>
       </c>
       <c r="C5" s="10"/>
       <c r="D5" s="10"/>
     </row>
     <row r="6" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B6" s="10" t="s">
-        <v>251</v>
+        <v>237</v>
       </c>
       <c r="C6" s="10"/>
       <c r="D6" s="10"/>
     </row>
-    <row r="7" ht="16" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="7" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B7" s="10" t="s">
-        <v>252</v>
+        <v>238</v>
       </c>
       <c r="C7" s="10"/>
       <c r="D7" s="10"/>
     </row>
     <row r="8" ht="45" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B8" s="10" t="s">
-        <v>253</v>
+        <v>239</v>
       </c>
       <c r="C8" s="10"/>
       <c r="D8" s="10"/>
     </row>
     <row r="9" ht="16" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B9" s="10" t="s">
-        <v>254</v>
+        <v>240</v>
       </c>
       <c r="C9" s="10"/>
       <c r="D9" s="10"/>
     </row>
     <row r="10" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B10" s="10" t="s">
-        <v>255</v>
+        <v>241</v>
       </c>
       <c r="C10" s="10"/>
       <c r="D10" s="10"/>
     </row>
-    <row r="11" ht="60" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="11" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B11" s="10" t="s">
-        <v>256</v>
+        <v>242</v>
       </c>
       <c r="C11" s="10"/>
       <c r="D11" s="10"/>
     </row>
     <row r="12" ht="60" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B12" s="10" t="s">
-        <v>257</v>
+        <v>243</v>
       </c>
       <c r="C12" s="10"/>
       <c r="D12" s="10"/>
     </row>
     <row r="13" ht="60" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B13" s="10" t="s">
-        <v>258</v>
+        <v>244</v>
       </c>
       <c r="C13" s="10"/>
       <c r="D13" s="10"/>
     </row>
-    <row r="14" ht="45" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="14" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B14" s="10" t="s">
-        <v>259</v>
+        <v>245</v>
       </c>
       <c r="C14" s="10"/>
       <c r="D14" s="10"/>
     </row>
     <row r="15" ht="60" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B15" s="10" t="s">
-        <v>260</v>
+        <v>246</v>
       </c>
       <c r="C15" s="10"/>
       <c r="D15" s="10"/>
     </row>
     <row r="16" ht="45" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B16" s="10" t="s">
-        <v>261</v>
+        <v>247</v>
       </c>
       <c r="C16" s="10"/>
       <c r="D16" s="10"/>
     </row>
     <row r="17" ht="45" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B17" s="10" t="s">
-        <v>262</v>
+        <v>248</v>
       </c>
       <c r="C17" s="10"/>
       <c r="D17" s="10"/>
     </row>
     <row r="19" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B19" s="11" t="s">
-        <v>263</v>
+        <v>249</v>
       </c>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.25">
@@ -8432,43 +8358,43 @@
         <v>21</v>
       </c>
       <c r="C20" t="s">
-        <v>264</v>
+        <v>250</v>
       </c>
       <c r="D20" s="13" t="s">
-        <v>265</v>
+        <v>251</v>
       </c>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B21" s="12" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="C21" t="s">
-        <v>266</v>
+        <v>252</v>
       </c>
       <c r="D21" s="14" t="s">
-        <v>267</v>
+        <v>253</v>
       </c>
     </row>
     <row r="22" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B22" s="12" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C22" t="s">
-        <v>268</v>
+        <v>254</v>
       </c>
       <c r="D22" s="15" t="s">
-        <v>269</v>
+        <v>255</v>
       </c>
     </row>
     <row r="23" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B23" s="12" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="C23" t="s">
-        <v>270</v>
+        <v>256</v>
       </c>
       <c r="D23" s="16" t="s">
-        <v>271</v>
+        <v>257</v>
       </c>
     </row>
     <row r="24" spans="2:4" x14ac:dyDescent="0.25">
@@ -8476,10 +8402,10 @@
         <v>23</v>
       </c>
       <c r="C24" t="s">
-        <v>272</v>
+        <v>258</v>
       </c>
       <c r="D24" s="17" t="s">
-        <v>273</v>
+        <v>259</v>
       </c>
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.25">
@@ -8487,108 +8413,108 @@
         <v>19</v>
       </c>
       <c r="C25" t="s">
-        <v>274</v>
+        <v>260</v>
       </c>
       <c r="D25" s="18" t="s">
-        <v>275</v>
+        <v>261</v>
       </c>
     </row>
     <row r="27" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B27" s="11" t="s">
-        <v>276</v>
+        <v>262</v>
       </c>
     </row>
     <row r="28" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B28" s="12" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C28" t="s">
-        <v>277</v>
+        <v>263</v>
       </c>
       <c r="D28" t="s">
-        <v>278</v>
+        <v>264</v>
       </c>
     </row>
     <row r="29" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B29" s="12" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C29" t="s">
-        <v>279</v>
+        <v>265</v>
       </c>
       <c r="D29" t="s">
-        <v>280</v>
+        <v>266</v>
       </c>
     </row>
     <row r="30" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B30" s="12" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="C30" t="s">
-        <v>281</v>
+        <v>267</v>
       </c>
       <c r="D30" t="s">
-        <v>282</v>
+        <v>268</v>
       </c>
     </row>
     <row r="31" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B31" s="12" t="s">
-        <v>283</v>
+        <v>269</v>
       </c>
       <c r="C31" t="s">
-        <v>284</v>
+        <v>270</v>
       </c>
       <c r="D31" t="s">
-        <v>285</v>
+        <v>271</v>
       </c>
     </row>
     <row r="33" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B33" s="11" t="s">
-        <v>286</v>
+        <v>272</v>
       </c>
     </row>
     <row r="34" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B34" s="12" t="s">
-        <v>229</v>
+        <v>214</v>
       </c>
       <c r="C34" t="s">
-        <v>287</v>
+        <v>273</v>
       </c>
       <c r="D34"/>
     </row>
     <row r="35" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B35" s="12" t="s">
-        <v>231</v>
+        <v>216</v>
       </c>
       <c r="C35" t="s">
-        <v>288</v>
+        <v>274</v>
       </c>
       <c r="D35"/>
     </row>
     <row r="36" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B36" s="12" t="s">
-        <v>233</v>
+        <v>218</v>
       </c>
       <c r="C36" t="s">
-        <v>289</v>
+        <v>275</v>
       </c>
       <c r="D36"/>
     </row>
     <row r="37" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B37" s="12" t="s">
-        <v>237</v>
+        <v>222</v>
       </c>
       <c r="C37" t="s">
-        <v>290</v>
+        <v>276</v>
       </c>
       <c r="D37"/>
     </row>
     <row r="38" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B38" s="12" t="s">
-        <v>241</v>
+        <v>227</v>
       </c>
       <c r="C38" t="s">
-        <v>291</v>
+        <v>277</v>
       </c>
       <c r="D38"/>
     </row>

</xml_diff>

<commit_message>
Etiquetas na planta junto de cada espaço; fichas viram "Visão simplificada"
Duas abas ao lado das plantas escolhem como mostrar as etiquetas (o app
lembra a última; o PNG sai na visão da tela):

- Na planta (padrão): cada pilha fica junto da parte do móvel a que
  pertence. Nos móveis com espaços, a pilha leva uma plaquinha com o nome
  do espaço (LADO A, MEIO B, FRENTE 2, PAINEL 1…) e sai da face dele, para
  o lado que ela olha, com linha-guia na cor da etiqueta até um ponto na
  face. Nos de um espaço só, fica em cima do móvel ou no lugar livre mais
  perto. A posição é escolhida por custo: distância, cobrir outros móveis
  (bem mais caro que cobrir o próprio), linhas cruzadas ou passando por
  outra pilha. Se faltar lugar, a planta e o slide (16:9) crescem.
- Visão simplificada: as fichas por móvel em colunas ao lado da planta,
  como na versão anterior.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017zCtX61WuLMgJTMdsRwq9V
</commit_message>
<xml_diff>
--- a/visualizador/Planilha base - Visualizador.xlsx
+++ b/visualizador/Planilha base - Visualizador.xlsx
@@ -723,7 +723,7 @@
     <t>Planilha base — Plano de Varejo</t>
   </si>
   <si>
-    <t>Gerada em 14/10/2026, 23:56:23 a partir do ciclo "Ciclo exemplo".</t>
+    <t>Gerada em 15/10/2026, 14:07:33 a partir do ciclo "Ciclo exemplo".</t>
   </si>
   <si>
     <t>Como preencher</t>
@@ -750,10 +750,10 @@
     <t>6.1 Gôndola, mesas, totem e móvel make são preenchidos espaço por espaço: não há linha do móvel inteiro (se houver, ela é ignorada). Espaço sem linha fica branco.</t>
   </si>
   <si>
-    <t>6.2 Gôndola: uma linha por espaço — GONDOLA 1/LADO-A, MEIO-A, MEIO-B e LADO-B ("A" é sempre o lado virado para quem olha a planta). Cada espaço mostra até 4 etiquetas, numa linha própria da ficha do móvel (ao lado da planta). Para dividir um meio em dois movimentos, preencha também a linha da metade 2 (ex.: GONDOLA 1/MEIO-A-2): a linha do meio passa a valer para a metade 1 e a planta mostra o meio dividido.</t>
-  </si>
-  <si>
-    <t>6.3 Mesa destaque (FRENTE-1 e 2), mesa 3 frentes (FRENTE-1 a 3), totem (PAINEL-1 a 3; o 1 é o de cima) e móvel make (TESTEIRA-1 a 4): uma linha por bloco, com cor e etiqueta próprias. Cada frente das mesas mostra até 4 etiquetas; cada painel e cada testeira, 1. Blocos vizinhos com as mesmas etiquetas e cor ficam numa linha só da ficha do móvel.</t>
+    <t>6.2 Gôndola: uma linha por espaço — GONDOLA 1/LADO-A, MEIO-A, MEIO-B e LADO-B ("A" é sempre o lado virado para quem olha a planta). Cada espaço mostra até 4 etiquetas, junto dele na planta, com o nome do espaço (LADO A, MEIO B…). Para dividir um meio em dois movimentos, preencha também a linha da metade 2 (ex.: GONDOLA 1/MEIO-A-2): a linha do meio passa a valer para a metade 1 e a planta mostra o meio dividido.</t>
+  </si>
+  <si>
+    <t>6.3 Mesa destaque (FRENTE-1 e 2), mesa 3 frentes (FRENTE-1 a 3), totem (PAINEL-1 a 3; o 1 é o de cima) e móvel make (TESTEIRA-1 a 4): uma linha por bloco, com cor e etiqueta próprias. Cada frente das mesas mostra até 4 etiquetas; cada painel e cada testeira, 1. Blocos vizinhos com as mesmas etiquetas e cor ficam com uma pilha só.</t>
   </si>
   <si>
     <t>6.4 Móveis de um espaço só (pirâmide, móvel de fila, móvel de parede, PDV, O.U.i…) têm uma linha. O balcão recepção também: um espaço só, com uma cor e até 3 etiquetas.</t>

</xml_diff>

<commit_message>
Espaço fixo com cadeado e borda dupla; sai o símbolo movimento
- FIXO: o losango vira um cadeado, e as etiquetas do espaço fixo ganham
  borda dupla (um contorno a mais por fora, na cor da etiqueta), na
  planta e na visão simplificada. Painel, legenda e planilha base usam
  o cadeado; a planilha aceita também 'cadeado' e 🔒.
- O símbolo MOVIMENTO (▶) sai de todo o código e do ciclo de exemplo;
  planilhas antigas que ainda o têm ficam sem símbolo, sem aviso.
- Arquivos gerados e planilha base do visualizador atualizados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RtdsxaTNVwVJtEiaKjKwmm
</commit_message>
<xml_diff>
--- a/visualizador/Planilha base - Visualizador.xlsx
+++ b/visualizador/Planilha base - Visualizador.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="925" uniqueCount="287">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="907" uniqueCount="282">
   <si>
     <t>Ciclo</t>
   </si>
@@ -70,13 +70,13 @@
     <t>MOVEL DE PAREDE 1</t>
   </si>
   <si>
-    <t>Móvel de parede 1 · vale para ER P, ER M, ER G, ER GG</t>
+    <t>Perf. Fem. BOT · vale para ER P, ER M, ER G, ER GG</t>
   </si>
   <si>
     <t>NEUTRO</t>
   </si>
   <si>
-    <t>CUIDADOS (NSPA)</t>
+    <t>PERF FEM</t>
   </si>
   <si>
     <t>BOT</t>
@@ -298,7 +298,7 @@
     <t>MOVEL DE PAREDE 2</t>
   </si>
   <si>
-    <t>Móvel de parede 2 · vale para ER P, ER M, ER G, ER GG</t>
+    <t>Perf. Masc. BOT · vale para ER P, ER M, ER G, ER GG</t>
   </si>
   <si>
     <t>PERF MASC</t>
@@ -307,19 +307,16 @@
     <t>MOVEL DE PAREDE 3</t>
   </si>
   <si>
-    <t>Móvel de parede 3 · vale para ER P, ER M, ER G, ER GG</t>
-  </si>
-  <si>
-    <t>CUIDADOS (CBEM)</t>
+    <t>Perf. Fem. EUD · vale para ER P, ER M, ER G, ER GG</t>
   </si>
   <si>
     <t>MOVEL DE PAREDE 4</t>
   </si>
   <si>
-    <t>Móvel de parede 4 · vale para ER P, ER M, ER G, ER GG</t>
-  </si>
-  <si>
-    <t>PERF FEM</t>
+    <t>CBEM/NSPA · vale para ER P, ER M, ER G, ER GG</t>
+  </si>
+  <si>
+    <t>CUIDADOS (CBEM/NSPA)</t>
   </si>
   <si>
     <t>ER M</t>
@@ -340,9 +337,6 @@
     <t>PERFUMARIA</t>
   </si>
   <si>
-    <t>MOVIMENTO</t>
-  </si>
-  <si>
     <t>GONDOLA 2/MEIO-A-2</t>
   </si>
   <si>
@@ -629,9 +623,6 @@
   </si>
   <si>
     <t>Pirâmide 5</t>
-  </si>
-  <si>
-    <t>Móvel de parede 4</t>
   </si>
   <si>
     <t>ILHA PREMIUM OUI 1</t>
@@ -745,7 +736,7 @@
     <t>Planilha base — Plano de Varejo</t>
   </si>
   <si>
-    <t>Gerada em 15/10/2026, 21:49:10 a partir do ciclo "Ciclo exemplo".</t>
+    <t>Gerada em 16/10/2026, 16:32:13 a partir do ciclo "Ciclo exemplo".</t>
   </si>
   <si>
     <t>Como preencher</t>
@@ -769,7 +760,7 @@
     <t>6. Na aba "Painéis" ficam os textos fora dos móveis: listas TV / A / C, caixas de destaque (CALLOUT, que podem apontar para um ID Móvel) e notas (NOTA).</t>
   </si>
   <si>
-    <t>6.0 Na aba "Tipos de movimento" ficam os movimentos do ciclo: uma linha por movimento (o texto da etiqueta, igual ao da aba Movimentos), com a "Classificação" (Lançamento, Promoção, Liquidação / outlet, Institucional / portfólio, Outro ou outro texto) e o "GMV esperado (R$)". Elas aparecem no painel "Espaço por marca", em "Por tipo de movimento". Maiúsculas e espaços a mais não importam.</t>
+    <t>6.0 Na aba "Tipos de movimento" ficam os movimentos do ciclo: uma linha por movimento (o texto da etiqueta, igual ao da aba Movimentos), com a "Classificação" (Lançamento, Promoção, Liquidação / outlet, Institucional / portfólio, Outro ou outro texto) e o "GMV esperado (R$)". Elas aparecem no painel "Espaço por marca", em "Por movimentos". Maiúsculas e espaços a mais não importam.</t>
   </si>
   <si>
     <t>6.1 Gôndola, mesas, totem e móvel make são preenchidos espaço por espaço: não há linha do móvel inteiro (se houver, ela é ignorada). Espaço sem linha fica branco.</t>
@@ -835,13 +826,7 @@
     <t>Símbolos</t>
   </si>
   <si>
-    <t>▶</t>
-  </si>
-  <si>
-    <t>Movimento definido nesta planta</t>
-  </si>
-  <si>
-    <t>◆</t>
+    <t>🔒</t>
   </si>
   <si>
     <t>Espaço fixo (sem mudança nos ciclos)</t>
@@ -1843,7 +1828,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O375"/>
+  <dimension ref="A1:O374"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="13" style="1" customWidth="1"/>
@@ -2775,10 +2760,10 @@
         <v>19</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>98</v>
+        <v>20</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="H28" s="1" t="s">
         <v>22</v>
@@ -2803,16 +2788,16 @@
         <v>16</v>
       </c>
       <c r="C29" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="D29" s="4" t="s">
         <v>99</v>
-      </c>
-      <c r="D29" s="4" t="s">
-        <v>100</v>
       </c>
       <c r="E29" s="1" t="s">
         <v>19</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G29" s="1" t="s">
         <v>21</v>
@@ -2837,13 +2822,13 @@
         <v>15</v>
       </c>
       <c r="B30" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="C30" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="D30" s="7" t="s">
         <v>103</v>
-      </c>
-      <c r="D30" s="7" t="s">
-        <v>104</v>
       </c>
       <c r="E30" s="1" t="s">
         <v>27</v>
@@ -2869,19 +2854,19 @@
         <v>15</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C31" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="D31" s="7" t="s">
         <v>105</v>
-      </c>
-      <c r="D31" s="7" t="s">
-        <v>106</v>
       </c>
       <c r="E31" s="1" t="s">
         <v>46</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G31" s="1" t="s">
         <v>46</v>
@@ -2890,7 +2875,7 @@
       <c r="K31" s="1"/>
       <c r="M31" s="1"/>
       <c r="N31" s="1" t="s">
-        <v>108</v>
+        <v>24</v>
       </c>
       <c r="O31" s="1" t="s">
         <v>24</v>
@@ -2901,13 +2886,13 @@
         <v>15</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D32" s="7" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E32" s="1" t="s">
         <v>21</v>
@@ -2922,7 +2907,7 @@
       <c r="K32" s="1"/>
       <c r="M32" s="1"/>
       <c r="N32" s="1" t="s">
-        <v>108</v>
+        <v>24</v>
       </c>
       <c r="O32" s="1" t="s">
         <v>24</v>
@@ -2933,19 +2918,19 @@
         <v>15</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E33" s="1" t="s">
         <v>46</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="G33" s="1" t="s">
         <v>46</v>
@@ -2954,7 +2939,7 @@
       <c r="K33" s="1"/>
       <c r="M33" s="1"/>
       <c r="N33" s="1" t="s">
-        <v>108</v>
+        <v>24</v>
       </c>
       <c r="O33" s="1" t="s">
         <v>24</v>
@@ -2965,13 +2950,13 @@
         <v>15</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="E34" s="1"/>
       <c r="G34" s="1"/>
@@ -2985,13 +2970,13 @@
         <v>15</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="E35" s="1" t="s">
         <v>46</v>
@@ -3006,7 +2991,7 @@
       <c r="K35" s="1"/>
       <c r="M35" s="1"/>
       <c r="N35" s="1" t="s">
-        <v>108</v>
+        <v>24</v>
       </c>
       <c r="O35" s="1" t="s">
         <v>24</v>
@@ -3017,13 +3002,13 @@
         <v>15</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D36" s="7" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="E36" s="1" t="s">
         <v>21</v>
@@ -3049,13 +3034,13 @@
         <v>15</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="D37" s="7" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="E37" s="1" t="s">
         <v>27</v>
@@ -3081,28 +3066,28 @@
         <v>15</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C38" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="D38" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="E38" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="D38" s="7" t="s">
+      <c r="F38" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="E38" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="F38" s="1" t="s">
-        <v>125</v>
-      </c>
       <c r="G38" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I38" s="1"/>
       <c r="K38" s="1"/>
       <c r="M38" s="1"/>
       <c r="N38" s="1" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="O38" s="1" t="s">
         <v>24</v>
@@ -3113,28 +3098,28 @@
         <v>15</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C39" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="D39" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="F39" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="D39" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="E39" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="F39" s="1" t="s">
-        <v>129</v>
-      </c>
       <c r="G39" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I39" s="1"/>
       <c r="K39" s="1"/>
       <c r="M39" s="1"/>
       <c r="N39" s="1" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="O39" s="1" t="s">
         <v>24</v>
@@ -3145,13 +3130,13 @@
         <v>15</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D40" s="7" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E40" s="1" t="s">
         <v>46</v>
@@ -3177,13 +3162,13 @@
         <v>15</v>
       </c>
       <c r="B41" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="D41" s="4" t="s">
         <v>132</v>
-      </c>
-      <c r="C41" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="D41" s="4" t="s">
-        <v>134</v>
       </c>
       <c r="E41" s="1" t="s">
         <v>21</v>
@@ -3209,13 +3194,13 @@
         <v>15</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="E42" s="1" t="s">
         <v>46</v>
@@ -3230,7 +3215,7 @@
       <c r="K42" s="1"/>
       <c r="M42" s="1"/>
       <c r="N42" s="1" t="s">
-        <v>108</v>
+        <v>24</v>
       </c>
       <c r="O42" s="1" t="s">
         <v>24</v>
@@ -3241,19 +3226,19 @@
         <v>15</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="E43" s="1" t="s">
         <v>46</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="G43" s="1" t="s">
         <v>46</v>
@@ -3262,7 +3247,7 @@
       <c r="K43" s="1"/>
       <c r="M43" s="1"/>
       <c r="N43" s="1" t="s">
-        <v>108</v>
+        <v>24</v>
       </c>
       <c r="O43" s="1" t="s">
         <v>24</v>
@@ -3273,13 +3258,13 @@
         <v>15</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="E44" s="1"/>
       <c r="G44" s="1"/>
@@ -3293,19 +3278,19 @@
         <v>15</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E45" s="1" t="s">
         <v>23</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="G45" s="1" t="s">
         <v>23</v>
@@ -3314,7 +3299,7 @@
       <c r="K45" s="1"/>
       <c r="M45" s="1"/>
       <c r="N45" s="1" t="s">
-        <v>108</v>
+        <v>24</v>
       </c>
       <c r="O45" s="1" t="s">
         <v>24</v>
@@ -3325,13 +3310,13 @@
         <v>15</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E46" s="1"/>
       <c r="G46" s="1"/>
@@ -3345,13 +3330,13 @@
         <v>15</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="E47" s="1" t="s">
         <v>23</v>
@@ -3361,7 +3346,7 @@
       <c r="K47" s="1"/>
       <c r="M47" s="1"/>
       <c r="N47" s="1" t="s">
-        <v>108</v>
+        <v>24</v>
       </c>
       <c r="O47" s="1" t="s">
         <v>24</v>
@@ -3372,13 +3357,13 @@
         <v>15</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="E48" s="1"/>
       <c r="G48" s="1"/>
@@ -3392,13 +3377,13 @@
         <v>15</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D49" s="4" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="E49" s="1"/>
       <c r="G49" s="1"/>
@@ -3412,13 +3397,13 @@
         <v>15</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="E50" s="1" t="s">
         <v>27</v>
@@ -3444,13 +3429,13 @@
         <v>15</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="E51" s="1" t="s">
         <v>21</v>
@@ -3476,19 +3461,19 @@
         <v>15</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="E52" s="1" t="s">
         <v>23</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="G52" s="1" t="s">
         <v>23</v>
@@ -3508,13 +3493,13 @@
         <v>15</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="E53" s="1" t="s">
         <v>46</v>
@@ -3540,28 +3525,28 @@
         <v>15</v>
       </c>
       <c r="B54" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="C54" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="D54" s="7" t="s">
         <v>161</v>
       </c>
-      <c r="C54" s="6" t="s">
+      <c r="E54" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="F54" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="D54" s="7" t="s">
-        <v>163</v>
-      </c>
-      <c r="E54" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="F54" s="1" t="s">
-        <v>164</v>
-      </c>
       <c r="G54" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I54" s="1"/>
       <c r="K54" s="1"/>
       <c r="M54" s="1"/>
       <c r="N54" s="1" t="s">
-        <v>108</v>
+        <v>24</v>
       </c>
       <c r="O54" s="1" t="s">
         <v>24</v>
@@ -3572,23 +3557,23 @@
         <v>15</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="D55" s="7" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G55" s="1"/>
       <c r="I55" s="1"/>
       <c r="K55" s="1"/>
       <c r="M55" s="1"/>
       <c r="N55" s="1" t="s">
-        <v>108</v>
+        <v>24</v>
       </c>
       <c r="O55" s="1" t="s">
         <v>24</v>
@@ -3599,13 +3584,13 @@
         <v>15</v>
       </c>
       <c r="B56" s="6" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="D56" s="7" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="E56" s="1"/>
       <c r="G56" s="1"/>
@@ -3619,23 +3604,23 @@
         <v>15</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="D57" s="7" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G57" s="1"/>
       <c r="I57" s="1"/>
       <c r="K57" s="1"/>
       <c r="M57" s="1"/>
       <c r="N57" s="1" t="s">
-        <v>108</v>
+        <v>24</v>
       </c>
       <c r="O57" s="1" t="s">
         <v>24</v>
@@ -3646,13 +3631,13 @@
         <v>15</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D58" s="7" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E58" s="1"/>
       <c r="G58" s="1"/>
@@ -3666,23 +3651,23 @@
         <v>15</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D59" s="7" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G59" s="1"/>
       <c r="I59" s="1"/>
       <c r="K59" s="1"/>
       <c r="M59" s="1"/>
       <c r="N59" s="1" t="s">
-        <v>108</v>
+        <v>24</v>
       </c>
       <c r="O59" s="1" t="s">
         <v>24</v>
@@ -3693,13 +3678,13 @@
         <v>15</v>
       </c>
       <c r="B60" s="6" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="D60" s="7" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="E60" s="1" t="s">
         <v>27</v>
@@ -3725,13 +3710,13 @@
         <v>15</v>
       </c>
       <c r="B61" s="6" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D61" s="7" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="E61" s="1" t="s">
         <v>27</v>
@@ -3752,13 +3737,13 @@
         <v>15</v>
       </c>
       <c r="B62" s="6" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D62" s="7" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="E62" s="1"/>
       <c r="G62" s="1"/>
@@ -3772,13 +3757,13 @@
         <v>15</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D63" s="7" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="E63" s="1" t="s">
         <v>27</v>
@@ -3799,13 +3784,13 @@
         <v>15</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="D64" s="7" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="E64" s="1"/>
       <c r="G64" s="1"/>
@@ -3819,13 +3804,13 @@
         <v>15</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D65" s="7" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="E65" s="1" t="s">
         <v>27</v>
@@ -3846,19 +3831,19 @@
         <v>15</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="D66" s="7" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="E66" s="1" t="s">
         <v>46</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="G66" s="1" t="s">
         <v>46</v>
@@ -3867,7 +3852,7 @@
       <c r="K66" s="1"/>
       <c r="M66" s="1"/>
       <c r="N66" s="1" t="s">
-        <v>108</v>
+        <v>24</v>
       </c>
       <c r="O66" s="1" t="s">
         <v>24</v>
@@ -3878,13 +3863,13 @@
         <v>15</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="D67" s="7" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="E67" s="1" t="s">
         <v>46</v>
@@ -3894,7 +3879,7 @@
       <c r="K67" s="1"/>
       <c r="M67" s="1"/>
       <c r="N67" s="1" t="s">
-        <v>108</v>
+        <v>24</v>
       </c>
       <c r="O67" s="1" t="s">
         <v>24</v>
@@ -3905,13 +3890,13 @@
         <v>15</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="D68" s="7" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="E68" s="1"/>
       <c r="G68" s="1"/>
@@ -3925,13 +3910,13 @@
         <v>15</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="D69" s="7" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E69" s="1" t="s">
         <v>46</v>
@@ -3941,7 +3926,7 @@
       <c r="K69" s="1"/>
       <c r="M69" s="1"/>
       <c r="N69" s="1" t="s">
-        <v>108</v>
+        <v>24</v>
       </c>
       <c r="O69" s="1" t="s">
         <v>24</v>
@@ -3952,13 +3937,13 @@
         <v>15</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C70" s="6" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="D70" s="7" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="E70" s="1"/>
       <c r="G70" s="1"/>
@@ -3972,13 +3957,13 @@
         <v>15</v>
       </c>
       <c r="B71" s="6" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C71" s="6" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D71" s="7" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="E71" s="1" t="s">
         <v>46</v>
@@ -3988,7 +3973,7 @@
       <c r="K71" s="1"/>
       <c r="M71" s="1"/>
       <c r="N71" s="1" t="s">
-        <v>108</v>
+        <v>24</v>
       </c>
       <c r="O71" s="1" t="s">
         <v>24</v>
@@ -3999,19 +3984,19 @@
         <v>15</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C72" s="6" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="D72" s="7" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="E72" s="1" t="s">
         <v>23</v>
       </c>
       <c r="F72" s="1" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="G72" s="1" t="s">
         <v>46</v>
@@ -4020,7 +4005,7 @@
       <c r="K72" s="1"/>
       <c r="M72" s="1"/>
       <c r="N72" s="1" t="s">
-        <v>108</v>
+        <v>24</v>
       </c>
       <c r="O72" s="1" t="s">
         <v>24</v>
@@ -4031,19 +4016,19 @@
         <v>15</v>
       </c>
       <c r="B73" s="6" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C73" s="6" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="D73" s="7" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="E73" s="1" t="s">
         <v>21</v>
       </c>
       <c r="F73" s="1" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="G73" s="1" t="s">
         <v>21</v>
@@ -4052,7 +4037,7 @@
       <c r="K73" s="1"/>
       <c r="M73" s="1"/>
       <c r="N73" s="1" t="s">
-        <v>108</v>
+        <v>24</v>
       </c>
       <c r="O73" s="1" t="s">
         <v>24</v>
@@ -4063,74 +4048,45 @@
         <v>15</v>
       </c>
       <c r="B74" s="6" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C74" s="6" t="s">
-        <v>99</v>
+        <v>203</v>
       </c>
       <c r="D74" s="7" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E74" s="1" t="s">
-        <v>19</v>
+        <v>122</v>
       </c>
       <c r="F74" s="1" t="s">
-        <v>20</v>
+        <v>123</v>
       </c>
       <c r="G74" s="1" t="s">
-        <v>21</v>
+        <v>122</v>
       </c>
       <c r="H74" s="1" t="s">
-        <v>22</v>
+        <v>127</v>
       </c>
       <c r="I74" s="1" t="s">
-        <v>23</v>
+        <v>122</v>
       </c>
       <c r="K74" s="1"/>
       <c r="M74" s="1"/>
       <c r="N74" s="1" t="s">
-        <v>24</v>
+        <v>124</v>
       </c>
       <c r="O74" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="75" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A75" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B75" s="6" t="s">
-        <v>161</v>
-      </c>
-      <c r="C75" s="6" t="s">
-        <v>206</v>
-      </c>
-      <c r="D75" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="E75" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="F75" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="G75" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="H75" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="I75" s="1" t="s">
-        <v>124</v>
-      </c>
+    <row r="75" spans="5:14" x14ac:dyDescent="0.25">
+      <c r="E75" s="1"/>
+      <c r="G75" s="1"/>
+      <c r="I75" s="1"/>
       <c r="K75" s="1"/>
       <c r="M75" s="1"/>
-      <c r="N75" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="O75" s="1" t="s">
-        <v>24</v>
-      </c>
+      <c r="N75" s="1"/>
     </row>
     <row r="76" spans="5:14" x14ac:dyDescent="0.25">
       <c r="E76" s="1"/>
@@ -6524,17 +6480,9 @@
       <c r="M374" s="1"/>
       <c r="N374" s="1"/>
     </row>
-    <row r="375" spans="5:14" x14ac:dyDescent="0.25">
-      <c r="E375" s="1"/>
-      <c r="G375" s="1"/>
-      <c r="I375" s="1"/>
-      <c r="K375" s="1"/>
-      <c r="M375" s="1"/>
-      <c r="N375" s="1"/>
-    </row>
   </sheetData>
   <autoFilter ref="A1:O1"/>
-  <conditionalFormatting sqref="E2:E375">
+  <conditionalFormatting sqref="E2:E374">
     <cfRule type="containsText" dxfId="0" priority="1">
       <formula>NOT(ISERROR(SEARCH("BOT",E2)))</formula>
     </cfRule>
@@ -6554,7 +6502,7 @@
       <formula>NOT(ISERROR(SEARCH("NEUTRO",E2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G375">
+  <conditionalFormatting sqref="G2:G374">
     <cfRule type="containsText" dxfId="6" priority="1">
       <formula>NOT(ISERROR(SEARCH("BOT",G2)))</formula>
     </cfRule>
@@ -6574,7 +6522,7 @@
       <formula>NOT(ISERROR(SEARCH("NEUTRO",G2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I375">
+  <conditionalFormatting sqref="I2:I374">
     <cfRule type="containsText" dxfId="12" priority="1">
       <formula>NOT(ISERROR(SEARCH("BOT",I2)))</formula>
     </cfRule>
@@ -6594,7 +6542,7 @@
       <formula>NOT(ISERROR(SEARCH("NEUTRO",I2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K2:K375">
+  <conditionalFormatting sqref="K2:K374">
     <cfRule type="containsText" dxfId="18" priority="1">
       <formula>NOT(ISERROR(SEARCH("BOT",K2)))</formula>
     </cfRule>
@@ -6614,7 +6562,7 @@
       <formula>NOT(ISERROR(SEARCH("NEUTRO",K2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M2:M375">
+  <conditionalFormatting sqref="M2:M374">
     <cfRule type="containsText" dxfId="24" priority="1">
       <formula>NOT(ISERROR(SEARCH("BOT",M2)))</formula>
     </cfRule>
@@ -6635,41 +6583,41 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="12">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca do Móvel" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca do Móvel" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="E10:E375">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca do Móvel" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca do Móvel" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="E10:E374">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca do Móvel" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca do Móvel" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="E2:E375">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca do Móvel" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca do Móvel" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="E2:E374">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 1" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 1" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="G10:G375">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 1" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 1" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="G10:G374">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 1" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 1" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="G2:G375">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 1" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 1" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="G2:G374">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 2" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 2" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="I10:I375">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 2" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 2" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="I10:I374">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 2" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 2" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="I2:I375">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 2" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 2" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="I2:I374">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 3" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 3" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="K10:K375">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 3" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 3" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="K10:K374">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 3" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 3" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="K2:K375">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 3" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 3" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="K2:K374">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 4" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 4" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="M10:M375">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 4" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 4" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="M10:M374">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 4" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 4" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="M2:M375">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 4" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 4" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="M2:M374">
       <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo" prompt="MOVIMENTO = Movimento definido nesta planta; FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo" error="MOVIMENTO = Movimento definido nesta planta; FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" sqref="N10:N375">
-      <formula1>"MOVIMENTO,FIXO,EXPOSICAO,NOVO"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" sqref="N10:N374">
+      <formula1>"FIXO,EXPOSICAO,NOVO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo" prompt="MOVIMENTO = Movimento definido nesta planta; FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo" error="MOVIMENTO = Movimento definido nesta planta; FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" sqref="N2:N375">
-      <formula1>"MOVIMENTO,FIXO,EXPOSICAO,NOVO"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" sqref="N2:N374">
+      <formula1>"FIXO,EXPOSICAO,NOVO"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6696,16 +6644,16 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>208</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -6713,13 +6661,13 @@
         <v>15</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>23</v>
@@ -6733,10 +6681,10 @@
         <v>15</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>212</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>215</v>
       </c>
       <c r="D3" s="8" t="s">
         <v>65</v>
@@ -6753,13 +6701,13 @@
         <v>15</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>215</v>
-      </c>
       <c r="D4" s="8" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>46</v>
@@ -6773,10 +6721,10 @@
         <v>15</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="D5" s="8" t="s">
         <v>71</v>
@@ -6793,10 +6741,10 @@
         <v>15</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="D6" s="8" t="s">
         <v>61</v>
@@ -6813,13 +6761,13 @@
         <v>15</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>46</v>
@@ -6833,16 +6781,16 @@
         <v>15</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>24</v>
@@ -6853,13 +6801,13 @@
         <v>15</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C9" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="D9" s="8" t="s">
         <v>217</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>220</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>23</v>
@@ -6873,19 +6821,19 @@
         <v>15</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>23</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -6893,13 +6841,13 @@
         <v>15</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C11" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="D11" s="8" t="s">
         <v>221</v>
-      </c>
-      <c r="D11" s="8" t="s">
-        <v>224</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>21</v>
@@ -6913,13 +6861,13 @@
         <v>15</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>46</v>
@@ -6936,10 +6884,10 @@
         <v>16</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>24</v>
@@ -6956,10 +6904,10 @@
         <v>16</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>24</v>
@@ -6973,13 +6921,13 @@
         <v>15</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C15" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="D15" s="8" t="s">
         <v>226</v>
-      </c>
-      <c r="D15" s="8" t="s">
-        <v>229</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>24</v>
@@ -6993,13 +6941,13 @@
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>24</v>
@@ -7013,13 +6961,13 @@
         <v>15</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C17" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="D17" s="8" t="s">
         <v>226</v>
-      </c>
-      <c r="D17" s="8" t="s">
-        <v>229</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>24</v>
@@ -7033,13 +6981,13 @@
         <v>15</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>24</v>
@@ -7053,13 +7001,13 @@
         <v>15</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C19" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="D19" s="8" t="s">
         <v>226</v>
-      </c>
-      <c r="D19" s="8" t="s">
-        <v>229</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>24</v>
@@ -7073,13 +7021,13 @@
         <v>15</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>24</v>
@@ -7093,13 +7041,13 @@
         <v>15</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>24</v>
@@ -8351,7 +8299,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E330"/>
+  <dimension ref="A1:E329"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" style="1" customWidth="1"/>
@@ -8365,13 +8313,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>14</v>
@@ -8382,10 +8330,10 @@
         <v>15</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="D2" s="9">
         <v>150000</v>
@@ -8402,7 +8350,7 @@
         <v>43</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="D3" s="9">
         <v>1200000</v>
@@ -8419,7 +8367,7 @@
         <v>32</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D4" s="9">
         <v>650000</v>
@@ -8436,7 +8384,7 @@
         <v>65</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="D5" s="9">
         <v>2400000</v>
@@ -8453,7 +8401,7 @@
         <v>80</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="D6" s="9">
         <v>430000</v>
@@ -8467,10 +8415,10 @@
         <v>15</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D7" s="9">
         <v>610000</v>
@@ -8484,7 +8432,7 @@
         <v>15</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>24</v>
@@ -8499,7 +8447,7 @@
         <v>15</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>20</v>
+        <v>187</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>24</v>
@@ -8514,7 +8462,7 @@
         <v>15</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>189</v>
+        <v>162</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>24</v>
@@ -8529,7 +8477,7 @@
         <v>15</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>164</v>
+        <v>127</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>24</v>
@@ -8544,12 +8492,14 @@
         <v>15</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>129</v>
+        <v>200</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="D12" s="9"/>
+        <v>235</v>
+      </c>
+      <c r="D12" s="9">
+        <v>380000</v>
+      </c>
       <c r="E12" s="1" t="s">
         <v>24</v>
       </c>
@@ -8559,13 +8509,13 @@
         <v>15</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>202</v>
+        <v>29</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="D13" s="9">
-        <v>380000</v>
+        <v>620000</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>24</v>
@@ -8576,13 +8526,13 @@
         <v>15</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>29</v>
+        <v>61</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="D14" s="9">
-        <v>620000</v>
+        <v>1800000</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>24</v>
@@ -8593,13 +8543,13 @@
         <v>15</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>61</v>
+        <v>71</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="D15" s="9">
-        <v>1800000</v>
+        <v>950000</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>24</v>
@@ -8610,13 +8560,13 @@
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="D16" s="9">
-        <v>950000</v>
+        <v>210000</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>24</v>
@@ -8627,13 +8577,13 @@
         <v>15</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>81</v>
+        <v>28</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D17" s="9">
-        <v>210000</v>
+        <v>900000</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>24</v>
@@ -8644,13 +8594,13 @@
         <v>15</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>28</v>
+        <v>123</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="D18" s="9">
-        <v>900000</v>
+        <v>260000</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>24</v>
@@ -8661,13 +8611,13 @@
         <v>15</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>125</v>
+        <v>22</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
       <c r="D19" s="9">
-        <v>260000</v>
+        <v>1500000</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>24</v>
@@ -8678,13 +8628,13 @@
         <v>15</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>22</v>
+        <v>68</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="D20" s="9">
-        <v>1500000</v>
+        <v>1100000</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>24</v>
@@ -8695,14 +8645,12 @@
         <v>15</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>68</v>
+        <v>20</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>238</v>
-      </c>
-      <c r="D21" s="9">
-        <v>1100000</v>
-      </c>
+        <v>24</v>
+      </c>
+      <c r="D21" s="9"/>
       <c r="E21" s="1" t="s">
         <v>24</v>
       </c>
@@ -8712,7 +8660,7 @@
         <v>15</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>24</v>
@@ -8727,12 +8675,14 @@
         <v>15</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>95</v>
+        <v>106</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="D23" s="9"/>
+        <v>234</v>
+      </c>
+      <c r="D23" s="9">
+        <v>870000</v>
+      </c>
       <c r="E23" s="1" t="s">
         <v>24</v>
       </c>
@@ -8742,13 +8692,13 @@
         <v>15</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>107</v>
+        <v>49</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="D24" s="9">
-        <v>870000</v>
+        <v>700000</v>
       </c>
       <c r="E24" s="1" t="s">
         <v>24</v>
@@ -8759,13 +8709,13 @@
         <v>15</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>236</v>
       </c>
       <c r="D25" s="9">
-        <v>700000</v>
+        <v>480000</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>24</v>
@@ -8776,13 +8726,13 @@
         <v>15</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="D26" s="9">
-        <v>480000</v>
+        <v>780000</v>
       </c>
       <c r="E26" s="1" t="s">
         <v>24</v>
@@ -8793,13 +8743,13 @@
         <v>15</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="D27" s="9">
-        <v>780000</v>
+        <v>540000</v>
       </c>
       <c r="E27" s="1" t="s">
         <v>24</v>
@@ -8810,13 +8760,13 @@
         <v>15</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="D28" s="9">
-        <v>540000</v>
+        <v>520000</v>
       </c>
       <c r="E28" s="1" t="s">
         <v>24</v>
@@ -8827,32 +8777,19 @@
         <v>15</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>38</v>
+        <v>156</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>237</v>
-      </c>
-      <c r="D29" s="9">
-        <v>520000</v>
-      </c>
+        <v>24</v>
+      </c>
+      <c r="D29" s="9"/>
       <c r="E29" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>24</v>
-      </c>
+    <row r="30" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C30" s="1"/>
       <c r="D30" s="9"/>
-      <c r="E30" s="1" t="s">
-        <v>24</v>
-      </c>
     </row>
     <row r="31" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C31" s="1"/>
@@ -10050,13 +9987,9 @@
       <c r="C329" s="1"/>
       <c r="D329" s="9"/>
     </row>
-    <row r="330" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C330" s="1"/>
-      <c r="D330" s="9"/>
-    </row>
   </sheetData>
   <autoFilter ref="A1:E1"/>
-  <conditionalFormatting sqref="C2:C330">
+  <conditionalFormatting sqref="C2:C329">
     <cfRule type="containsText" dxfId="36" priority="1">
       <formula>NOT(ISERROR(SEARCH("Lançamento",C2)))</formula>
     </cfRule>
@@ -10074,10 +10007,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Classificação" prompt="Tipo do movimento: Lançamento, Promoção, Liquidação / outlet, Institucional / portfólio, Outro. Também aceita outro texto." showErrorMessage="1" errorStyle="warning" errorTitle="Classificação" error="Tipo do movimento: Lançamento, Promoção, Liquidação / outlet, Institucional / portfólio, Outro. Também aceita outro texto." sqref="C10:C330">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Classificação" prompt="Tipo do movimento: Lançamento, Promoção, Liquidação / outlet, Institucional / portfólio, Outro. Também aceita outro texto." showErrorMessage="1" errorStyle="warning" errorTitle="Classificação" error="Tipo do movimento: Lançamento, Promoção, Liquidação / outlet, Institucional / portfólio, Outro. Também aceita outro texto." sqref="C10:C329">
       <formula1>"Lançamento,Promoção,Liquidação / outlet,Institucional / portfólio,Outro"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Classificação" prompt="Tipo do movimento: Lançamento, Promoção, Liquidação / outlet, Institucional / portfólio, Outro. Também aceita outro texto." showErrorMessage="1" errorStyle="warning" errorTitle="Classificação" error="Tipo do movimento: Lançamento, Promoção, Liquidação / outlet, Institucional / portfólio, Outro. Também aceita outro texto." sqref="C2:C330">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Classificação" prompt="Tipo do movimento: Lançamento, Promoção, Liquidação / outlet, Institucional / portfólio, Outro. Também aceita outro texto." showErrorMessage="1" errorStyle="warning" errorTitle="Classificação" error="Tipo do movimento: Lançamento, Promoção, Liquidação / outlet, Institucional / portfólio, Outro. Também aceita outro texto." sqref="C2:C329">
       <formula1>"Lançamento,Promoção,Liquidação / outlet,Institucional / portfólio,Outro"</formula1>
     </dataValidation>
   </dataValidations>
@@ -10088,7 +10021,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:D46"/>
+  <dimension ref="B1:D45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -10099,122 +10032,122 @@
   <sheetData>
     <row r="1" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B1" s="11" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B2" s="12" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12"/>
     </row>
     <row r="4" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B4" s="13" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B5" s="12" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="C5" s="12"/>
       <c r="D5" s="12"/>
     </row>
     <row r="6" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B6" s="12" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="C6" s="12"/>
       <c r="D6" s="12"/>
     </row>
     <row r="7" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B7" s="12" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="12"/>
     </row>
     <row r="8" ht="45" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B8" s="12" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="C8" s="12"/>
       <c r="D8" s="12"/>
     </row>
     <row r="9" ht="16" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B9" s="12" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="C9" s="12"/>
       <c r="D9" s="12"/>
     </row>
     <row r="10" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B10" s="12" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="C10" s="12"/>
       <c r="D10" s="12"/>
     </row>
     <row r="11" ht="60" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B11" s="12" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="C11" s="12"/>
       <c r="D11" s="12"/>
     </row>
     <row r="12" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B12" s="12" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="C12" s="12"/>
       <c r="D12" s="12"/>
     </row>
     <row r="13" ht="60" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B13" s="12" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="C13" s="12"/>
       <c r="D13" s="12"/>
     </row>
     <row r="14" ht="60" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B14" s="12" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="C14" s="12"/>
       <c r="D14" s="12"/>
     </row>
     <row r="15" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B15" s="12" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="C15" s="12"/>
       <c r="D15" s="12"/>
     </row>
     <row r="16" ht="60" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B16" s="12" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="C16" s="12"/>
       <c r="D16" s="12"/>
     </row>
     <row r="17" ht="45" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B17" s="12" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="C17" s="12"/>
       <c r="D17" s="12"/>
     </row>
     <row r="18" ht="45" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B18" s="12" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="C18" s="12"/>
       <c r="D18" s="12"/>
     </row>
     <row r="20" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B20" s="13" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.25">
@@ -10222,10 +10155,10 @@
         <v>21</v>
       </c>
       <c r="C21" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="D21" s="15" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
     </row>
     <row r="22" spans="2:4" x14ac:dyDescent="0.25">
@@ -10233,10 +10166,10 @@
         <v>27</v>
       </c>
       <c r="C22" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
     </row>
     <row r="23" spans="2:4" x14ac:dyDescent="0.25">
@@ -10244,21 +10177,21 @@
         <v>46</v>
       </c>
       <c r="C23" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="D23" s="17" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
     </row>
     <row r="24" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B24" s="14" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C24" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D24" s="18" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.25">
@@ -10266,10 +10199,10 @@
         <v>23</v>
       </c>
       <c r="C25" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="D25" s="19" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
     </row>
     <row r="26" spans="2:4" x14ac:dyDescent="0.25">
@@ -10277,140 +10210,129 @@
         <v>19</v>
       </c>
       <c r="C26" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="D26" s="20" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="28" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B28" s="13" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
     </row>
     <row r="29" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B29" s="14" t="s">
-        <v>108</v>
+        <v>33</v>
       </c>
       <c r="C29" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="D29" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
     </row>
     <row r="30" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B30" s="14" t="s">
-        <v>33</v>
+        <v>124</v>
       </c>
       <c r="C30" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="D30" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
     </row>
     <row r="31" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B31" s="14" t="s">
-        <v>126</v>
+        <v>272</v>
       </c>
       <c r="C31" t="s">
+        <v>273</v>
+      </c>
+      <c r="D31" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="33" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B33" s="13" t="s">
         <v>275</v>
       </c>
-      <c r="D31" t="s">
+    </row>
+    <row r="34" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B34" s="21" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="35" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B35" s="22" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="36" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B36" s="23" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="37" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B37" s="24" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="38" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B38" s="25" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="40" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B40" s="13" t="s">
         <v>276</v>
       </c>
     </row>
-    <row r="32" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B32" s="14" t="s">
+    <row r="41" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B41" s="14" t="s">
+        <v>210</v>
+      </c>
+      <c r="C41" t="s">
         <v>277</v>
       </c>
-      <c r="C32" t="s">
-        <v>278</v>
-      </c>
-      <c r="D32" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="34" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B34" s="13" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="35" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B35" s="21" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="36" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B36" s="22" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="37" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B37" s="23" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="38" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B38" s="24" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="39" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B39" s="25" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="41" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B41" s="13" t="s">
-        <v>281</v>
-      </c>
+      <c r="D41"/>
     </row>
     <row r="42" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B42" s="14" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C42" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="D42"/>
     </row>
     <row r="43" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B43" s="14" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C43" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="D43"/>
     </row>
     <row r="44" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B44" s="14" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C44" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="D44"/>
     </row>
     <row r="45" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B45" s="14" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C45" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="D45"/>
-    </row>
-    <row r="46" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B46" s="14" t="s">
-        <v>226</v>
-      </c>
-      <c r="C46" t="s">
-        <v>286</v>
-      </c>
-      <c r="D46"/>
     </row>
   </sheetData>
   <mergeCells count="20">
@@ -10429,11 +10351,11 @@
     <mergeCell ref="B16:D16"/>
     <mergeCell ref="B17:D17"/>
     <mergeCell ref="B18:D18"/>
+    <mergeCell ref="C41:D41"/>
     <mergeCell ref="C42:D42"/>
     <mergeCell ref="C43:D43"/>
     <mergeCell ref="C44:D44"/>
     <mergeCell ref="C45:D45"/>
-    <mergeCell ref="C46:D46"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Construção do ciclo: meio da gôndola em 2, etiquetas sob demanda e cores das marcas
- Fixos copiados aparecem na planta em construção: a comparação de ciclos sai ao montar um ciclo
- Dividir em 2 / Juntar metades nos meios da gôndola, no painel de construção
- Cada espaço começa com uma etiqueta; "+ Adicionar etiqueta" até o limite (4) e "×" para tirar
- Selects de marca com a cor da marca no fundo (construção e antecipação)
- Ordem das marcas BOT | EUD | QDB | OUI | MM em todo o app
- Visualizador sem a comparação de ciclos
- Testes, documentação e arquivos gerados atualizados

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GqpAiGcpzkPePwg7sgDhuP
</commit_message>
<xml_diff>
--- a/visualizador/Planilha base - Visualizador.xlsx
+++ b/visualizador/Planilha base - Visualizador.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="907" uniqueCount="282">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="927" uniqueCount="282">
   <si>
     <t>Ciclo</t>
   </si>
@@ -91,10 +91,10 @@
     <t/>
   </si>
   <si>
-    <t>GONDOLA 1/LADO-A</t>
-  </si>
-  <si>
-    <t>Gôndola 1 – Lado A · vale para ER P, ER M, ER G, ER GG</t>
+    <t>GONDOLA 1/PONTA-A</t>
+  </si>
+  <si>
+    <t>Gôndola 1 – Ponta A · vale para ER P, ER M, ER G, ER GG</t>
   </si>
   <si>
     <t>QDB</t>
@@ -139,10 +139,10 @@
     <t>Gôndola 1 – Meio B – metade 2 (preencha só para dividir o meio em dois)</t>
   </si>
   <si>
-    <t>GONDOLA 1/LADO-B</t>
-  </si>
-  <si>
-    <t>Gôndola 1 – Lado B</t>
+    <t>GONDOLA 1/PONTA-B</t>
+  </si>
+  <si>
+    <t>Gôndola 1 – Ponta B</t>
   </si>
   <si>
     <t>BOTI PROMO</t>
@@ -166,6 +166,9 @@
     <t>PRINCIPAIS OPORTUNIDADES</t>
   </si>
   <si>
+    <t>BOTIPROMO</t>
+  </si>
+  <si>
     <t>MESA DESTAQUE 1/FRENTE-1</t>
   </si>
   <si>
@@ -184,6 +187,15 @@
     <t>SIÀGE GLORIFICADO</t>
   </si>
   <si>
+    <t>MESA DESTAQUE 1/VERSO</t>
+  </si>
+  <si>
+    <t>Mesa destaque 1 – Verso</t>
+  </si>
+  <si>
+    <t>LÇTO UOMINI</t>
+  </si>
+  <si>
     <t>PDV MOVEL 1</t>
   </si>
   <si>
@@ -211,9 +223,6 @@
     <t>Móvel de fila 2 · vale para ER P, ER M, ER G, ER GG</t>
   </si>
   <si>
-    <t>BOTIPROMO</t>
-  </si>
-  <si>
     <t>MOVEL DE FILA 1</t>
   </si>
   <si>
@@ -229,9 +238,6 @@
     <t>Totem 1 – Painel 1 · vale para ER P, ER M, ER G, ER GG</t>
   </si>
   <si>
-    <t>LÇTO UOMINI</t>
-  </si>
-  <si>
     <t>TOTEM 1/PAINEL-2</t>
   </si>
   <si>
@@ -322,10 +328,10 @@
     <t>ER M</t>
   </si>
   <si>
-    <t>GONDOLA 2/LADO-A</t>
-  </si>
-  <si>
-    <t>Gôndola 2 – Lado A · vale para ER M, ER G, ER GG</t>
+    <t>GONDOLA 2/PONTA-A</t>
+  </si>
+  <si>
+    <t>Gôndola 2 – Ponta A · vale para ER M, ER G, ER GG</t>
   </si>
   <si>
     <t>GONDOLA 2/MEIO-A</t>
@@ -358,10 +364,10 @@
     <t>Gôndola 2 – Meio B – metade 2 (preencha só para dividir o meio em dois)</t>
   </si>
   <si>
-    <t>GONDOLA 2/LADO-B</t>
-  </si>
-  <si>
-    <t>Gôndola 2 – Lado B</t>
+    <t>GONDOLA 2/PONTA-B</t>
+  </si>
+  <si>
+    <t>Gôndola 2 – Ponta B</t>
   </si>
   <si>
     <t>MOVEL DE FILA 3</t>
@@ -415,10 +421,10 @@
     <t>Móvel de fila 6 · vale para ER G, ER GG</t>
   </si>
   <si>
-    <t>GONDOLA 3/LADO-A</t>
-  </si>
-  <si>
-    <t>Gôndola 3 – Lado A · vale para ER G, ER GG</t>
+    <t>GONDOLA 3/PONTA-A</t>
+  </si>
+  <si>
+    <t>Gôndola 3 – Ponta A · vale para ER G, ER GG</t>
   </si>
   <si>
     <t>GONDOLA 3/MEIO-A</t>
@@ -448,10 +454,10 @@
     <t>Gôndola 3 – Meio B – metade 2 (preencha só para dividir o meio em dois)</t>
   </si>
   <si>
-    <t>GONDOLA 3/LADO-B</t>
-  </si>
-  <si>
-    <t>Gôndola 3 – Lado B</t>
+    <t>GONDOLA 3/PONTA-B</t>
+  </si>
+  <si>
+    <t>Gôndola 3 – Ponta B</t>
   </si>
   <si>
     <t>MOVEL DE FILA 7</t>
@@ -493,13 +499,19 @@
     <t>Mesa destaque 3 frentes 1 – Frente 3</t>
   </si>
   <si>
+    <t>MESA DESTAQUE 3 FRENTES 1/VERSO</t>
+  </si>
+  <si>
+    <t>Mesa destaque 3 frentes 1 – Verso</t>
+  </si>
+  <si>
     <t>ER GG</t>
   </si>
   <si>
-    <t>GONDOLA 4/LADO-A</t>
-  </si>
-  <si>
-    <t>Gôndola 4 – Lado A</t>
+    <t>GONDOLA 4/PONTA-A</t>
+  </si>
+  <si>
+    <t>Gôndola 4 – Ponta A</t>
   </si>
   <si>
     <t>EXAUSTÃO OUI</t>
@@ -529,16 +541,16 @@
     <t>Gôndola 4 – Meio B – metade 2 (preencha só para dividir o meio em dois)</t>
   </si>
   <si>
-    <t>GONDOLA 4/LADO-B</t>
-  </si>
-  <si>
-    <t>Gôndola 4 – Lado B</t>
-  </si>
-  <si>
-    <t>GONDOLA 5/LADO-A</t>
-  </si>
-  <si>
-    <t>Gôndola 5 – Lado A</t>
+    <t>GONDOLA 4/PONTA-B</t>
+  </si>
+  <si>
+    <t>Gôndola 4 – Ponta B</t>
+  </si>
+  <si>
+    <t>GONDOLA 5/PONTA-A</t>
+  </si>
+  <si>
+    <t>Gôndola 5 – Ponta A</t>
   </si>
   <si>
     <t>GONDOLA 5/MEIO-A</t>
@@ -565,16 +577,16 @@
     <t>Gôndola 5 – Meio B – metade 2 (preencha só para dividir o meio em dois)</t>
   </si>
   <si>
-    <t>GONDOLA 5/LADO-B</t>
-  </si>
-  <si>
-    <t>Gôndola 5 – Lado B</t>
-  </si>
-  <si>
-    <t>GONDOLA 6/LADO-A</t>
-  </si>
-  <si>
-    <t>Gôndola 6 – Lado A</t>
+    <t>GONDOLA 5/PONTA-B</t>
+  </si>
+  <si>
+    <t>Gôndola 5 – Ponta B</t>
+  </si>
+  <si>
+    <t>GONDOLA 6/PONTA-A</t>
+  </si>
+  <si>
+    <t>Gôndola 6 – Ponta A</t>
   </si>
   <si>
     <t>EXAUSTÃO EUD</t>
@@ -604,10 +616,10 @@
     <t>Gôndola 6 – Meio B – metade 2 (preencha só para dividir o meio em dois)</t>
   </si>
   <si>
-    <t>GONDOLA 6/LADO-B</t>
-  </si>
-  <si>
-    <t>Gôndola 6 – Lado B</t>
+    <t>GONDOLA 6/PONTA-B</t>
+  </si>
+  <si>
+    <t>Gôndola 6 – Ponta B</t>
   </si>
   <si>
     <t>PIRAMIDE 4</t>
@@ -736,7 +748,7 @@
     <t>Planilha base — Plano de Varejo</t>
   </si>
   <si>
-    <t>Gerada em 16/10/2026, 19:38:08 a partir do ciclo "Ciclo exemplo".</t>
+    <t>Gerada em 20/10/2026, 21:39:36 a partir do ciclo "Ciclo exemplo".</t>
   </si>
   <si>
     <t>Como preencher</t>
@@ -760,16 +772,16 @@
     <t>6. Na aba "Painéis" ficam os textos fora dos móveis: listas TV / A / C, caixas de destaque (CALLOUT, que podem apontar para um ID Móvel) e notas (NOTA).</t>
   </si>
   <si>
-    <t>6.0 Na aba "Tipos de movimento" ficam os movimentos do ciclo: uma linha por movimento (o texto da etiqueta, igual ao da aba Movimentos), com a "Classificação" (Lançamento, Promoção, Liquidação / outlet, Institucional / portfólio, Outro ou outro texto) e o "GMV esperado (R$)". Elas aparecem no painel "Espaço por marca", em "Por movimentos". Maiúsculas e espaços a mais não importam.</t>
+    <t>6.0 Na aba "Tipos de movimento" ficam os movimentos do ciclo: uma linha por movimento (o texto da etiqueta, igual ao da aba Movimentos), com a "Classificação" (Lançamento, Promoção, Liquidação / outlet, Institucional / portfólio, Outro ou outro texto) e o "GMV esperado (R$)". Elas aparecem no Analytics (movimentos, classificações e GMV esperado de cada ER). Maiúsculas e espaços a mais não importam.</t>
   </si>
   <si>
     <t>6.1 Gôndola, mesas, totem e móvel make são preenchidos espaço por espaço: não há linha do móvel inteiro (se houver, ela é ignorada). Espaço sem linha fica branco.</t>
   </si>
   <si>
-    <t>6.2 Gôndola: uma linha por espaço — GONDOLA 1/LADO-A, MEIO-A, MEIO-B e LADO-B ("A" é sempre o lado virado para quem olha a planta). Cada espaço mostra até 4 etiquetas, junto dele na planta, com o nome do espaço (LADO A, MEIO B…). Para dividir um meio em dois movimentos, preencha também a linha da metade 2 (ex.: GONDOLA 1/MEIO-A-2): a linha do meio passa a valer para a metade 1 e a planta mostra o meio dividido.</t>
-  </si>
-  <si>
-    <t>6.3 Mesa destaque (FRENTE-1 e 2), mesa 3 frentes (FRENTE-1 a 3), totem (PAINEL-1 a 3; o 1 é o de cima) e móvel make (TESTEIRA-1 a 4): uma linha por bloco, com cor e etiqueta próprias. Cada frente das mesas mostra até 4 etiquetas; cada painel e cada testeira, 1. Blocos vizinhos com as mesmas etiquetas e cor ficam com uma pilha só.</t>
+    <t>6.2 Gôndola: uma linha por espaço — GONDOLA 1/PONTA-A, MEIO-A, MEIO-B e PONTA-B ("A" é sempre o lado virado para quem olha a planta). Cada espaço mostra até 4 etiquetas, junto dele na planta, com o nome do espaço (PONTA A, MEIO B…). Para dividir um meio em dois movimentos, preencha também a linha da metade 2 (ex.: GONDOLA 1/MEIO-A-2): a linha do meio passa a valer para a metade 1 e a planta mostra o meio dividido.</t>
+  </si>
+  <si>
+    <t>6.3 Mesa destaque (FRENTE-1 e 2, e VERSO, atrás das lâminas), mesa 3 frentes (FRENTE-1 a 3 e VERSO), totem (PAINEL-1 a 3; o 1 é o de cima) e móvel make (TESTEIRA-1 a 4): uma linha por bloco, com cor e etiqueta próprias. Cada frente e o verso das mesas mostram até 4 etiquetas; cada painel e cada testeira, 1. Blocos vizinhos com as mesmas etiquetas e cor ficam com uma pilha só.</t>
   </si>
   <si>
     <t>6.4 Móveis de um espaço só (pirâmide, móvel de fila, móvel de parede, PDV, O.U.i…) têm uma linha. O balcão recepção também: um espaço só, com uma cor e até 3 etiquetas.</t>
@@ -787,31 +799,19 @@
     <t>Marcas (cores)</t>
   </si>
   <si>
-    <t>Boticário</t>
-  </si>
-  <si>
     <t>Etiqueta #3E9D6B  ·  Móvel #7CC9A0</t>
   </si>
   <si>
-    <t>Quem disse, berenice?</t>
+    <t>Etiqueta #A11FC9  ·  Móvel #B666D8</t>
   </si>
   <si>
     <t>Etiqueta #E23FB4  ·  Móvel #F07ACD</t>
   </si>
   <si>
-    <t>Eudora</t>
-  </si>
-  <si>
-    <t>Etiqueta #A11FC9  ·  Móvel #B666D8</t>
-  </si>
-  <si>
-    <t>O.U.i</t>
-  </si>
-  <si>
     <t>Etiqueta #E1262F  ·  Móvel #C9343F</t>
   </si>
   <si>
-    <t>Multimarca</t>
+    <t>MM</t>
   </si>
   <si>
     <t>Etiqueta #2B4DE3  ·  Móvel #7D90EC</t>
@@ -941,12 +941,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE23FB4"/>
+        <fgColor rgb="FFA11FC9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFA11FC9"/>
+        <fgColor rgb="FFE23FB4"/>
       </patternFill>
     </fill>
     <fill>
@@ -1060,7 +1060,7 @@
       </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFE23FB4"/>
+          <bgColor rgb="FFA11FC9"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1071,7 +1071,7 @@
       </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFA11FC9"/>
+          <bgColor rgb="FFE23FB4"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1126,7 +1126,7 @@
       </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFE23FB4"/>
+          <bgColor rgb="FFA11FC9"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1137,7 +1137,7 @@
       </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFA11FC9"/>
+          <bgColor rgb="FFE23FB4"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1192,7 +1192,7 @@
       </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFE23FB4"/>
+          <bgColor rgb="FFA11FC9"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1203,7 +1203,7 @@
       </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFA11FC9"/>
+          <bgColor rgb="FFE23FB4"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1258,7 +1258,7 @@
       </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFE23FB4"/>
+          <bgColor rgb="FFA11FC9"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1269,7 +1269,7 @@
       </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFA11FC9"/>
+          <bgColor rgb="FFE23FB4"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1324,7 +1324,7 @@
       </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFE23FB4"/>
+          <bgColor rgb="FFA11FC9"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1335,7 +1335,7 @@
       </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFA11FC9"/>
+          <bgColor rgb="FFE23FB4"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1390,7 +1390,7 @@
       </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFE23FB4"/>
+          <bgColor rgb="FFA11FC9"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1401,7 +1401,7 @@
       </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFA11FC9"/>
+          <bgColor rgb="FFE23FB4"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1828,7 +1828,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O374"/>
+  <dimension ref="A1:O376"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="13" style="1" customWidth="1"/>
@@ -2157,7 +2157,12 @@
       <c r="G10" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="I10" s="1"/>
+      <c r="H10" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>21</v>
+      </c>
       <c r="K10" s="1"/>
       <c r="M10" s="1"/>
       <c r="N10" s="1" t="s">
@@ -2175,16 +2180,16 @@
         <v>16</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>21</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G11" s="1" t="s">
         <v>21</v>
@@ -2207,16 +2212,16 @@
         <v>16</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>46</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G12" s="1" t="s">
         <v>46</v>
@@ -2239,19 +2244,19 @@
         <v>16</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>46</v>
+        <v>21</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>46</v>
+        <v>21</v>
       </c>
       <c r="I13" s="1"/>
       <c r="K13" s="1"/>
@@ -2271,34 +2276,23 @@
         <v>16</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="H14" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="I14" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J14" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="K14" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="L14" s="5"/>
-      <c r="M14" s="5"/>
+      <c r="I14" s="1"/>
+      <c r="K14" s="1"/>
+      <c r="M14" s="1"/>
       <c r="N14" s="1" t="s">
         <v>24</v>
       </c>
@@ -2326,11 +2320,22 @@
         <v>65</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="I15" s="1"/>
-      <c r="K15" s="1"/>
-      <c r="M15" s="1"/>
+        <v>66</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J15" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="K15" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="L15" s="5"/>
+      <c r="M15" s="5"/>
       <c r="N15" s="1" t="s">
         <v>24</v>
       </c>
@@ -2346,19 +2351,19 @@
         <v>16</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>46</v>
+        <v>21</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>46</v>
+        <v>21</v>
       </c>
       <c r="I16" s="1"/>
       <c r="K16" s="1"/>
@@ -2384,20 +2389,17 @@
         <v>70</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>71</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="H17" s="5"/>
-      <c r="I17" s="5"/>
-      <c r="J17" s="5"/>
-      <c r="K17" s="5"/>
-      <c r="L17" s="5"/>
-      <c r="M17" s="5"/>
+        <v>46</v>
+      </c>
+      <c r="I17" s="1"/>
+      <c r="K17" s="1"/>
+      <c r="M17" s="1"/>
       <c r="N17" s="1" t="s">
         <v>24</v>
       </c>
@@ -2422,7 +2424,7 @@
         <v>21</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="G18" s="1" t="s">
         <v>21</v>
@@ -2454,13 +2456,13 @@
         <v>75</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>28</v>
+        <v>50</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="H19" s="5"/>
       <c r="I19" s="5"/>
@@ -2489,17 +2491,20 @@
         <v>77</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>61</v>
+        <v>28</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="I20" s="1"/>
-      <c r="K20" s="1"/>
-      <c r="M20" s="1"/>
+        <v>27</v>
+      </c>
+      <c r="H20" s="5"/>
+      <c r="I20" s="5"/>
+      <c r="J20" s="5"/>
+      <c r="K20" s="5"/>
+      <c r="L20" s="5"/>
+      <c r="M20" s="5"/>
       <c r="N20" s="1" t="s">
         <v>24</v>
       </c>
@@ -2524,17 +2529,12 @@
         <v>19</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="H21" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="I21" s="1" t="s">
-        <v>27</v>
-      </c>
+        <v>66</v>
+      </c>
+      <c r="I21" s="1"/>
       <c r="K21" s="1"/>
       <c r="M21" s="1"/>
       <c r="N21" s="1" t="s">
@@ -2552,21 +2552,26 @@
         <v>16</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E22" s="1" t="s">
         <v>19</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>58</v>
+        <v>82</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="I22" s="1"/>
+        <v>21</v>
+      </c>
+      <c r="H22" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="I22" s="1" t="s">
+        <v>27</v>
+      </c>
       <c r="K22" s="1"/>
       <c r="M22" s="1"/>
       <c r="N22" s="1" t="s">
@@ -2590,15 +2595,17 @@
         <v>85</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="G23" s="1"/>
-      <c r="H23" s="5"/>
-      <c r="I23" s="5"/>
-      <c r="J23" s="5"/>
-      <c r="K23" s="5"/>
-      <c r="L23" s="5"/>
-      <c r="M23" s="5"/>
+        <v>19</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="I23" s="1"/>
+      <c r="K23" s="1"/>
+      <c r="M23" s="1"/>
       <c r="N23" s="1" t="s">
         <v>24</v>
       </c>
@@ -2614,20 +2621,15 @@
         <v>16</v>
       </c>
       <c r="C24" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="D24" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="E24" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="E24" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F24" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="G24" s="1" t="s">
-        <v>21</v>
-      </c>
+      <c r="G24" s="1"/>
       <c r="H24" s="5"/>
       <c r="I24" s="5"/>
       <c r="J24" s="5"/>
@@ -2658,7 +2660,7 @@
         <v>21</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G25" s="1" t="s">
         <v>21</v>
@@ -2690,9 +2692,14 @@
         <v>92</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="G26" s="1"/>
+        <v>21</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>21</v>
+      </c>
       <c r="H26" s="5"/>
       <c r="I26" s="5"/>
       <c r="J26" s="5"/>
@@ -2720,22 +2727,15 @@
         <v>94</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F27" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="G27" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="H27" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="I27" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="K27" s="1"/>
-      <c r="M27" s="1"/>
+        <v>46</v>
+      </c>
+      <c r="G27" s="1"/>
+      <c r="H27" s="5"/>
+      <c r="I27" s="5"/>
+      <c r="J27" s="5"/>
+      <c r="K27" s="5"/>
+      <c r="L27" s="5"/>
+      <c r="M27" s="5"/>
       <c r="N27" s="1" t="s">
         <v>24</v>
       </c>
@@ -2751,19 +2751,19 @@
         <v>16</v>
       </c>
       <c r="C28" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="D28" s="4" t="s">
         <v>96</v>
-      </c>
-      <c r="D28" s="4" t="s">
-        <v>97</v>
       </c>
       <c r="E28" s="1" t="s">
         <v>19</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>20</v>
+        <v>97</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>46</v>
+        <v>21</v>
       </c>
       <c r="H28" s="1" t="s">
         <v>22</v>
@@ -2797,10 +2797,10 @@
         <v>19</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="H29" s="1" t="s">
         <v>22</v>
@@ -2818,28 +2818,33 @@
       </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A30" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B30" s="6" t="s">
+      <c r="A30" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="D30" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="E30" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F30" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="D30" s="7" t="s">
-        <v>103</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="F30" s="1" t="s">
-        <v>28</v>
-      </c>
       <c r="G30" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="I30" s="1"/>
+        <v>21</v>
+      </c>
+      <c r="H30" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I30" s="1" t="s">
+        <v>23</v>
+      </c>
       <c r="K30" s="1"/>
       <c r="M30" s="1"/>
       <c r="N30" s="1" t="s">
@@ -2854,7 +2859,7 @@
         <v>15</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C31" s="6" t="s">
         <v>104</v>
@@ -2863,13 +2868,13 @@
         <v>105</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>46</v>
+        <v>27</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>106</v>
+        <v>28</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>46</v>
+        <v>27</v>
       </c>
       <c r="I31" s="1"/>
       <c r="K31" s="1"/>
@@ -2886,22 +2891,22 @@
         <v>15</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C32" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="D32" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="D32" s="7" t="s">
+      <c r="E32" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F32" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="E32" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F32" s="1" t="s">
-        <v>43</v>
-      </c>
       <c r="G32" s="1" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="I32" s="1"/>
       <c r="K32" s="1"/>
@@ -2918,7 +2923,7 @@
         <v>15</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C33" s="6" t="s">
         <v>109</v>
@@ -2927,13 +2932,13 @@
         <v>110</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>46</v>
+        <v>21</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>111</v>
+        <v>43</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>46</v>
+        <v>21</v>
       </c>
       <c r="I33" s="1"/>
       <c r="K33" s="1"/>
@@ -2945,32 +2950,44 @@
         <v>24</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C34" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="D34" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="D34" s="7" t="s">
+      <c r="E34" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F34" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="E34" s="1"/>
-      <c r="G34" s="1"/>
+      <c r="G34" s="1" t="s">
+        <v>46</v>
+      </c>
       <c r="I34" s="1"/>
       <c r="K34" s="1"/>
       <c r="M34" s="1"/>
-      <c r="N34" s="1"/>
-    </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N34" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O34" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C35" s="6" t="s">
         <v>114</v>
@@ -2978,31 +2995,19 @@
       <c r="D35" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="E35" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="F35" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="G35" s="1" t="s">
-        <v>46</v>
-      </c>
+      <c r="E35" s="1"/>
+      <c r="G35" s="1"/>
       <c r="I35" s="1"/>
       <c r="K35" s="1"/>
       <c r="M35" s="1"/>
-      <c r="N35" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="O35" s="1" t="s">
-        <v>24</v>
-      </c>
+      <c r="N35" s="1"/>
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C36" s="6" t="s">
         <v>116</v>
@@ -3011,13 +3016,13 @@
         <v>117</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="I36" s="1"/>
       <c r="K36" s="1"/>
@@ -3034,7 +3039,7 @@
         <v>15</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C37" s="6" t="s">
         <v>118</v>
@@ -3043,13 +3048,13 @@
         <v>119</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>28</v>
+        <v>50</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="I37" s="1"/>
       <c r="K37" s="1"/>
@@ -3066,7 +3071,7 @@
         <v>15</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C38" s="6" t="s">
         <v>120</v>
@@ -3075,19 +3080,19 @@
         <v>121</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>122</v>
+        <v>27</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>123</v>
+        <v>28</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>122</v>
+        <v>27</v>
       </c>
       <c r="I38" s="1"/>
       <c r="K38" s="1"/>
       <c r="M38" s="1"/>
       <c r="N38" s="1" t="s">
-        <v>124</v>
+        <v>24</v>
       </c>
       <c r="O38" s="1" t="s">
         <v>24</v>
@@ -3098,28 +3103,28 @@
         <v>15</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C39" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="D39" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="F39" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="D39" s="7" t="s">
-        <v>126</v>
-      </c>
-      <c r="E39" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="F39" s="1" t="s">
-        <v>127</v>
-      </c>
       <c r="G39" s="1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="I39" s="1"/>
       <c r="K39" s="1"/>
       <c r="M39" s="1"/>
       <c r="N39" s="1" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="O39" s="1" t="s">
         <v>24</v>
@@ -3130,54 +3135,54 @@
         <v>15</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C40" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="D40" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="D40" s="7" t="s">
+      <c r="E40" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="F40" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="E40" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="F40" s="1" t="s">
-        <v>22</v>
-      </c>
       <c r="G40" s="1" t="s">
-        <v>23</v>
+        <v>124</v>
       </c>
       <c r="I40" s="1"/>
       <c r="K40" s="1"/>
       <c r="M40" s="1"/>
       <c r="N40" s="1" t="s">
-        <v>24</v>
+        <v>126</v>
       </c>
       <c r="O40" s="1" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A41" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B41" s="3" t="s">
+      <c r="A41" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="C41" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="C41" s="3" t="s">
+      <c r="D41" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="D41" s="4" t="s">
-        <v>132</v>
-      </c>
       <c r="E41" s="1" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>65</v>
+        <v>22</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I41" s="1"/>
       <c r="K41" s="1"/>
@@ -3194,7 +3199,7 @@
         <v>15</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C42" s="3" t="s">
         <v>133</v>
@@ -3203,13 +3208,13 @@
         <v>134</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>46</v>
+        <v>21</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>46</v>
+        <v>21</v>
       </c>
       <c r="I42" s="1"/>
       <c r="K42" s="1"/>
@@ -3226,7 +3231,7 @@
         <v>15</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C43" s="3" t="s">
         <v>135</v>
@@ -3238,7 +3243,7 @@
         <v>46</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>111</v>
+        <v>71</v>
       </c>
       <c r="G43" s="1" t="s">
         <v>46</v>
@@ -3253,12 +3258,12 @@
         <v>24</v>
       </c>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C44" s="3" t="s">
         <v>137</v>
@@ -3266,19 +3271,31 @@
       <c r="D44" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="E44" s="1"/>
-      <c r="G44" s="1"/>
+      <c r="E44" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="G44" s="1" t="s">
+        <v>46</v>
+      </c>
       <c r="I44" s="1"/>
       <c r="K44" s="1"/>
       <c r="M44" s="1"/>
-      <c r="N44" s="1"/>
-    </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N44" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O44" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C45" s="3" t="s">
         <v>139</v>
@@ -3286,51 +3303,51 @@
       <c r="D45" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="E45" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F45" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="G45" s="1" t="s">
-        <v>23</v>
-      </c>
+      <c r="E45" s="1"/>
+      <c r="G45" s="1"/>
       <c r="I45" s="1"/>
       <c r="K45" s="1"/>
       <c r="M45" s="1"/>
-      <c r="N45" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="O45" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N45" s="1"/>
+    </row>
+    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C46" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="D46" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="D46" s="4" t="s">
+      <c r="E46" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F46" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="E46" s="1"/>
-      <c r="G46" s="1"/>
+      <c r="G46" s="1" t="s">
+        <v>23</v>
+      </c>
       <c r="I46" s="1"/>
       <c r="K46" s="1"/>
       <c r="M46" s="1"/>
-      <c r="N46" s="1"/>
-    </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N46" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O46" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C47" s="3" t="s">
         <v>144</v>
@@ -3338,26 +3355,19 @@
       <c r="D47" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="E47" s="1" t="s">
-        <v>23</v>
-      </c>
+      <c r="E47" s="1"/>
       <c r="G47" s="1"/>
       <c r="I47" s="1"/>
       <c r="K47" s="1"/>
       <c r="M47" s="1"/>
-      <c r="N47" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="O47" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N47" s="1"/>
+    </row>
+    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C48" s="3" t="s">
         <v>146</v>
@@ -3365,19 +3375,26 @@
       <c r="D48" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="E48" s="1"/>
+      <c r="E48" s="1" t="s">
+        <v>23</v>
+      </c>
       <c r="G48" s="1"/>
       <c r="I48" s="1"/>
       <c r="K48" s="1"/>
       <c r="M48" s="1"/>
-      <c r="N48" s="1"/>
+      <c r="N48" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O48" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C49" s="3" t="s">
         <v>148</v>
@@ -3392,12 +3409,12 @@
       <c r="M49" s="1"/>
       <c r="N49" s="1"/>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C50" s="3" t="s">
         <v>150</v>
@@ -3405,31 +3422,19 @@
       <c r="D50" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="E50" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="F50" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="G50" s="1" t="s">
-        <v>27</v>
-      </c>
+      <c r="E50" s="1"/>
+      <c r="G50" s="1"/>
       <c r="I50" s="1"/>
       <c r="K50" s="1"/>
       <c r="M50" s="1"/>
-      <c r="N50" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="O50" s="1" t="s">
-        <v>24</v>
-      </c>
+      <c r="N50" s="1"/>
     </row>
     <row r="51" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C51" s="3" t="s">
         <v>152</v>
@@ -3438,13 +3443,13 @@
         <v>153</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="G51" s="1" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="I51" s="1"/>
       <c r="K51" s="1"/>
@@ -3461,7 +3466,7 @@
         <v>15</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C52" s="3" t="s">
         <v>154</v>
@@ -3470,13 +3475,13 @@
         <v>155</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>156</v>
+        <v>53</v>
       </c>
       <c r="G52" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I52" s="1"/>
       <c r="K52" s="1"/>
@@ -3493,22 +3498,22 @@
         <v>15</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C53" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="D53" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="D53" s="4" t="s">
+      <c r="E53" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F53" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="E53" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="F53" s="1" t="s">
-        <v>55</v>
-      </c>
       <c r="G53" s="1" t="s">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="I53" s="1"/>
       <c r="K53" s="1"/>
@@ -3521,26 +3526,26 @@
       </c>
     </row>
     <row r="54" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A54" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B54" s="6" t="s">
+      <c r="A54" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="C54" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="C54" s="6" t="s">
+      <c r="D54" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="D54" s="7" t="s">
-        <v>161</v>
-      </c>
       <c r="E54" s="1" t="s">
-        <v>122</v>
+        <v>46</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>162</v>
+        <v>56</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>122</v>
+        <v>46</v>
       </c>
       <c r="I54" s="1"/>
       <c r="K54" s="1"/>
@@ -3553,22 +3558,27 @@
       </c>
     </row>
     <row r="55" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A55" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B55" s="6" t="s">
-        <v>159</v>
-      </c>
-      <c r="C55" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="D55" s="7" t="s">
-        <v>164</v>
+      <c r="A55" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="C55" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>162</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="G55" s="1"/>
+        <v>46</v>
+      </c>
+      <c r="F55" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="G55" s="1" t="s">
+        <v>46</v>
+      </c>
       <c r="I55" s="1"/>
       <c r="K55" s="1"/>
       <c r="M55" s="1"/>
@@ -3579,32 +3589,44 @@
         <v>24</v>
       </c>
     </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A56" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B56" s="6" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="C56" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="D56" s="7" t="s">
         <v>165</v>
       </c>
-      <c r="D56" s="7" t="s">
+      <c r="E56" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="F56" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="E56" s="1"/>
-      <c r="G56" s="1"/>
+      <c r="G56" s="1" t="s">
+        <v>124</v>
+      </c>
       <c r="I56" s="1"/>
       <c r="K56" s="1"/>
       <c r="M56" s="1"/>
-      <c r="N56" s="1"/>
+      <c r="N56" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O56" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="57" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A57" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="C57" s="6" t="s">
         <v>167</v>
@@ -3613,7 +3635,7 @@
         <v>168</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="G57" s="1"/>
       <c r="I57" s="1"/>
@@ -3631,7 +3653,7 @@
         <v>15</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="C58" s="6" t="s">
         <v>169</v>
@@ -3651,7 +3673,7 @@
         <v>15</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="C59" s="6" t="s">
         <v>171</v>
@@ -3660,7 +3682,7 @@
         <v>172</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="G59" s="1"/>
       <c r="I59" s="1"/>
@@ -3673,12 +3695,12 @@
         <v>24</v>
       </c>
     </row>
-    <row r="60" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A60" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B60" s="6" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="C60" s="6" t="s">
         <v>173</v>
@@ -3686,31 +3708,19 @@
       <c r="D60" s="7" t="s">
         <v>174</v>
       </c>
-      <c r="E60" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="F60" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="G60" s="1" t="s">
-        <v>27</v>
-      </c>
+      <c r="E60" s="1"/>
+      <c r="G60" s="1"/>
       <c r="I60" s="1"/>
       <c r="K60" s="1"/>
       <c r="M60" s="1"/>
-      <c r="N60" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="O60" s="1" t="s">
-        <v>24</v>
-      </c>
+      <c r="N60" s="1"/>
     </row>
     <row r="61" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A61" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B61" s="6" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="C61" s="6" t="s">
         <v>175</v>
@@ -3719,7 +3729,7 @@
         <v>176</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>27</v>
+        <v>124</v>
       </c>
       <c r="G61" s="1"/>
       <c r="I61" s="1"/>
@@ -3732,12 +3742,12 @@
         <v>24</v>
       </c>
     </row>
-    <row r="62" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A62" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B62" s="6" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="C62" s="6" t="s">
         <v>177</v>
@@ -3745,19 +3755,31 @@
       <c r="D62" s="7" t="s">
         <v>178</v>
       </c>
-      <c r="E62" s="1"/>
-      <c r="G62" s="1"/>
+      <c r="E62" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F62" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G62" s="1" t="s">
+        <v>27</v>
+      </c>
       <c r="I62" s="1"/>
       <c r="K62" s="1"/>
       <c r="M62" s="1"/>
-      <c r="N62" s="1"/>
+      <c r="N62" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O62" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="63" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A63" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="C63" s="6" t="s">
         <v>179</v>
@@ -3784,7 +3806,7 @@
         <v>15</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="C64" s="6" t="s">
         <v>181</v>
@@ -3804,7 +3826,7 @@
         <v>15</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="C65" s="6" t="s">
         <v>183</v>
@@ -3826,12 +3848,12 @@
         <v>24</v>
       </c>
     </row>
-    <row r="66" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A66" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="C66" s="6" t="s">
         <v>185</v>
@@ -3839,40 +3861,28 @@
       <c r="D66" s="7" t="s">
         <v>186</v>
       </c>
-      <c r="E66" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="F66" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="G66" s="1" t="s">
-        <v>46</v>
-      </c>
+      <c r="E66" s="1"/>
+      <c r="G66" s="1"/>
       <c r="I66" s="1"/>
       <c r="K66" s="1"/>
       <c r="M66" s="1"/>
-      <c r="N66" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="O66" s="1" t="s">
-        <v>24</v>
-      </c>
+      <c r="N66" s="1"/>
     </row>
     <row r="67" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A67" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="C67" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="D67" s="7" t="s">
         <v>188</v>
       </c>
-      <c r="D67" s="7" t="s">
-        <v>189</v>
-      </c>
       <c r="E67" s="1" t="s">
-        <v>46</v>
+        <v>27</v>
       </c>
       <c r="G67" s="1"/>
       <c r="I67" s="1"/>
@@ -3885,32 +3895,44 @@
         <v>24</v>
       </c>
     </row>
-    <row r="68" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A68" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="C68" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="D68" s="7" t="s">
         <v>190</v>
       </c>
-      <c r="D68" s="7" t="s">
+      <c r="E68" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F68" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="E68" s="1"/>
-      <c r="G68" s="1"/>
+      <c r="G68" s="1" t="s">
+        <v>46</v>
+      </c>
       <c r="I68" s="1"/>
       <c r="K68" s="1"/>
       <c r="M68" s="1"/>
-      <c r="N68" s="1"/>
+      <c r="N68" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O68" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="69" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A69" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="C69" s="6" t="s">
         <v>192</v>
@@ -3937,7 +3959,7 @@
         <v>15</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="C70" s="6" t="s">
         <v>194</v>
@@ -3957,7 +3979,7 @@
         <v>15</v>
       </c>
       <c r="B71" s="6" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="C71" s="6" t="s">
         <v>196</v>
@@ -3979,12 +4001,12 @@
         <v>24</v>
       </c>
     </row>
-    <row r="72" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A72" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="C72" s="6" t="s">
         <v>198</v>
@@ -3992,47 +4014,30 @@
       <c r="D72" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="E72" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F72" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="G72" s="1" t="s">
-        <v>46</v>
-      </c>
+      <c r="E72" s="1"/>
+      <c r="G72" s="1"/>
       <c r="I72" s="1"/>
       <c r="K72" s="1"/>
       <c r="M72" s="1"/>
-      <c r="N72" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="O72" s="1" t="s">
-        <v>24</v>
-      </c>
+      <c r="N72" s="1"/>
     </row>
     <row r="73" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A73" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B73" s="6" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="C73" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="D73" s="7" t="s">
         <v>201</v>
       </c>
-      <c r="D73" s="7" t="s">
-        <v>202</v>
-      </c>
       <c r="E73" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F73" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="G73" s="1" t="s">
-        <v>21</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="G73" s="1"/>
       <c r="I73" s="1"/>
       <c r="K73" s="1"/>
       <c r="M73" s="1"/>
@@ -4048,53 +4053,101 @@
         <v>15</v>
       </c>
       <c r="B74" s="6" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="C74" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="D74" s="7" t="s">
         <v>203</v>
       </c>
-      <c r="D74" s="7" t="s">
+      <c r="E74" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F74" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="E74" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="F74" s="1" t="s">
-        <v>123</v>
-      </c>
       <c r="G74" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="H74" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="I74" s="1" t="s">
-        <v>122</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="I74" s="1"/>
       <c r="K74" s="1"/>
       <c r="M74" s="1"/>
       <c r="N74" s="1" t="s">
-        <v>124</v>
+        <v>24</v>
       </c>
       <c r="O74" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="75" spans="5:14" x14ac:dyDescent="0.25">
-      <c r="E75" s="1"/>
-      <c r="G75" s="1"/>
+    <row r="75" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A75" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B75" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="C75" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="D75" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="E75" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F75" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="G75" s="1" t="s">
+        <v>21</v>
+      </c>
       <c r="I75" s="1"/>
       <c r="K75" s="1"/>
       <c r="M75" s="1"/>
-      <c r="N75" s="1"/>
-    </row>
-    <row r="76" spans="5:14" x14ac:dyDescent="0.25">
-      <c r="E76" s="1"/>
-      <c r="G76" s="1"/>
-      <c r="I76" s="1"/>
+      <c r="N75" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O75" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="76" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A76" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B76" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="C76" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="D76" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="E76" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="F76" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="G76" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="H76" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="I76" s="1" t="s">
+        <v>124</v>
+      </c>
       <c r="K76" s="1"/>
       <c r="M76" s="1"/>
-      <c r="N76" s="1"/>
+      <c r="N76" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="O76" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="77" spans="5:14" x14ac:dyDescent="0.25">
       <c r="E77" s="1"/>
@@ -6480,17 +6533,33 @@
       <c r="M374" s="1"/>
       <c r="N374" s="1"/>
     </row>
+    <row r="375" spans="5:14" x14ac:dyDescent="0.25">
+      <c r="E375" s="1"/>
+      <c r="G375" s="1"/>
+      <c r="I375" s="1"/>
+      <c r="K375" s="1"/>
+      <c r="M375" s="1"/>
+      <c r="N375" s="1"/>
+    </row>
+    <row r="376" spans="5:14" x14ac:dyDescent="0.25">
+      <c r="E376" s="1"/>
+      <c r="G376" s="1"/>
+      <c r="I376" s="1"/>
+      <c r="K376" s="1"/>
+      <c r="M376" s="1"/>
+      <c r="N376" s="1"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O1"/>
-  <conditionalFormatting sqref="E2:E374">
+  <conditionalFormatting sqref="E2:E376">
     <cfRule type="containsText" dxfId="0" priority="1">
       <formula>NOT(ISERROR(SEARCH("BOT",E2)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="1" priority="2">
-      <formula>NOT(ISERROR(SEARCH("QDB",E2)))</formula>
+      <formula>NOT(ISERROR(SEARCH("EUD",E2)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="2" priority="3">
-      <formula>NOT(ISERROR(SEARCH("EUD",E2)))</formula>
+      <formula>NOT(ISERROR(SEARCH("QDB",E2)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="3" priority="4">
       <formula>NOT(ISERROR(SEARCH("OUI",E2)))</formula>
@@ -6502,15 +6571,15 @@
       <formula>NOT(ISERROR(SEARCH("NEUTRO",E2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G374">
+  <conditionalFormatting sqref="G2:G376">
     <cfRule type="containsText" dxfId="6" priority="1">
       <formula>NOT(ISERROR(SEARCH("BOT",G2)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="7" priority="2">
-      <formula>NOT(ISERROR(SEARCH("QDB",G2)))</formula>
+      <formula>NOT(ISERROR(SEARCH("EUD",G2)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="8" priority="3">
-      <formula>NOT(ISERROR(SEARCH("EUD",G2)))</formula>
+      <formula>NOT(ISERROR(SEARCH("QDB",G2)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="9" priority="4">
       <formula>NOT(ISERROR(SEARCH("OUI",G2)))</formula>
@@ -6522,15 +6591,15 @@
       <formula>NOT(ISERROR(SEARCH("NEUTRO",G2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I374">
+  <conditionalFormatting sqref="I2:I376">
     <cfRule type="containsText" dxfId="12" priority="1">
       <formula>NOT(ISERROR(SEARCH("BOT",I2)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="13" priority="2">
-      <formula>NOT(ISERROR(SEARCH("QDB",I2)))</formula>
+      <formula>NOT(ISERROR(SEARCH("EUD",I2)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="14" priority="3">
-      <formula>NOT(ISERROR(SEARCH("EUD",I2)))</formula>
+      <formula>NOT(ISERROR(SEARCH("QDB",I2)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="15" priority="4">
       <formula>NOT(ISERROR(SEARCH("OUI",I2)))</formula>
@@ -6542,15 +6611,15 @@
       <formula>NOT(ISERROR(SEARCH("NEUTRO",I2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K2:K374">
+  <conditionalFormatting sqref="K2:K376">
     <cfRule type="containsText" dxfId="18" priority="1">
       <formula>NOT(ISERROR(SEARCH("BOT",K2)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="19" priority="2">
-      <formula>NOT(ISERROR(SEARCH("QDB",K2)))</formula>
+      <formula>NOT(ISERROR(SEARCH("EUD",K2)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="20" priority="3">
-      <formula>NOT(ISERROR(SEARCH("EUD",K2)))</formula>
+      <formula>NOT(ISERROR(SEARCH("QDB",K2)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="21" priority="4">
       <formula>NOT(ISERROR(SEARCH("OUI",K2)))</formula>
@@ -6562,15 +6631,15 @@
       <formula>NOT(ISERROR(SEARCH("NEUTRO",K2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M2:M374">
+  <conditionalFormatting sqref="M2:M376">
     <cfRule type="containsText" dxfId="24" priority="1">
       <formula>NOT(ISERROR(SEARCH("BOT",M2)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="25" priority="2">
-      <formula>NOT(ISERROR(SEARCH("QDB",M2)))</formula>
+      <formula>NOT(ISERROR(SEARCH("EUD",M2)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="26" priority="3">
-      <formula>NOT(ISERROR(SEARCH("EUD",M2)))</formula>
+      <formula>NOT(ISERROR(SEARCH("QDB",M2)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="27" priority="4">
       <formula>NOT(ISERROR(SEARCH("OUI",M2)))</formula>
@@ -6583,40 +6652,40 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="12">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca do Móvel" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca do Móvel" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="E10:E374">
-      <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca do Móvel" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca do Móvel" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="E10:E376">
+      <formula1>"BOT,EUD,QDB,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca do Móvel" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca do Móvel" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="E2:E374">
-      <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca do Móvel" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca do Móvel" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="E2:E376">
+      <formula1>"BOT,EUD,QDB,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 1" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 1" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="G10:G374">
-      <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 1" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 1" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="G10:G376">
+      <formula1>"BOT,EUD,QDB,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 1" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 1" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="G2:G374">
-      <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 1" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 1" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="G2:G376">
+      <formula1>"BOT,EUD,QDB,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 2" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 2" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="I10:I374">
-      <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 2" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 2" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="I10:I376">
+      <formula1>"BOT,EUD,QDB,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 2" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 2" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="I2:I374">
-      <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 2" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 2" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="I2:I376">
+      <formula1>"BOT,EUD,QDB,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 3" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 3" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="K10:K374">
-      <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 3" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 3" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="K10:K376">
+      <formula1>"BOT,EUD,QDB,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 3" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 3" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="K2:K374">
-      <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 3" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 3" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="K2:K376">
+      <formula1>"BOT,EUD,QDB,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 4" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 4" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="M10:M374">
-      <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 4" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 4" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="M10:M376">
+      <formula1>"BOT,EUD,QDB,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 4" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 4" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="M2:M374">
-      <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 4" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 4" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="M2:M376">
+      <formula1>"BOT,EUD,QDB,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" sqref="N10:N374">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" sqref="N10:N376">
       <formula1>"FIXO,EXPOSICAO,NOVO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" sqref="N2:N374">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" sqref="N2:N376">
       <formula1>"FIXO,EXPOSICAO,NOVO"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6644,16 +6713,16 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -6661,13 +6730,13 @@
         <v>15</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>23</v>
@@ -6681,13 +6750,13 @@
         <v>15</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>21</v>
@@ -6701,13 +6770,13 @@
         <v>15</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>46</v>
@@ -6721,13 +6790,13 @@
         <v>15</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>71</v>
+        <v>59</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>21</v>
@@ -6741,13 +6810,13 @@
         <v>15</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>21</v>
@@ -6761,13 +6830,13 @@
         <v>15</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>46</v>
@@ -6781,16 +6850,16 @@
         <v>15</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>24</v>
@@ -6801,13 +6870,13 @@
         <v>15</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>23</v>
@@ -6821,19 +6890,19 @@
         <v>15</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>23</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -6841,19 +6910,19 @@
         <v>15</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>21</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -6861,19 +6930,19 @@
         <v>15</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>46</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -6884,10 +6953,10 @@
         <v>16</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>24</v>
@@ -6904,10 +6973,10 @@
         <v>16</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>24</v>
@@ -6921,13 +6990,13 @@
         <v>15</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>24</v>
@@ -6941,13 +7010,13 @@
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>24</v>
@@ -6961,13 +7030,13 @@
         <v>15</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>24</v>
@@ -6981,13 +7050,13 @@
         <v>15</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>24</v>
@@ -7001,13 +7070,13 @@
         <v>15</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>24</v>
@@ -7021,13 +7090,13 @@
         <v>15</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>24</v>
@@ -7041,13 +7110,13 @@
         <v>15</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>24</v>
@@ -8263,10 +8332,10 @@
       <formula>NOT(ISERROR(SEARCH("BOT",E2)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="31" priority="2">
-      <formula>NOT(ISERROR(SEARCH("QDB",E2)))</formula>
+      <formula>NOT(ISERROR(SEARCH("EUD",E2)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="32" priority="3">
-      <formula>NOT(ISERROR(SEARCH("EUD",E2)))</formula>
+      <formula>NOT(ISERROR(SEARCH("QDB",E2)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="33" priority="4">
       <formula>NOT(ISERROR(SEARCH("OUI",E2)))</formula>
@@ -8285,11 +8354,11 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Seção" prompt="TV = Lista ao lado dos ícones de TV / rádio; A = Lista ao lado do ícone (A); C = Lista ao lado do ícone (C); CALLOUT = Caixa de destaque sobre a planta (pode apontar para um móvel); NOTA = Nota no canto inferior esquerdo (texto antes de &quot;:&quot; fica em n" showErrorMessage="1" errorStyle="warning" errorTitle="Seção" error="TV = Lista ao lado dos ícones de TV / rádio; A = Lista ao lado do ícone (A); C = Lista ao lado do ícone (C); CALLOUT = Caixa de destaque sobre a planta (pode apontar para um móvel); NOTA = Nota no canto inferior esquerdo (texto antes de &quot;:&quot; fica em negrito)" sqref="C2:C321">
       <formula1>"TV,A,C,CALLOUT,NOTA"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="E10:E321">
-      <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="E10:E321">
+      <formula1>"BOT,EUD,QDB,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca" prompt="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca" error="Use BOT, QDB, EUD, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="E2:E321">
-      <formula1>"BOT,QDB,EUD,OUI,MULTI,NEUTRO"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="E2:E321">
+      <formula1>"BOT,EUD,QDB,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8313,13 +8382,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>14</v>
@@ -8330,10 +8399,10 @@
         <v>15</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="D2" s="9">
         <v>150000</v>
@@ -8350,7 +8419,7 @@
         <v>43</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="D3" s="9">
         <v>1200000</v>
@@ -8367,7 +8436,7 @@
         <v>32</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="D4" s="9">
         <v>650000</v>
@@ -8381,10 +8450,10 @@
         <v>15</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="D5" s="9">
         <v>2400000</v>
@@ -8398,10 +8467,10 @@
         <v>15</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="D6" s="9">
         <v>430000</v>
@@ -8415,10 +8484,10 @@
         <v>15</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="D7" s="9">
         <v>610000</v>
@@ -8432,7 +8501,7 @@
         <v>15</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>24</v>
@@ -8447,7 +8516,7 @@
         <v>15</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>24</v>
@@ -8462,7 +8531,7 @@
         <v>15</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>24</v>
@@ -8477,7 +8546,7 @@
         <v>15</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>24</v>
@@ -8492,10 +8561,10 @@
         <v>15</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="D12" s="9">
         <v>380000</v>
@@ -8512,7 +8581,7 @@
         <v>29</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="D13" s="9">
         <v>620000</v>
@@ -8526,10 +8595,10 @@
         <v>15</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="D14" s="9">
         <v>1800000</v>
@@ -8543,10 +8612,10 @@
         <v>15</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>71</v>
+        <v>59</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="D15" s="9">
         <v>950000</v>
@@ -8560,10 +8629,10 @@
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="D16" s="9">
         <v>210000</v>
@@ -8580,7 +8649,7 @@
         <v>28</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="D17" s="9">
         <v>900000</v>
@@ -8594,10 +8663,10 @@
         <v>15</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="D18" s="9">
         <v>260000</v>
@@ -8614,7 +8683,7 @@
         <v>22</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="D19" s="9">
         <v>1500000</v>
@@ -8628,10 +8697,10 @@
         <v>15</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="D20" s="9">
         <v>1100000</v>
@@ -8660,7 +8729,7 @@
         <v>15</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>24</v>
@@ -8675,10 +8744,10 @@
         <v>15</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="D23" s="9">
         <v>870000</v>
@@ -8695,7 +8764,7 @@
         <v>49</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="D24" s="9">
         <v>700000</v>
@@ -8709,10 +8778,10 @@
         <v>15</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="D25" s="9">
         <v>480000</v>
@@ -8726,10 +8795,10 @@
         <v>15</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="D26" s="9">
         <v>780000</v>
@@ -8743,10 +8812,10 @@
         <v>15</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="D27" s="9">
         <v>540000</v>
@@ -8763,7 +8832,7 @@
         <v>38</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="D28" s="9">
         <v>520000</v>
@@ -8777,7 +8846,7 @@
         <v>15</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>24</v>
@@ -10032,122 +10101,122 @@
   <sheetData>
     <row r="1" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B1" s="11" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B2" s="12" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12"/>
     </row>
     <row r="4" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B4" s="13" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B5" s="12" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="C5" s="12"/>
       <c r="D5" s="12"/>
     </row>
     <row r="6" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B6" s="12" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="C6" s="12"/>
       <c r="D6" s="12"/>
     </row>
     <row r="7" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B7" s="12" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="12"/>
     </row>
     <row r="8" ht="45" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B8" s="12" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="C8" s="12"/>
       <c r="D8" s="12"/>
     </row>
     <row r="9" ht="16" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B9" s="12" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="C9" s="12"/>
       <c r="D9" s="12"/>
     </row>
     <row r="10" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B10" s="12" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="C10" s="12"/>
       <c r="D10" s="12"/>
     </row>
     <row r="11" ht="60" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B11" s="12" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="C11" s="12"/>
       <c r="D11" s="12"/>
     </row>
     <row r="12" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B12" s="12" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="C12" s="12"/>
       <c r="D12" s="12"/>
     </row>
     <row r="13" ht="60" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B13" s="12" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="C13" s="12"/>
       <c r="D13" s="12"/>
     </row>
     <row r="14" ht="60" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B14" s="12" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="C14" s="12"/>
       <c r="D14" s="12"/>
     </row>
     <row r="15" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B15" s="12" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="C15" s="12"/>
       <c r="D15" s="12"/>
     </row>
     <row r="16" ht="60" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B16" s="12" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="C16" s="12"/>
       <c r="D16" s="12"/>
     </row>
     <row r="17" ht="45" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B17" s="12" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="C17" s="12"/>
       <c r="D17" s="12"/>
     </row>
     <row r="18" ht="45" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B18" s="12" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="C18" s="12"/>
       <c r="D18" s="12"/>
     </row>
     <row r="20" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B20" s="13" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.25">
@@ -10155,40 +10224,40 @@
         <v>21</v>
       </c>
       <c r="C21" t="s">
-        <v>255</v>
+        <v>21</v>
       </c>
       <c r="D21" s="15" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
     </row>
     <row r="22" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B22" s="14" t="s">
-        <v>27</v>
+        <v>46</v>
       </c>
       <c r="C22" t="s">
-        <v>257</v>
+        <v>46</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
     </row>
     <row r="23" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B23" s="14" t="s">
-        <v>46</v>
+        <v>27</v>
       </c>
       <c r="C23" t="s">
-        <v>259</v>
+        <v>27</v>
       </c>
       <c r="D23" s="17" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="24" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B24" s="14" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C24" t="s">
-        <v>261</v>
+        <v>124</v>
       </c>
       <c r="D24" s="18" t="s">
         <v>262</v>
@@ -10234,7 +10303,7 @@
     </row>
     <row r="30" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B30" s="14" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C30" t="s">
         <v>270</v>
@@ -10261,27 +10330,27 @@
     </row>
     <row r="34" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B34" s="21" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
     </row>
     <row r="35" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B35" s="22" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
     </row>
     <row r="36" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B36" s="23" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
     </row>
     <row r="37" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B37" s="24" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
     </row>
     <row r="38" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B38" s="25" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
     </row>
     <row r="40" spans="2:2" x14ac:dyDescent="0.25">
@@ -10291,7 +10360,7 @@
     </row>
     <row r="41" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B41" s="14" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="C41" t="s">
         <v>277</v>
@@ -10300,7 +10369,7 @@
     </row>
     <row r="42" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B42" s="14" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="C42" t="s">
         <v>278</v>
@@ -10309,7 +10378,7 @@
     </row>
     <row r="43" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B43" s="14" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="C43" t="s">
         <v>279</v>
@@ -10318,7 +10387,7 @@
     </row>
     <row r="44" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B44" s="14" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="C44" t="s">
         <v>280</v>
@@ -10327,7 +10396,7 @@
     </row>
     <row r="45" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B45" s="14" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="C45" t="s">
         <v>281</v>

</xml_diff>

<commit_message>
Classificação "Institucional / portfólio" passa a se chamar Baseline
O código interno continua INSTITUCIONAL e o nome antigo segue aceito na planilha
(aparece como Baseline). Planilha base do visualizador gerada de novo.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MHQRMyvP3NMZPhZq474WCH
</commit_message>
<xml_diff>
--- a/visualizador/Planilha base - Visualizador.xlsx
+++ b/visualizador/Planilha base - Visualizador.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="935" uniqueCount="290">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="988" uniqueCount="297">
   <si>
     <t>Ciclo</t>
   </si>
@@ -166,192 +166,201 @@
     <t>GONDOLA 1/PONTA-B</t>
   </si>
   <si>
-    <t>Gôndola 1 – Ponta B</t>
+    <t>Gôndola 1 – Ponta B · Fixo O.U.i (só ER P)</t>
+  </si>
+  <si>
+    <t>OUI</t>
+  </si>
+  <si>
+    <t>MON AMIE + LOÇÃO</t>
+  </si>
+  <si>
+    <t>PIRAMIDE 1</t>
+  </si>
+  <si>
+    <t>Pirâmide 1 · vale para ER P, ER M, ER G, ER GG</t>
+  </si>
+  <si>
+    <t>EUD</t>
+  </si>
+  <si>
+    <t>PIRAMIDE 2</t>
+  </si>
+  <si>
+    <t>Pirâmide 2 · vale para ER P, ER M, ER G, ER GG</t>
+  </si>
+  <si>
+    <t>PRINCIPAIS OPORTUNIDADES</t>
+  </si>
+  <si>
+    <t>BOTIPROMO</t>
+  </si>
+  <si>
+    <t>MESA DESTAQUE 1/FRENTE-1</t>
+  </si>
+  <si>
+    <t>Mesa destaque 1 – Frente 1 · vale para ER P, ER M</t>
+  </si>
+  <si>
+    <t>UOMINI GLORIFICADO</t>
+  </si>
+  <si>
+    <t>MESA DESTAQUE 1/FRENTE-2</t>
+  </si>
+  <si>
+    <t>Mesa destaque 1 – Frente 2</t>
+  </si>
+  <si>
+    <t>SIÀGE GLORIFICADO</t>
+  </si>
+  <si>
+    <t>MESA DESTAQUE 1/VERSO</t>
+  </si>
+  <si>
+    <t>Mesa destaque 1 – Verso</t>
+  </si>
+  <si>
+    <t>LÇTO UOMINI</t>
+  </si>
+  <si>
+    <t>PDV MOVEL 1</t>
+  </si>
+  <si>
+    <t>PDV móvel 1 · vale para ER P, ER M, ER G, ER GG</t>
+  </si>
+  <si>
+    <t>SIÀGE ULTIMATE</t>
+  </si>
+  <si>
+    <t>BALCAO RECEPCAO 1</t>
+  </si>
+  <si>
+    <t>Balcão recepção 1 · vale para ER P, ER M, ER G, ER GG</t>
+  </si>
+  <si>
+    <t>LÇTO EGEO</t>
+  </si>
+  <si>
+    <t>BOT+QDB</t>
+  </si>
+  <si>
+    <t>MOVEL DE FILA 2</t>
+  </si>
+  <si>
+    <t>Móvel de fila 2 · vale para ER P, ER M, ER G, ER GG</t>
+  </si>
+  <si>
+    <t>MOVEL DE FILA 1</t>
+  </si>
+  <si>
+    <t>Móvel de fila 1 · vale para ER P, ER M, ER G, ER GG</t>
+  </si>
+  <si>
+    <t>OUTLET EUD</t>
+  </si>
+  <si>
+    <t>TOTEM 1/PAINEL-1</t>
+  </si>
+  <si>
+    <t>Totem 1 – Painel 1 · vale para ER P, ER M, ER G, ER GG</t>
+  </si>
+  <si>
+    <t>TOTEM 1/PAINEL-2</t>
+  </si>
+  <si>
+    <t>Totem 1 – Painel 2</t>
+  </si>
+  <si>
+    <t>TOTEM 1/PAINEL-3</t>
+  </si>
+  <si>
+    <t>Totem 1 – Painel 3</t>
+  </si>
+  <si>
+    <t>EXTRA-CESTINHAS</t>
+  </si>
+  <si>
+    <t>Cestinhas · vale para ER P, ER M, ER G, ER GG</t>
+  </si>
+  <si>
+    <t>EXTRA-BELEZA</t>
+  </si>
+  <si>
+    <t>Espaço da Beleza · vale para ER P, ER M, ER G, ER GG</t>
+  </si>
+  <si>
+    <t>BOTIPROMO MAKE B.</t>
+  </si>
+  <si>
+    <t>LIQUIDA MAKE</t>
+  </si>
+  <si>
+    <t>EXTRA-CAVALETE</t>
+  </si>
+  <si>
+    <t>Cavalete · vale para ER P, ER M, ER G, ER GG</t>
+  </si>
+  <si>
+    <t>MOVEL MAKE 1/TESTEIRA-1</t>
+  </si>
+  <si>
+    <t>Móvel make 1 – Testeira 1 · vale para ER P, ER M, ER G, ER GG</t>
+  </si>
+  <si>
+    <t>#1F1F1F</t>
+  </si>
+  <si>
+    <t>MOVEL MAKE 1/TESTEIRA-2</t>
+  </si>
+  <si>
+    <t>Móvel make 1 – Testeira 2</t>
+  </si>
+  <si>
+    <t>MOVEL MAKE 1/TESTEIRA-3</t>
+  </si>
+  <si>
+    <t>Móvel make 1 – Testeira 3</t>
+  </si>
+  <si>
+    <t>MOVEL MAKE 1/TESTEIRA-4</t>
+  </si>
+  <si>
+    <t>Móvel make 1 – Testeira 4</t>
+  </si>
+  <si>
+    <t>MOVEL DE PAREDE 2</t>
+  </si>
+  <si>
+    <t>Perf. Masc. BOT · vale para ER P, ER M, ER G, ER GG</t>
+  </si>
+  <si>
+    <t>PERF MASC</t>
+  </si>
+  <si>
+    <t>MOVEL DE PAREDE 3</t>
+  </si>
+  <si>
+    <t>Perf. Fem. EUD · vale para ER P, ER M, ER G, ER GG</t>
+  </si>
+  <si>
+    <t>MOVEL DE PAREDE 4</t>
+  </si>
+  <si>
+    <t>CBEM/NSPA · vale para ER P, ER M, ER G, ER GG</t>
+  </si>
+  <si>
+    <t>CUIDADOS (CBEM/NSPA)</t>
+  </si>
+  <si>
+    <t>ER M</t>
+  </si>
+  <si>
+    <t>Gôndola 1 – Ponta B · Livre (vale para ER M, ER G, ER GG)</t>
   </si>
   <si>
     <t>BOTI PROMO</t>
   </si>
   <si>
-    <t>PIRAMIDE 1</t>
-  </si>
-  <si>
-    <t>Pirâmide 1 · vale para ER P, ER M, ER G, ER GG</t>
-  </si>
-  <si>
-    <t>EUD</t>
-  </si>
-  <si>
-    <t>PIRAMIDE 2</t>
-  </si>
-  <si>
-    <t>Pirâmide 2 · vale para ER P, ER M, ER G, ER GG</t>
-  </si>
-  <si>
-    <t>PRINCIPAIS OPORTUNIDADES</t>
-  </si>
-  <si>
-    <t>BOTIPROMO</t>
-  </si>
-  <si>
-    <t>MESA DESTAQUE 1/FRENTE-1</t>
-  </si>
-  <si>
-    <t>Mesa destaque 1 – Frente 1 · vale para ER P, ER M</t>
-  </si>
-  <si>
-    <t>UOMINI GLORIFICADO</t>
-  </si>
-  <si>
-    <t>MESA DESTAQUE 1/FRENTE-2</t>
-  </si>
-  <si>
-    <t>Mesa destaque 1 – Frente 2</t>
-  </si>
-  <si>
-    <t>SIÀGE GLORIFICADO</t>
-  </si>
-  <si>
-    <t>MESA DESTAQUE 1/VERSO</t>
-  </si>
-  <si>
-    <t>Mesa destaque 1 – Verso</t>
-  </si>
-  <si>
-    <t>LÇTO UOMINI</t>
-  </si>
-  <si>
-    <t>PDV MOVEL 1</t>
-  </si>
-  <si>
-    <t>PDV móvel 1 · vale para ER P, ER M, ER G, ER GG</t>
-  </si>
-  <si>
-    <t>SIÀGE ULTIMATE</t>
-  </si>
-  <si>
-    <t>BALCAO RECEPCAO 1</t>
-  </si>
-  <si>
-    <t>Balcão recepção 1 · vale para ER P, ER M, ER G, ER GG</t>
-  </si>
-  <si>
-    <t>LÇTO EGEO</t>
-  </si>
-  <si>
-    <t>BOT+QDB</t>
-  </si>
-  <si>
-    <t>MOVEL DE FILA 2</t>
-  </si>
-  <si>
-    <t>Móvel de fila 2 · vale para ER P, ER M, ER G, ER GG</t>
-  </si>
-  <si>
-    <t>MOVEL DE FILA 1</t>
-  </si>
-  <si>
-    <t>Móvel de fila 1 · vale para ER P, ER M, ER G, ER GG</t>
-  </si>
-  <si>
-    <t>OUTLET EUD</t>
-  </si>
-  <si>
-    <t>TOTEM 1/PAINEL-1</t>
-  </si>
-  <si>
-    <t>Totem 1 – Painel 1 · vale para ER P, ER M, ER G, ER GG</t>
-  </si>
-  <si>
-    <t>TOTEM 1/PAINEL-2</t>
-  </si>
-  <si>
-    <t>Totem 1 – Painel 2</t>
-  </si>
-  <si>
-    <t>TOTEM 1/PAINEL-3</t>
-  </si>
-  <si>
-    <t>Totem 1 – Painel 3</t>
-  </si>
-  <si>
-    <t>EXTRA-CESTINHAS</t>
-  </si>
-  <si>
-    <t>Cestinhas · vale para ER P, ER M, ER G, ER GG</t>
-  </si>
-  <si>
-    <t>EXTRA-BELEZA</t>
-  </si>
-  <si>
-    <t>Espaço da Beleza · vale para ER P, ER M, ER G, ER GG</t>
-  </si>
-  <si>
-    <t>BOTIPROMO MAKE B.</t>
-  </si>
-  <si>
-    <t>LIQUIDA MAKE</t>
-  </si>
-  <si>
-    <t>EXTRA-CAVALETE</t>
-  </si>
-  <si>
-    <t>Cavalete · vale para ER P, ER M, ER G, ER GG</t>
-  </si>
-  <si>
-    <t>MOVEL MAKE 1/TESTEIRA-1</t>
-  </si>
-  <si>
-    <t>Móvel make 1 – Testeira 1 · vale para ER P, ER M, ER G, ER GG</t>
-  </si>
-  <si>
-    <t>#1F1F1F</t>
-  </si>
-  <si>
-    <t>MOVEL MAKE 1/TESTEIRA-2</t>
-  </si>
-  <si>
-    <t>Móvel make 1 – Testeira 2</t>
-  </si>
-  <si>
-    <t>MOVEL MAKE 1/TESTEIRA-3</t>
-  </si>
-  <si>
-    <t>Móvel make 1 – Testeira 3</t>
-  </si>
-  <si>
-    <t>MOVEL MAKE 1/TESTEIRA-4</t>
-  </si>
-  <si>
-    <t>Móvel make 1 – Testeira 4</t>
-  </si>
-  <si>
-    <t>MOVEL DE PAREDE 2</t>
-  </si>
-  <si>
-    <t>Perf. Masc. BOT · vale para ER P, ER M, ER G, ER GG</t>
-  </si>
-  <si>
-    <t>PERF MASC</t>
-  </si>
-  <si>
-    <t>MOVEL DE PAREDE 3</t>
-  </si>
-  <si>
-    <t>Perf. Fem. EUD · vale para ER P, ER M, ER G, ER GG</t>
-  </si>
-  <si>
-    <t>MOVEL DE PAREDE 4</t>
-  </si>
-  <si>
-    <t>CBEM/NSPA · vale para ER P, ER M, ER G, ER GG</t>
-  </si>
-  <si>
-    <t>CUIDADOS (CBEM/NSPA)</t>
-  </si>
-  <si>
-    <t>ER M</t>
-  </si>
-  <si>
     <t>GONDOLA 2/PONTA-A</t>
   </si>
   <si>
@@ -412,12 +421,6 @@
     <t>Parede O.U.i 1 · vale para ER M, ER G</t>
   </si>
   <si>
-    <t>OUI</t>
-  </si>
-  <si>
-    <t>MON AMIE + LOÇÃO</t>
-  </si>
-  <si>
     <t>EXPOSICAO</t>
   </si>
   <si>
@@ -439,28 +442,46 @@
     <t>ER G</t>
   </si>
   <si>
+    <t>Gôndola 1 – Meio B (ou metade 1, se a metade 2 for preenchida) · defina de novo (não vem da ER M)</t>
+  </si>
+  <si>
+    <t>Gôndola 1 – Meio B – metade 2 (preencha só para dividir o meio em dois) · defina de novo (não vem da ER M)</t>
+  </si>
+  <si>
+    <t>Gôndola 1 – Ponta B · Livre (vale para ER M, ER G, ER GG) · defina de novo (não vem da ER M)</t>
+  </si>
+  <si>
     <t>MOVEL DE FILA 6</t>
   </si>
   <si>
     <t>Móvel de fila 6 · vale para ER G, ER GG</t>
   </si>
   <si>
+    <t>Gôndola 2 – Meio B (ou metade 1, se a metade 2 for preenchida) · defina de novo (não vem da ER M)</t>
+  </si>
+  <si>
+    <t>Gôndola 2 – Meio B – metade 2 (preencha só para dividir o meio em dois) · defina de novo (não vem da ER M)</t>
+  </si>
+  <si>
+    <t>Gôndola 2 – Ponta B · defina de novo (não vem da ER M)</t>
+  </si>
+  <si>
     <t>GONDOLA 3/PONTA-A</t>
   </si>
   <si>
-    <t>Gôndola 3 – Ponta A · vale para ER G, ER GG</t>
+    <t>Gôndola 3 – Ponta A · vale para ER G, ER GG · vem de GONDOLA 2/PONTA-B da ER M</t>
   </si>
   <si>
     <t>GONDOLA 3/MEIO-A</t>
   </si>
   <si>
-    <t>Gôndola 3 – Meio A (ou metade 1, se a metade 2 for preenchida)</t>
+    <t>Gôndola 3 – Meio A (ou metade 1, se a metade 2 for preenchida) · vem de GONDOLA 2/MEIO-B da ER M</t>
   </si>
   <si>
     <t>GONDOLA 3/MEIO-A-2</t>
   </si>
   <si>
-    <t>Gôndola 3 – Meio A – metade 2 (preencha só para dividir o meio em dois)</t>
+    <t>Gôndola 3 – Meio A – metade 2 (preencha só para dividir o meio em dois) · vem de GONDOLA 2/MEIO-B-2 da ER M</t>
   </si>
   <si>
     <t>GONDOLA 3/MEIO-B</t>
@@ -760,7 +781,7 @@
     <t>Promoção</t>
   </si>
   <si>
-    <t>Institucional / portfólio</t>
+    <t>Baseline</t>
   </si>
   <si>
     <t>Liquidação / outlet</t>
@@ -772,7 +793,7 @@
     <t>Planilha base — Plano de Varejo</t>
   </si>
   <si>
-    <t>Gerada em 20/10/2026, 22:56:30 a partir do ciclo "Ciclo exemplo".</t>
+    <t>Gerada em 23/10/2026, 14:32:12 a partir do ciclo "Ciclo exemplo".</t>
   </si>
   <si>
     <t>Como preencher</t>
@@ -796,7 +817,7 @@
     <t>6. Na aba "Painéis" ficam os textos fora dos móveis: listas TV / A / C, caixas de destaque (CALLOUT, que podem apontar para um ID Móvel) e notas (NOTA).</t>
   </si>
   <si>
-    <t>6.0 Na aba "Tipos de movimento" ficam os movimentos do ciclo: uma linha por movimento (o texto da etiqueta, igual ao da aba Movimentos), com a "Classificação" (Lançamento, Promoção, Liquidação / outlet, Institucional / portfólio, Outro ou outro texto) e o "GMV esperado (R$)". Elas aparecem no Analytics (movimentos, classificações e GMV esperado de cada ER). Maiúsculas e espaços a mais não importam.</t>
+    <t>6.0 Na aba "Tipos de movimento" ficam os movimentos do ciclo: uma linha por movimento (o texto da etiqueta, igual ao da aba Movimentos), com a "Classificação" (Lançamento, Promoção, Liquidação / outlet, Baseline, Outro ou outro texto) e o "GMV esperado (R$)". Elas aparecem no Analytics (movimentos, classificações e GMV esperado de cada ER). Maiúsculas e espaços a mais não importam.</t>
   </si>
   <si>
     <t>6.1 Gôndola, mesas, totem e móvel make são preenchidos espaço por espaço: não há linha do móvel inteiro (se houver, ela é ignorada). Espaço sem linha fica branco.</t>
@@ -811,7 +832,7 @@
     <t>6.4 Móveis de um espaço só (pirâmide, móvel de fila, móvel de parede, PDV, O.U.i…) têm uma linha. O balcão recepção também: um espaço só, com uma cor e até 3 etiquetas.</t>
   </si>
   <si>
-    <t>7. Na coluna "Planta" vale o nome (ex.: ER P) ou o número (01). Cascata: o que é definido numa planta vale também para as seguintes (ER P → ER M → ER G → ER GG), por isso cada móvel aparece uma vez só, na primeira planta que o tem ("vale para…" na coluna Móvel). Para mudar um móvel só a partir de uma planta, acrescente uma linha com o mesmo ID Móvel e essa planta. Planta = TODAS vale para todas.</t>
+    <t>7. Na coluna "Planta" vale o nome (ex.: ER P) ou o número (01). Cascata: o que é definido numa planta vale também para as seguintes (ER P → ER M → ER G → ER GG), por isso cada móvel aparece uma vez só, na primeira planta que o tem ("vale para…" na coluna Móvel). Para mudar um móvel só a partir de uma planta, acrescente uma linha com o mesmo ID Móvel e essa planta. Planta = TODAS vale para todas. Exceção: a ponta B da gôndola 1 é fixa de O.U.i na ER P e livre nas ERs maiores — a linha da ER P (Fixo O.U.i) não passa para elas; a da ER M (Livre) vale para a ER M. Da ER M para a ER G: a ponta B e o meio B da gôndola 2 da ER M viram a ponta A e o meio A da gôndola 3 da ER G; a ponta B e o meio B das gôndolas 1 e 2 são definidos de novo na ER G (não vêm da ER M).</t>
   </si>
   <si>
     <t>8. Todos os ciclos ficam nesta mesma planilha. Para criar um ciclo novo, copie as linhas de um ciclo existente (nas abas "Movimentos", "Painéis" e "Tipos de movimento"), cole no fim e troque o "Ciclo". Cada nome diferente de ciclo aparece no seletor do visualizador.</t>
@@ -1852,7 +1873,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:W376"/>
+  <dimension ref="A1:W383"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="13" style="1" customWidth="1"/>
@@ -2160,13 +2181,13 @@
         <v>50</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>29</v>
+        <v>51</v>
       </c>
       <c r="F8" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="G8" s="1" t="s">
         <v>51</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>29</v>
       </c>
       <c r="H8" s="1"/>
       <c r="K8" s="1"/>
@@ -2190,13 +2211,13 @@
         <v>24</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>30</v>
@@ -2226,23 +2247,23 @@
         <v>24</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>29</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G10" s="1" t="s">
         <v>29</v>
       </c>
       <c r="H10" s="1"/>
       <c r="J10" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="K10" s="1" t="s">
         <v>29</v>
@@ -2267,16 +2288,16 @@
         <v>24</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G11" s="1" t="s">
         <v>29</v>
@@ -2303,19 +2324,19 @@
         <v>24</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H12" s="1"/>
       <c r="K12" s="1"/>
@@ -2339,16 +2360,16 @@
         <v>24</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>29</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G13" s="1" t="s">
         <v>29</v>
@@ -2375,19 +2396,19 @@
         <v>24</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H14" s="1"/>
       <c r="K14" s="1"/>
@@ -2411,19 +2432,19 @@
         <v>24</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>29</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H15" s="1"/>
       <c r="J15" s="1" t="s">
@@ -2434,10 +2455,10 @@
       </c>
       <c r="L15" s="1"/>
       <c r="N15" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="O15" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="P15" s="1"/>
       <c r="R15" s="5"/>
@@ -2459,16 +2480,16 @@
         <v>24</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>29</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G16" s="1" t="s">
         <v>29</v>
@@ -2495,19 +2516,19 @@
         <v>24</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H17" s="1"/>
       <c r="K17" s="1"/>
@@ -2531,16 +2552,16 @@
         <v>24</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>29</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G18" s="1" t="s">
         <v>29</v>
@@ -2573,16 +2594,16 @@
         <v>24</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>29</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G19" s="1" t="s">
         <v>29</v>
@@ -2615,10 +2636,10 @@
         <v>24</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>35</v>
@@ -2657,19 +2678,19 @@
         <v>24</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>27</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H21" s="1"/>
       <c r="K21" s="1"/>
@@ -2693,23 +2714,23 @@
         <v>24</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E22" s="1" t="s">
         <v>27</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G22" s="1" t="s">
         <v>29</v>
       </c>
       <c r="H22" s="1"/>
       <c r="J22" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K22" s="1" t="s">
         <v>35</v>
@@ -2734,19 +2755,19 @@
         <v>24</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>27</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H23" s="1"/>
       <c r="K23" s="1"/>
@@ -2770,13 +2791,13 @@
         <v>24</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G24" s="1"/>
       <c r="H24" s="1"/>
@@ -2807,16 +2828,16 @@
         <v>24</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>29</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G25" s="1" t="s">
         <v>29</v>
@@ -2849,16 +2870,16 @@
         <v>24</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E26" s="1" t="s">
         <v>29</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G26" s="1" t="s">
         <v>29</v>
@@ -2891,13 +2912,13 @@
         <v>24</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G27" s="1"/>
       <c r="H27" s="1"/>
@@ -2928,16 +2949,16 @@
         <v>24</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E28" s="1" t="s">
         <v>27</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G28" s="1" t="s">
         <v>29</v>
@@ -2969,10 +2990,10 @@
         <v>24</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E29" s="1" t="s">
         <v>27</v>
@@ -2981,7 +3002,7 @@
         <v>28</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H29" s="1"/>
       <c r="J29" s="1" t="s">
@@ -3010,16 +3031,16 @@
         <v>24</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E30" s="1" t="s">
         <v>27</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G30" s="1" t="s">
         <v>29</v>
@@ -3048,22 +3069,22 @@
         <v>23</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>112</v>
+        <v>49</v>
       </c>
       <c r="D31" s="7" t="s">
         <v>113</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>36</v>
+        <v>114</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="H31" s="1"/>
       <c r="K31" s="1"/>
@@ -3084,22 +3105,22 @@
         <v>23</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D32" s="7" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>54</v>
+        <v>35</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>116</v>
+        <v>36</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>54</v>
+        <v>35</v>
       </c>
       <c r="H32" s="1"/>
       <c r="K32" s="1"/>
@@ -3120,7 +3141,7 @@
         <v>23</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C33" s="6" t="s">
         <v>117</v>
@@ -3129,13 +3150,13 @@
         <v>118</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>29</v>
+        <v>55</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>51</v>
+        <v>119</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>29</v>
+        <v>55</v>
       </c>
       <c r="H33" s="1"/>
       <c r="K33" s="1"/>
@@ -3156,22 +3177,22 @@
         <v>23</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>54</v>
+        <v>29</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>54</v>
+        <v>29</v>
       </c>
       <c r="H34" s="1"/>
       <c r="K34" s="1"/>
@@ -3187,12 +3208,12 @@
         <v>32</v>
       </c>
     </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C35" s="6" t="s">
         <v>122</v>
@@ -3200,8 +3221,15 @@
       <c r="D35" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="E35" s="1"/>
-      <c r="G35" s="1"/>
+      <c r="E35" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>55</v>
+      </c>
       <c r="H35" s="1"/>
       <c r="K35" s="1"/>
       <c r="L35" s="1"/>
@@ -3209,30 +3237,28 @@
       <c r="P35" s="1"/>
       <c r="S35" s="1"/>
       <c r="T35" s="1"/>
-      <c r="V35" s="1"/>
-    </row>
-    <row r="36" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="V35" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="W35" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="36" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D36" s="7" t="s">
-        <v>125</v>
-      </c>
-      <c r="E36" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="F36" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="G36" s="1" t="s">
-        <v>54</v>
-      </c>
+        <v>126</v>
+      </c>
+      <c r="E36" s="1"/>
+      <c r="G36" s="1"/>
       <c r="H36" s="1"/>
       <c r="K36" s="1"/>
       <c r="L36" s="1"/>
@@ -3240,34 +3266,29 @@
       <c r="P36" s="1"/>
       <c r="S36" s="1"/>
       <c r="T36" s="1"/>
-      <c r="V36" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="W36" s="1" t="s">
-        <v>32</v>
-      </c>
+      <c r="V36" s="1"/>
     </row>
     <row r="37" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D37" s="7" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>29</v>
+        <v>55</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>58</v>
+        <v>80</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>29</v>
+        <v>55</v>
       </c>
       <c r="H37" s="1"/>
       <c r="K37" s="1"/>
@@ -3288,22 +3309,22 @@
         <v>23</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D38" s="7" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="H38" s="1"/>
       <c r="K38" s="1"/>
@@ -3324,22 +3345,22 @@
         <v>23</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>132</v>
+        <v>35</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>133</v>
+        <v>36</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>132</v>
+        <v>35</v>
       </c>
       <c r="H39" s="1"/>
       <c r="K39" s="1"/>
@@ -3349,7 +3370,7 @@
       <c r="S39" s="1"/>
       <c r="T39" s="1"/>
       <c r="V39" s="1" t="s">
-        <v>134</v>
+        <v>32</v>
       </c>
       <c r="W39" s="1" t="s">
         <v>32</v>
@@ -3360,22 +3381,22 @@
         <v>23</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D40" s="7" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>132</v>
+        <v>51</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>137</v>
+        <v>52</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>132</v>
+        <v>51</v>
       </c>
       <c r="H40" s="1"/>
       <c r="K40" s="1"/>
@@ -3385,7 +3406,7 @@
       <c r="S40" s="1"/>
       <c r="T40" s="1"/>
       <c r="V40" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="W40" s="1" t="s">
         <v>32</v>
@@ -3396,22 +3417,22 @@
         <v>23</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C41" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="D41" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="F41" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="D41" s="7" t="s">
-        <v>139</v>
-      </c>
-      <c r="E41" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="F41" s="1" t="s">
-        <v>30</v>
-      </c>
       <c r="G41" s="1" t="s">
-        <v>31</v>
+        <v>51</v>
       </c>
       <c r="H41" s="1"/>
       <c r="K41" s="1"/>
@@ -3421,33 +3442,33 @@
       <c r="S41" s="1"/>
       <c r="T41" s="1"/>
       <c r="V41" s="1" t="s">
-        <v>32</v>
+        <v>135</v>
       </c>
       <c r="W41" s="1" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="42" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A42" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B42" s="3" t="s">
+      <c r="A42" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B42" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="D42" s="7" t="s">
         <v>140</v>
       </c>
-      <c r="C42" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="D42" s="4" t="s">
-        <v>142</v>
-      </c>
       <c r="E42" s="1" t="s">
-        <v>29</v>
+        <v>55</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>58</v>
+        <v>30</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="H42" s="1"/>
       <c r="K42" s="1"/>
@@ -3468,22 +3489,22 @@
         <v>23</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>143</v>
+        <v>44</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>54</v>
+        <v>29</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>79</v>
+        <v>46</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>54</v>
+        <v>29</v>
       </c>
       <c r="H43" s="1"/>
       <c r="K43" s="1"/>
@@ -3493,34 +3514,27 @@
       <c r="S43" s="1"/>
       <c r="T43" s="1"/>
       <c r="V43" s="1" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="W43" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="44" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
         <v>23</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>145</v>
+        <v>47</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="E44" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="F44" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="G44" s="1" t="s">
-        <v>54</v>
-      </c>
+        <v>143</v>
+      </c>
+      <c r="E44" s="1"/>
+      <c r="G44" s="1"/>
       <c r="H44" s="1"/>
       <c r="K44" s="1"/>
       <c r="L44" s="1"/>
@@ -3528,28 +3542,30 @@
       <c r="P44" s="1"/>
       <c r="S44" s="1"/>
       <c r="T44" s="1"/>
-      <c r="V44" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="W44" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="V44" s="1"/>
+    </row>
+    <row r="45" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
         <v>23</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>147</v>
+        <v>49</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>148</v>
-      </c>
-      <c r="E45" s="1"/>
-      <c r="G45" s="1"/>
+        <v>144</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="G45" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="H45" s="1"/>
       <c r="K45" s="1"/>
       <c r="L45" s="1"/>
@@ -3557,29 +3573,34 @@
       <c r="P45" s="1"/>
       <c r="S45" s="1"/>
       <c r="T45" s="1"/>
-      <c r="V45" s="1"/>
+      <c r="V45" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="W45" s="1" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="46" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
         <v>23</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>151</v>
+        <v>59</v>
       </c>
       <c r="G46" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="H46" s="1"/>
       <c r="K46" s="1"/>
@@ -3595,21 +3616,28 @@
         <v>32</v>
       </c>
     </row>
-    <row r="47" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
         <v>23</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>152</v>
+        <v>122</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="E47" s="1"/>
-      <c r="G47" s="1"/>
+        <v>147</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F47" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="G47" s="1" t="s">
+        <v>55</v>
+      </c>
       <c r="H47" s="1"/>
       <c r="K47" s="1"/>
       <c r="L47" s="1"/>
@@ -3617,24 +3645,27 @@
       <c r="P47" s="1"/>
       <c r="S47" s="1"/>
       <c r="T47" s="1"/>
-      <c r="V47" s="1"/>
-    </row>
-    <row r="48" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="V47" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="W47" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="48" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
         <v>23</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>154</v>
+        <v>125</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="E48" s="1" t="s">
-        <v>31</v>
-      </c>
+        <v>148</v>
+      </c>
+      <c r="E48" s="1"/>
       <c r="G48" s="1"/>
       <c r="H48" s="1"/>
       <c r="K48" s="1"/>
@@ -3643,28 +3674,30 @@
       <c r="P48" s="1"/>
       <c r="S48" s="1"/>
       <c r="T48" s="1"/>
-      <c r="V48" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="W48" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="49" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="V48" s="1"/>
+    </row>
+    <row r="49" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
         <v>23</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>156</v>
+        <v>127</v>
       </c>
       <c r="D49" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="E49" s="1"/>
-      <c r="G49" s="1"/>
+        <v>149</v>
+      </c>
+      <c r="E49" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="F49" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="G49" s="1" t="s">
+        <v>35</v>
+      </c>
       <c r="H49" s="1"/>
       <c r="K49" s="1"/>
       <c r="L49" s="1"/>
@@ -3672,23 +3705,35 @@
       <c r="P49" s="1"/>
       <c r="S49" s="1"/>
       <c r="T49" s="1"/>
-      <c r="V49" s="1"/>
-    </row>
-    <row r="50" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="V49" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="W49" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="50" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
         <v>23</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="E50" s="1"/>
-      <c r="G50" s="1"/>
+        <v>151</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F50" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="G50" s="1" t="s">
+        <v>55</v>
+      </c>
       <c r="H50" s="1"/>
       <c r="K50" s="1"/>
       <c r="L50" s="1"/>
@@ -3696,29 +3741,34 @@
       <c r="P50" s="1"/>
       <c r="S50" s="1"/>
       <c r="T50" s="1"/>
-      <c r="V50" s="1"/>
+      <c r="V50" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="W50" s="1" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="51" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
         <v>23</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>36</v>
+        <v>124</v>
       </c>
       <c r="G51" s="1" t="s">
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="H51" s="1"/>
       <c r="K51" s="1"/>
@@ -3734,28 +3784,21 @@
         <v>32</v>
       </c>
     </row>
-    <row r="52" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
         <v>23</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>163</v>
-      </c>
-      <c r="E52" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="F52" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="G52" s="1" t="s">
-        <v>29</v>
-      </c>
+        <v>155</v>
+      </c>
+      <c r="E52" s="1"/>
+      <c r="G52" s="1"/>
       <c r="H52" s="1"/>
       <c r="K52" s="1"/>
       <c r="L52" s="1"/>
@@ -3763,31 +3806,26 @@
       <c r="P52" s="1"/>
       <c r="S52" s="1"/>
       <c r="T52" s="1"/>
-      <c r="V52" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="W52" s="1" t="s">
-        <v>32</v>
-      </c>
+      <c r="V52" s="1"/>
     </row>
     <row r="53" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
         <v>23</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="E53" s="1" t="s">
         <v>31</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="G53" s="1" t="s">
         <v>31</v>
@@ -3806,28 +3844,21 @@
         <v>32</v>
       </c>
     </row>
-    <row r="54" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
         <v>23</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="D54" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="E54" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="F54" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="G54" s="1" t="s">
-        <v>54</v>
-      </c>
+        <v>160</v>
+      </c>
+      <c r="E54" s="1"/>
+      <c r="G54" s="1"/>
       <c r="H54" s="1"/>
       <c r="K54" s="1"/>
       <c r="L54" s="1"/>
@@ -3835,35 +3866,25 @@
       <c r="P54" s="1"/>
       <c r="S54" s="1"/>
       <c r="T54" s="1"/>
-      <c r="V54" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="W54" s="1" t="s">
-        <v>32</v>
-      </c>
+      <c r="V54" s="1"/>
     </row>
     <row r="55" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
         <v>23</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="D55" s="4" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="F55" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="G55" s="1" t="s">
-        <v>54</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="G55" s="1"/>
       <c r="H55" s="1"/>
       <c r="K55" s="1"/>
       <c r="L55" s="1"/>
@@ -3878,28 +3899,21 @@
         <v>32</v>
       </c>
     </row>
-    <row r="56" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A56" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="B56" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="C56" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="D56" s="7" t="s">
-        <v>173</v>
-      </c>
-      <c r="E56" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="F56" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="G56" s="1" t="s">
-        <v>132</v>
-      </c>
+    <row r="56" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A56" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B56" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="C56" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="E56" s="1"/>
+      <c r="G56" s="1"/>
       <c r="H56" s="1"/>
       <c r="K56" s="1"/>
       <c r="L56" s="1"/>
@@ -3907,29 +3921,22 @@
       <c r="P56" s="1"/>
       <c r="S56" s="1"/>
       <c r="T56" s="1"/>
-      <c r="V56" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="W56" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="57" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A57" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="B57" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="C57" s="6" t="s">
-        <v>175</v>
-      </c>
-      <c r="D57" s="7" t="s">
-        <v>176</v>
-      </c>
-      <c r="E57" s="1" t="s">
-        <v>132</v>
-      </c>
+      <c r="V56" s="1"/>
+    </row>
+    <row r="57" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A57" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B57" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="C57" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="D57" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="E57" s="1"/>
       <c r="G57" s="1"/>
       <c r="H57" s="1"/>
       <c r="K57" s="1"/>
@@ -3938,28 +3945,30 @@
       <c r="P57" s="1"/>
       <c r="S57" s="1"/>
       <c r="T57" s="1"/>
-      <c r="V57" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="W57" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="58" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A58" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="B58" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="C58" s="6" t="s">
-        <v>177</v>
-      </c>
-      <c r="D58" s="7" t="s">
-        <v>178</v>
-      </c>
-      <c r="E58" s="1"/>
-      <c r="G58" s="1"/>
+      <c r="V57" s="1"/>
+    </row>
+    <row r="58" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A58" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B58" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="C58" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="D58" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="E58" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="F58" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G58" s="1" t="s">
+        <v>35</v>
+      </c>
       <c r="H58" s="1"/>
       <c r="K58" s="1"/>
       <c r="L58" s="1"/>
@@ -3967,25 +3976,35 @@
       <c r="P58" s="1"/>
       <c r="S58" s="1"/>
       <c r="T58" s="1"/>
-      <c r="V58" s="1"/>
+      <c r="V58" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="W58" s="1" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="59" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A59" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="B59" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="C59" s="6" t="s">
-        <v>179</v>
-      </c>
-      <c r="D59" s="7" t="s">
-        <v>180</v>
+      <c r="A59" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="C59" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="D59" s="4" t="s">
+        <v>170</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="G59" s="1"/>
+        <v>29</v>
+      </c>
+      <c r="F59" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="G59" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="H59" s="1"/>
       <c r="K59" s="1"/>
       <c r="L59" s="1"/>
@@ -4000,21 +4019,28 @@
         <v>32</v>
       </c>
     </row>
-    <row r="60" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A60" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="B60" s="6" t="s">
+    <row r="60" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A60" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="C60" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="C60" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="D60" s="7" t="s">
-        <v>182</v>
-      </c>
-      <c r="E60" s="1"/>
-      <c r="G60" s="1"/>
+      <c r="D60" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F60" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="G60" s="1" t="s">
+        <v>31</v>
+      </c>
       <c r="H60" s="1"/>
       <c r="K60" s="1"/>
       <c r="L60" s="1"/>
@@ -4022,25 +4048,35 @@
       <c r="P60" s="1"/>
       <c r="S60" s="1"/>
       <c r="T60" s="1"/>
-      <c r="V60" s="1"/>
+      <c r="V60" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="W60" s="1" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="61" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A61" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="B61" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="C61" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="D61" s="7" t="s">
-        <v>184</v>
+      <c r="A61" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B61" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="C61" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="D61" s="4" t="s">
+        <v>175</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="G61" s="1"/>
+        <v>55</v>
+      </c>
+      <c r="F61" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="G61" s="1" t="s">
+        <v>55</v>
+      </c>
       <c r="H61" s="1"/>
       <c r="K61" s="1"/>
       <c r="L61" s="1"/>
@@ -4056,26 +4092,26 @@
       </c>
     </row>
     <row r="62" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A62" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="B62" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="C62" s="6" t="s">
-        <v>185</v>
-      </c>
-      <c r="D62" s="7" t="s">
-        <v>186</v>
+      <c r="A62" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B62" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="C62" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="D62" s="4" t="s">
+        <v>177</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>36</v>
+        <v>71</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="H62" s="1"/>
       <c r="K62" s="1"/>
@@ -4096,18 +4132,23 @@
         <v>23</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="D63" s="7" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="G63" s="1"/>
+        <v>51</v>
+      </c>
+      <c r="F63" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="G63" s="1" t="s">
+        <v>51</v>
+      </c>
       <c r="H63" s="1"/>
       <c r="K63" s="1"/>
       <c r="L63" s="1"/>
@@ -4122,20 +4163,22 @@
         <v>32</v>
       </c>
     </row>
-    <row r="64" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A64" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="D64" s="7" t="s">
-        <v>190</v>
-      </c>
-      <c r="E64" s="1"/>
+        <v>183</v>
+      </c>
+      <c r="E64" s="1" t="s">
+        <v>51</v>
+      </c>
       <c r="G64" s="1"/>
       <c r="H64" s="1"/>
       <c r="K64" s="1"/>
@@ -4144,24 +4187,27 @@
       <c r="P64" s="1"/>
       <c r="S64" s="1"/>
       <c r="T64" s="1"/>
-      <c r="V64" s="1"/>
-    </row>
-    <row r="65" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="V64" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="W64" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="65" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A65" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="D65" s="7" t="s">
-        <v>192</v>
-      </c>
-      <c r="E65" s="1" t="s">
-        <v>35</v>
-      </c>
+        <v>185</v>
+      </c>
+      <c r="E65" s="1"/>
       <c r="G65" s="1"/>
       <c r="H65" s="1"/>
       <c r="K65" s="1"/>
@@ -4170,27 +4216,24 @@
       <c r="P65" s="1"/>
       <c r="S65" s="1"/>
       <c r="T65" s="1"/>
-      <c r="V65" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="W65" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="66" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="V65" s="1"/>
+    </row>
+    <row r="66" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A66" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="D66" s="7" t="s">
-        <v>194</v>
-      </c>
-      <c r="E66" s="1"/>
+        <v>187</v>
+      </c>
+      <c r="E66" s="1" t="s">
+        <v>51</v>
+      </c>
       <c r="G66" s="1"/>
       <c r="H66" s="1"/>
       <c r="K66" s="1"/>
@@ -4199,24 +4242,27 @@
       <c r="P66" s="1"/>
       <c r="S66" s="1"/>
       <c r="T66" s="1"/>
-      <c r="V66" s="1"/>
-    </row>
-    <row r="67" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="V66" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="W66" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="67" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A67" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="D67" s="7" t="s">
-        <v>196</v>
-      </c>
-      <c r="E67" s="1" t="s">
-        <v>35</v>
-      </c>
+        <v>189</v>
+      </c>
+      <c r="E67" s="1"/>
       <c r="G67" s="1"/>
       <c r="H67" s="1"/>
       <c r="K67" s="1"/>
@@ -4225,35 +4271,25 @@
       <c r="P67" s="1"/>
       <c r="S67" s="1"/>
       <c r="T67" s="1"/>
-      <c r="V67" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="W67" s="1" t="s">
-        <v>32</v>
-      </c>
+      <c r="V67" s="1"/>
     </row>
     <row r="68" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A68" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="D68" s="7" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="F68" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="G68" s="1" t="s">
-        <v>54</v>
-      </c>
+        <v>51</v>
+      </c>
+      <c r="G68" s="1"/>
       <c r="H68" s="1"/>
       <c r="K68" s="1"/>
       <c r="L68" s="1"/>
@@ -4273,18 +4309,23 @@
         <v>23</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="D69" s="7" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="G69" s="1"/>
+        <v>35</v>
+      </c>
+      <c r="F69" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G69" s="1" t="s">
+        <v>35</v>
+      </c>
       <c r="H69" s="1"/>
       <c r="K69" s="1"/>
       <c r="L69" s="1"/>
@@ -4299,20 +4340,22 @@
         <v>32</v>
       </c>
     </row>
-    <row r="70" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A70" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="C70" s="6" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="D70" s="7" t="s">
-        <v>203</v>
-      </c>
-      <c r="E70" s="1"/>
+        <v>195</v>
+      </c>
+      <c r="E70" s="1" t="s">
+        <v>35</v>
+      </c>
       <c r="G70" s="1"/>
       <c r="H70" s="1"/>
       <c r="K70" s="1"/>
@@ -4321,24 +4364,27 @@
       <c r="P70" s="1"/>
       <c r="S70" s="1"/>
       <c r="T70" s="1"/>
-      <c r="V70" s="1"/>
-    </row>
-    <row r="71" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="V70" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="W70" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="71" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A71" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B71" s="6" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="C71" s="6" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="D71" s="7" t="s">
-        <v>205</v>
-      </c>
-      <c r="E71" s="1" t="s">
-        <v>54</v>
-      </c>
+        <v>197</v>
+      </c>
+      <c r="E71" s="1"/>
       <c r="G71" s="1"/>
       <c r="H71" s="1"/>
       <c r="K71" s="1"/>
@@ -4347,27 +4393,24 @@
       <c r="P71" s="1"/>
       <c r="S71" s="1"/>
       <c r="T71" s="1"/>
-      <c r="V71" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="W71" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="72" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="V71" s="1"/>
+    </row>
+    <row r="72" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A72" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="C72" s="6" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="D72" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="E72" s="1"/>
+        <v>199</v>
+      </c>
+      <c r="E72" s="1" t="s">
+        <v>35</v>
+      </c>
       <c r="G72" s="1"/>
       <c r="H72" s="1"/>
       <c r="K72" s="1"/>
@@ -4376,24 +4419,27 @@
       <c r="P72" s="1"/>
       <c r="S72" s="1"/>
       <c r="T72" s="1"/>
-      <c r="V72" s="1"/>
-    </row>
-    <row r="73" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="V72" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="W72" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="73" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A73" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B73" s="6" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="C73" s="6" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="D73" s="7" t="s">
-        <v>209</v>
-      </c>
-      <c r="E73" s="1" t="s">
-        <v>54</v>
-      </c>
+        <v>201</v>
+      </c>
+      <c r="E73" s="1"/>
       <c r="G73" s="1"/>
       <c r="H73" s="1"/>
       <c r="K73" s="1"/>
@@ -4402,35 +4448,25 @@
       <c r="P73" s="1"/>
       <c r="S73" s="1"/>
       <c r="T73" s="1"/>
-      <c r="V73" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="W73" s="1" t="s">
-        <v>32</v>
-      </c>
+      <c r="V73" s="1"/>
     </row>
     <row r="74" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A74" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B74" s="6" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="C74" s="6" t="s">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="D74" s="7" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="E74" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="F74" s="1" t="s">
-        <v>212</v>
-      </c>
-      <c r="G74" s="1" t="s">
-        <v>54</v>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="G74" s="1"/>
       <c r="H74" s="1"/>
       <c r="K74" s="1"/>
       <c r="L74" s="1"/>
@@ -4450,22 +4486,22 @@
         <v>23</v>
       </c>
       <c r="B75" s="6" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="C75" s="6" t="s">
-        <v>213</v>
+        <v>204</v>
       </c>
       <c r="D75" s="7" t="s">
-        <v>214</v>
+        <v>205</v>
       </c>
       <c r="E75" s="1" t="s">
-        <v>29</v>
+        <v>55</v>
       </c>
       <c r="F75" s="1" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="G75" s="1" t="s">
-        <v>29</v>
+        <v>55</v>
       </c>
       <c r="H75" s="1"/>
       <c r="K75" s="1"/>
@@ -4486,43 +4522,45 @@
         <v>23</v>
       </c>
       <c r="B76" s="6" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="C76" s="6" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="D76" s="7" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="E76" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="F76" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="G76" s="1" t="s">
-        <v>132</v>
-      </c>
+        <v>55</v>
+      </c>
+      <c r="G76" s="1"/>
       <c r="H76" s="1"/>
-      <c r="J76" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="K76" s="1" t="s">
-        <v>132</v>
-      </c>
+      <c r="K76" s="1"/>
       <c r="L76" s="1"/>
       <c r="O76" s="1"/>
       <c r="P76" s="1"/>
       <c r="S76" s="1"/>
       <c r="T76" s="1"/>
       <c r="V76" s="1" t="s">
-        <v>134</v>
+        <v>32</v>
       </c>
       <c r="W76" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="77" spans="5:22" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A77" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B77" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="C77" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="D77" s="7" t="s">
+        <v>210</v>
+      </c>
       <c r="E77" s="1"/>
       <c r="G77" s="1"/>
       <c r="H77" s="1"/>
@@ -4534,8 +4572,22 @@
       <c r="T77" s="1"/>
       <c r="V77" s="1"/>
     </row>
-    <row r="78" spans="5:22" x14ac:dyDescent="0.25">
-      <c r="E78" s="1"/>
+    <row r="78" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A78" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B78" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="C78" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="D78" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="E78" s="1" t="s">
+        <v>55</v>
+      </c>
       <c r="G78" s="1"/>
       <c r="H78" s="1"/>
       <c r="K78" s="1"/>
@@ -4544,9 +4596,26 @@
       <c r="P78" s="1"/>
       <c r="S78" s="1"/>
       <c r="T78" s="1"/>
-      <c r="V78" s="1"/>
-    </row>
-    <row r="79" spans="5:22" x14ac:dyDescent="0.25">
+      <c r="V78" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="W78" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="79" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A79" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B79" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="C79" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="D79" s="7" t="s">
+        <v>214</v>
+      </c>
       <c r="E79" s="1"/>
       <c r="G79" s="1"/>
       <c r="H79" s="1"/>
@@ -4558,8 +4627,22 @@
       <c r="T79" s="1"/>
       <c r="V79" s="1"/>
     </row>
-    <row r="80" spans="5:22" x14ac:dyDescent="0.25">
-      <c r="E80" s="1"/>
+    <row r="80" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A80" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B80" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="C80" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="D80" s="7" t="s">
+        <v>216</v>
+      </c>
+      <c r="E80" s="1" t="s">
+        <v>55</v>
+      </c>
       <c r="G80" s="1"/>
       <c r="H80" s="1"/>
       <c r="K80" s="1"/>
@@ -4568,11 +4651,35 @@
       <c r="P80" s="1"/>
       <c r="S80" s="1"/>
       <c r="T80" s="1"/>
-      <c r="V80" s="1"/>
-    </row>
-    <row r="81" spans="5:22" x14ac:dyDescent="0.25">
-      <c r="E81" s="1"/>
-      <c r="G81" s="1"/>
+      <c r="V80" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="W80" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="81" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A81" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B81" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="C81" s="6" t="s">
+        <v>217</v>
+      </c>
+      <c r="D81" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="E81" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F81" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="G81" s="1" t="s">
+        <v>55</v>
+      </c>
       <c r="H81" s="1"/>
       <c r="K81" s="1"/>
       <c r="L81" s="1"/>
@@ -4580,11 +4687,35 @@
       <c r="P81" s="1"/>
       <c r="S81" s="1"/>
       <c r="T81" s="1"/>
-      <c r="V81" s="1"/>
-    </row>
-    <row r="82" spans="5:22" x14ac:dyDescent="0.25">
-      <c r="E82" s="1"/>
-      <c r="G82" s="1"/>
+      <c r="V81" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="W81" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="82" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A82" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B82" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="C82" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="D82" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="E82" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F82" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="G82" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="H82" s="1"/>
       <c r="K82" s="1"/>
       <c r="L82" s="1"/>
@@ -4592,19 +4723,53 @@
       <c r="P82" s="1"/>
       <c r="S82" s="1"/>
       <c r="T82" s="1"/>
-      <c r="V82" s="1"/>
-    </row>
-    <row r="83" spans="5:22" x14ac:dyDescent="0.25">
-      <c r="E83" s="1"/>
-      <c r="G83" s="1"/>
+      <c r="V82" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="W82" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="83" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A83" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B83" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="C83" s="6" t="s">
+        <v>222</v>
+      </c>
+      <c r="D83" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="E83" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="F83" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="G83" s="1" t="s">
+        <v>51</v>
+      </c>
       <c r="H83" s="1"/>
-      <c r="K83" s="1"/>
+      <c r="J83" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="K83" s="1" t="s">
+        <v>51</v>
+      </c>
       <c r="L83" s="1"/>
       <c r="O83" s="1"/>
       <c r="P83" s="1"/>
       <c r="S83" s="1"/>
       <c r="T83" s="1"/>
-      <c r="V83" s="1"/>
+      <c r="V83" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="W83" s="1" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="84" spans="5:22" x14ac:dyDescent="0.25">
       <c r="E84" s="1"/>
@@ -8122,9 +8287,93 @@
       <c r="T376" s="1"/>
       <c r="V376" s="1"/>
     </row>
+    <row r="377" spans="5:22" x14ac:dyDescent="0.25">
+      <c r="E377" s="1"/>
+      <c r="G377" s="1"/>
+      <c r="H377" s="1"/>
+      <c r="K377" s="1"/>
+      <c r="L377" s="1"/>
+      <c r="O377" s="1"/>
+      <c r="P377" s="1"/>
+      <c r="S377" s="1"/>
+      <c r="T377" s="1"/>
+      <c r="V377" s="1"/>
+    </row>
+    <row r="378" spans="5:22" x14ac:dyDescent="0.25">
+      <c r="E378" s="1"/>
+      <c r="G378" s="1"/>
+      <c r="H378" s="1"/>
+      <c r="K378" s="1"/>
+      <c r="L378" s="1"/>
+      <c r="O378" s="1"/>
+      <c r="P378" s="1"/>
+      <c r="S378" s="1"/>
+      <c r="T378" s="1"/>
+      <c r="V378" s="1"/>
+    </row>
+    <row r="379" spans="5:22" x14ac:dyDescent="0.25">
+      <c r="E379" s="1"/>
+      <c r="G379" s="1"/>
+      <c r="H379" s="1"/>
+      <c r="K379" s="1"/>
+      <c r="L379" s="1"/>
+      <c r="O379" s="1"/>
+      <c r="P379" s="1"/>
+      <c r="S379" s="1"/>
+      <c r="T379" s="1"/>
+      <c r="V379" s="1"/>
+    </row>
+    <row r="380" spans="5:22" x14ac:dyDescent="0.25">
+      <c r="E380" s="1"/>
+      <c r="G380" s="1"/>
+      <c r="H380" s="1"/>
+      <c r="K380" s="1"/>
+      <c r="L380" s="1"/>
+      <c r="O380" s="1"/>
+      <c r="P380" s="1"/>
+      <c r="S380" s="1"/>
+      <c r="T380" s="1"/>
+      <c r="V380" s="1"/>
+    </row>
+    <row r="381" spans="5:22" x14ac:dyDescent="0.25">
+      <c r="E381" s="1"/>
+      <c r="G381" s="1"/>
+      <c r="H381" s="1"/>
+      <c r="K381" s="1"/>
+      <c r="L381" s="1"/>
+      <c r="O381" s="1"/>
+      <c r="P381" s="1"/>
+      <c r="S381" s="1"/>
+      <c r="T381" s="1"/>
+      <c r="V381" s="1"/>
+    </row>
+    <row r="382" spans="5:22" x14ac:dyDescent="0.25">
+      <c r="E382" s="1"/>
+      <c r="G382" s="1"/>
+      <c r="H382" s="1"/>
+      <c r="K382" s="1"/>
+      <c r="L382" s="1"/>
+      <c r="O382" s="1"/>
+      <c r="P382" s="1"/>
+      <c r="S382" s="1"/>
+      <c r="T382" s="1"/>
+      <c r="V382" s="1"/>
+    </row>
+    <row r="383" spans="5:22" x14ac:dyDescent="0.25">
+      <c r="E383" s="1"/>
+      <c r="G383" s="1"/>
+      <c r="H383" s="1"/>
+      <c r="K383" s="1"/>
+      <c r="L383" s="1"/>
+      <c r="O383" s="1"/>
+      <c r="P383" s="1"/>
+      <c r="S383" s="1"/>
+      <c r="T383" s="1"/>
+      <c r="V383" s="1"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:W1"/>
-  <conditionalFormatting sqref="E2:E376">
+  <conditionalFormatting sqref="E2:E383">
     <cfRule type="containsText" dxfId="0" priority="1">
       <formula>NOT(ISERROR(SEARCH("BOT",E2)))</formula>
     </cfRule>
@@ -8144,7 +8393,7 @@
       <formula>NOT(ISERROR(SEARCH("NEUTRO",E2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G376">
+  <conditionalFormatting sqref="G2:G383">
     <cfRule type="containsText" dxfId="6" priority="1">
       <formula>NOT(ISERROR(SEARCH("BOT",G2)))</formula>
     </cfRule>
@@ -8164,7 +8413,7 @@
       <formula>NOT(ISERROR(SEARCH("NEUTRO",G2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K2:K376">
+  <conditionalFormatting sqref="K2:K383">
     <cfRule type="containsText" dxfId="12" priority="1">
       <formula>NOT(ISERROR(SEARCH("BOT",K2)))</formula>
     </cfRule>
@@ -8184,7 +8433,7 @@
       <formula>NOT(ISERROR(SEARCH("NEUTRO",K2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O2:O376">
+  <conditionalFormatting sqref="O2:O383">
     <cfRule type="containsText" dxfId="18" priority="1">
       <formula>NOT(ISERROR(SEARCH("BOT",O2)))</formula>
     </cfRule>
@@ -8204,7 +8453,7 @@
       <formula>NOT(ISERROR(SEARCH("NEUTRO",O2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S2:S376">
+  <conditionalFormatting sqref="S2:S383">
     <cfRule type="containsText" dxfId="24" priority="1">
       <formula>NOT(ISERROR(SEARCH("BOT",S2)))</formula>
     </cfRule>
@@ -8225,64 +8474,64 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="20">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca do Móvel" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca do Móvel" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="E10:E376">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca do Móvel" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca do Móvel" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="E10:E383">
       <formula1>"BOT,EUD,QDB,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca do Móvel" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca do Móvel" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="E2:E376">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca do Móvel" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca do Móvel" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="E2:E383">
       <formula1>"BOT,EUD,QDB,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 1" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 1" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="G10:G376">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 1" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 1" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="G10:G383">
       <formula1>"BOT,EUD,QDB,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 1" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 1" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="G2:G376">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 1" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 1" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="G2:G383">
       <formula1>"BOT,EUD,QDB,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo Etiqueta 1" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo Etiqueta 1" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." sqref="H10:H376">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo Etiqueta 1" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo Etiqueta 1" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." sqref="H10:H383">
       <formula1>"FIXO,EXPOSICAO,NOVO,ANTECIPADO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo Etiqueta 1" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo Etiqueta 1" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." sqref="H2:H376">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo Etiqueta 1" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo Etiqueta 1" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." sqref="H2:H383">
       <formula1>"FIXO,EXPOSICAO,NOVO,ANTECIPADO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 2" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 2" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="K10:K376">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 2" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 2" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="K10:K383">
       <formula1>"BOT,EUD,QDB,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 2" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 2" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="K2:K376">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 2" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 2" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="K2:K383">
       <formula1>"BOT,EUD,QDB,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo Etiqueta 2" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo Etiqueta 2" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." sqref="L10:L376">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo Etiqueta 2" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo Etiqueta 2" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." sqref="L10:L383">
       <formula1>"FIXO,EXPOSICAO,NOVO,ANTECIPADO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo Etiqueta 2" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo Etiqueta 2" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." sqref="L2:L376">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo Etiqueta 2" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo Etiqueta 2" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." sqref="L2:L383">
       <formula1>"FIXO,EXPOSICAO,NOVO,ANTECIPADO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 3" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 3" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="O10:O376">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 3" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 3" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="O10:O383">
       <formula1>"BOT,EUD,QDB,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 3" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 3" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="O2:O376">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 3" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 3" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="O2:O383">
       <formula1>"BOT,EUD,QDB,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo Etiqueta 3" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo Etiqueta 3" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." sqref="P10:P376">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo Etiqueta 3" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo Etiqueta 3" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." sqref="P10:P383">
       <formula1>"FIXO,EXPOSICAO,NOVO,ANTECIPADO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo Etiqueta 3" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo Etiqueta 3" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." sqref="P2:P376">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo Etiqueta 3" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo Etiqueta 3" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." sqref="P2:P383">
       <formula1>"FIXO,EXPOSICAO,NOVO,ANTECIPADO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 4" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 4" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="S10:S376">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 4" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 4" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="S10:S383">
       <formula1>"BOT,EUD,QDB,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 4" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 4" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="S2:S376">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 4" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 4" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="S2:S383">
       <formula1>"BOT,EUD,QDB,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo Etiqueta 4" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo Etiqueta 4" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." sqref="T10:T376">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo Etiqueta 4" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo Etiqueta 4" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." sqref="T10:T383">
       <formula1>"FIXO,EXPOSICAO,NOVO,ANTECIPADO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo Etiqueta 4" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo Etiqueta 4" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." sqref="T2:T376">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo Etiqueta 4" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo Etiqueta 4" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." sqref="T2:T383">
       <formula1>"FIXO,EXPOSICAO,NOVO,ANTECIPADO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" sqref="V10:V376">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" sqref="V10:V383">
       <formula1>"FIXO,EXPOSICAO,NOVO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" sqref="V2:V376">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" sqref="V2:V383">
       <formula1>"FIXO,EXPOSICAO,NOVO"</formula1>
     </dataValidation>
   </dataValidations>
@@ -8310,16 +8559,16 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>218</v>
+        <v>225</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -8327,13 +8576,13 @@
         <v>23</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>222</v>
+        <v>229</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>31</v>
@@ -8347,13 +8596,13 @@
         <v>23</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>29</v>
@@ -8367,16 +8616,16 @@
         <v>23</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>225</v>
+        <v>232</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>32</v>
@@ -8387,13 +8636,13 @@
         <v>23</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>29</v>
@@ -8407,13 +8656,13 @@
         <v>23</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>29</v>
@@ -8427,16 +8676,16 @@
         <v>23</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>227</v>
+        <v>234</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>32</v>
@@ -8447,16 +8696,16 @@
         <v>23</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>228</v>
+        <v>235</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>132</v>
+        <v>51</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>32</v>
@@ -8467,13 +8716,13 @@
         <v>23</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>229</v>
+        <v>236</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>31</v>
@@ -8487,19 +8736,19 @@
         <v>23</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>231</v>
+        <v>238</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>31</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>232</v>
+        <v>239</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -8507,19 +8756,19 @@
         <v>23</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>233</v>
+        <v>240</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -8527,19 +8776,19 @@
         <v>23</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>234</v>
+        <v>241</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -8550,10 +8799,10 @@
         <v>24</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>32</v>
@@ -8570,10 +8819,10 @@
         <v>24</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>237</v>
+        <v>244</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>32</v>
@@ -8587,13 +8836,13 @@
         <v>23</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>32</v>
@@ -8607,13 +8856,13 @@
         <v>23</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>32</v>
@@ -8627,13 +8876,13 @@
         <v>23</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>32</v>
@@ -8647,13 +8896,13 @@
         <v>23</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>32</v>
@@ -8667,13 +8916,13 @@
         <v>23</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>32</v>
@@ -8687,13 +8936,13 @@
         <v>23</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>240</v>
+        <v>247</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>32</v>
@@ -8707,13 +8956,13 @@
         <v>23</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>32</v>
@@ -9979,13 +10228,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>241</v>
+        <v>248</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>242</v>
+        <v>249</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>243</v>
+        <v>250</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>22</v>
@@ -9996,10 +10245,10 @@
         <v>23</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>244</v>
+        <v>251</v>
       </c>
       <c r="D2" s="9">
         <v>150000</v>
@@ -10013,10 +10262,10 @@
         <v>23</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>51</v>
+        <v>114</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>245</v>
+        <v>252</v>
       </c>
       <c r="D3" s="9">
         <v>1200000</v>
@@ -10033,7 +10282,7 @@
         <v>40</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="D4" s="9">
         <v>650000</v>
@@ -10047,10 +10296,10 @@
         <v>23</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>245</v>
+        <v>252</v>
       </c>
       <c r="D5" s="9">
         <v>2400000</v>
@@ -10064,10 +10313,10 @@
         <v>23</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>245</v>
+        <v>252</v>
       </c>
       <c r="D6" s="9">
         <v>430000</v>
@@ -10081,10 +10330,10 @@
         <v>23</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="D7" s="9">
         <v>610000</v>
@@ -10098,7 +10347,7 @@
         <v>23</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>32</v>
@@ -10113,7 +10362,7 @@
         <v>23</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>32</v>
@@ -10128,7 +10377,7 @@
         <v>23</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>174</v>
+        <v>181</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>32</v>
@@ -10143,7 +10392,7 @@
         <v>23</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>32</v>
@@ -10158,10 +10407,10 @@
         <v>23</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="D12" s="9">
         <v>380000</v>
@@ -10178,7 +10427,7 @@
         <v>37</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
       <c r="D13" s="9">
         <v>620000</v>
@@ -10192,10 +10441,10 @@
         <v>23</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
       <c r="D14" s="9">
         <v>1800000</v>
@@ -10209,10 +10458,10 @@
         <v>23</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
       <c r="D15" s="9">
         <v>950000</v>
@@ -10226,10 +10475,10 @@
         <v>23</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="D16" s="9">
         <v>210000</v>
@@ -10246,7 +10495,7 @@
         <v>36</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="D17" s="9">
         <v>900000</v>
@@ -10260,10 +10509,10 @@
         <v>23</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>133</v>
+        <v>52</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
       <c r="D18" s="9">
         <v>260000</v>
@@ -10280,7 +10529,7 @@
         <v>30</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>245</v>
+        <v>252</v>
       </c>
       <c r="D19" s="9">
         <v>1500000</v>
@@ -10294,10 +10543,10 @@
         <v>23</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="D20" s="9">
         <v>1100000</v>
@@ -10326,7 +10575,7 @@
         <v>23</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>32</v>
@@ -10341,10 +10590,10 @@
         <v>23</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="D23" s="9">
         <v>870000</v>
@@ -10358,10 +10607,10 @@
         <v>23</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>245</v>
+        <v>252</v>
       </c>
       <c r="D24" s="9">
         <v>700000</v>
@@ -10375,10 +10624,10 @@
         <v>23</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
       <c r="D25" s="9">
         <v>480000</v>
@@ -10392,10 +10641,10 @@
         <v>23</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
       <c r="D26" s="9">
         <v>780000</v>
@@ -10409,10 +10658,10 @@
         <v>23</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
       <c r="D27" s="9">
         <v>540000</v>
@@ -10429,7 +10678,7 @@
         <v>46</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="D28" s="9">
         <v>520000</v>
@@ -10443,7 +10692,7 @@
         <v>23</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>32</v>
@@ -11666,18 +11915,18 @@
       <formula>NOT(ISERROR(SEARCH("Liquidação / outlet",C2)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="39" priority="4">
-      <formula>NOT(ISERROR(SEARCH("Institucional / portfólio",C2)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Baseline",C2)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="40" priority="5">
       <formula>NOT(ISERROR(SEARCH("Outro",C2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Classificação" prompt="Tipo do movimento: Lançamento, Promoção, Liquidação / outlet, Institucional / portfólio, Outro. Também aceita outro texto." showErrorMessage="1" errorStyle="warning" errorTitle="Classificação" error="Tipo do movimento: Lançamento, Promoção, Liquidação / outlet, Institucional / portfólio, Outro. Também aceita outro texto." sqref="C10:C329">
-      <formula1>"Lançamento,Promoção,Liquidação / outlet,Institucional / portfólio,Outro"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Classificação" prompt="Tipo do movimento: Lançamento, Promoção, Liquidação / outlet, Baseline, Outro. Também aceita outro texto." showErrorMessage="1" errorStyle="warning" errorTitle="Classificação" error="Tipo do movimento: Lançamento, Promoção, Liquidação / outlet, Baseline, Outro. Também aceita outro texto." sqref="C10:C329">
+      <formula1>"Lançamento,Promoção,Liquidação / outlet,Baseline,Outro"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Classificação" prompt="Tipo do movimento: Lançamento, Promoção, Liquidação / outlet, Institucional / portfólio, Outro. Também aceita outro texto." showErrorMessage="1" errorStyle="warning" errorTitle="Classificação" error="Tipo do movimento: Lançamento, Promoção, Liquidação / outlet, Institucional / portfólio, Outro. Também aceita outro texto." sqref="C2:C329">
-      <formula1>"Lançamento,Promoção,Liquidação / outlet,Institucional / portfólio,Outro"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Classificação" prompt="Tipo do movimento: Lançamento, Promoção, Liquidação / outlet, Baseline, Outro. Também aceita outro texto." showErrorMessage="1" errorStyle="warning" errorTitle="Classificação" error="Tipo do movimento: Lançamento, Promoção, Liquidação / outlet, Baseline, Outro. Também aceita outro texto." sqref="C2:C329">
+      <formula1>"Lançamento,Promoção,Liquidação / outlet,Baseline,Outro"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -11698,122 +11947,122 @@
   <sheetData>
     <row r="1" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B1" s="11" t="s">
-        <v>249</v>
+        <v>256</v>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B2" s="12" t="s">
-        <v>250</v>
+        <v>257</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12"/>
     </row>
     <row r="4" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B4" s="13" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B5" s="12" t="s">
-        <v>252</v>
+        <v>259</v>
       </c>
       <c r="C5" s="12"/>
       <c r="D5" s="12"/>
     </row>
     <row r="6" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B6" s="12" t="s">
-        <v>253</v>
+        <v>260</v>
       </c>
       <c r="C6" s="12"/>
       <c r="D6" s="12"/>
     </row>
     <row r="7" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B7" s="12" t="s">
-        <v>254</v>
+        <v>261</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="12"/>
     </row>
     <row r="8" ht="45" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B8" s="12" t="s">
-        <v>255</v>
+        <v>262</v>
       </c>
       <c r="C8" s="12"/>
       <c r="D8" s="12"/>
     </row>
     <row r="9" ht="16" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B9" s="12" t="s">
-        <v>256</v>
+        <v>263</v>
       </c>
       <c r="C9" s="12"/>
       <c r="D9" s="12"/>
     </row>
     <row r="10" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B10" s="12" t="s">
-        <v>257</v>
+        <v>264</v>
       </c>
       <c r="C10" s="12"/>
       <c r="D10" s="12"/>
     </row>
     <row r="11" ht="60" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B11" s="12" t="s">
-        <v>258</v>
+        <v>265</v>
       </c>
       <c r="C11" s="12"/>
       <c r="D11" s="12"/>
     </row>
     <row r="12" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B12" s="12" t="s">
-        <v>259</v>
+        <v>266</v>
       </c>
       <c r="C12" s="12"/>
       <c r="D12" s="12"/>
     </row>
     <row r="13" ht="60" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B13" s="12" t="s">
-        <v>260</v>
+        <v>267</v>
       </c>
       <c r="C13" s="12"/>
       <c r="D13" s="12"/>
     </row>
     <row r="14" ht="60" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B14" s="12" t="s">
-        <v>261</v>
+        <v>268</v>
       </c>
       <c r="C14" s="12"/>
       <c r="D14" s="12"/>
     </row>
     <row r="15" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B15" s="12" t="s">
-        <v>262</v>
+        <v>269</v>
       </c>
       <c r="C15" s="12"/>
       <c r="D15" s="12"/>
     </row>
-    <row r="16" ht="60" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="16" ht="105" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B16" s="12" t="s">
-        <v>263</v>
+        <v>270</v>
       </c>
       <c r="C16" s="12"/>
       <c r="D16" s="12"/>
     </row>
     <row r="17" ht="45" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B17" s="12" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="C17" s="12"/>
       <c r="D17" s="12"/>
     </row>
     <row r="18" ht="45" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B18" s="12" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
       <c r="C18" s="12"/>
       <c r="D18" s="12"/>
     </row>
     <row r="20" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B20" s="13" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.25">
@@ -11824,18 +12073,18 @@
         <v>29</v>
       </c>
       <c r="D21" s="15" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
     </row>
     <row r="22" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B22" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C22" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
     </row>
     <row r="23" spans="2:4" x14ac:dyDescent="0.25">
@@ -11846,18 +12095,18 @@
         <v>35</v>
       </c>
       <c r="D23" s="17" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
     </row>
     <row r="24" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B24" s="14" t="s">
-        <v>132</v>
+        <v>51</v>
       </c>
       <c r="C24" t="s">
-        <v>132</v>
+        <v>51</v>
       </c>
       <c r="D24" s="18" t="s">
-        <v>270</v>
+        <v>277</v>
       </c>
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.25">
@@ -11865,10 +12114,10 @@
         <v>31</v>
       </c>
       <c r="C25" t="s">
-        <v>271</v>
+        <v>278</v>
       </c>
       <c r="D25" s="19" t="s">
-        <v>272</v>
+        <v>279</v>
       </c>
     </row>
     <row r="26" spans="2:4" x14ac:dyDescent="0.25">
@@ -11876,15 +12125,15 @@
         <v>27</v>
       </c>
       <c r="C26" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="D26" s="20" t="s">
-        <v>274</v>
+        <v>281</v>
       </c>
     </row>
     <row r="28" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B28" s="13" t="s">
-        <v>275</v>
+        <v>282</v>
       </c>
     </row>
     <row r="29" spans="2:4" x14ac:dyDescent="0.25">
@@ -11892,111 +12141,111 @@
         <v>41</v>
       </c>
       <c r="C29" t="s">
-        <v>276</v>
+        <v>283</v>
       </c>
       <c r="D29" t="s">
-        <v>277</v>
+        <v>284</v>
       </c>
     </row>
     <row r="30" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B30" s="14" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C30" t="s">
-        <v>278</v>
+        <v>285</v>
       </c>
       <c r="D30" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
     </row>
     <row r="31" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B31" s="14" t="s">
-        <v>280</v>
+        <v>287</v>
       </c>
       <c r="C31" t="s">
-        <v>281</v>
+        <v>288</v>
       </c>
       <c r="D31" t="s">
-        <v>282</v>
+        <v>289</v>
       </c>
     </row>
     <row r="33" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B33" s="13" t="s">
-        <v>283</v>
+        <v>290</v>
       </c>
     </row>
     <row r="34" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B34" s="21" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
     </row>
     <row r="35" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B35" s="22" t="s">
-        <v>245</v>
+        <v>252</v>
       </c>
     </row>
     <row r="36" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B36" s="23" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
     </row>
     <row r="37" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B37" s="24" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
     </row>
     <row r="38" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B38" s="25" t="s">
-        <v>244</v>
+        <v>251</v>
       </c>
     </row>
     <row r="40" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B40" s="13" t="s">
-        <v>284</v>
+        <v>291</v>
       </c>
     </row>
     <row r="41" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B41" s="14" t="s">
-        <v>222</v>
+        <v>229</v>
       </c>
       <c r="C41" t="s">
-        <v>285</v>
+        <v>292</v>
       </c>
       <c r="D41"/>
     </row>
     <row r="42" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B42" s="14" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
       <c r="C42" t="s">
-        <v>286</v>
+        <v>293</v>
       </c>
       <c r="D42"/>
     </row>
     <row r="43" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B43" s="14" t="s">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="C43" t="s">
-        <v>287</v>
+        <v>294</v>
       </c>
       <c r="D43"/>
     </row>
     <row r="44" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B44" s="14" t="s">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="C44" t="s">
-        <v>288</v>
+        <v>295</v>
       </c>
       <c r="D44"/>
     </row>
     <row r="45" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B45" s="14" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="C45" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="D45"/>
     </row>

</xml_diff>

<commit_message>
Gôndola 1 volta a seguir a cascata na ER G: meio B e ponta B livre até a ER GG
Só o lado B da gôndola 2 continua definido de novo na ER G (HERANCA_ENTRE_ERS).
O ciclo de exemplo perde as linhas da gôndola 1 na ER G, que só existiam por
causa da regra.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MHQRMyvP3NMZPhZq474WCH
</commit_message>
<xml_diff>
--- a/visualizador/Planilha base - Visualizador.xlsx
+++ b/visualizador/Planilha base - Visualizador.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="988" uniqueCount="297">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="966" uniqueCount="294">
   <si>
     <t>Ciclo</t>
   </si>
@@ -440,15 +440,6 @@
   </si>
   <si>
     <t>ER G</t>
-  </si>
-  <si>
-    <t>Gôndola 1 – Meio B (ou metade 1, se a metade 2 for preenchida) · defina de novo (não vem da ER M)</t>
-  </si>
-  <si>
-    <t>Gôndola 1 – Meio B – metade 2 (preencha só para dividir o meio em dois) · defina de novo (não vem da ER M)</t>
-  </si>
-  <si>
-    <t>Gôndola 1 – Ponta B · Livre (vale para ER M, ER G, ER GG) · defina de novo (não vem da ER M)</t>
   </si>
   <si>
     <t>MOVEL DE FILA 6</t>
@@ -793,7 +784,7 @@
     <t>Planilha base — Plano de Varejo</t>
   </si>
   <si>
-    <t>Gerada em 23/10/2026, 14:32:12 a partir do ciclo "Ciclo exemplo".</t>
+    <t>Gerada em 23/10/2026, 14:49:43 a partir do ciclo "Ciclo exemplo".</t>
   </si>
   <si>
     <t>Como preencher</t>
@@ -832,7 +823,7 @@
     <t>6.4 Móveis de um espaço só (pirâmide, móvel de fila, móvel de parede, PDV, O.U.i…) têm uma linha. O balcão recepção também: um espaço só, com uma cor e até 3 etiquetas.</t>
   </si>
   <si>
-    <t>7. Na coluna "Planta" vale o nome (ex.: ER P) ou o número (01). Cascata: o que é definido numa planta vale também para as seguintes (ER P → ER M → ER G → ER GG), por isso cada móvel aparece uma vez só, na primeira planta que o tem ("vale para…" na coluna Móvel). Para mudar um móvel só a partir de uma planta, acrescente uma linha com o mesmo ID Móvel e essa planta. Planta = TODAS vale para todas. Exceção: a ponta B da gôndola 1 é fixa de O.U.i na ER P e livre nas ERs maiores — a linha da ER P (Fixo O.U.i) não passa para elas; a da ER M (Livre) vale para a ER M. Da ER M para a ER G: a ponta B e o meio B da gôndola 2 da ER M viram a ponta A e o meio A da gôndola 3 da ER G; a ponta B e o meio B das gôndolas 1 e 2 são definidos de novo na ER G (não vêm da ER M).</t>
+    <t>7. Na coluna "Planta" vale o nome (ex.: ER P) ou o número (01). Cascata: o que é definido numa planta vale também para as seguintes (ER P → ER M → ER G → ER GG), por isso cada móvel aparece uma vez só, na primeira planta que o tem ("vale para…" na coluna Móvel). Para mudar um móvel só a partir de uma planta, acrescente uma linha com o mesmo ID Móvel e essa planta. Planta = TODAS vale para todas. Exceção: a ponta B da gôndola 1 é fixa de O.U.i na ER P e livre nas ERs maiores — a linha da ER P (Fixo O.U.i) não passa para elas; a da ER M (Livre) vale para a ER M, a ER G e a ER GG. Da ER M para a ER G: a ponta B e o meio B da gôndola 2 da ER M viram a ponta A e o meio A da gôndola 3 da ER G; a ponta B e o meio B da gôndola 2 são definidos de novo na ER G (não vêm da ER M). A gôndola 1 segue a cascata normal.</t>
   </si>
   <si>
     <t>8. Todos os ciclos ficam nesta mesma planilha. Para criar um ciclo novo, copie as linhas de um ciclo existente (nas abas "Movimentos", "Painéis" e "Tipos de movimento"), cole no fim e troque o "Ciclo". Cada nome diferente de ciclo aparece no seletor do visualizador.</t>
@@ -1873,7 +1864,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:W383"/>
+  <dimension ref="A1:W380"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="13" style="1" customWidth="1"/>
@@ -3492,16 +3483,16 @@
         <v>141</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>44</v>
+        <v>142</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E43" s="1" t="s">
         <v>29</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="G43" s="1" t="s">
         <v>29</v>
@@ -3514,13 +3505,13 @@
       <c r="S43" s="1"/>
       <c r="T43" s="1"/>
       <c r="V43" s="1" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="W43" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
         <v>23</v>
       </c>
@@ -3528,13 +3519,20 @@
         <v>141</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>47</v>
+        <v>122</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="E44" s="1"/>
-      <c r="G44" s="1"/>
+        <v>144</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="G44" s="1" t="s">
+        <v>55</v>
+      </c>
       <c r="H44" s="1"/>
       <c r="K44" s="1"/>
       <c r="L44" s="1"/>
@@ -3542,9 +3540,14 @@
       <c r="P44" s="1"/>
       <c r="S44" s="1"/>
       <c r="T44" s="1"/>
-      <c r="V44" s="1"/>
-    </row>
-    <row r="45" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="V44" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="W44" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="45" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
         <v>23</v>
       </c>
@@ -3552,20 +3555,13 @@
         <v>141</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>49</v>
+        <v>125</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="E45" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="F45" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="G45" s="1" t="s">
-        <v>29</v>
-      </c>
+        <v>145</v>
+      </c>
+      <c r="E45" s="1"/>
+      <c r="G45" s="1"/>
       <c r="H45" s="1"/>
       <c r="K45" s="1"/>
       <c r="L45" s="1"/>
@@ -3573,12 +3569,7 @@
       <c r="P45" s="1"/>
       <c r="S45" s="1"/>
       <c r="T45" s="1"/>
-      <c r="V45" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="W45" s="1" t="s">
-        <v>32</v>
-      </c>
+      <c r="V45" s="1"/>
     </row>
     <row r="46" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
@@ -3588,19 +3579,19 @@
         <v>141</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>145</v>
+        <v>127</v>
       </c>
       <c r="D46" s="4" t="s">
         <v>146</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>59</v>
+        <v>37</v>
       </c>
       <c r="G46" s="1" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="H46" s="1"/>
       <c r="K46" s="1"/>
@@ -3624,16 +3615,16 @@
         <v>141</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>122</v>
+        <v>147</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E47" s="1" t="s">
         <v>55</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>119</v>
+        <v>80</v>
       </c>
       <c r="G47" s="1" t="s">
         <v>55</v>
@@ -3652,7 +3643,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="48" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
         <v>23</v>
       </c>
@@ -3660,13 +3651,20 @@
         <v>141</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>125</v>
+        <v>149</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>148</v>
-      </c>
-      <c r="E48" s="1"/>
-      <c r="G48" s="1"/>
+        <v>150</v>
+      </c>
+      <c r="E48" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F48" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="G48" s="1" t="s">
+        <v>55</v>
+      </c>
       <c r="H48" s="1"/>
       <c r="K48" s="1"/>
       <c r="L48" s="1"/>
@@ -3674,9 +3672,14 @@
       <c r="P48" s="1"/>
       <c r="S48" s="1"/>
       <c r="T48" s="1"/>
-      <c r="V48" s="1"/>
-    </row>
-    <row r="49" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="V48" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="W48" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="49" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
         <v>23</v>
       </c>
@@ -3684,20 +3687,13 @@
         <v>141</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>127</v>
+        <v>151</v>
       </c>
       <c r="D49" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="E49" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="F49" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="G49" s="1" t="s">
-        <v>35</v>
-      </c>
+        <v>152</v>
+      </c>
+      <c r="E49" s="1"/>
+      <c r="G49" s="1"/>
       <c r="H49" s="1"/>
       <c r="K49" s="1"/>
       <c r="L49" s="1"/>
@@ -3705,12 +3701,7 @@
       <c r="P49" s="1"/>
       <c r="S49" s="1"/>
       <c r="T49" s="1"/>
-      <c r="V49" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="W49" s="1" t="s">
-        <v>32</v>
-      </c>
+      <c r="V49" s="1"/>
     </row>
     <row r="50" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
@@ -3720,19 +3711,19 @@
         <v>141</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>55</v>
+        <v>31</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>80</v>
+        <v>155</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>55</v>
+        <v>31</v>
       </c>
       <c r="H50" s="1"/>
       <c r="K50" s="1"/>
@@ -3748,7 +3739,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="51" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
         <v>23</v>
       </c>
@@ -3756,20 +3747,13 @@
         <v>141</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="E51" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="F51" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="G51" s="1" t="s">
-        <v>55</v>
-      </c>
+        <v>157</v>
+      </c>
+      <c r="E51" s="1"/>
+      <c r="G51" s="1"/>
       <c r="H51" s="1"/>
       <c r="K51" s="1"/>
       <c r="L51" s="1"/>
@@ -3777,14 +3761,9 @@
       <c r="P51" s="1"/>
       <c r="S51" s="1"/>
       <c r="T51" s="1"/>
-      <c r="V51" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="W51" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="52" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="V51" s="1"/>
+    </row>
+    <row r="52" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
         <v>23</v>
       </c>
@@ -3792,12 +3771,14 @@
         <v>141</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="E52" s="1"/>
+        <v>159</v>
+      </c>
+      <c r="E52" s="1" t="s">
+        <v>31</v>
+      </c>
       <c r="G52" s="1"/>
       <c r="H52" s="1"/>
       <c r="K52" s="1"/>
@@ -3806,9 +3787,14 @@
       <c r="P52" s="1"/>
       <c r="S52" s="1"/>
       <c r="T52" s="1"/>
-      <c r="V52" s="1"/>
-    </row>
-    <row r="53" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="V52" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="W52" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="53" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
         <v>23</v>
       </c>
@@ -3816,20 +3802,13 @@
         <v>141</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="E53" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="F53" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="G53" s="1" t="s">
-        <v>31</v>
-      </c>
+        <v>161</v>
+      </c>
+      <c r="E53" s="1"/>
+      <c r="G53" s="1"/>
       <c r="H53" s="1"/>
       <c r="K53" s="1"/>
       <c r="L53" s="1"/>
@@ -3837,12 +3816,7 @@
       <c r="P53" s="1"/>
       <c r="S53" s="1"/>
       <c r="T53" s="1"/>
-      <c r="V53" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="W53" s="1" t="s">
-        <v>32</v>
-      </c>
+      <c r="V53" s="1"/>
     </row>
     <row r="54" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
@@ -3852,10 +3826,10 @@
         <v>141</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="D54" s="4" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="E54" s="1"/>
       <c r="G54" s="1"/>
@@ -3876,15 +3850,20 @@
         <v>141</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="D55" s="4" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="G55" s="1"/>
+        <v>35</v>
+      </c>
+      <c r="F55" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G55" s="1" t="s">
+        <v>35</v>
+      </c>
       <c r="H55" s="1"/>
       <c r="K55" s="1"/>
       <c r="L55" s="1"/>
@@ -3899,7 +3878,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="56" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
         <v>23</v>
       </c>
@@ -3907,13 +3886,20 @@
         <v>141</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="D56" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="E56" s="1"/>
-      <c r="G56" s="1"/>
+        <v>167</v>
+      </c>
+      <c r="E56" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F56" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="G56" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="H56" s="1"/>
       <c r="K56" s="1"/>
       <c r="L56" s="1"/>
@@ -3921,9 +3907,14 @@
       <c r="P56" s="1"/>
       <c r="S56" s="1"/>
       <c r="T56" s="1"/>
-      <c r="V56" s="1"/>
-    </row>
-    <row r="57" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="V56" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="W56" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="57" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="s">
         <v>23</v>
       </c>
@@ -3931,13 +3922,20 @@
         <v>141</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="D57" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="E57" s="1"/>
-      <c r="G57" s="1"/>
+        <v>169</v>
+      </c>
+      <c r="E57" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F57" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="G57" s="1" t="s">
+        <v>31</v>
+      </c>
       <c r="H57" s="1"/>
       <c r="K57" s="1"/>
       <c r="L57" s="1"/>
@@ -3945,7 +3943,12 @@
       <c r="P57" s="1"/>
       <c r="S57" s="1"/>
       <c r="T57" s="1"/>
-      <c r="V57" s="1"/>
+      <c r="V57" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="W57" s="1" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="58" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
@@ -3955,19 +3958,19 @@
         <v>141</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="D58" s="4" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>36</v>
+        <v>65</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="H58" s="1"/>
       <c r="K58" s="1"/>
@@ -3991,19 +3994,19 @@
         <v>141</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="D59" s="4" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>29</v>
+        <v>55</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>29</v>
+        <v>55</v>
       </c>
       <c r="H59" s="1"/>
       <c r="K59" s="1"/>
@@ -4020,26 +4023,26 @@
       </c>
     </row>
     <row r="60" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A60" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B60" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="C60" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="D60" s="4" t="s">
-        <v>172</v>
+      <c r="A60" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B60" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="C60" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="D60" s="7" t="s">
+        <v>177</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>31</v>
+        <v>51</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>31</v>
+        <v>51</v>
       </c>
       <c r="H60" s="1"/>
       <c r="K60" s="1"/>
@@ -4056,27 +4059,22 @@
       </c>
     </row>
     <row r="61" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A61" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B61" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="C61" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="D61" s="4" t="s">
+      <c r="A61" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B61" s="6" t="s">
         <v>175</v>
       </c>
+      <c r="C61" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="D61" s="7" t="s">
+        <v>180</v>
+      </c>
       <c r="E61" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="F61" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="G61" s="1" t="s">
-        <v>55</v>
-      </c>
+        <v>51</v>
+      </c>
+      <c r="G61" s="1"/>
       <c r="H61" s="1"/>
       <c r="K61" s="1"/>
       <c r="L61" s="1"/>
@@ -4091,28 +4089,21 @@
         <v>32</v>
       </c>
     </row>
-    <row r="62" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A62" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B62" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="C62" s="3" t="s">
-        <v>176</v>
-      </c>
-      <c r="D62" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="E62" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="F62" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="G62" s="1" t="s">
-        <v>55</v>
-      </c>
+    <row r="62" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A62" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B62" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="C62" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="D62" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="E62" s="1"/>
+      <c r="G62" s="1"/>
       <c r="H62" s="1"/>
       <c r="K62" s="1"/>
       <c r="L62" s="1"/>
@@ -4120,35 +4111,25 @@
       <c r="P62" s="1"/>
       <c r="S62" s="1"/>
       <c r="T62" s="1"/>
-      <c r="V62" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="W62" s="1" t="s">
-        <v>32</v>
-      </c>
+      <c r="V62" s="1"/>
     </row>
     <row r="63" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A63" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="D63" s="7" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="E63" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="F63" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="G63" s="1" t="s">
-        <v>51</v>
-      </c>
+      <c r="G63" s="1"/>
       <c r="H63" s="1"/>
       <c r="K63" s="1"/>
       <c r="L63" s="1"/>
@@ -4163,22 +4144,20 @@
         <v>32</v>
       </c>
     </row>
-    <row r="64" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A64" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="D64" s="7" t="s">
-        <v>183</v>
-      </c>
-      <c r="E64" s="1" t="s">
-        <v>51</v>
-      </c>
+        <v>186</v>
+      </c>
+      <c r="E64" s="1"/>
       <c r="G64" s="1"/>
       <c r="H64" s="1"/>
       <c r="K64" s="1"/>
@@ -4187,27 +4166,24 @@
       <c r="P64" s="1"/>
       <c r="S64" s="1"/>
       <c r="T64" s="1"/>
-      <c r="V64" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="W64" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="65" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="V64" s="1"/>
+    </row>
+    <row r="65" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A65" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D65" s="7" t="s">
-        <v>185</v>
-      </c>
-      <c r="E65" s="1"/>
+        <v>188</v>
+      </c>
+      <c r="E65" s="1" t="s">
+        <v>51</v>
+      </c>
       <c r="G65" s="1"/>
       <c r="H65" s="1"/>
       <c r="K65" s="1"/>
@@ -4216,25 +4192,35 @@
       <c r="P65" s="1"/>
       <c r="S65" s="1"/>
       <c r="T65" s="1"/>
-      <c r="V65" s="1"/>
+      <c r="V65" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="W65" s="1" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="66" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A66" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="D66" s="7" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="G66" s="1"/>
+        <v>35</v>
+      </c>
+      <c r="F66" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G66" s="1" t="s">
+        <v>35</v>
+      </c>
       <c r="H66" s="1"/>
       <c r="K66" s="1"/>
       <c r="L66" s="1"/>
@@ -4249,20 +4235,22 @@
         <v>32</v>
       </c>
     </row>
-    <row r="67" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A67" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="D67" s="7" t="s">
-        <v>189</v>
-      </c>
-      <c r="E67" s="1"/>
+        <v>192</v>
+      </c>
+      <c r="E67" s="1" t="s">
+        <v>35</v>
+      </c>
       <c r="G67" s="1"/>
       <c r="H67" s="1"/>
       <c r="K67" s="1"/>
@@ -4271,24 +4259,27 @@
       <c r="P67" s="1"/>
       <c r="S67" s="1"/>
       <c r="T67" s="1"/>
-      <c r="V67" s="1"/>
-    </row>
-    <row r="68" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="V67" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="W67" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="68" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A68" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="D68" s="7" t="s">
-        <v>191</v>
-      </c>
-      <c r="E68" s="1" t="s">
-        <v>51</v>
-      </c>
+        <v>194</v>
+      </c>
+      <c r="E68" s="1"/>
       <c r="G68" s="1"/>
       <c r="H68" s="1"/>
       <c r="K68" s="1"/>
@@ -4297,35 +4288,25 @@
       <c r="P68" s="1"/>
       <c r="S68" s="1"/>
       <c r="T68" s="1"/>
-      <c r="V68" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="W68" s="1" t="s">
-        <v>32</v>
-      </c>
+      <c r="V68" s="1"/>
     </row>
     <row r="69" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A69" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="D69" s="7" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="E69" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="F69" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="G69" s="1" t="s">
-        <v>35</v>
-      </c>
+      <c r="G69" s="1"/>
       <c r="H69" s="1"/>
       <c r="K69" s="1"/>
       <c r="L69" s="1"/>
@@ -4340,22 +4321,20 @@
         <v>32</v>
       </c>
     </row>
-    <row r="70" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A70" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="C70" s="6" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="D70" s="7" t="s">
-        <v>195</v>
-      </c>
-      <c r="E70" s="1" t="s">
-        <v>35</v>
-      </c>
+        <v>198</v>
+      </c>
+      <c r="E70" s="1"/>
       <c r="G70" s="1"/>
       <c r="H70" s="1"/>
       <c r="K70" s="1"/>
@@ -4364,27 +4343,24 @@
       <c r="P70" s="1"/>
       <c r="S70" s="1"/>
       <c r="T70" s="1"/>
-      <c r="V70" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="W70" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="71" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="V70" s="1"/>
+    </row>
+    <row r="71" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A71" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B71" s="6" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="C71" s="6" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="D71" s="7" t="s">
-        <v>197</v>
-      </c>
-      <c r="E71" s="1"/>
+        <v>200</v>
+      </c>
+      <c r="E71" s="1" t="s">
+        <v>35</v>
+      </c>
       <c r="G71" s="1"/>
       <c r="H71" s="1"/>
       <c r="K71" s="1"/>
@@ -4393,25 +4369,35 @@
       <c r="P71" s="1"/>
       <c r="S71" s="1"/>
       <c r="T71" s="1"/>
-      <c r="V71" s="1"/>
+      <c r="V71" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="W71" s="1" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="72" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A72" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="C72" s="6" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="D72" s="7" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="G72" s="1"/>
+        <v>55</v>
+      </c>
+      <c r="F72" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="G72" s="1" t="s">
+        <v>55</v>
+      </c>
       <c r="H72" s="1"/>
       <c r="K72" s="1"/>
       <c r="L72" s="1"/>
@@ -4426,20 +4412,22 @@
         <v>32</v>
       </c>
     </row>
-    <row r="73" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A73" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B73" s="6" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="C73" s="6" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="D73" s="7" t="s">
-        <v>201</v>
-      </c>
-      <c r="E73" s="1"/>
+        <v>205</v>
+      </c>
+      <c r="E73" s="1" t="s">
+        <v>55</v>
+      </c>
       <c r="G73" s="1"/>
       <c r="H73" s="1"/>
       <c r="K73" s="1"/>
@@ -4448,24 +4436,27 @@
       <c r="P73" s="1"/>
       <c r="S73" s="1"/>
       <c r="T73" s="1"/>
-      <c r="V73" s="1"/>
-    </row>
-    <row r="74" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="V73" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="W73" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="74" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A74" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B74" s="6" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="C74" s="6" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="D74" s="7" t="s">
-        <v>203</v>
-      </c>
-      <c r="E74" s="1" t="s">
-        <v>35</v>
-      </c>
+        <v>207</v>
+      </c>
+      <c r="E74" s="1"/>
       <c r="G74" s="1"/>
       <c r="H74" s="1"/>
       <c r="K74" s="1"/>
@@ -4474,35 +4465,25 @@
       <c r="P74" s="1"/>
       <c r="S74" s="1"/>
       <c r="T74" s="1"/>
-      <c r="V74" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="W74" s="1" t="s">
-        <v>32</v>
-      </c>
+      <c r="V74" s="1"/>
     </row>
     <row r="75" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A75" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B75" s="6" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="C75" s="6" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="D75" s="7" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="E75" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="F75" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="G75" s="1" t="s">
-        <v>55</v>
-      </c>
+      <c r="G75" s="1"/>
       <c r="H75" s="1"/>
       <c r="K75" s="1"/>
       <c r="L75" s="1"/>
@@ -4517,22 +4498,20 @@
         <v>32</v>
       </c>
     </row>
-    <row r="76" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A76" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B76" s="6" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="C76" s="6" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="D76" s="7" t="s">
-        <v>208</v>
-      </c>
-      <c r="E76" s="1" t="s">
-        <v>55</v>
-      </c>
+        <v>211</v>
+      </c>
+      <c r="E76" s="1"/>
       <c r="G76" s="1"/>
       <c r="H76" s="1"/>
       <c r="K76" s="1"/>
@@ -4541,27 +4520,24 @@
       <c r="P76" s="1"/>
       <c r="S76" s="1"/>
       <c r="T76" s="1"/>
-      <c r="V76" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="W76" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="77" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="V76" s="1"/>
+    </row>
+    <row r="77" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A77" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B77" s="6" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="C77" s="6" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="D77" s="7" t="s">
-        <v>210</v>
-      </c>
-      <c r="E77" s="1"/>
+        <v>213</v>
+      </c>
+      <c r="E77" s="1" t="s">
+        <v>55</v>
+      </c>
       <c r="G77" s="1"/>
       <c r="H77" s="1"/>
       <c r="K77" s="1"/>
@@ -4570,25 +4546,35 @@
       <c r="P77" s="1"/>
       <c r="S77" s="1"/>
       <c r="T77" s="1"/>
-      <c r="V77" s="1"/>
+      <c r="V77" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="W77" s="1" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="78" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A78" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B78" s="6" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="C78" s="6" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="D78" s="7" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="E78" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F78" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="G78" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="G78" s="1"/>
       <c r="H78" s="1"/>
       <c r="K78" s="1"/>
       <c r="L78" s="1"/>
@@ -4603,21 +4589,28 @@
         <v>32</v>
       </c>
     </row>
-    <row r="79" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A79" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B79" s="6" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="C79" s="6" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="D79" s="7" t="s">
-        <v>214</v>
-      </c>
-      <c r="E79" s="1"/>
-      <c r="G79" s="1"/>
+        <v>218</v>
+      </c>
+      <c r="E79" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F79" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="G79" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="H79" s="1"/>
       <c r="K79" s="1"/>
       <c r="L79" s="1"/>
@@ -4625,61 +4618,57 @@
       <c r="P79" s="1"/>
       <c r="S79" s="1"/>
       <c r="T79" s="1"/>
-      <c r="V79" s="1"/>
+      <c r="V79" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="W79" s="1" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="80" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A80" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B80" s="6" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="C80" s="6" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="D80" s="7" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="E80" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="G80" s="1"/>
+        <v>51</v>
+      </c>
+      <c r="F80" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="G80" s="1" t="s">
+        <v>51</v>
+      </c>
       <c r="H80" s="1"/>
-      <c r="K80" s="1"/>
+      <c r="J80" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="K80" s="1" t="s">
+        <v>51</v>
+      </c>
       <c r="L80" s="1"/>
       <c r="O80" s="1"/>
       <c r="P80" s="1"/>
       <c r="S80" s="1"/>
       <c r="T80" s="1"/>
       <c r="V80" s="1" t="s">
-        <v>32</v>
+        <v>135</v>
       </c>
       <c r="W80" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="81" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A81" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="B81" s="6" t="s">
-        <v>178</v>
-      </c>
-      <c r="C81" s="6" t="s">
-        <v>217</v>
-      </c>
-      <c r="D81" s="7" t="s">
-        <v>218</v>
-      </c>
-      <c r="E81" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="F81" s="1" t="s">
-        <v>219</v>
-      </c>
-      <c r="G81" s="1" t="s">
-        <v>55</v>
-      </c>
+    <row r="81" spans="5:22" x14ac:dyDescent="0.25">
+      <c r="E81" s="1"/>
+      <c r="G81" s="1"/>
       <c r="H81" s="1"/>
       <c r="K81" s="1"/>
       <c r="L81" s="1"/>
@@ -4687,35 +4676,11 @@
       <c r="P81" s="1"/>
       <c r="S81" s="1"/>
       <c r="T81" s="1"/>
-      <c r="V81" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="W81" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="82" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A82" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="B82" s="6" t="s">
-        <v>178</v>
-      </c>
-      <c r="C82" s="6" t="s">
-        <v>220</v>
-      </c>
-      <c r="D82" s="7" t="s">
-        <v>221</v>
-      </c>
-      <c r="E82" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="F82" s="1" t="s">
-        <v>219</v>
-      </c>
-      <c r="G82" s="1" t="s">
-        <v>29</v>
-      </c>
+      <c r="V81" s="1"/>
+    </row>
+    <row r="82" spans="5:22" x14ac:dyDescent="0.25">
+      <c r="E82" s="1"/>
+      <c r="G82" s="1"/>
       <c r="H82" s="1"/>
       <c r="K82" s="1"/>
       <c r="L82" s="1"/>
@@ -4723,53 +4688,19 @@
       <c r="P82" s="1"/>
       <c r="S82" s="1"/>
       <c r="T82" s="1"/>
-      <c r="V82" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="W82" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="83" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A83" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="B83" s="6" t="s">
-        <v>178</v>
-      </c>
-      <c r="C83" s="6" t="s">
-        <v>222</v>
-      </c>
-      <c r="D83" s="7" t="s">
-        <v>223</v>
-      </c>
-      <c r="E83" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="F83" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="G83" s="1" t="s">
-        <v>51</v>
-      </c>
+      <c r="V82" s="1"/>
+    </row>
+    <row r="83" spans="5:22" x14ac:dyDescent="0.25">
+      <c r="E83" s="1"/>
+      <c r="G83" s="1"/>
       <c r="H83" s="1"/>
-      <c r="J83" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="K83" s="1" t="s">
-        <v>51</v>
-      </c>
+      <c r="K83" s="1"/>
       <c r="L83" s="1"/>
       <c r="O83" s="1"/>
       <c r="P83" s="1"/>
       <c r="S83" s="1"/>
       <c r="T83" s="1"/>
-      <c r="V83" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="W83" s="1" t="s">
-        <v>32</v>
-      </c>
+      <c r="V83" s="1"/>
     </row>
     <row r="84" spans="5:22" x14ac:dyDescent="0.25">
       <c r="E84" s="1"/>
@@ -8335,45 +8266,9 @@
       <c r="T380" s="1"/>
       <c r="V380" s="1"/>
     </row>
-    <row r="381" spans="5:22" x14ac:dyDescent="0.25">
-      <c r="E381" s="1"/>
-      <c r="G381" s="1"/>
-      <c r="H381" s="1"/>
-      <c r="K381" s="1"/>
-      <c r="L381" s="1"/>
-      <c r="O381" s="1"/>
-      <c r="P381" s="1"/>
-      <c r="S381" s="1"/>
-      <c r="T381" s="1"/>
-      <c r="V381" s="1"/>
-    </row>
-    <row r="382" spans="5:22" x14ac:dyDescent="0.25">
-      <c r="E382" s="1"/>
-      <c r="G382" s="1"/>
-      <c r="H382" s="1"/>
-      <c r="K382" s="1"/>
-      <c r="L382" s="1"/>
-      <c r="O382" s="1"/>
-      <c r="P382" s="1"/>
-      <c r="S382" s="1"/>
-      <c r="T382" s="1"/>
-      <c r="V382" s="1"/>
-    </row>
-    <row r="383" spans="5:22" x14ac:dyDescent="0.25">
-      <c r="E383" s="1"/>
-      <c r="G383" s="1"/>
-      <c r="H383" s="1"/>
-      <c r="K383" s="1"/>
-      <c r="L383" s="1"/>
-      <c r="O383" s="1"/>
-      <c r="P383" s="1"/>
-      <c r="S383" s="1"/>
-      <c r="T383" s="1"/>
-      <c r="V383" s="1"/>
-    </row>
   </sheetData>
   <autoFilter ref="A1:W1"/>
-  <conditionalFormatting sqref="E2:E383">
+  <conditionalFormatting sqref="E2:E380">
     <cfRule type="containsText" dxfId="0" priority="1">
       <formula>NOT(ISERROR(SEARCH("BOT",E2)))</formula>
     </cfRule>
@@ -8393,7 +8288,7 @@
       <formula>NOT(ISERROR(SEARCH("NEUTRO",E2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G383">
+  <conditionalFormatting sqref="G2:G380">
     <cfRule type="containsText" dxfId="6" priority="1">
       <formula>NOT(ISERROR(SEARCH("BOT",G2)))</formula>
     </cfRule>
@@ -8413,7 +8308,7 @@
       <formula>NOT(ISERROR(SEARCH("NEUTRO",G2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K2:K383">
+  <conditionalFormatting sqref="K2:K380">
     <cfRule type="containsText" dxfId="12" priority="1">
       <formula>NOT(ISERROR(SEARCH("BOT",K2)))</formula>
     </cfRule>
@@ -8433,7 +8328,7 @@
       <formula>NOT(ISERROR(SEARCH("NEUTRO",K2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O2:O383">
+  <conditionalFormatting sqref="O2:O380">
     <cfRule type="containsText" dxfId="18" priority="1">
       <formula>NOT(ISERROR(SEARCH("BOT",O2)))</formula>
     </cfRule>
@@ -8453,7 +8348,7 @@
       <formula>NOT(ISERROR(SEARCH("NEUTRO",O2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S2:S383">
+  <conditionalFormatting sqref="S2:S380">
     <cfRule type="containsText" dxfId="24" priority="1">
       <formula>NOT(ISERROR(SEARCH("BOT",S2)))</formula>
     </cfRule>
@@ -8474,64 +8369,64 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="20">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca do Móvel" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca do Móvel" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="E10:E383">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca do Móvel" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca do Móvel" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="E10:E380">
       <formula1>"BOT,EUD,QDB,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca do Móvel" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca do Móvel" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="E2:E383">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca do Móvel" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca do Móvel" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="E2:E380">
       <formula1>"BOT,EUD,QDB,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 1" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 1" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="G10:G383">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 1" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 1" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="G10:G380">
       <formula1>"BOT,EUD,QDB,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 1" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 1" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="G2:G383">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 1" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 1" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="G2:G380">
       <formula1>"BOT,EUD,QDB,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo Etiqueta 1" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo Etiqueta 1" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." sqref="H10:H383">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo Etiqueta 1" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo Etiqueta 1" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." sqref="H10:H380">
       <formula1>"FIXO,EXPOSICAO,NOVO,ANTECIPADO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo Etiqueta 1" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo Etiqueta 1" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." sqref="H2:H383">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo Etiqueta 1" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo Etiqueta 1" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." sqref="H2:H380">
       <formula1>"FIXO,EXPOSICAO,NOVO,ANTECIPADO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 2" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 2" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="K10:K383">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 2" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 2" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="K10:K380">
       <formula1>"BOT,EUD,QDB,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 2" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 2" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="K2:K383">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 2" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 2" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="K2:K380">
       <formula1>"BOT,EUD,QDB,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo Etiqueta 2" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo Etiqueta 2" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." sqref="L10:L383">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo Etiqueta 2" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo Etiqueta 2" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." sqref="L10:L380">
       <formula1>"FIXO,EXPOSICAO,NOVO,ANTECIPADO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo Etiqueta 2" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo Etiqueta 2" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." sqref="L2:L383">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo Etiqueta 2" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo Etiqueta 2" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." sqref="L2:L380">
       <formula1>"FIXO,EXPOSICAO,NOVO,ANTECIPADO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 3" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 3" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="O10:O383">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 3" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 3" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="O10:O380">
       <formula1>"BOT,EUD,QDB,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 3" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 3" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="O2:O383">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 3" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 3" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="O2:O380">
       <formula1>"BOT,EUD,QDB,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo Etiqueta 3" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo Etiqueta 3" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." sqref="P10:P383">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo Etiqueta 3" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo Etiqueta 3" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." sqref="P10:P380">
       <formula1>"FIXO,EXPOSICAO,NOVO,ANTECIPADO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo Etiqueta 3" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo Etiqueta 3" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." sqref="P2:P383">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo Etiqueta 3" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo Etiqueta 3" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." sqref="P2:P380">
       <formula1>"FIXO,EXPOSICAO,NOVO,ANTECIPADO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 4" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 4" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="S10:S383">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 4" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 4" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="S10:S380">
       <formula1>"BOT,EUD,QDB,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 4" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 4" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="S2:S383">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Marca Etiqueta 4" prompt="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." showErrorMessage="1" errorStyle="warning" errorTitle="Marca Etiqueta 4" error="Use BOT, EUD, QDB, OUI, MULTI, NEUTRO. Combinações com &quot;+&quot; (ex.: BOT+QDB) geram degradê; também aceita cor #RRGGBB." sqref="S2:S380">
       <formula1>"BOT,EUD,QDB,OUI,MULTI,NEUTRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo Etiqueta 4" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo Etiqueta 4" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." sqref="T10:T383">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo Etiqueta 4" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo Etiqueta 4" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." sqref="T10:T380">
       <formula1>"FIXO,EXPOSICAO,NOVO,ANTECIPADO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo Etiqueta 4" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo Etiqueta 4" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." sqref="T2:T383">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo Etiqueta 4" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo Etiqueta 4" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade; ANTECIPADO = Antecipação (item adiantado do próximo ciclo). Com ANTECIPADO, a data vai na coluna ao lado (dd/mm/aaaa)." sqref="T2:T380">
       <formula1>"FIXO,EXPOSICAO,NOVO,ANTECIPADO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" sqref="V10:V383">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" sqref="V10:V380">
       <formula1>"FIXO,EXPOSICAO,NOVO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" sqref="V2:V383">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Símbolo" prompt="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" showErrorMessage="1" errorStyle="warning" errorTitle="Símbolo" error="FIXO = Espaço fixo (sem mudança nos ciclos); EXPOSICAO = Exposição, sem comunicação; NOVO = Novidade" sqref="V2:V380">
       <formula1>"FIXO,EXPOSICAO,NOVO"</formula1>
     </dataValidation>
   </dataValidations>
@@ -8559,16 +8454,16 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>224</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>227</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -8576,13 +8471,13 @@
         <v>23</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>31</v>
@@ -8596,10 +8491,10 @@
         <v>23</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>228</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>231</v>
       </c>
       <c r="D3" s="8" t="s">
         <v>59</v>
@@ -8616,13 +8511,13 @@
         <v>23</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>231</v>
-      </c>
       <c r="D4" s="8" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>55</v>
@@ -8636,10 +8531,10 @@
         <v>23</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="D5" s="8" t="s">
         <v>68</v>
@@ -8656,10 +8551,10 @@
         <v>23</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="D6" s="8" t="s">
         <v>74</v>
@@ -8676,13 +8571,13 @@
         <v>23</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>55</v>
@@ -8696,13 +8591,13 @@
         <v>23</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>51</v>
@@ -8716,13 +8611,13 @@
         <v>23</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="C9" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="D9" s="8" t="s">
         <v>233</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>236</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>31</v>
@@ -8736,19 +8631,19 @@
         <v>23</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>31</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -8756,13 +8651,13 @@
         <v>23</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="C11" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="D11" s="8" t="s">
         <v>237</v>
-      </c>
-      <c r="D11" s="8" t="s">
-        <v>240</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>29</v>
@@ -8776,13 +8671,13 @@
         <v>23</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>55</v>
@@ -8799,10 +8694,10 @@
         <v>24</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>32</v>
@@ -8819,10 +8714,10 @@
         <v>24</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>32</v>
@@ -8839,10 +8734,10 @@
         <v>112</v>
       </c>
       <c r="C15" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="D15" s="8" t="s">
         <v>242</v>
-      </c>
-      <c r="D15" s="8" t="s">
-        <v>245</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>32</v>
@@ -8859,10 +8754,10 @@
         <v>112</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>32</v>
@@ -8879,10 +8774,10 @@
         <v>141</v>
       </c>
       <c r="C17" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="D17" s="8" t="s">
         <v>242</v>
-      </c>
-      <c r="D17" s="8" t="s">
-        <v>245</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>32</v>
@@ -8899,10 +8794,10 @@
         <v>141</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>32</v>
@@ -8916,13 +8811,13 @@
         <v>23</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="C19" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="D19" s="8" t="s">
         <v>242</v>
-      </c>
-      <c r="D19" s="8" t="s">
-        <v>245</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>32</v>
@@ -8936,13 +8831,13 @@
         <v>23</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>32</v>
@@ -8956,13 +8851,13 @@
         <v>23</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>32</v>
@@ -10228,13 +10123,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>22</v>
@@ -10245,10 +10140,10 @@
         <v>23</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="D2" s="9">
         <v>150000</v>
@@ -10265,7 +10160,7 @@
         <v>114</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D3" s="9">
         <v>1200000</v>
@@ -10282,7 +10177,7 @@
         <v>40</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D4" s="9">
         <v>650000</v>
@@ -10299,7 +10194,7 @@
         <v>59</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D5" s="9">
         <v>2400000</v>
@@ -10316,7 +10211,7 @@
         <v>91</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D6" s="9">
         <v>430000</v>
@@ -10333,7 +10228,7 @@
         <v>124</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D7" s="9">
         <v>610000</v>
@@ -10362,7 +10257,7 @@
         <v>23</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>32</v>
@@ -10377,7 +10272,7 @@
         <v>23</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>32</v>
@@ -10407,10 +10302,10 @@
         <v>23</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="D12" s="9">
         <v>380000</v>
@@ -10427,7 +10322,7 @@
         <v>37</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="D13" s="9">
         <v>620000</v>
@@ -10444,7 +10339,7 @@
         <v>74</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="D14" s="9">
         <v>1800000</v>
@@ -10461,7 +10356,7 @@
         <v>68</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="D15" s="9">
         <v>950000</v>
@@ -10478,7 +10373,7 @@
         <v>92</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="D16" s="9">
         <v>210000</v>
@@ -10495,7 +10390,7 @@
         <v>36</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="D17" s="9">
         <v>900000</v>
@@ -10512,7 +10407,7 @@
         <v>52</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="D18" s="9">
         <v>260000</v>
@@ -10529,7 +10424,7 @@
         <v>30</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D19" s="9">
         <v>1500000</v>
@@ -10546,7 +10441,7 @@
         <v>80</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="D20" s="9">
         <v>1100000</v>
@@ -10593,7 +10488,7 @@
         <v>119</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D23" s="9">
         <v>870000</v>
@@ -10610,7 +10505,7 @@
         <v>58</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D24" s="9">
         <v>700000</v>
@@ -10627,7 +10522,7 @@
         <v>65</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="D25" s="9">
         <v>480000</v>
@@ -10644,7 +10539,7 @@
         <v>71</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="D26" s="9">
         <v>780000</v>
@@ -10661,7 +10556,7 @@
         <v>62</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="D27" s="9">
         <v>540000</v>
@@ -10678,7 +10573,7 @@
         <v>46</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D28" s="9">
         <v>520000</v>
@@ -10692,7 +10587,7 @@
         <v>23</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>32</v>
@@ -11947,122 +11842,122 @@
   <sheetData>
     <row r="1" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B1" s="11" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B2" s="12" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12"/>
     </row>
     <row r="4" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B4" s="13" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B5" s="12" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="C5" s="12"/>
       <c r="D5" s="12"/>
     </row>
     <row r="6" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B6" s="12" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="C6" s="12"/>
       <c r="D6" s="12"/>
     </row>
     <row r="7" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B7" s="12" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="12"/>
     </row>
     <row r="8" ht="45" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B8" s="12" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="C8" s="12"/>
       <c r="D8" s="12"/>
     </row>
     <row r="9" ht="16" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B9" s="12" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="C9" s="12"/>
       <c r="D9" s="12"/>
     </row>
     <row r="10" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B10" s="12" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="C10" s="12"/>
       <c r="D10" s="12"/>
     </row>
     <row r="11" ht="60" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B11" s="12" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="C11" s="12"/>
       <c r="D11" s="12"/>
     </row>
     <row r="12" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B12" s="12" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="C12" s="12"/>
       <c r="D12" s="12"/>
     </row>
     <row r="13" ht="60" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B13" s="12" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="C13" s="12"/>
       <c r="D13" s="12"/>
     </row>
     <row r="14" ht="60" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B14" s="12" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="C14" s="12"/>
       <c r="D14" s="12"/>
     </row>
     <row r="15" ht="30" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B15" s="12" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="C15" s="12"/>
       <c r="D15" s="12"/>
     </row>
-    <row r="16" ht="105" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="16" ht="120" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B16" s="12" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="C16" s="12"/>
       <c r="D16" s="12"/>
     </row>
     <row r="17" ht="45" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B17" s="12" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="C17" s="12"/>
       <c r="D17" s="12"/>
     </row>
     <row r="18" ht="45" customHeight="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B18" s="12" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="C18" s="12"/>
       <c r="D18" s="12"/>
     </row>
     <row r="20" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B20" s="13" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.25">
@@ -12073,7 +11968,7 @@
         <v>29</v>
       </c>
       <c r="D21" s="15" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
     </row>
     <row r="22" spans="2:4" x14ac:dyDescent="0.25">
@@ -12084,7 +11979,7 @@
         <v>55</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
     </row>
     <row r="23" spans="2:4" x14ac:dyDescent="0.25">
@@ -12095,7 +11990,7 @@
         <v>35</v>
       </c>
       <c r="D23" s="17" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
     </row>
     <row r="24" spans="2:4" x14ac:dyDescent="0.25">
@@ -12106,7 +12001,7 @@
         <v>51</v>
       </c>
       <c r="D24" s="18" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.25">
@@ -12114,10 +12009,10 @@
         <v>31</v>
       </c>
       <c r="C25" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="D25" s="19" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
     </row>
     <row r="26" spans="2:4" x14ac:dyDescent="0.25">
@@ -12125,15 +12020,15 @@
         <v>27</v>
       </c>
       <c r="C26" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="D26" s="20" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
     </row>
     <row r="28" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B28" s="13" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
     </row>
     <row r="29" spans="2:4" x14ac:dyDescent="0.25">
@@ -12141,10 +12036,10 @@
         <v>41</v>
       </c>
       <c r="C29" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="D29" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
     </row>
     <row r="30" spans="2:4" x14ac:dyDescent="0.25">
@@ -12152,100 +12047,100 @@
         <v>135</v>
       </c>
       <c r="C30" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="D30" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
     </row>
     <row r="31" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B31" s="14" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="C31" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="D31" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
     </row>
     <row r="33" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B33" s="13" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
     </row>
     <row r="34" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B34" s="21" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
     </row>
     <row r="35" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B35" s="22" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
     </row>
     <row r="36" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B36" s="23" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
     </row>
     <row r="37" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B37" s="24" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
     </row>
     <row r="38" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B38" s="25" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
     </row>
     <row r="40" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B40" s="13" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
     </row>
     <row r="41" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B41" s="14" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="C41" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="D41"/>
     </row>
     <row r="42" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B42" s="14" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="C42" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="D42"/>
     </row>
     <row r="43" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B43" s="14" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="C43" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="D43"/>
     </row>
     <row r="44" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B44" s="14" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="C44" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="D44"/>
     </row>
     <row r="45" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B45" s="14" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="C45" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="D45"/>
     </row>

</xml_diff>